<commit_message>
feat(F-NAR-009): ramifiées AUT-001, 002, 013
Monde d’abord, 86 passages, plus de « On va apprendre ».
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-AUT-001.xlsx
+++ b/stories/arbres/TREE-AUT-001.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -552,7 +552,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Préparer son sac — dans la chambre</t>
+          <t>Le sac d'Amir sur le tapis rayé</t>
         </is>
       </c>
     </row>
@@ -843,6 +843,18 @@
       <c r="B30" t="inlineStr">
         <is>
           <t>voix-roles-v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fil_rouge</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Amir prépare son sac sur le tapis rayé. Papa et maman disent ce qu'il met. Ensuite il joue.</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1197,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Lina est dans la chambre, avec maman. Papa plie un pull. Lina prépare son sac. Maman parle, tout doux. On met dans le sac ce que l'adulte a dit.</t>
+          <t>Sur le toit, la gouttière fait plic ploc. La maison a un volet jaune. Le volet claque tout doux. Dans le village, les pavés brillent. Ils sont encore mouillés. Une odeur de soupe entre par la fenêtre. Le tapis de la chambre est rayé. Il est bleu et crème. Un rayon de soleil touche le plancher. Papa plie un pull marine. Le pull est encore un peu chaud. Le pull est prêt, Amir. Il est tout doux. Maman ouvre un peu la fenêtre. Tu as senti la soupe ? Oui, maman. Le sac d'Amir attend sur le tapis. Le sac est vide. La fermeture brille. Je veux jouer ! D'accord. On prépare le sac d'abord. On met dans le sac ce que maman a dit. Ou ce que papa a dit. Amir pose la main sur le sac. En ce moment, il a trop envie de jouer.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1325,7 +1337,32 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Lina est dans la chambre, avec maman. Papa plie un pull. Lina prépare son sac. Maman parle, tout doux. On met dans le sac ce que l'adulte a dit.</t>
+          <t>narrateur|Sur le toit, la gouttière fait plic ploc.
+narrateur|La maison a un volet jaune.
+narrateur|Le volet claque tout doux.
+narrateur|Dans le village, les pavés brillent.
+narrateur|Ils sont encore mouillés.
+narrateur|Une odeur de soupe entre par la fenêtre.
+narrateur|Le tapis de la chambre est rayé.
+narrateur|Il est bleu et crème.
+narrateur|Un rayon de soleil touche le plancher.
+narrateur|Papa plie un pull marine.
+narrateur|Le pull est encore un peu chaud.
+papa|Le pull est prêt, Amir.
+papa|Il est tout doux.
+narrateur|Maman ouvre un peu la fenêtre.
+maman|Tu as senti la soupe ?
+enfant-m|Oui, maman.
+narrateur|Le sac d'Amir attend sur le tapis.
+narrateur|Le sac est vide.
+narrateur|La fermeture brille.
+enfant-m|Je veux jouer !
+maman|D'accord.
+maman|On prépare le sac d'abord.
+papa|On met dans le sac ce que maman a dit.
+papa|Ou ce que papa a dit.
+narrateur|Amir pose la main sur le sac.
+narrateur|En ce moment, il a trop envie de jouer.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr"/>
@@ -1353,7 +1390,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre une pomme, un yaourt, ou un morceau de pain.</t>
+          <t>On peut mettre une pomme, un yaourt, ou un morceau de pain.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1521,7 +1558,7 @@
       <c r="AV3" s="2" t="inlineStr"/>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre une pomme, un yaourt, ou un morceau de pain.</t>
+          <t>narrateur|On peut mettre une pomme, un yaourt, ou un morceau de pain.</t>
         </is>
       </c>
       <c r="AX3" t="inlineStr"/>
@@ -1549,7 +1586,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Lina met une pomme dans le sac. Maman La pomme. On met dans le sac ce que l'adulte a dit. Lina appuie un peu. Ça sent le fruit. C'est ça.</t>
+          <t>Dans la coupe, une pomme rouge brille. Elle sent le fruit. La peau est lisse et froide. La pomme dans le sac, Amir. La pomme. Amir la prend à deux mains. Il la glisse dans le sac. Le fond du sac fait un petit bruit. Bravo. Tu as mis ce que maman a dit. Tu as fini de mettre la pomme ? Oui. Amir appuie un peu. Ça sent encore le fruit.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1689,10 +1726,20 @@
       <c r="AV4" s="2" t="inlineStr"/>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Lina met une pomme dans le sac. Maman
-enfant-f|La pomme. On met dans le sac ce que l'adulte a dit.
-narrateur|Lina appuie un peu. Ça sent le fruit.
-papa|C'est ça.</t>
+          <t>narrateur|Dans la coupe, une pomme rouge brille.
+narrateur|Elle sent le fruit.
+narrateur|La peau est lisse et froide.
+maman|La pomme dans le sac, Amir.
+enfant-m|La pomme.
+narrateur|Amir la prend à deux mains.
+narrateur|Il la glisse dans le sac.
+narrateur|Le fond du sac fait un petit bruit.
+papa|Bravo.
+papa|Tu as mis ce que maman a dit.
+maman|Tu as fini de mettre la pomme ?
+enfant-m|Oui.
+narrateur|Amir appuie un peu.
+narrateur|Ça sent encore le fruit.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr"/>
@@ -1908,7 +1955,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Oui. On met dans le sac ce que l'adulte a dit. Lina respire. Maman est là. On met dans le sac ce que l'adulte a dit.</t>
+          <t>Oui. On met dans le sac ce que maman a dit. Amir regarde la pomme dans le sac. Bravo, Amir. Tu as écouté. C'est du bon travail. Le sac a ce que l'adulte a dit. La pomme est dedans. On continue ensemble ? Oui.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -2052,7 +2099,16 @@
       </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Oui. On met dans le sac ce que l'adulte a dit. Lina respire. Maman est là. On met dans le sac ce que l'adulte a dit.</t>
+          <t>narrateur|Oui.
+narrateur|On met dans le sac ce que maman a dit.
+narrateur|Amir regarde la pomme dans le sac.
+maman|Bravo, Amir.
+maman|Tu as écouté.
+papa|C'est du bon travail.
+papa|Le sac a ce que l'adulte a dit.
+enfant-m|La pomme est dedans.
+maman|On continue ensemble ?
+enfant-m|Oui.</t>
         </is>
       </c>
       <c r="AX6" t="inlineStr"/>
@@ -2080,7 +2136,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre la cuisine, le jardin, ou la chambre.</t>
+          <t>On peut aller dans la cuisine, le jardin, ou la chambre.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -2244,7 +2300,7 @@
       <c r="AV7" s="2" t="inlineStr"/>
       <c r="AW7" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre la cuisine, le jardin, ou la chambre.</t>
+          <t>narrateur|On peut aller dans la cuisine, le jardin, ou la chambre.</t>
         </is>
       </c>
       <c r="AX7" t="inlineStr"/>
@@ -2272,7 +2328,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Ensuite Lina va dans la cuisine. Elle met les cubes près du sac. On met dans le sac ce que l'adulte a dit. Les cubes, oui. Maman montre le geste, lentement. On met dans le sac ce que l'adulte a dit.</t>
+          <t>Amir emporte le sac vers la cuisine. Le carrelage est un peu froid. La soupe fume encore dans la casserole. La petite serviette, Amir. On la met dans le sac. La serviette. Elle est douce et pliée. Amir la glisse près de la pomme. Bravo. Tu as mis ce que maman a dit. Une miette reste sur la table. On la ramasse après le jeu.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -2412,8 +2468,18 @@
       <c r="AV8" s="2" t="inlineStr"/>
       <c r="AW8" t="inlineStr">
         <is>
-          <t>narrateur|Ensuite Lina va dans la cuisine. Elle met les cubes près du sac. On met dans le sac ce que l'adulte a dit.
-maman|Les cubes, oui. Maman montre le geste, lentement. On met dans le sac ce que l'adulte a dit.</t>
+          <t>narrateur|Amir emporte le sac vers la cuisine.
+narrateur|Le carrelage est un peu froid.
+narrateur|La soupe fume encore dans la casserole.
+maman|La petite serviette, Amir.
+maman|On la met dans le sac.
+enfant-m|La serviette.
+narrateur|Elle est douce et pliée.
+narrateur|Amir la glisse près de la pomme.
+papa|Bravo.
+papa|Tu as mis ce que maman a dit.
+narrateur|Une miette reste sur la table.
+maman|On la ramasse après le jeu.</t>
         </is>
       </c>
       <c r="AX8" t="inlineStr"/>
@@ -2633,7 +2699,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Lina a choisi une pomme. Puis la cuisine. Puis les cubes. Un vélo passe au loin. Lina prend la main de maman. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>Les cubes bleus attendent près de l'assiette. Ils tapent un peu sur le bois. Deux cubes dans le sac, Amir. Deux cubes. Amir les empile, puis les glisse près de la pomme. Bravo. Tu as mis ce que maman a dit. La soupe fume encore, tout doux. On jouera aux cubes plus tard. D'accord.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -2773,7 +2839,16 @@
       <c r="AV10" s="2" t="inlineStr"/>
       <c r="AW10" t="inlineStr">
         <is>
-          <t>narrateur|Lina a choisi une pomme. Puis la cuisine. Puis les cubes. Un vélo passe au loin. Lina prend la main de maman. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|Les cubes bleus attendent près de l'assiette.
+narrateur|Ils tapent un peu sur le bois.
+maman|Deux cubes dans le sac, Amir.
+enfant-m|Deux cubes.
+narrateur|Amir les empile, puis les glisse près de la pomme.
+papa|Bravo.
+papa|Tu as mis ce que maman a dit.
+narrateur|La soupe fume encore, tout doux.
+maman|On jouera aux cubes plus tard.
+enfant-m|D'accord.</t>
         </is>
       </c>
       <c r="AX10" t="inlineStr"/>
@@ -2801,7 +2876,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Amir ferme le sac. Ça fait zzz. Le sac est prêt. Bravo, Amir. Tu as fait du bon travail. Merci. La cuisine sent encore la soupe. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -2941,7 +3016,14 @@
       <c r="AV11" s="2" t="inlineStr"/>
       <c r="AW11" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir ferme le sac.
+narrateur|Ça fait zzz.
+papa|Le sac est prêt.
+maman|Bravo, Amir.
+maman|Tu as fait du bon travail.
+enfant-m|Merci.
+narrateur|La cuisine sent encore la soupe.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX11" t="inlineStr"/>
@@ -2969,7 +3051,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Lina s'arrête près de le livre. la cuisine est rangé. On entend un oiseau. Papa n'est pas loin. Lina les rejoint. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>Un petit livre est posé près du sel. Les pages sentent le papier. Le livre dans le sac, Amir. Le livre. Amir le glisse à plat, près de la pomme. Bravo. Tu as mis ce que papa a dit. Une farine légère reste sur la table. On essuie après. Le livre est dedans.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -3109,7 +3191,16 @@
       <c r="AV12" s="2" t="inlineStr"/>
       <c r="AW12" t="inlineStr">
         <is>
-          <t>narrateur|Lina s'arrête près de le livre. la cuisine est rangé. On entend un oiseau. Papa n'est pas loin. Lina les rejoint. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|Un petit livre est posé près du sel.
+narrateur|Les pages sentent le papier.
+papa|Le livre dans le sac, Amir.
+enfant-m|Le livre.
+narrateur|Amir le glisse à plat, près de la pomme.
+maman|Bravo.
+maman|Tu as mis ce que papa a dit.
+narrateur|Une farine légère reste sur la table.
+papa|On essuie après.
+enfant-m|Le livre est dedans.</t>
         </is>
       </c>
       <c r="AX12" t="inlineStr"/>
@@ -3137,7 +3228,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Amir appuie sur la fermeture. Tu as mis le livre. Et la pomme. C'est ce que l'adulte a dit. Le sac est prêt. Bravo. Ils restent un moment près de la table. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -3277,7 +3368,14 @@
       <c r="AV13" s="2" t="inlineStr"/>
       <c r="AW13" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir appuie sur la fermeture.
+maman|Tu as mis le livre.
+papa|Et la pomme.
+maman|C'est ce que l'adulte a dit.
+enfant-m|Le sac est prêt.
+papa|Bravo.
+narrateur|Ils restent un moment près de la table.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX13" t="inlineStr"/>
@@ -3305,7 +3403,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Lina se souvient de une pomme. Et de la cuisine. Et de la dînette. La couverture est douce. Lina enfile ses chaussons. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>La petite tasse de dînette cliquette. Elle est rouge, près de l'évier. La tasse dans le sac, Amir. La tasse. Amir la pose tout doux près de la pomme. Bravo. Tu as mis ce que maman a dit. Ça sonne comme un tout petit verre. On fera la dînette après le goûter. Oui, maman.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -3445,7 +3543,16 @@
       <c r="AV14" s="2" t="inlineStr"/>
       <c r="AW14" t="inlineStr">
         <is>
-          <t>narrateur|Lina se souvient de une pomme. Et de la cuisine. Et de la dînette. La couverture est douce. Lina enfile ses chaussons. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|La petite tasse de dînette cliquette.
+narrateur|Elle est rouge, près de l'évier.
+maman|La tasse dans le sac, Amir.
+enfant-m|La tasse.
+narrateur|Amir la pose tout doux près de la pomme.
+papa|Bravo.
+papa|Tu as mis ce que maman a dit.
+narrateur|Ça sonne comme un tout petit verre.
+maman|On fera la dînette après le goûter.
+enfant-m|Oui, maman.</t>
         </is>
       </c>
       <c r="AX14" t="inlineStr"/>
@@ -3473,7 +3580,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Le sac a la pomme et la tasse. Bravo, Amir. Tu as écouté. Merci, papa. Une goutte tombe dans l'évier. On va jouer. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -3613,7 +3720,13 @@
       <c r="AV15" s="2" t="inlineStr"/>
       <c r="AW15" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Le sac a la pomme et la tasse.
+maman|Bravo, Amir.
+papa|Tu as écouté.
+enfant-m|Merci, papa.
+narrateur|Une goutte tombe dans l'évier.
+maman|On va jouer.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX15" t="inlineStr"/>
@@ -3641,7 +3754,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Ensuite Lina va dans la cuisine. Elle met le livre près du sac. On met dans le sac ce que l'adulte a dit. Le livre, oui. Je suis là. On met dans le sac ce que l'adulte a dit.</t>
+          <t>Amir pousse la porte du jardin. L'herbe est encore mouillée. Une feuille colle à sa chaussette. Le petit linge, Amir. On le met dans le sac. Le linge. Le linge sent l'air frais. Amir le pose près de la pomme. Bravo. Tu as mis ce que papa a dit. Un oiseau chante sur le mur. Tu as entendu l'oiseau ? Oui, papa.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -3781,9 +3894,19 @@
       <c r="AV16" s="2" t="inlineStr"/>
       <c r="AW16" t="inlineStr">
         <is>
-          <t>narrateur|Ensuite Lina va dans la cuisine. Elle met le livre près du sac. On met dans le sac ce que l'adulte a dit.
-maman|Le livre, oui.
-maman|Je suis là. On met dans le sac ce que l'adulte a dit.</t>
+          <t>narrateur|Amir pousse la porte du jardin.
+narrateur|L'herbe est encore mouillée.
+narrateur|Une feuille colle à sa chaussette.
+papa|Le petit linge, Amir.
+papa|On le met dans le sac.
+enfant-m|Le linge.
+narrateur|Le linge sent l'air frais.
+narrateur|Amir le pose près de la pomme.
+maman|Bravo.
+maman|Tu as mis ce que papa a dit.
+narrateur|Un oiseau chante sur le mur.
+papa|Tu as entendu l'oiseau ?
+enfant-m|Oui, papa.</t>
         </is>
       </c>
       <c r="AX16" t="inlineStr"/>
@@ -4003,7 +4126,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Avec les cubes. Après le jardin. Près de une pomme. Lina s'arrête. Il y a des miettes sur la table. Lina tend les cubes à papa. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>Les cubes sont sur la pierre chaude. Ils sentent un peu le soleil. Un cube dans le sac, Amir. Un cube. Amir l'essuie sur son pantalon. Il le met près de la pomme. Bravo. Tu as mis ce que papa a dit. Une abeille passe, tout loin. On laisse l'abeille au jardin.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -4143,7 +4266,16 @@
       <c r="AV18" s="2" t="inlineStr"/>
       <c r="AW18" t="inlineStr">
         <is>
-          <t>narrateur|Avec les cubes. Après le jardin. Près de une pomme. Lina s'arrête. Il y a des miettes sur la table. Lina tend les cubes à papa. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|Les cubes sont sur la pierre chaude.
+narrateur|Ils sentent un peu le soleil.
+papa|Un cube dans le sac, Amir.
+enfant-m|Un cube.
+narrateur|Amir l'essuie sur son pantalon.
+narrateur|Il le met près de la pomme.
+maman|Bravo.
+maman|Tu as mis ce que papa a dit.
+narrateur|Une abeille passe, tout loin.
+papa|On laisse l'abeille au jardin.</t>
         </is>
       </c>
       <c r="AX18" t="inlineStr"/>
@@ -4171,7 +4303,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Amir referme le sac sur l'herbe. Bravo. Le sac a ce que l'adulte a dit. Merci. La feuille reste collée à la chaussette. On l'enlève à la maison. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -4311,7 +4443,13 @@
       <c r="AV19" s="2" t="inlineStr"/>
       <c r="AW19" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir referme le sac sur l'herbe.
+papa|Bravo.
+maman|Le sac a ce que l'adulte a dit.
+enfant-m|Merci.
+narrateur|La feuille reste collée à la chaussette.
+papa|On l'enlève à la maison.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX19" t="inlineStr"/>
@@ -4339,7 +4477,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Lina range le jardin. le livre reste près de une pomme. La lumière est claire. Lina s'assoit près de maman. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>Le livre est à l'ombre, sous le banc. L'herbe chatouille les chevilles. Le livre dans le sac, Amir. Le livre. Les pages sont un peu fraîches. Amir le glisse près de la pomme. Bravo. Tu as mis ce que maman a dit. On lira plus tard, au calme. D'accord.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -4479,7 +4617,16 @@
       <c r="AV20" s="2" t="inlineStr"/>
       <c r="AW20" t="inlineStr">
         <is>
-          <t>narrateur|Lina range le jardin. le livre reste près de une pomme. La lumière est claire. Lina s'assoit près de maman. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|Le livre est à l'ombre, sous le banc.
+narrateur|L'herbe chatouille les chevilles.
+maman|Le livre dans le sac, Amir.
+enfant-m|Le livre.
+narrateur|Les pages sont un peu fraîches.
+narrateur|Amir le glisse près de la pomme.
+papa|Bravo.
+papa|Tu as mis ce que maman a dit.
+maman|On lira plus tard, au calme.
+enfant-m|D'accord.</t>
         </is>
       </c>
       <c r="AX20" t="inlineStr"/>
@@ -4507,7 +4654,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Le sac est posé sur le banc. Bravo, Amir. Tu as fait du bon travail. Le livre est dedans. Un oiseau s'envole du mur. On rentre avec le sac. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -4647,7 +4794,13 @@
       <c r="AV21" s="2" t="inlineStr"/>
       <c r="AW21" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Le sac est posé sur le banc.
+maman|Bravo, Amir.
+papa|Tu as fait du bon travail.
+enfant-m|Le livre est dedans.
+narrateur|Un oiseau s'envole du mur.
+maman|On rentre avec le sac.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX21" t="inlineStr"/>
@@ -4675,7 +4828,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>La dînette est là. le jardin aussi. une pomme reste dans le souvenir. On attend son tour. Lina ferme la porte, tout doux. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>La dînette est sur un linge, dans l'herbe. Une assiette minuscule brille. L'assiette dans le sac, Amir. L'assiette. Amir la pose à plat près de la pomme. Bravo. Tu as mis ce que papa a dit. Le linge sent l'herbe mouillée. On plie le linge après. Oui, papa.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -4815,7 +4968,16 @@
       <c r="AV22" s="2" t="inlineStr"/>
       <c r="AW22" t="inlineStr">
         <is>
-          <t>narrateur|La dînette est là. le jardin aussi. une pomme reste dans le souvenir. On attend son tour. Lina ferme la porte, tout doux. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|La dînette est sur un linge, dans l'herbe.
+narrateur|Une assiette minuscule brille.
+papa|L'assiette dans le sac, Amir.
+enfant-m|L'assiette.
+narrateur|Amir la pose à plat près de la pomme.
+maman|Bravo.
+maman|Tu as mis ce que papa a dit.
+narrateur|Le linge sent l'herbe mouillée.
+papa|On plie le linge après.
+enfant-m|Oui, papa.</t>
         </is>
       </c>
       <c r="AX22" t="inlineStr"/>
@@ -4843,7 +5005,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Amir tient le sac contre lui. Le sac est prêt. Bravo. Merci, maman. Une goutte tombe de la gouttière. Plic ploc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -4983,7 +5145,13 @@
       <c r="AV23" s="2" t="inlineStr"/>
       <c r="AW23" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir tient le sac contre lui.
+papa|Le sac est prêt.
+maman|Bravo.
+enfant-m|Merci, maman.
+narrateur|Une goutte tombe de la gouttière.
+papa|Plic ploc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX23" t="inlineStr"/>
@@ -5011,7 +5179,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Ensuite Lina va dans la cuisine. Elle met la dînette près du sac. On met dans le sac ce que l'adulte a dit. Une tasse seulement. Maman reste tout près. On met dans le sac ce que l'adulte a dit.</t>
+          <t>Amir revient dans la chambre. Le tapis rayé est tiède. Le pull marine attend sur le lit. Le pull, Amir. On le met dans le sac. Le pull. Le pull est doux sous la main. Amir le tasse près de la pomme. Bravo. Tu as mis ce que maman a dit. Le volet claque encore un peu. On le ferme après.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -5151,8 +5319,18 @@
       <c r="AV24" s="2" t="inlineStr"/>
       <c r="AW24" t="inlineStr">
         <is>
-          <t>narrateur|Ensuite Lina va dans la cuisine. Elle met la dînette près du sac. On met dans le sac ce que l'adulte a dit.
-maman|Une tasse seulement. Maman reste tout près. On met dans le sac ce que l'adulte a dit.</t>
+          <t>narrateur|Amir revient dans la chambre.
+narrateur|Le tapis rayé est tiède.
+narrateur|Le pull marine attend sur le lit.
+maman|Le pull, Amir.
+maman|On le met dans le sac.
+enfant-m|Le pull.
+narrateur|Le pull est doux sous la main.
+narrateur|Amir le tasse près de la pomme.
+papa|Bravo.
+papa|Tu as mis ce que maman a dit.
+maman|Le volet claque encore un peu.
+papa|On le ferme après.</t>
         </is>
       </c>
       <c r="AX24" t="inlineStr"/>
@@ -5372,7 +5550,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Lina rejoint les cubes. la chambre est rangé. une pomme est fini. Une cloche tinte, tout loin. Lina chuchote : c'est fini. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>Les cubes sont sur le tapis rayé. Le bleu du tapis les cache un peu. Les cubes dans le sac, Amir. Les cubes. Ils tapent doucement contre le pull. Bravo. Tu as mis ce que maman a dit. Le rayon de soleil touche un cube rouge. Tu as vu la lumière ? Oui.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -5512,7 +5690,16 @@
       <c r="AV26" s="2" t="inlineStr"/>
       <c r="AW26" t="inlineStr">
         <is>
-          <t>narrateur|Lina rejoint les cubes. la chambre est rangé. une pomme est fini. Une cloche tinte, tout loin. Lina chuchote : c'est fini. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|Les cubes sont sur le tapis rayé.
+narrateur|Le bleu du tapis les cache un peu.
+maman|Les cubes dans le sac, Amir.
+enfant-m|Les cubes.
+narrateur|Ils tapent doucement contre le pull.
+papa|Bravo.
+papa|Tu as mis ce que maman a dit.
+narrateur|Le rayon de soleil touche un cube rouge.
+maman|Tu as vu la lumière ?
+enfant-m|Oui.</t>
         </is>
       </c>
       <c r="AX26" t="inlineStr"/>
@@ -5540,7 +5727,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Amir ferme le sac sur le tapis. Bravo, Amir. Tu as écouté. Le sac est prêt. Le volet jaune ne claque plus. On peut jouer maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -5680,7 +5867,13 @@
       <c r="AV27" s="2" t="inlineStr"/>
       <c r="AW27" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir ferme le sac sur le tapis.
+maman|Bravo, Amir.
+papa|Tu as écouté.
+enfant-m|Le sac est prêt.
+narrateur|Le volet jaune ne claque plus.
+maman|On peut jouer maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX27" t="inlineStr"/>
@@ -5708,7 +5901,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Près de le livre. Lina pose la chambre. une pomme est derrière. On écoute jusqu'au bout. Lina dit merci à maman. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>Le livre est sous l'oreiller. L'oreiller est chaud. Le livre dans le sac, Amir. Le livre. Amir le tire tout doux. Il le glisse près de la pomme. Bravo. Tu as mis ce que papa a dit. La couverture retombe, toute ronde. On la lissera après.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -5848,7 +6041,16 @@
       <c r="AV28" s="2" t="inlineStr"/>
       <c r="AW28" t="inlineStr">
         <is>
-          <t>narrateur|Près de le livre. Lina pose la chambre. une pomme est derrière. On écoute jusqu'au bout. Lina dit merci à maman. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|Le livre est sous l'oreiller.
+narrateur|L'oreiller est chaud.
+papa|Le livre dans le sac, Amir.
+enfant-m|Le livre.
+narrateur|Amir le tire tout doux.
+narrateur|Il le glisse près de la pomme.
+maman|Bravo.
+maman|Tu as mis ce que papa a dit.
+narrateur|La couverture retombe, toute ronde.
+papa|On la lissera après.</t>
         </is>
       </c>
       <c r="AX28" t="inlineStr"/>
@@ -5876,7 +6078,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Le sac repose au pied du lit. Bravo. C'est du bon travail. Merci. Le pull marine n'est plus sur le lit. Il est dans le sac, avec le livre. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -6016,7 +6218,13 @@
       <c r="AV29" s="2" t="inlineStr"/>
       <c r="AW29" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Le sac repose au pied du lit.
+papa|Bravo.
+maman|C'est du bon travail.
+enfant-m|Merci.
+narrateur|Le pull marine n'est plus sur le lit.
+papa|Il est dans le sac, avec le livre.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX29" t="inlineStr"/>
@@ -6044,7 +6252,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Lina montre la dînette. Maman a vu une pomme. Et la chambre. Un crochet tient bien le manteau. Lina ferme le sac. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>La dînette est sur la couverture. Une petite casserole roule un peu. La casserole dans le sac, Amir. La casserole. Amir la rattrape, puis la met près de la pomme. Bravo. Tu as mis ce que maman a dit. Ça sonne tout petit, dans le sac. On fera un goûter de dînette plus tard. Oui.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -6184,7 +6392,16 @@
       <c r="AV30" s="2" t="inlineStr"/>
       <c r="AW30" t="inlineStr">
         <is>
-          <t>narrateur|Lina montre la dînette. Maman a vu une pomme. Et la chambre. Un crochet tient bien le manteau. Lina ferme le sac. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|La dînette est sur la couverture.
+narrateur|Une petite casserole roule un peu.
+maman|La casserole dans le sac, Amir.
+enfant-m|La casserole.
+narrateur|Amir la rattrape, puis la met près de la pomme.
+papa|Bravo.
+papa|Tu as mis ce que maman a dit.
+narrateur|Ça sonne tout petit, dans le sac.
+maman|On fera un goûter de dînette plus tard.
+enfant-m|Oui.</t>
         </is>
       </c>
       <c r="AX30" t="inlineStr"/>
@@ -6212,7 +6429,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Amir s'assoit près du sac. Bravo, Amir. Tu as mis ce que l'adulte a dit. La pomme est dedans. Le tapis est doux sous les genoux. On reste un moment. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -6352,7 +6569,13 @@
       <c r="AV31" s="2" t="inlineStr"/>
       <c r="AW31" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir s'assoit près du sac.
+maman|Bravo, Amir.
+papa|Tu as mis ce que l'adulte a dit.
+enfant-m|La pomme est dedans.
+narrateur|Le tapis est doux sous les genoux.
+maman|On reste un moment.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX31" t="inlineStr"/>
@@ -6380,7 +6603,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Lina met un yaourt dans le sac. Maman Le yaourt. On met dans le sac ce que l'adulte a dit. Le pot est frais. Lina le cale. Papa ferme un coin du sac.</t>
+          <t>Papa ouvre le frigo. Un air frais sort. Un petit yaourt attend sur la tablette. Le yaourt dans le sac, Amir. Le yaourt. Le pot est frais sous les doigts. Amir le pose dans le sac. Le sac se creuse un peu. Bravo. Tu as mis ce que papa a dit. Tu as fini de mettre le yaourt ? Oui, papa. Amir referme un peu le sac.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -6520,9 +6743,19 @@
       <c r="AV32" s="2" t="inlineStr"/>
       <c r="AW32" t="inlineStr">
         <is>
-          <t>narrateur|Lina met un yaourt dans le sac. Maman
-enfant-f|Le yaourt. On met dans le sac ce que l'adulte a dit.
-narrateur|Le pot est frais. Lina le cale. Papa ferme un coin du sac.</t>
+          <t>narrateur|Papa ouvre le frigo.
+narrateur|Un air frais sort.
+narrateur|Un petit yaourt attend sur la tablette.
+papa|Le yaourt dans le sac, Amir.
+enfant-m|Le yaourt.
+narrateur|Le pot est frais sous les doigts.
+narrateur|Amir le pose dans le sac.
+narrateur|Le sac se creuse un peu.
+maman|Bravo.
+maman|Tu as mis ce que papa a dit.
+papa|Tu as fini de mettre le yaourt ?
+enfant-m|Oui, papa.
+narrateur|Amir referme un peu le sac.</t>
         </is>
       </c>
       <c r="AX32" t="inlineStr"/>
@@ -6738,7 +6971,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Oui. On met dans le sac ce que l'adulte a dit. Lina retient le geste. Maman sourit. On met dans le sac ce que l'adulte a dit.</t>
+          <t>Oui. On met dans le sac ce que papa a dit. Le yaourt reste au fond, bien droit. Bravo, Amir. Tu as écouté. C'est du bon travail. Le sac a ce que l'adulte a dit. Le yaourt est dedans. On continue ensemble ? Oui.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -6882,7 +7115,16 @@
       </c>
       <c r="AW34" t="inlineStr">
         <is>
-          <t>narrateur|Oui. On met dans le sac ce que l'adulte a dit. Lina retient le geste. Maman sourit. On met dans le sac ce que l'adulte a dit.</t>
+          <t>narrateur|Oui.
+narrateur|On met dans le sac ce que papa a dit.
+narrateur|Le yaourt reste au fond, bien droit.
+papa|Bravo, Amir.
+papa|Tu as écouté.
+maman|C'est du bon travail.
+maman|Le sac a ce que l'adulte a dit.
+enfant-m|Le yaourt est dedans.
+papa|On continue ensemble ?
+enfant-m|Oui.</t>
         </is>
       </c>
       <c r="AX34" t="inlineStr"/>
@@ -6910,7 +7152,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre la cuisine, le jardin, ou la chambre.</t>
+          <t>On peut aller dans la cuisine, le jardin, ou la chambre.</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -7074,7 +7316,7 @@
       <c r="AV35" s="2" t="inlineStr"/>
       <c r="AW35" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre la cuisine, le jardin, ou la chambre.</t>
+          <t>narrateur|On peut aller dans la cuisine, le jardin, ou la chambre.</t>
         </is>
       </c>
       <c r="AX35" t="inlineStr"/>
@@ -7102,7 +7344,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Ensuite Lina va dans le jardin. Elle met les cubes au soleil, puis dans le sac. On met dans le sac ce que l'adulte a dit. Je suis là. On met dans le sac ce que l'adulte a dit.</t>
+          <t>Amir pose le sac sur la table de la cuisine. Le yaourt reste bien droit. Le frigo ronronne tout bas. La cuillère, Amir. On la met dans le sac. La cuillère. Elle est lisse et froide. Amir la glisse à côté du yaourt. Bravo. Tu as mis ce que papa a dit. Ça sent encore la soupe. On goûtera plus tard.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -7242,8 +7484,18 @@
       <c r="AV36" s="2" t="inlineStr"/>
       <c r="AW36" t="inlineStr">
         <is>
-          <t>narrateur|Ensuite Lina va dans le jardin. Elle met les cubes au soleil, puis dans le sac. On met dans le sac ce que l'adulte a dit.
-maman|Je suis là. On met dans le sac ce que l'adulte a dit.</t>
+          <t>narrateur|Amir pose le sac sur la table de la cuisine.
+narrateur|Le yaourt reste bien droit.
+narrateur|Le frigo ronronne tout bas.
+papa|La cuillère, Amir.
+papa|On la met dans le sac.
+enfant-m|La cuillère.
+narrateur|Elle est lisse et froide.
+narrateur|Amir la glisse à côté du yaourt.
+maman|Bravo.
+maman|Tu as mis ce que papa a dit.
+narrateur|Ça sent encore la soupe.
+maman|On goûtera plus tard.</t>
         </is>
       </c>
       <c r="AX36" t="inlineStr"/>
@@ -7463,7 +7715,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Lina a choisi un yaourt. Puis la cuisine. Puis les cubes. Un galet est encore chaud. Lina plie un pull. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>Les cubes sont près du yaourt, sur la table. Le bois est lisse et un peu collant. Trois cubes dans le sac, Amir. Trois cubes. Amir les compte tout bas. Il les met près du yaourt. Bravo. Tu as mis ce que papa a dit. Le frigo ronronne encore. Tu as bien compté.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -7603,7 +7855,16 @@
       <c r="AV38" s="2" t="inlineStr"/>
       <c r="AW38" t="inlineStr">
         <is>
-          <t>narrateur|Lina a choisi un yaourt. Puis la cuisine. Puis les cubes. Un galet est encore chaud. Lina plie un pull. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|Les cubes sont près du yaourt, sur la table.
+narrateur|Le bois est lisse et un peu collant.
+papa|Trois cubes dans le sac, Amir.
+enfant-m|Trois cubes.
+narrateur|Amir les compte tout bas.
+narrateur|Il les met près du yaourt.
+maman|Bravo.
+maman|Tu as mis ce que papa a dit.
+narrateur|Le frigo ronronne encore.
+papa|Tu as bien compté.</t>
         </is>
       </c>
       <c r="AX38" t="inlineStr"/>
@@ -7631,7 +7892,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Amir ferme le sac près de l'évier. Bravo. Le yaourt et les cubes sont dedans. Merci, maman. Une cuillère brille encore sur la table. Elle aussi, on l'a mise. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -7771,7 +8032,13 @@
       <c r="AV39" s="2" t="inlineStr"/>
       <c r="AW39" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir ferme le sac près de l'évier.
+papa|Bravo.
+maman|Le yaourt et les cubes sont dedans.
+enfant-m|Merci, maman.
+narrateur|Une cuillère brille encore sur la table.
+papa|Elle aussi, on l'a mise.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX39" t="inlineStr"/>
@@ -7799,7 +8066,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Lina s'arrête près de le livre. la cuisine est rangé. On rit un peu. Lina raccroche un linge. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>Le livre est contre le pot de farine. Une page est un peu cornée. Le livre dans le sac, Amir. Le livre. Amir le glisse à côté du yaourt. Bravo. Tu as mis ce que maman a dit. Ça sent le lait froid et le papier. On lira après le goûter. D'accord.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -7939,7 +8206,16 @@
       <c r="AV40" s="2" t="inlineStr"/>
       <c r="AW40" t="inlineStr">
         <is>
-          <t>narrateur|Lina s'arrête près de le livre. la cuisine est rangé. On rit un peu. Lina raccroche un linge. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|Le livre est contre le pot de farine.
+narrateur|Une page est un peu cornée.
+maman|Le livre dans le sac, Amir.
+enfant-m|Le livre.
+narrateur|Amir le glisse à côté du yaourt.
+papa|Bravo.
+papa|Tu as mis ce que maman a dit.
+narrateur|Ça sent le lait froid et le papier.
+maman|On lira après le goûter.
+enfant-m|D'accord.</t>
         </is>
       </c>
       <c r="AX40" t="inlineStr"/>
@@ -7967,7 +8243,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Le sac est lourd d'un côté. Bravo, Amir. Tu as écouté. Le livre est dedans. La soupe ne fume plus. On peut jouer. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -8107,7 +8383,13 @@
       <c r="AV41" s="2" t="inlineStr"/>
       <c r="AW41" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Le sac est lourd d'un côté.
+maman|Bravo, Amir.
+papa|Tu as écouté.
+enfant-m|Le livre est dedans.
+narrateur|La soupe ne fume plus.
+maman|On peut jouer.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX41" t="inlineStr"/>
@@ -8135,7 +8417,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Lina se souvient de un yaourt. Et de la cuisine. Et de la dînette. On souffle doucement. Lina écoute maman encore une fois. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>Une petite cuillère de dînette attend près de l'évier. Elle est jaune et légère. La petite cuillère dans le sac, Amir. La cuillère. Amir la pose près du vrai yaourt. Bravo. Tu as mis ce que papa a dit. Deux cuillères, une grande, une petite. On les a mises toutes les deux. Oui.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -8275,7 +8557,16 @@
       <c r="AV42" s="2" t="inlineStr"/>
       <c r="AW42" t="inlineStr">
         <is>
-          <t>narrateur|Lina se souvient de un yaourt. Et de la cuisine. Et de la dînette. On souffle doucement. Lina écoute maman encore une fois. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|Une petite cuillère de dînette attend près de l'évier.
+narrateur|Elle est jaune et légère.
+papa|La petite cuillère dans le sac, Amir.
+enfant-m|La cuillère.
+narrateur|Amir la pose près du vrai yaourt.
+maman|Bravo.
+maman|Tu as mis ce que papa a dit.
+narrateur|Deux cuillères, une grande, une petite.
+papa|On les a mises toutes les deux.
+enfant-m|Oui.</t>
         </is>
       </c>
       <c r="AX42" t="inlineStr"/>
@@ -8303,7 +8594,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Amir appuie sur la fermeture. Le sac est prêt. Bravo. Merci, papa. Le carrelage n'est plus si froid. On a bien travaillé. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -8443,7 +8734,13 @@
       <c r="AV43" s="2" t="inlineStr"/>
       <c r="AW43" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir appuie sur la fermeture.
+papa|Le sac est prêt.
+maman|Bravo.
+enfant-m|Merci, papa.
+narrateur|Le carrelage n'est plus si froid.
+maman|On a bien travaillé.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX43" t="inlineStr"/>
@@ -8471,7 +8768,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Ensuite Lina va dans le jardin. Elle met le livre à l'ombre, puis dans le sac. On met dans le sac ce que l'adulte a dit. Maman reste tout près. On met dans le sac ce que l'adulte a dit.</t>
+          <t>Amir marche dans le jardin avec le sac. Le yaourt reste au fond, au frais. Un galet est encore chaud au soleil. Le petit gant, Amir. On le met dans le sac. Le gant. Le gant est un peu rêche. Amir le pose près du yaourt. Bravo. Tu as mis ce que maman a dit. Une goutte tombe de la gouttière. Plic ploc, tu as entendu ? Oui.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -8611,7 +8908,19 @@
       <c r="AV44" s="2" t="inlineStr"/>
       <c r="AW44" t="inlineStr">
         <is>
-          <t>narrateur|Ensuite Lina va dans le jardin. Elle met le livre à l'ombre, puis dans le sac. On met dans le sac ce que l'adulte a dit. Maman reste tout près. On met dans le sac ce que l'adulte a dit.</t>
+          <t>narrateur|Amir marche dans le jardin avec le sac.
+narrateur|Le yaourt reste au fond, au frais.
+narrateur|Un galet est encore chaud au soleil.
+maman|Le petit gant, Amir.
+maman|On le met dans le sac.
+enfant-m|Le gant.
+narrateur|Le gant est un peu rêche.
+narrateur|Amir le pose près du yaourt.
+papa|Bravo.
+papa|Tu as mis ce que maman a dit.
+narrateur|Une goutte tombe de la gouttière.
+papa|Plic ploc, tu as entendu ?
+enfant-m|Oui.</t>
         </is>
       </c>
       <c r="AX44" t="inlineStr"/>
@@ -8831,7 +9140,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Avec les cubes. Après le jardin. Près de un yaourt. Lina s'arrête. On range un objet. Lina montre les cubes à maman. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>Les cubes sont dans l'herbe, près du galet. Un cube vert est un peu humide. Les cubes secs dans le sac, Amir. Les cubes secs. Amir choisit deux cubes secs. Il les met près du yaourt. Bravo. Tu as mis ce que maman a dit. Le galet reste au jardin. Le galet n'est pas pour le sac.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -8971,7 +9280,16 @@
       <c r="AV46" s="2" t="inlineStr"/>
       <c r="AW46" t="inlineStr">
         <is>
-          <t>narrateur|Avec les cubes. Après le jardin. Près de un yaourt. Lina s'arrête. On range un objet. Lina montre les cubes à maman. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|Les cubes sont dans l'herbe, près du galet.
+narrateur|Un cube vert est un peu humide.
+maman|Les cubes secs dans le sac, Amir.
+enfant-m|Les cubes secs.
+narrateur|Amir choisit deux cubes secs.
+narrateur|Il les met près du yaourt.
+papa|Bravo.
+papa|Tu as mis ce que maman a dit.
+narrateur|Le galet reste au jardin.
+maman|Le galet n'est pas pour le sac.</t>
         </is>
       </c>
       <c r="AX46" t="inlineStr"/>
@@ -8999,7 +9317,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Amir essuie ses mains sur le linge. Bravo, Amir. Le sac a ce que l'adulte a dit. Merci. La gouttière fait encore plic ploc. On rentre. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -9139,7 +9457,13 @@
       <c r="AV47" s="2" t="inlineStr"/>
       <c r="AW47" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir essuie ses mains sur le linge.
+maman|Bravo, Amir.
+papa|Le sac a ce que l'adulte a dit.
+enfant-m|Merci.
+narrateur|La gouttière fait encore plic ploc.
+papa|On rentre.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX47" t="inlineStr"/>
@@ -9167,7 +9491,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Lina range le jardin. le livre reste près de un yaourt. On dit merci. Lina souffle, puis sourit à maman. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>Le livre est sur le muret, au soleil. La couverture est un peu chaude. Le livre dans le sac, Amir. Le livre. Amir le souffle, puis le glisse près du yaourt. Bravo. Tu as mis ce que papa a dit. Une fourmi passe sur le muret. On laisse la fourmi. Oui, papa.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -9307,7 +9631,16 @@
       <c r="AV48" s="2" t="inlineStr"/>
       <c r="AW48" t="inlineStr">
         <is>
-          <t>narrateur|Lina range le jardin. le livre reste près de un yaourt. On dit merci. Lina souffle, puis sourit à maman. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|Le livre est sur le muret, au soleil.
+narrateur|La couverture est un peu chaude.
+papa|Le livre dans le sac, Amir.
+enfant-m|Le livre.
+narrateur|Amir le souffle, puis le glisse près du yaourt.
+maman|Bravo.
+maman|Tu as mis ce que papa a dit.
+narrateur|Une fourmi passe sur le muret.
+papa|On laisse la fourmi.
+enfant-m|Oui, papa.</t>
         </is>
       </c>
       <c r="AX48" t="inlineStr"/>
@@ -9335,7 +9668,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Le sac est posé sur le muret. Bravo. Tu as fait du bon travail. Le livre est dedans. Le vent est doux dans les cheveux. On rentre avec le sac. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -9475,7 +9808,13 @@
       <c r="AV49" s="2" t="inlineStr"/>
       <c r="AW49" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Le sac est posé sur le muret.
+papa|Bravo.
+maman|Tu as fait du bon travail.
+enfant-m|Le livre est dedans.
+narrateur|Le vent est doux dans les cheveux.
+maman|On rentre avec le sac.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX49" t="inlineStr"/>
@@ -9503,7 +9842,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>La dînette est là. le jardin aussi. un yaourt reste dans le souvenir. Un ballon s'immobilise. Lina essuie ses mains. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>Une tasse de dînette est retournée dans l'herbe. Une goutte d'eau brille dedans. La tasse dans le sac, Amir. La tasse. Amir la vide, puis la met près du yaourt. Bravo. Tu as mis ce que maman a dit. L'herbe reste collée un instant. On l'enlève d'un doigt. C'est fait.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -9643,7 +9982,16 @@
       <c r="AV50" s="2" t="inlineStr"/>
       <c r="AW50" t="inlineStr">
         <is>
-          <t>narrateur|La dînette est là. le jardin aussi. un yaourt reste dans le souvenir. Un ballon s'immobilise. Lina essuie ses mains. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|Une tasse de dînette est retournée dans l'herbe.
+narrateur|Une goutte d'eau brille dedans.
+maman|La tasse dans le sac, Amir.
+enfant-m|La tasse.
+narrateur|Amir la vide, puis la met près du yaourt.
+papa|Bravo.
+papa|Tu as mis ce que maman a dit.
+narrateur|L'herbe reste collée un instant.
+maman|On l'enlève d'un doigt.
+enfant-m|C'est fait.</t>
         </is>
       </c>
       <c r="AX50" t="inlineStr"/>
@@ -9671,7 +10019,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Amir tient le sac à deux mains. Bravo, Amir. Tu as écouté. Merci. Le jardin sent l'herbe mouillée. On rentre. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -9811,7 +10159,13 @@
       <c r="AV51" s="2" t="inlineStr"/>
       <c r="AW51" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir tient le sac à deux mains.
+maman|Bravo, Amir.
+papa|Tu as écouté.
+enfant-m|Merci.
+narrateur|Le jardin sent l'herbe mouillée.
+papa|On rentre.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX51" t="inlineStr"/>
@@ -9839,7 +10193,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Ensuite Lina va dans le jardin. Elle met une tasse de dînette, puis dans le sac. On met dans le sac ce que l'adulte a dit. Maman montre le geste, lentement. On met dans le sac ce que l'adulte a dit.</t>
+          <t>Amir s'assoit sur le tapis de la chambre. Le yaourt fait un petit rond dans le sac. La couverture est douce contre le genou. Les chaussons, Amir. On les met dans le sac. Les chaussons. Ils sont chauds et mous. Amir les glisse près du yaourt. Bravo. Tu as mis ce que papa a dit. Le rayon de soleil a bougé. Il touche maintenant le sac.</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -9979,7 +10333,18 @@
       <c r="AV52" s="2" t="inlineStr"/>
       <c r="AW52" t="inlineStr">
         <is>
-          <t>narrateur|Ensuite Lina va dans le jardin. Elle met une tasse de dînette, puis dans le sac. On met dans le sac ce que l'adulte a dit. Maman montre le geste, lentement. On met dans le sac ce que l'adulte a dit.</t>
+          <t>narrateur|Amir s'assoit sur le tapis de la chambre.
+narrateur|Le yaourt fait un petit rond dans le sac.
+narrateur|La couverture est douce contre le genou.
+papa|Les chaussons, Amir.
+papa|On les met dans le sac.
+enfant-m|Les chaussons.
+narrateur|Ils sont chauds et mous.
+narrateur|Amir les glisse près du yaourt.
+maman|Bravo.
+maman|Tu as mis ce que papa a dit.
+narrateur|Le rayon de soleil a bougé.
+maman|Il touche maintenant le sac.</t>
         </is>
       </c>
       <c r="AX52" t="inlineStr"/>
@@ -10199,7 +10564,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Lina rejoint les cubes. la chambre est rangé. un yaourt est fini. Une tasse cliquette. J'ai appris. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>Les cubes sont sous la chaise, dans la chambre. Un cube rouge a roulé loin. Les cubes dans le sac, Amir. Les cubes. Amir ramasse le cube rouge. Il les met près du yaourt. Bravo. Tu as mis ce que papa a dit. La chaise ne bouge plus. Tu as tout retrouvé.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -10339,9 +10704,16 @@
       <c r="AV54" s="2" t="inlineStr"/>
       <c r="AW54" t="inlineStr">
         <is>
-          <t>narrateur|Lina rejoint les cubes. la chambre est rangé. un yaourt est fini. Une tasse cliquette.
-enfant-f|J'ai appris. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit.
-narrateur|Lina dit merci à maman.</t>
+          <t>narrateur|Les cubes sont sous la chaise, dans la chambre.
+narrateur|Un cube rouge a roulé loin.
+papa|Les cubes dans le sac, Amir.
+enfant-m|Les cubes.
+narrateur|Amir ramasse le cube rouge.
+narrateur|Il les met près du yaourt.
+maman|Bravo.
+maman|Tu as mis ce que papa a dit.
+narrateur|La chaise ne bouge plus.
+papa|Tu as tout retrouvé.</t>
         </is>
       </c>
       <c r="AX54" t="inlineStr"/>
@@ -10369,7 +10741,7 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Amir ferme le sac au pied du lit. Bravo. Les chaussons et les cubes sont dedans. Le sac est prêt. Le tapis rayé est calme. On peut jouer. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -10509,7 +10881,13 @@
       <c r="AV55" s="2" t="inlineStr"/>
       <c r="AW55" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir ferme le sac au pied du lit.
+papa|Bravo.
+maman|Les chaussons et les cubes sont dedans.
+enfant-m|Le sac est prêt.
+narrateur|Le tapis rayé est calme.
+maman|On peut jouer.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX55" t="inlineStr"/>
@@ -10537,7 +10915,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Près de le livre. Lina pose la chambre. un yaourt est derrière. Un chat miaule une fois. Lina range encore un peu, près de maman. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>Le livre est ouvert sur la commode. Une image montre un bateau. Le livre dans le sac, Amir. Le livre. Amir le ferme tout doux. Il le glisse près du yaourt. Bravo. Tu as mis ce que maman a dit. Le bateau disparaît entre les pages. On le reverra plus tard.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -10677,7 +11055,16 @@
       <c r="AV56" s="2" t="inlineStr"/>
       <c r="AW56" t="inlineStr">
         <is>
-          <t>narrateur|Près de le livre. Lina pose la chambre. un yaourt est derrière. Un chat miaule une fois. Lina range encore un peu, près de maman. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|Le livre est ouvert sur la commode.
+narrateur|Une image montre un bateau.
+maman|Le livre dans le sac, Amir.
+enfant-m|Le livre.
+narrateur|Amir le ferme tout doux.
+narrateur|Il le glisse près du yaourt.
+papa|Bravo.
+papa|Tu as mis ce que maman a dit.
+narrateur|Le bateau disparaît entre les pages.
+maman|On le reverra plus tard.</t>
         </is>
       </c>
       <c r="AX56" t="inlineStr"/>
@@ -10705,7 +11092,7 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Le sac est sur la commode, une seconde. Bravo, Amir. C'est du bon travail. Merci, papa. Le rayon de soleil a quitté le tapis. On va jouer. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -10845,7 +11232,13 @@
       <c r="AV57" s="2" t="inlineStr"/>
       <c r="AW57" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Le sac est sur la commode, une seconde.
+maman|Bravo, Amir.
+papa|C'est du bon travail.
+enfant-m|Merci, papa.
+narrateur|Le rayon de soleil a quitté le tapis.
+maman|On va jouer.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX57" t="inlineStr"/>
@@ -10873,7 +11266,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Lina montre la dînette. Maman a vu un yaourt. Et la chambre. Le sol est un peu froid. Lina caresse le doudou. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>La dînette est dans la caisse, sous le lit. Une petite assiette dépasse. L'assiette dans le sac, Amir. L'assiette. Amir la tire, puis la met près du yaourt. Bravo. Tu as mis ce que papa a dit. La caisse sent le bois. On laisse le reste dans la caisse. D'accord.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -11013,7 +11406,16 @@
       <c r="AV58" s="2" t="inlineStr"/>
       <c r="AW58" t="inlineStr">
         <is>
-          <t>narrateur|Lina montre la dînette. Maman a vu un yaourt. Et la chambre. Le sol est un peu froid. Lina caresse le doudou. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|La dînette est dans la caisse, sous le lit.
+narrateur|Une petite assiette dépasse.
+papa|L'assiette dans le sac, Amir.
+enfant-m|L'assiette.
+narrateur|Amir la tire, puis la met près du yaourt.
+maman|Bravo.
+maman|Tu as mis ce que papa a dit.
+narrateur|La caisse sent le bois.
+papa|On laisse le reste dans la caisse.
+enfant-m|D'accord.</t>
         </is>
       </c>
       <c r="AX58" t="inlineStr"/>
@@ -11041,7 +11443,7 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Amir s'assoit sur le tapis. Le sac est prêt. Bravo. Merci, maman. La couverture retombe sur le lit. On a mis ce que l'adulte a dit. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -11181,7 +11583,13 @@
       <c r="AV59" s="2" t="inlineStr"/>
       <c r="AW59" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir s'assoit sur le tapis.
+papa|Le sac est prêt.
+maman|Bravo.
+enfant-m|Merci, maman.
+narrateur|La couverture retombe sur le lit.
+papa|On a mis ce que l'adulte a dit.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX59" t="inlineStr"/>
@@ -11209,7 +11617,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Lina met un morceau de pain dans le sac. Maman Le pain. On met dans le sac ce que l'adulte a dit. Le pain est un peu dur. Lina le glisse sur le côté.</t>
+          <t>Sur la planche, un morceau de pain attend. La croûte fait un petit bruit. Ça sent le four, encore un peu. Le pain dans le sac, Amir. Le pain. Amir le prend avec précaution. Il le glisse à côté de la paroi. Bravo. Tu as mis ce que maman a dit. Tu as fini de mettre le pain ? Oui, maman. Une miette reste sur le tapis. On la range après.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -11349,9 +11757,19 @@
       <c r="AV60" s="2" t="inlineStr"/>
       <c r="AW60" t="inlineStr">
         <is>
-          <t>narrateur|Lina met un morceau de pain dans le sac. Maman
-enfant-f|Le pain. On met dans le sac ce que l'adulte a dit.
-narrateur|Le pain est un peu dur. Lina le glisse sur le côté.</t>
+          <t>narrateur|Sur la planche, un morceau de pain attend.
+narrateur|La croûte fait un petit bruit.
+narrateur|Ça sent le four, encore un peu.
+maman|Le pain dans le sac, Amir.
+enfant-m|Le pain.
+narrateur|Amir le prend avec précaution.
+narrateur|Il le glisse à côté de la paroi.
+papa|Bravo.
+papa|Tu as mis ce que maman a dit.
+maman|Tu as fini de mettre le pain ?
+enfant-m|Oui, maman.
+narrateur|Une miette reste sur le tapis.
+papa|On la range après.</t>
         </is>
       </c>
       <c r="AX60" t="inlineStr"/>
@@ -11567,7 +11985,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Oui. On met dans le sac ce que l'adulte a dit. Lina hoche la tête. On continue, avec maman. On met dans le sac ce que l'adulte a dit.</t>
+          <t>Oui. Papa ou maman dit ce qu'on met. On met dans le sac ce que l'adulte a dit. Bravo, Amir. Tu as écouté. C'est du bon travail. Le pain est dedans. On continue ensemble ? Oui.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -11711,7 +12129,15 @@
       </c>
       <c r="AW62" t="inlineStr">
         <is>
-          <t>narrateur|Oui. On met dans le sac ce que l'adulte a dit. Lina hoche la tête. On continue, avec maman. On met dans le sac ce que l'adulte a dit.</t>
+          <t>narrateur|Oui.
+narrateur|Papa ou maman dit ce qu'on met.
+narrateur|On met dans le sac ce que l'adulte a dit.
+maman|Bravo, Amir.
+maman|Tu as écouté.
+papa|C'est du bon travail.
+enfant-m|Le pain est dedans.
+maman|On continue ensemble ?
+enfant-m|Oui.</t>
         </is>
       </c>
       <c r="AX62" t="inlineStr"/>
@@ -11739,7 +12165,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre la cuisine, le jardin, ou la chambre.</t>
+          <t>On peut aller dans la cuisine, le jardin, ou la chambre.</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -11903,7 +12329,7 @@
       <c r="AV63" s="2" t="inlineStr"/>
       <c r="AW63" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre la cuisine, le jardin, ou la chambre.</t>
+          <t>narrateur|On peut aller dans la cuisine, le jardin, ou la chambre.</t>
         </is>
       </c>
       <c r="AX63" t="inlineStr"/>
@@ -11931,7 +12357,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Ensuite Lina reste dans la chambre. Elle met les cubes dans le sac. On met dans le sac ce que l'adulte a dit. Papa tient le sac. Maman reste tout près. On met dans le sac ce que l'adulte a dit.</t>
+          <t>Amir pose le sac près de l'évier. Le pain sent encore le four. L'eau fait un tout petit bruit. La boîte à goûter, Amir. On la met dans le sac. La boîte. La boîte est lisse et bleue. Amir y glisse le pain, puis la boîte dans le sac. Bravo. Tu as mis ce que maman a dit. Tu as fini ? Oui, maman.</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -12071,7 +12497,18 @@
       <c r="AV64" s="2" t="inlineStr"/>
       <c r="AW64" t="inlineStr">
         <is>
-          <t>narrateur|Ensuite Lina reste dans la chambre. Elle met les cubes dans le sac. On met dans le sac ce que l'adulte a dit. Papa tient le sac. Maman reste tout près. On met dans le sac ce que l'adulte a dit.</t>
+          <t>narrateur|Amir pose le sac près de l'évier.
+narrateur|Le pain sent encore le four.
+narrateur|L'eau fait un tout petit bruit.
+maman|La boîte à goûter, Amir.
+maman|On la met dans le sac.
+enfant-m|La boîte.
+narrateur|La boîte est lisse et bleue.
+narrateur|Amir y glisse le pain, puis la boîte dans le sac.
+papa|Bravo.
+papa|Tu as mis ce que maman a dit.
+maman|Tu as fini ?
+enfant-m|Oui, maman.</t>
         </is>
       </c>
       <c r="AX64" t="inlineStr"/>
@@ -12291,7 +12728,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Lina a choisi un morceau de pain. Puis la cuisine. Puis les cubes. L'eau coule, tout petit bruit. Lina répète tout bas le geste. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>Les cubes sont près de la boîte à goûter. Ils font une petite tour. La tour, non. Deux cubes dans le sac, Amir. Deux cubes. Amir défait la tour tout doux. Il met deux cubes près du pain. Bravo. Tu as mis ce que maman a dit. La tour n'est plus là. On en fera une autre plus tard.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -12431,7 +12868,17 @@
       <c r="AV66" s="2" t="inlineStr"/>
       <c r="AW66" t="inlineStr">
         <is>
-          <t>narrateur|Lina a choisi un morceau de pain. Puis la cuisine. Puis les cubes. L'eau coule, tout petit bruit. Lina répète tout bas le geste. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|Les cubes sont près de la boîte à goûter.
+narrateur|Ils font une petite tour.
+maman|La tour, non.
+maman|Deux cubes dans le sac, Amir.
+enfant-m|Deux cubes.
+narrateur|Amir défait la tour tout doux.
+narrateur|Il met deux cubes près du pain.
+papa|Bravo.
+papa|Tu as mis ce que maman a dit.
+narrateur|La tour n'est plus là.
+maman|On en fera une autre plus tard.</t>
         </is>
       </c>
       <c r="AX66" t="inlineStr"/>
@@ -12459,7 +12906,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Amir ferme le sac près de l'évier. Bravo, Amir. Le pain est dans la boîte. Les cubes aussi. L'eau ne coule plus. On a fini le sac. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -12599,7 +13046,13 @@
       <c r="AV67" s="2" t="inlineStr"/>
       <c r="AW67" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir ferme le sac près de l'évier.
+maman|Bravo, Amir.
+papa|Le pain est dans la boîte.
+enfant-m|Les cubes aussi.
+narrateur|L'eau ne coule plus.
+maman|On a fini le sac.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX67" t="inlineStr"/>
@@ -12627,7 +13080,7 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Lina s'arrête près de le livre. la cuisine est rangé. Une feuille tombe. Lina range un morceau de pain dans sa tête, comme un souvenir. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>Le livre est sous un torchon, dans la cuisine. Le torchon sent le propre. Le livre dans le sac, Amir. Le livre. Amir le sort du torchon. Il le glisse près du pain. Bravo. Tu as mis ce que papa a dit. Le torchon reste sur la table. Le torchon n'est pas pour le sac.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -12767,7 +13220,16 @@
       <c r="AV68" s="2" t="inlineStr"/>
       <c r="AW68" t="inlineStr">
         <is>
-          <t>narrateur|Lina s'arrête près de le livre. la cuisine est rangé. Une feuille tombe. Lina range un morceau de pain dans sa tête, comme un souvenir. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|Le livre est sous un torchon, dans la cuisine.
+narrateur|Le torchon sent le propre.
+papa|Le livre dans le sac, Amir.
+enfant-m|Le livre.
+narrateur|Amir le sort du torchon.
+narrateur|Il le glisse près du pain.
+maman|Bravo.
+maman|Tu as mis ce que papa a dit.
+narrateur|Le torchon reste sur la table.
+papa|Le torchon n'est pas pour le sac.</t>
         </is>
       </c>
       <c r="AX68" t="inlineStr"/>
@@ -12795,7 +13257,7 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Le sac est posé contre la chaise. Bravo. Tu as écouté. Merci. Ça sent encore un peu le four. On va jouer. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
@@ -12935,7 +13397,13 @@
       <c r="AV69" s="2" t="inlineStr"/>
       <c r="AW69" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Le sac est posé contre la chaise.
+papa|Bravo.
+maman|Tu as écouté.
+enfant-m|Merci.
+narrateur|Ça sent encore un peu le four.
+papa|On va jouer.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX69" t="inlineStr"/>
@@ -12963,7 +13431,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Lina se souvient de un morceau de pain. Et de la cuisine. Et de la dînette. Le vent est doux. Lina boit une gorgée d'eau. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>La dînette est dans le tiroir du bas. Une casserole minuscule brille. La casserole dans le sac, Amir. La casserole. Amir ouvre le tiroir tout doux. Il met la casserole près du pain. Bravo. Tu as mis ce que maman a dit. Le tiroir se referme sans bruit. Tu as bien fermé.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -13103,7 +13571,16 @@
       <c r="AV70" s="2" t="inlineStr"/>
       <c r="AW70" t="inlineStr">
         <is>
-          <t>narrateur|Lina se souvient de un morceau de pain. Et de la cuisine. Et de la dînette. Le vent est doux. Lina boit une gorgée d'eau. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|La dînette est dans le tiroir du bas.
+narrateur|Une casserole minuscule brille.
+maman|La casserole dans le sac, Amir.
+enfant-m|La casserole.
+narrateur|Amir ouvre le tiroir tout doux.
+narrateur|Il met la casserole près du pain.
+papa|Bravo.
+papa|Tu as mis ce que maman a dit.
+narrateur|Le tiroir se referme sans bruit.
+maman|Tu as bien fermé.</t>
         </is>
       </c>
       <c r="AX70" t="inlineStr"/>
@@ -13131,7 +13608,7 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Amir tient la sangle du sac. Bravo, Amir. C'est du bon travail. Le sac est prêt. La cuisine est calme. On a mis ce que l'adulte a dit. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -13271,7 +13748,13 @@
       <c r="AV71" s="2" t="inlineStr"/>
       <c r="AW71" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir tient la sangle du sac.
+maman|Bravo, Amir.
+papa|C'est du bon travail.
+enfant-m|Le sac est prêt.
+narrateur|La cuisine est calme.
+maman|On a mis ce que l'adulte a dit.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX71" t="inlineStr"/>
@@ -13299,7 +13782,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Ensuite Lina reste dans la chambre. Elle met le livre dans le sac. On met dans le sac ce que l'adulte a dit. Papa tient le sac. Maman montre le geste, lentement. On met dans le sac ce que l'adulte a dit.</t>
+          <t>Amir descend la marche du jardin. Le pain reste au fond du sac. Le vent est doux sur les joues. Le petit chapeau, Amir. On le met dans le sac. Le chapeau. Le chapeau est souple. Amir le tasse près du pain. Bravo. Tu as mis ce que papa a dit. Une feuille tourne au-dessus du bac. On la laisse au jardin.</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -13439,7 +13922,18 @@
       <c r="AV72" s="2" t="inlineStr"/>
       <c r="AW72" t="inlineStr">
         <is>
-          <t>narrateur|Ensuite Lina reste dans la chambre. Elle met le livre dans le sac. On met dans le sac ce que l'adulte a dit. Papa tient le sac. Maman montre le geste, lentement. On met dans le sac ce que l'adulte a dit.</t>
+          <t>narrateur|Amir descend la marche du jardin.
+narrateur|Le pain reste au fond du sac.
+narrateur|Le vent est doux sur les joues.
+papa|Le petit chapeau, Amir.
+papa|On le met dans le sac.
+enfant-m|Le chapeau.
+narrateur|Le chapeau est souple.
+narrateur|Amir le tasse près du pain.
+maman|Bravo.
+maman|Tu as mis ce que papa a dit.
+narrateur|Une feuille tourne au-dessus du bac.
+papa|On la laisse au jardin.</t>
         </is>
       </c>
       <c r="AX72" t="inlineStr"/>
@@ -13659,7 +14153,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Avec les cubes. Après le jardin. Près de un morceau de pain. Lina s'arrête. Le savon sent bon. Lina pose sa tête un moment. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>Les cubes sont dans le bac à sable, au jardin. Un cube a un peu de sable. Le cube propre dans le sac, Amir. Le cube propre. Amir le frotte, puis le met près du pain. Bravo. Tu as mis ce que papa a dit. Le chapeau bouge dans le sac. Le sable reste au jardin. Oui.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -13799,7 +14293,16 @@
       <c r="AV74" s="2" t="inlineStr"/>
       <c r="AW74" t="inlineStr">
         <is>
-          <t>narrateur|Avec les cubes. Après le jardin. Près de un morceau de pain. Lina s'arrête. Le savon sent bon. Lina pose sa tête un moment. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|Les cubes sont dans le bac à sable, au jardin.
+narrateur|Un cube a un peu de sable.
+papa|Le cube propre dans le sac, Amir.
+enfant-m|Le cube propre.
+narrateur|Amir le frotte, puis le met près du pain.
+maman|Bravo.
+maman|Tu as mis ce que papa a dit.
+narrateur|Le chapeau bouge dans le sac.
+papa|Le sable reste au jardin.
+enfant-m|Oui.</t>
         </is>
       </c>
       <c r="AX74" t="inlineStr"/>
@@ -13827,7 +14330,7 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Amir remonte la marche avec le sac. Bravo. Tu as fait du bon travail. Merci, papa. Une feuille reste sur le bac. On rentre. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -13967,7 +14470,13 @@
       <c r="AV75" s="2" t="inlineStr"/>
       <c r="AW75" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir remonte la marche avec le sac.
+papa|Bravo.
+maman|Tu as fait du bon travail.
+enfant-m|Merci, papa.
+narrateur|Une feuille reste sur le bac.
+maman|On rentre.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX75" t="inlineStr"/>
@@ -13995,7 +14504,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Lina range le jardin. le livre reste près de un morceau de pain. Un panier est posé sur le banc. Lina sourit. Maman sourit aussi. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>Le livre est sous le chapeau, sur le banc. Une page tremble au vent. Le livre dans le sac, Amir. Le livre. Amir le met près du pain, puis le chapeau par-dessus. Bravo. Tu as mis ce que maman a dit. Le vent n'attrape plus les pages. Le livre est à l'abri. Oui, maman.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -14135,7 +14644,16 @@
       <c r="AV76" s="2" t="inlineStr"/>
       <c r="AW76" t="inlineStr">
         <is>
-          <t>narrateur|Lina range le jardin. le livre reste près de un morceau de pain. Un panier est posé sur le banc. Lina sourit. Maman sourit aussi. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|Le livre est sous le chapeau, sur le banc.
+narrateur|Une page tremble au vent.
+maman|Le livre dans le sac, Amir.
+enfant-m|Le livre.
+narrateur|Amir le met près du pain, puis le chapeau par-dessus.
+papa|Bravo.
+papa|Tu as mis ce que maman a dit.
+narrateur|Le vent n'attrape plus les pages.
+maman|Le livre est à l'abri.
+enfant-m|Oui, maman.</t>
         </is>
       </c>
       <c r="AX76" t="inlineStr"/>
@@ -14163,7 +14681,7 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Le sac est lourd, un peu. Bravo, Amir. Tu as écouté. Merci. Le jardin sent la terre mouillée. On rentre avec le sac. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -14303,7 +14821,13 @@
       <c r="AV77" s="2" t="inlineStr"/>
       <c r="AW77" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Le sac est lourd, un peu.
+maman|Bravo, Amir.
+papa|Tu as écouté.
+enfant-m|Merci.
+narrateur|Le jardin sent la terre mouillée.
+papa|On rentre avec le sac.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX77" t="inlineStr"/>
@@ -14331,7 +14855,7 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>La dînette est là. le jardin aussi. un morceau de pain reste dans le souvenir. Un linge sèche à l'air. Lina range la tasse. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>Une assiette de dînette est sur le muret. Une feuille sèche est posée dessus. L'assiette dans le sac, Amir. L'assiette. Amir enlève la feuille. Il met l'assiette près du pain. Bravo. Tu as mis ce que papa a dit. La feuille s'envole. Elle reste au jardin.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -14471,7 +14995,16 @@
       <c r="AV78" s="2" t="inlineStr"/>
       <c r="AW78" t="inlineStr">
         <is>
-          <t>narrateur|La dînette est là. le jardin aussi. un morceau de pain reste dans le souvenir. Un linge sèche à l'air. Lina range la tasse. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|Une assiette de dînette est sur le muret.
+narrateur|Une feuille sèche est posée dessus.
+papa|L'assiette dans le sac, Amir.
+enfant-m|L'assiette.
+narrateur|Amir enlève la feuille.
+narrateur|Il met l'assiette près du pain.
+maman|Bravo.
+maman|Tu as mis ce que papa a dit.
+narrateur|La feuille s'envole.
+papa|Elle reste au jardin.</t>
         </is>
       </c>
       <c r="AX78" t="inlineStr"/>
@@ -14499,7 +15032,7 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Amir serre le sac contre lui. Le sac est prêt. Bravo. Merci, maman. Le vent est plus calme. On a mis ce que l'adulte a dit. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -14639,7 +15172,13 @@
       <c r="AV79" s="2" t="inlineStr"/>
       <c r="AW79" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir serre le sac contre lui.
+papa|Le sac est prêt.
+maman|Bravo.
+enfant-m|Merci, maman.
+narrateur|Le vent est plus calme.
+papa|On a mis ce que l'adulte a dit.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX79" t="inlineStr"/>
@@ -14667,7 +15206,7 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Ensuite Lina reste dans la chambre. Elle met une tasse de dînette dans le sac. On met dans le sac ce que l'adulte a dit. Je suis là. On met dans le sac ce que l'adulte a dit.</t>
+          <t>Amir repose le sac sur le tapis rayé. Le pain fait un petit bruit de croûte. Le volet jaune claque une fois. Le doudou du sac, Amir. On le met dans le sac. Le doudou. Le doudou est chaud et un peu plat. Amir le glisse près du pain. Bravo. Tu as mis ce que maman a dit. Le sac se remplit bien. Il est presque prêt.</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -14807,8 +15346,18 @@
       <c r="AV80" s="2" t="inlineStr"/>
       <c r="AW80" t="inlineStr">
         <is>
-          <t>narrateur|Ensuite Lina reste dans la chambre. Elle met une tasse de dînette dans le sac. On met dans le sac ce que l'adulte a dit.
-maman|Je suis là. On met dans le sac ce que l'adulte a dit.</t>
+          <t>narrateur|Amir repose le sac sur le tapis rayé.
+narrateur|Le pain fait un petit bruit de croûte.
+narrateur|Le volet jaune claque une fois.
+maman|Le doudou du sac, Amir.
+maman|On le met dans le sac.
+enfant-m|Le doudou.
+narrateur|Le doudou est chaud et un peu plat.
+narrateur|Amir le glisse près du pain.
+papa|Bravo.
+papa|Tu as mis ce que maman a dit.
+maman|Le sac se remplit bien.
+enfant-m|Il est presque prêt.</t>
         </is>
       </c>
       <c r="AX80" t="inlineStr"/>
@@ -15028,7 +15577,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Lina rejoint les cubes. la chambre est rangé. un morceau de pain est fini. Les chaussures font toc toc. Lina serre la main de maman. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>Les cubes sont près du doudou, sur le tapis. Un cube touche la patte du doudou. Les cubes dans le sac, Amir. Les cubes. Amir les met près du pain et du doudou. Bravo. Tu as mis ce que maman a dit. Le doudou ne tombe pas. Tu as été doux. Oui.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -15168,7 +15717,16 @@
       <c r="AV82" s="2" t="inlineStr"/>
       <c r="AW82" t="inlineStr">
         <is>
-          <t>narrateur|Lina rejoint les cubes. la chambre est rangé. un morceau de pain est fini. Les chaussures font toc toc. Lina serre la main de maman. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|Les cubes sont près du doudou, sur le tapis.
+narrateur|Un cube touche la patte du doudou.
+maman|Les cubes dans le sac, Amir.
+enfant-m|Les cubes.
+narrateur|Amir les met près du pain et du doudou.
+papa|Bravo.
+papa|Tu as mis ce que maman a dit.
+narrateur|Le doudou ne tombe pas.
+maman|Tu as été doux.
+enfant-m|Oui.</t>
         </is>
       </c>
       <c r="AX82" t="inlineStr"/>
@@ -15196,7 +15754,7 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Amir ferme le sac sur le tapis rayé. Bravo, Amir. Tu as fait du bon travail. Le sac est prêt. Le volet jaune est calme. On peut jouer maintenant. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -15336,7 +15894,13 @@
       <c r="AV83" s="2" t="inlineStr"/>
       <c r="AW83" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir ferme le sac sur le tapis rayé.
+maman|Bravo, Amir.
+papa|Tu as fait du bon travail.
+enfant-m|Le sac est prêt.
+narrateur|Le volet jaune est calme.
+maman|On peut jouer maintenant.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX83" t="inlineStr"/>
@@ -15364,7 +15928,7 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Près de le livre. Lina pose la chambre. un morceau de pain est derrière. Une pomme brille un peu. Lina marche près de maman. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>Le livre est coincé entre deux peluches. Amir le tire tout doux. Le livre dans le sac, Amir. Le livre. Il le glisse près du pain. Bravo. Tu as mis ce que papa a dit. Les peluches restent sur le lit. Elles ne vont pas dans le sac. D'accord.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -15504,7 +16068,16 @@
       <c r="AV84" s="2" t="inlineStr"/>
       <c r="AW84" t="inlineStr">
         <is>
-          <t>narrateur|Près de le livre. Lina pose la chambre. un morceau de pain est derrière. Une pomme brille un peu. Lina marche près de maman. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|Le livre est coincé entre deux peluches.
+narrateur|Amir le tire tout doux.
+papa|Le livre dans le sac, Amir.
+enfant-m|Le livre.
+narrateur|Il le glisse près du pain.
+maman|Bravo.
+maman|Tu as mis ce que papa a dit.
+narrateur|Les peluches restent sur le lit.
+papa|Elles ne vont pas dans le sac.
+enfant-m|D'accord.</t>
         </is>
       </c>
       <c r="AX84" t="inlineStr"/>
@@ -15532,7 +16105,7 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Le sac attend près de la porte de la chambre. Bravo. Tu as écouté. Merci, papa. Le tapis n'a plus de cubes. On a mis ce que l'adulte a dit. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -15672,7 +16245,13 @@
       <c r="AV85" s="2" t="inlineStr"/>
       <c r="AW85" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Le sac attend près de la porte de la chambre.
+papa|Bravo.
+maman|Tu as écouté.
+enfant-m|Merci, papa.
+narrateur|Le tapis n'a plus de cubes.
+maman|On a mis ce que l'adulte a dit.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX85" t="inlineStr"/>
@@ -15700,7 +16279,7 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Lina montre la dînette. Maman a vu un morceau de pain. Et la chambre. On se tient la main. Lina pose la chambre à sa place. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>La dînette est dans le panier, près du lit. Une tasse et une assiette s'entrechoquent. La tasse seulement, Amir. On la met dans le sac. La tasse. Amir prend la tasse, pas l'assiette. Il la met près du pain. Bravo. Tu as mis ce que maman a dit. L'assiette reste dans le panier. C'est ça.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -15840,7 +16419,17 @@
       <c r="AV86" s="2" t="inlineStr"/>
       <c r="AW86" t="inlineStr">
         <is>
-          <t>narrateur|Lina montre la dînette. Maman a vu un morceau de pain. Et la chambre. On se tient la main. Lina pose la chambre à sa place. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.</t>
+          <t>narrateur|La dînette est dans le panier, près du lit.
+narrateur|Une tasse et une assiette s'entrechoquent.
+maman|La tasse seulement, Amir.
+maman|On la met dans le sac.
+enfant-m|La tasse.
+narrateur|Amir prend la tasse, pas l'assiette.
+narrateur|Il la met près du pain.
+papa|Bravo.
+papa|Tu as mis ce que maman a dit.
+narrateur|L'assiette reste dans le panier.
+maman|C'est ça.</t>
         </is>
       </c>
       <c r="AX86" t="inlineStr"/>
@@ -15868,7 +16457,7 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Amir s'assoit, le sac sur les genoux. Bravo, Amir. C'est du bon travail. Merci. La chambre sent encore la soupe, un peu. Le sac est prêt. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
@@ -16008,7 +16597,13 @@
       <c r="AV87" s="2" t="inlineStr"/>
       <c r="AW87" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir s'assoit, le sac sur les genoux.
+maman|Bravo, Amir.
+papa|C'est du bon travail.
+enfant-m|Merci.
+narrateur|La chambre sent encore la soupe, un peu.
+maman|Le sac est prêt.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX87" t="inlineStr"/>
@@ -16030,7 +16625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16068,6 +16663,13 @@
       <c r="A5" t="inlineStr">
         <is>
           <t>F-AUD-007 colonne sons ; vide = silence ; jamais parler dans le bruit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F-NAR-016): texte F-NAR-010…015 sur TREE-AUT-001 et TREE-COL-001
Désir du héros, branches à conséquences, chaînes de questions, troupe D16.
Sans audio.
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-AUT-001.xlsx
+++ b/stories/arbres/TREE-AUT-001.xlsx
@@ -696,7 +696,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Lina, maman, papa</t>
+          <t>Amir, maman, papa</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amir prépare son sac sur le tapis rayé. Papa et maman disent ce qu'il met. Ensuite il joue.</t>
+          <t>Amir veut aller jouer. Son sac est vide sur le tapis rayé. Il demande à papa et maman. Il met la pomme, le yaourt ou le pain, puis ce qu'ils nomment. Quand le sac est fermé, il joue enfin.</t>
         </is>
       </c>
     </row>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Sur le toit, la gouttière fait plic ploc. La maison a un volet jaune. Le volet claque tout doux. Dans le village, les pavés brillent. Ils sont encore mouillés. Une odeur de soupe entre par la fenêtre. Le tapis de la chambre est rayé. Il est bleu et crème. Un rayon de soleil touche le plancher. Papa plie un pull marine. Le pull est encore un peu chaud. Le pull est prêt, Amir. Il est tout doux. Maman ouvre un peu la fenêtre. Tu as senti la soupe ? Oui, maman. Le sac d'Amir attend sur le tapis. Le sac est vide. La fermeture brille. Je veux jouer ! D'accord. On prépare le sac d'abord. On met dans le sac ce que maman a dit. Ou ce que papa a dit. Amir pose la main sur le sac. En ce moment, il a trop envie de jouer.</t>
+          <t>Sur le toit, la gouttière fait encore plic ploc. La pluie vient de s'arrêter. La maison a un volet jaune. Le volet claque tout doux. Dans la rue, les pavés brillent. Ils sont encore mouillés. Une odeur de soupe entre par la fenêtre. Le tapis de la chambre est rayé. Il est bleu et crème. Un rayon de soleil touche le plancher. Papa pose un pull sur le lit. Il est encore un peu chaud. Maman ouvre un peu la fenêtre. Tu as senti la soupe ? Oui, maman. En ce moment, Amir veut aller jouer. Son sac attend sur le tapis. Amir tire la fermeture. Ça fait zzz. Le sac est vide. Je veux jouer ! D'accord. On prépare ton sac d'abord. Tu mets quoi, Amir ? Je ne sais pas. Demande. On t'aide. Amir pose la main sur le sac.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1337,35 +1337,35 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Sur le toit, la gouttière fait plic ploc.
+          <t>narrateur|Sur le toit, la gouttière fait encore plic ploc.
+narrateur|La pluie vient de s'arrêter.
 narrateur|La maison a un volet jaune.
 narrateur|Le volet claque tout doux.
-narrateur|Dans le village, les pavés brillent.
+narrateur|Dans la rue, les pavés brillent.
 narrateur|Ils sont encore mouillés.
 narrateur|Une odeur de soupe entre par la fenêtre.
 narrateur|Le tapis de la chambre est rayé.
 narrateur|Il est bleu et crème.
 narrateur|Un rayon de soleil touche le plancher.
-narrateur|Papa plie un pull marine.
-narrateur|Le pull est encore un peu chaud.
-papa|Le pull est prêt, Amir.
-papa|Il est tout doux.
+narrateur|Papa pose un pull sur le lit.
+papa|Il est encore un peu chaud.
 narrateur|Maman ouvre un peu la fenêtre.
 maman|Tu as senti la soupe ?
 enfant-m|Oui, maman.
-narrateur|Le sac d'Amir attend sur le tapis.
+narrateur|En ce moment, Amir veut aller jouer.
+narrateur|Son sac attend sur le tapis.
+narrateur|Amir tire la fermeture.
+narrateur|Ça fait zzz.
 narrateur|Le sac est vide.
-narrateur|La fermeture brille.
 enfant-m|Je veux jouer !
 maman|D'accord.
-maman|On prépare le sac d'abord.
-papa|On met dans le sac ce que maman a dit.
-papa|Ou ce que papa a dit.
-narrateur|Amir pose la main sur le sac.
-narrateur|En ce moment, il a trop envie de jouer.</t>
-        </is>
-      </c>
-      <c r="AX2" t="inlineStr"/>
+maman|On prépare ton sac d'abord.
+papa|Tu mets quoi, Amir ?
+enfant-m|Je ne sais pas.
+maman|Demande. On t'aide.
+narrateur|Amir pose la main sur le sac.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1390,7 +1390,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>On peut mettre une pomme, un yaourt, ou un morceau de pain.</t>
+          <t>Pour le goûter, on peut choisir. Une pomme, un yaourt, ou un morceau de pain.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1558,10 +1558,10 @@
       <c r="AV3" s="2" t="inlineStr"/>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|On peut mettre une pomme, un yaourt, ou un morceau de pain.</t>
-        </is>
-      </c>
-      <c r="AX3" t="inlineStr"/>
+          <t>narrateur|Pour le goûter, on peut choisir.
+narrateur|Une pomme, un yaourt, ou un morceau de pain.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Dans la coupe, une pomme rouge brille. Elle sent le fruit. La peau est lisse et froide. La pomme dans le sac, Amir. La pomme. Amir la prend à deux mains. Il la glisse dans le sac. Le fond du sac fait un petit bruit. Bravo. Tu as mis ce que maman a dit. Tu as fini de mettre la pomme ? Oui. Amir appuie un peu. Ça sent encore le fruit.</t>
+          <t>Dans la coupe, une pomme rouge brille. Elle sent le fruit. Amir tend la main. La pomme roule sur la table. Il la rattrape contre son ventre. La peau est lisse et froide. Celle-là, dans le sac. La pomme. Amir la glisse au fond. Le sac fait un petit toc. Elle est bien au fond ? Oui. Ça sent encore le fruit.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1728,21 +1728,19 @@
         <is>
           <t>narrateur|Dans la coupe, une pomme rouge brille.
 narrateur|Elle sent le fruit.
+narrateur|Amir tend la main.
+narrateur|La pomme roule sur la table.
+narrateur|Il la rattrape contre son ventre.
 narrateur|La peau est lisse et froide.
-maman|La pomme dans le sac, Amir.
+maman|Celle-là, dans le sac.
 enfant-m|La pomme.
-narrateur|Amir la prend à deux mains.
-narrateur|Il la glisse dans le sac.
-narrateur|Le fond du sac fait un petit bruit.
-papa|Bravo.
-papa|Tu as mis ce que maman a dit.
-maman|Tu as fini de mettre la pomme ?
+narrateur|Amir la glisse au fond.
+narrateur|Le sac fait un petit toc.
+maman|Elle est bien au fond ?
 enfant-m|Oui.
-narrateur|Amir appuie un peu.
 narrateur|Ça sent encore le fruit.</t>
         </is>
       </c>
-      <c r="AX4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1782,27 +1780,27 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>le sac</t>
+          <t>la pomme</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>le sac | mettre | ce que l'adulte a dit</t>
+          <t>la pomme | une pomme | pomme | le fruit</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Oui, c'est la bonne réponse.</t>
+          <t>Oui.</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Tu étais presque.</t>
+          <t>C'est dans le sac. La pomme.</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Dis : le sac.</t>
+          <t>Dis : la pomme.</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr"/>
@@ -1930,7 +1928,6 @@
           <t>narrateur|On met quoi dans le sac ?</t>
         </is>
       </c>
-      <c r="AX5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1955,7 +1952,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Oui. On met dans le sac ce que maman a dit. Amir regarde la pomme dans le sac. Bravo, Amir. Tu as écouté. C'est du bon travail. Le sac a ce que l'adulte a dit. La pomme est dedans. On continue ensemble ? Oui.</t>
+          <t>La pomme est dans le sac. Elle fait un petit rond. Amir touche la fermeture. Pas encore. Il manque encore des choses. Quoi ? On va voir ensemble.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -2099,19 +2096,15 @@
       </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Oui.
-narrateur|On met dans le sac ce que maman a dit.
-narrateur|Amir regarde la pomme dans le sac.
-maman|Bravo, Amir.
-maman|Tu as écouté.
-papa|C'est du bon travail.
-papa|Le sac a ce que l'adulte a dit.
-enfant-m|La pomme est dedans.
-maman|On continue ensemble ?
-enfant-m|Oui.</t>
-        </is>
-      </c>
-      <c r="AX6" t="inlineStr"/>
+          <t>narrateur|La pomme est dans le sac.
+narrateur|Elle fait un petit rond.
+narrateur|Amir touche la fermeture.
+maman|Pas encore.
+maman|Il manque encore des choses.
+enfant-m|Quoi ?
+maman|On va voir ensemble.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2136,7 +2129,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>On peut aller dans la cuisine, le jardin, ou la chambre.</t>
+          <t>On peut aller où ? La cuisine, le jardin, ou la chambre.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -2300,10 +2293,10 @@
       <c r="AV7" s="2" t="inlineStr"/>
       <c r="AW7" t="inlineStr">
         <is>
-          <t>narrateur|On peut aller dans la cuisine, le jardin, ou la chambre.</t>
-        </is>
-      </c>
-      <c r="AX7" t="inlineStr"/>
+          <t>narrateur|On peut aller où ?
+narrateur|La cuisine, le jardin, ou la chambre.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2328,7 +2321,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Amir emporte le sac vers la cuisine. Le carrelage est un peu froid. La soupe fume encore dans la casserole. La petite serviette, Amir. On la met dans le sac. La serviette. Elle est douce et pliée. Amir la glisse près de la pomme. Bravo. Tu as mis ce que maman a dit. Une miette reste sur la table. On la ramasse après le jeu.</t>
+          <t>Amir emporte le sac vers la cuisine. Le carrelage est un peu froid. La soupe fume encore dans la casserole. Une serviette dépasse sous une cuillère. Amir tire le coin tout doux. La petite serviette, dans le sac. La serviette. Elle est douce et pliée. Il la glisse près de la pomme. Tu as fini de la mettre ? Oui, maman. Une miette reste sur la table.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -2471,18 +2464,17 @@
           <t>narrateur|Amir emporte le sac vers la cuisine.
 narrateur|Le carrelage est un peu froid.
 narrateur|La soupe fume encore dans la casserole.
-maman|La petite serviette, Amir.
-maman|On la met dans le sac.
+narrateur|Une serviette dépasse sous une cuillère.
+narrateur|Amir tire le coin tout doux.
+maman|La petite serviette, dans le sac.
 enfant-m|La serviette.
 narrateur|Elle est douce et pliée.
-narrateur|Amir la glisse près de la pomme.
-papa|Bravo.
-papa|Tu as mis ce que maman a dit.
-narrateur|Une miette reste sur la table.
-maman|On la ramasse après le jeu.</t>
-        </is>
-      </c>
-      <c r="AX8" t="inlineStr"/>
+narrateur|Il la glisse près de la pomme.
+maman|Tu as fini de la mettre ?
+enfant-m|Oui, maman.
+narrateur|Une miette reste sur la table.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2507,7 +2499,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre les cubes, le livre, ou la dînette.</t>
+          <t>On peut prendre quoi ? Les cubes, le livre, ou la dînette.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -2671,10 +2663,10 @@
       <c r="AV9" s="2" t="inlineStr"/>
       <c r="AW9" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre les cubes, le livre, ou la dînette.</t>
-        </is>
-      </c>
-      <c r="AX9" t="inlineStr"/>
+          <t>narrateur|On peut prendre quoi ?
+narrateur|Les cubes, le livre, ou la dînette.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2699,7 +2691,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Les cubes bleus attendent près de l'assiette. Ils tapent un peu sur le bois. Deux cubes dans le sac, Amir. Deux cubes. Amir les empile, puis les glisse près de la pomme. Bravo. Tu as mis ce que maman a dit. La soupe fume encore, tout doux. On jouera aux cubes plus tard. D'accord.</t>
+          <t>Les cubes bleus attendent près de l'assiette. Ils tapent un peu sur le bois. Amir en empile deux. La tour penche vers la pomme. Deux cubes dans le sac. Deux cubes. Il défait la tour tout doux. Il les glisse près de la pomme. Ils tiennent ? Ils tiennent.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -2841,17 +2833,16 @@
         <is>
           <t>narrateur|Les cubes bleus attendent près de l'assiette.
 narrateur|Ils tapent un peu sur le bois.
-maman|Deux cubes dans le sac, Amir.
+narrateur|Amir en empile deux.
+narrateur|La tour penche vers la pomme.
+maman|Deux cubes dans le sac.
 enfant-m|Deux cubes.
-narrateur|Amir les empile, puis les glisse près de la pomme.
-papa|Bravo.
-papa|Tu as mis ce que maman a dit.
-narrateur|La soupe fume encore, tout doux.
-maman|On jouera aux cubes plus tard.
-enfant-m|D'accord.</t>
-        </is>
-      </c>
-      <c r="AX10" t="inlineStr"/>
+narrateur|Il défait la tour tout doux.
+narrateur|Il les glisse près de la pomme.
+papa|Ils tiennent ?
+enfant-m|Ils tiennent.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2876,7 +2867,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Amir ferme le sac. Ça fait zzz. Le sac est prêt. Bravo, Amir. Tu as fait du bon travail. Merci. La cuisine sent encore la soupe. L'histoire est finie.</t>
+          <t>Amir ferme le sac près de la table. Ça fait zzz. Le sac est prêt. On peut jouer ? Oui. Les cubes, après. Amir sort un cube. Il le pose sur la table. Toc. La cuisine sent encore la soupe. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -3016,17 +3007,18 @@
       <c r="AV11" s="2" t="inlineStr"/>
       <c r="AW11" t="inlineStr">
         <is>
-          <t>narrateur|Amir ferme le sac.
+          <t>narrateur|Amir ferme le sac près de la table.
 narrateur|Ça fait zzz.
 papa|Le sac est prêt.
-maman|Bravo, Amir.
-maman|Tu as fait du bon travail.
-enfant-m|Merci.
+enfant-m|On peut jouer ?
+maman|Oui. Les cubes, après.
+narrateur|Amir sort un cube.
+narrateur|Il le pose sur la table.
+narrateur|Toc.
 narrateur|La cuisine sent encore la soupe.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3051,7 +3043,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Un petit livre est posé près du sel. Les pages sentent le papier. Le livre dans le sac, Amir. Le livre. Amir le glisse à plat, près de la pomme. Bravo. Tu as mis ce que papa a dit. Une farine légère reste sur la table. On essuie après. Le livre est dedans.</t>
+          <t>Un petit livre est posé près du sel. Les pages sentent le papier. Une page colle un peu. Amir souffle dessus. Le livre, à plat dans le sac. Le livre. Il le glisse près de la pomme. Il est à plat ? À plat.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -3193,17 +3185,15 @@
         <is>
           <t>narrateur|Un petit livre est posé près du sel.
 narrateur|Les pages sentent le papier.
-papa|Le livre dans le sac, Amir.
+narrateur|Une page colle un peu.
+narrateur|Amir souffle dessus.
+papa|Le livre, à plat dans le sac.
 enfant-m|Le livre.
-narrateur|Amir le glisse à plat, près de la pomme.
-maman|Bravo.
-maman|Tu as mis ce que papa a dit.
-narrateur|Une farine légère reste sur la table.
-papa|On essuie après.
-enfant-m|Le livre est dedans.</t>
-        </is>
-      </c>
-      <c r="AX12" t="inlineStr"/>
+narrateur|Il le glisse près de la pomme.
+papa|Il est à plat ?
+enfant-m|À plat.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3228,7 +3218,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Amir appuie sur la fermeture. Tu as mis le livre. Et la pomme. C'est ce que l'adulte a dit. Le sac est prêt. Bravo. Ils restent un moment près de la table. L'histoire est finie.</t>
+          <t>Amir appuie sur la fermeture. Tu as mis le livre. Et la pomme. Le sac est prêt. On ouvre juste la couverture ? Oui. Amir montre un bateau sur la page. Puis il referme le sac. Ils restent un moment près de la table. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -3371,14 +3361,15 @@
           <t>narrateur|Amir appuie sur la fermeture.
 maman|Tu as mis le livre.
 papa|Et la pomme.
-maman|C'est ce que l'adulte a dit.
 enfant-m|Le sac est prêt.
-papa|Bravo.
+maman|On ouvre juste la couverture ?
+enfant-m|Oui.
+narrateur|Amir montre un bateau sur la page.
+narrateur|Puis il referme le sac.
 narrateur|Ils restent un moment près de la table.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3403,7 +3394,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>La petite tasse de dînette cliquette. Elle est rouge, près de l'évier. La tasse dans le sac, Amir. La tasse. Amir la pose tout doux près de la pomme. Bravo. Tu as mis ce que maman a dit. Ça sonne comme un tout petit verre. On fera la dînette après le goûter. Oui, maman.</t>
+          <t>La petite tasse de dînette cliquette. Elle est rouge, près de l'évier. Une goutte brille au fond. Amir la verse dans l'évier. La tasse, dans le sac. La tasse. Il la pose tout doux près de la pomme. Ça sonne comme un tout petit verre. On fera la dînette après. Oui, maman.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -3545,17 +3536,16 @@
         <is>
           <t>narrateur|La petite tasse de dînette cliquette.
 narrateur|Elle est rouge, près de l'évier.
-maman|La tasse dans le sac, Amir.
+narrateur|Une goutte brille au fond.
+narrateur|Amir la verse dans l'évier.
+maman|La tasse, dans le sac.
 enfant-m|La tasse.
-narrateur|Amir la pose tout doux près de la pomme.
-papa|Bravo.
-papa|Tu as mis ce que maman a dit.
+narrateur|Il la pose tout doux près de la pomme.
 narrateur|Ça sonne comme un tout petit verre.
-maman|On fera la dînette après le goûter.
+maman|On fera la dînette après.
 enfant-m|Oui, maman.</t>
         </is>
       </c>
-      <c r="AX14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3580,7 +3570,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Le sac a la pomme et la tasse. Bravo, Amir. Tu as écouté. Merci, papa. Une goutte tombe dans l'évier. On va jouer. L'histoire est finie.</t>
+          <t>Le sac a la pomme et la tasse. Amir le serre contre lui. On va jouer ? Oui. Il sort la tasse. Il fait semblant de boire. À plus tard, petite tasse. Une goutte tombe dans l'évier. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -3721,15 +3711,16 @@
       <c r="AW15" t="inlineStr">
         <is>
           <t>narrateur|Le sac a la pomme et la tasse.
-maman|Bravo, Amir.
-papa|Tu as écouté.
-enfant-m|Merci, papa.
+narrateur|Amir le serre contre lui.
+papa|On va jouer ?
+enfant-m|Oui.
+narrateur|Il sort la tasse.
+narrateur|Il fait semblant de boire.
+maman|À plus tard, petite tasse.
 narrateur|Une goutte tombe dans l'évier.
-maman|On va jouer.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3754,7 +3745,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Amir pousse la porte du jardin. L'herbe est encore mouillée. Une feuille colle à sa chaussette. Le petit linge, Amir. On le met dans le sac. Le linge. Le linge sent l'air frais. Amir le pose près de la pomme. Bravo. Tu as mis ce que papa a dit. Un oiseau chante sur le mur. Tu as entendu l'oiseau ? Oui, papa.</t>
+          <t>Amir pousse la porte du jardin. L'herbe est encore mouillée. Une feuille colle à sa chaussette. Un petit linge sèche sur le banc. Le petit linge, Amir. On le met dans le sac. Le linge. Le linge sent l'air frais. Amir le pose près de la pomme. Un oiseau chante sur le mur. Tu as entendu l'oiseau ? Oui, papa.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -3897,19 +3888,17 @@
           <t>narrateur|Amir pousse la porte du jardin.
 narrateur|L'herbe est encore mouillée.
 narrateur|Une feuille colle à sa chaussette.
+narrateur|Un petit linge sèche sur le banc.
 papa|Le petit linge, Amir.
 papa|On le met dans le sac.
 enfant-m|Le linge.
 narrateur|Le linge sent l'air frais.
 narrateur|Amir le pose près de la pomme.
-maman|Bravo.
-maman|Tu as mis ce que papa a dit.
 narrateur|Un oiseau chante sur le mur.
 papa|Tu as entendu l'oiseau ?
 enfant-m|Oui, papa.</t>
         </is>
       </c>
-      <c r="AX16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3934,7 +3923,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre les cubes, le livre, ou la dînette.</t>
+          <t>On peut prendre quoi ? Les cubes, le livre, ou la dînette.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -4098,10 +4087,10 @@
       <c r="AV17" s="2" t="inlineStr"/>
       <c r="AW17" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre les cubes, le livre, ou la dînette.</t>
-        </is>
-      </c>
-      <c r="AX17" t="inlineStr"/>
+          <t>narrateur|On peut prendre quoi ?
+narrateur|Les cubes, le livre, ou la dînette.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -4126,7 +4115,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Les cubes sont sur la pierre chaude. Ils sentent un peu le soleil. Un cube dans le sac, Amir. Un cube. Amir l'essuie sur son pantalon. Il le met près de la pomme. Bravo. Tu as mis ce que papa a dit. Une abeille passe, tout loin. On laisse l'abeille au jardin.</t>
+          <t>Les cubes sont sur la pierre chaude. Ils sentent un peu le soleil. Un cube a une goutte dessus. Amir l'essuie sur son pantalon. Un cube dans le sac. Un cube. Il le met près de la pomme. Une abeille passe, tout loin. On laisse l'abeille au jardin.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -4268,17 +4257,15 @@
         <is>
           <t>narrateur|Les cubes sont sur la pierre chaude.
 narrateur|Ils sentent un peu le soleil.
-papa|Un cube dans le sac, Amir.
+narrateur|Un cube a une goutte dessus.
+narrateur|Amir l'essuie sur son pantalon.
+papa|Un cube dans le sac.
 enfant-m|Un cube.
-narrateur|Amir l'essuie sur son pantalon.
 narrateur|Il le met près de la pomme.
-maman|Bravo.
-maman|Tu as mis ce que papa a dit.
 narrateur|Une abeille passe, tout loin.
 papa|On laisse l'abeille au jardin.</t>
         </is>
       </c>
-      <c r="AX18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -4303,7 +4290,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Amir referme le sac sur l'herbe. Bravo. Le sac a ce que l'adulte a dit. Merci. La feuille reste collée à la chaussette. On l'enlève à la maison. L'histoire est finie.</t>
+          <t>Amir referme le sac sur l'herbe. C'est prêt. On enlève la feuille, d'abord. Amir ôte la feuille de sa chaussette. Il sort le cube. Il le pose sur la pierre. On rentre quand tu veux. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -4444,15 +4431,15 @@
       <c r="AW19" t="inlineStr">
         <is>
           <t>narrateur|Amir referme le sac sur l'herbe.
-papa|Bravo.
-maman|Le sac a ce que l'adulte a dit.
-enfant-m|Merci.
-narrateur|La feuille reste collée à la chaussette.
-papa|On l'enlève à la maison.
+enfant-m|C'est prêt.
+papa|On enlève la feuille, d'abord.
+narrateur|Amir ôte la feuille de sa chaussette.
+narrateur|Il sort le cube.
+narrateur|Il le pose sur la pierre.
+maman|On rentre quand tu veux.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -4477,7 +4464,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Le livre est à l'ombre, sous le banc. L'herbe chatouille les chevilles. Le livre dans le sac, Amir. Le livre. Les pages sont un peu fraîches. Amir le glisse près de la pomme. Bravo. Tu as mis ce que maman a dit. On lira plus tard, au calme. D'accord.</t>
+          <t>Le livre est à l'ombre, sous le banc. L'herbe chatouille les chevilles. Amir se penche. Les pages sont un peu fraîches. Le livre dans le sac, Amir. Le livre. Il le glisse près de la pomme. On lira plus tard, au calme. D'accord.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -4619,17 +4606,15 @@
         <is>
           <t>narrateur|Le livre est à l'ombre, sous le banc.
 narrateur|L'herbe chatouille les chevilles.
+narrateur|Amir se penche.
+narrateur|Les pages sont un peu fraîches.
 maman|Le livre dans le sac, Amir.
 enfant-m|Le livre.
-narrateur|Les pages sont un peu fraîches.
-narrateur|Amir le glisse près de la pomme.
-papa|Bravo.
-papa|Tu as mis ce que maman a dit.
+narrateur|Il le glisse près de la pomme.
 maman|On lira plus tard, au calme.
 enfant-m|D'accord.</t>
         </is>
       </c>
-      <c r="AX20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -4654,7 +4639,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Le sac est posé sur le banc. Bravo, Amir. Tu as fait du bon travail. Le livre est dedans. Un oiseau s'envole du mur. On rentre avec le sac. L'histoire est finie.</t>
+          <t>Le sac est posé sur le banc. Amir ouvre un tout petit coin. Il regarde une page. On rentre avec le sac. Oui. Un oiseau s'envole du mur. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -4795,15 +4780,14 @@
       <c r="AW21" t="inlineStr">
         <is>
           <t>narrateur|Le sac est posé sur le banc.
-maman|Bravo, Amir.
-papa|Tu as fait du bon travail.
-enfant-m|Le livre est dedans.
+narrateur|Amir ouvre un tout petit coin.
+narrateur|Il regarde une page.
+papa|On rentre avec le sac.
+enfant-m|Oui.
 narrateur|Un oiseau s'envole du mur.
-maman|On rentre avec le sac.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -4828,7 +4812,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>La dînette est sur un linge, dans l'herbe. Une assiette minuscule brille. L'assiette dans le sac, Amir. L'assiette. Amir la pose à plat près de la pomme. Bravo. Tu as mis ce que papa a dit. Le linge sent l'herbe mouillée. On plie le linge après. Oui, papa.</t>
+          <t>La dînette est sur un linge, dans l'herbe. Une assiette minuscule brille. Une feuille sèche est posée dessus. Amir enlève la feuille. L'assiette dans le sac, Amir. L'assiette. Il la pose à plat près de la pomme. Elle est à plat ? Oui.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -4970,17 +4954,15 @@
         <is>
           <t>narrateur|La dînette est sur un linge, dans l'herbe.
 narrateur|Une assiette minuscule brille.
-papa|L'assiette dans le sac, Amir.
+narrateur|Une feuille sèche est posée dessus.
+narrateur|Amir enlève la feuille.
+maman|L'assiette dans le sac, Amir.
 enfant-m|L'assiette.
-narrateur|Amir la pose à plat près de la pomme.
-maman|Bravo.
-maman|Tu as mis ce que papa a dit.
-narrateur|Le linge sent l'herbe mouillée.
-papa|On plie le linge après.
-enfant-m|Oui, papa.</t>
-        </is>
-      </c>
-      <c r="AX22" t="inlineStr"/>
+narrateur|Il la pose à plat près de la pomme.
+papa|Elle est à plat ?
+enfant-m|Oui.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -5005,7 +4987,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Amir tient le sac contre lui. Le sac est prêt. Bravo. Merci, maman. Une goutte tombe de la gouttière. Plic ploc. L'histoire est finie.</t>
+          <t>Amir tient le sac contre lui. Le sac est prêt. On goûte la pomme dehors ? Après. Il sort l'assiette. Il pose la pomme dessus, un instant. Puis tout rentre dans le sac. Une goutte tombe de la gouttière. Plic ploc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -5146,15 +5128,17 @@
       <c r="AW23" t="inlineStr">
         <is>
           <t>narrateur|Amir tient le sac contre lui.
-papa|Le sac est prêt.
-maman|Bravo.
-enfant-m|Merci, maman.
+enfant-m|Le sac est prêt.
+maman|On goûte la pomme dehors ?
+enfant-m|Après.
+narrateur|Il sort l'assiette.
+narrateur|Il pose la pomme dessus, un instant.
+narrateur|Puis tout rentre dans le sac.
 narrateur|Une goutte tombe de la gouttière.
-papa|Plic ploc.
+narrateur|Plic ploc.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -5179,7 +5163,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Amir revient dans la chambre. Le tapis rayé est tiède. Le pull marine attend sur le lit. Le pull, Amir. On le met dans le sac. Le pull. Le pull est doux sous la main. Amir le tasse près de la pomme. Bravo. Tu as mis ce que maman a dit. Le volet claque encore un peu. On le ferme après.</t>
+          <t>Amir revient dans la chambre. Le tapis rayé est tiède. Le pull marine attend sur le lit. Amir essaie de le plier. Une manche dépasse. Le pull, dans le sac. Le pull. Il le tasse près de la pomme. La manche est rentrée ? Presque. Le volet claque encore un peu.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -5322,18 +5306,16 @@
           <t>narrateur|Amir revient dans la chambre.
 narrateur|Le tapis rayé est tiède.
 narrateur|Le pull marine attend sur le lit.
-maman|Le pull, Amir.
-maman|On le met dans le sac.
+narrateur|Amir essaie de le plier.
+narrateur|Une manche dépasse.
+papa|Le pull, dans le sac.
 enfant-m|Le pull.
-narrateur|Le pull est doux sous la main.
-narrateur|Amir le tasse près de la pomme.
-papa|Bravo.
-papa|Tu as mis ce que maman a dit.
-maman|Le volet claque encore un peu.
-papa|On le ferme après.</t>
-        </is>
-      </c>
-      <c r="AX24" t="inlineStr"/>
+narrateur|Il le tasse près de la pomme.
+papa|La manche est rentrée ?
+enfant-m|Presque.
+narrateur|Le volet claque encore un peu.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -5358,7 +5340,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre les cubes, le livre, ou la dînette.</t>
+          <t>On peut prendre quoi ? Les cubes, le livre, ou la dînette.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -5522,10 +5504,10 @@
       <c r="AV25" s="2" t="inlineStr"/>
       <c r="AW25" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre les cubes, le livre, ou la dînette.</t>
-        </is>
-      </c>
-      <c r="AX25" t="inlineStr"/>
+          <t>narrateur|On peut prendre quoi ?
+narrateur|Les cubes, le livre, ou la dînette.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -5550,7 +5532,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Les cubes sont sur le tapis rayé. Le bleu du tapis les cache un peu. Les cubes dans le sac, Amir. Les cubes. Ils tapent doucement contre le pull. Bravo. Tu as mis ce que maman a dit. Le rayon de soleil touche un cube rouge. Tu as vu la lumière ? Oui.</t>
+          <t>Les cubes sont sous la chaise. Un cube rouge a roulé loin. Amir rampe sur le tapis. Il rattrape le cube rouge. Les cubes dans le sac. Les cubes. Il les met près de la pomme. Tu as le rouge ? Oui.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -5690,19 +5672,17 @@
       <c r="AV26" s="2" t="inlineStr"/>
       <c r="AW26" t="inlineStr">
         <is>
-          <t>narrateur|Les cubes sont sur le tapis rayé.
-narrateur|Le bleu du tapis les cache un peu.
-maman|Les cubes dans le sac, Amir.
+          <t>narrateur|Les cubes sont sous la chaise.
+narrateur|Un cube rouge a roulé loin.
+narrateur|Amir rampe sur le tapis.
+narrateur|Il rattrape le cube rouge.
+maman|Les cubes dans le sac.
 enfant-m|Les cubes.
-narrateur|Ils tapent doucement contre le pull.
-papa|Bravo.
-papa|Tu as mis ce que maman a dit.
-narrateur|Le rayon de soleil touche un cube rouge.
-maman|Tu as vu la lumière ?
+narrateur|Il les met près de la pomme.
+maman|Tu as le rouge ?
 enfant-m|Oui.</t>
         </is>
       </c>
-      <c r="AX26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -5727,7 +5707,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Amir ferme le sac sur le tapis. Bravo, Amir. Tu as écouté. Le sac est prêt. Le volet jaune ne claque plus. On peut jouer maintenant. L'histoire est finie.</t>
+          <t>Amir ferme le sac au pied du lit. On peut jouer ? Oui. Sur le tapis. Amir sort deux cubes. Il les pose sur une rayure crème. Le tapis rayé est calme. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -5867,16 +5847,15 @@
       <c r="AV27" s="2" t="inlineStr"/>
       <c r="AW27" t="inlineStr">
         <is>
-          <t>narrateur|Amir ferme le sac sur le tapis.
-maman|Bravo, Amir.
-papa|Tu as écouté.
-enfant-m|Le sac est prêt.
-narrateur|Le volet jaune ne claque plus.
-maman|On peut jouer maintenant.
+          <t>narrateur|Amir ferme le sac au pied du lit.
+enfant-m|On peut jouer ?
+papa|Oui. Sur le tapis.
+narrateur|Amir sort deux cubes.
+narrateur|Il les pose sur une rayure crème.
+narrateur|Le tapis rayé est calme.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -5901,7 +5880,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Le livre est sous l'oreiller. L'oreiller est chaud. Le livre dans le sac, Amir. Le livre. Amir le tire tout doux. Il le glisse près de la pomme. Bravo. Tu as mis ce que papa a dit. La couverture retombe, toute ronde. On la lissera après.</t>
+          <t>Le livre est ouvert sur la commode. Une image montre un bateau. Amir le ferme tout doux. Le livre dans le sac, Amir. Le livre. Il le glisse près de la pomme. Le bateau est dedans aussi. Oui.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -6041,19 +6020,16 @@
       <c r="AV28" s="2" t="inlineStr"/>
       <c r="AW28" t="inlineStr">
         <is>
-          <t>narrateur|Le livre est sous l'oreiller.
-narrateur|L'oreiller est chaud.
+          <t>narrateur|Le livre est ouvert sur la commode.
+narrateur|Une image montre un bateau.
+narrateur|Amir le ferme tout doux.
 papa|Le livre dans le sac, Amir.
 enfant-m|Le livre.
-narrateur|Amir le tire tout doux.
 narrateur|Il le glisse près de la pomme.
-maman|Bravo.
-maman|Tu as mis ce que papa a dit.
-narrateur|La couverture retombe, toute ronde.
-papa|On la lissera après.</t>
-        </is>
-      </c>
-      <c r="AX28" t="inlineStr"/>
+papa|Le bateau est dedans aussi.
+enfant-m|Oui.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -6078,7 +6054,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Le sac repose au pied du lit. Bravo. C'est du bon travail. Merci. Le pull marine n'est plus sur le lit. Il est dans le sac, avec le livre. L'histoire est finie.</t>
+          <t>Le sac est sur la commode, une seconde. On va jouer ? Oui. Amir ouvre le sac. Il touche la couverture du livre. Le rayon de soleil a quitté le tapis. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -6218,16 +6194,15 @@
       <c r="AV29" s="2" t="inlineStr"/>
       <c r="AW29" t="inlineStr">
         <is>
-          <t>narrateur|Le sac repose au pied du lit.
-papa|Bravo.
-maman|C'est du bon travail.
-enfant-m|Merci.
-narrateur|Le pull marine n'est plus sur le lit.
-papa|Il est dans le sac, avec le livre.
+          <t>narrateur|Le sac est sur la commode, une seconde.
+maman|On va jouer ?
+enfant-m|Oui.
+narrateur|Amir ouvre le sac.
+narrateur|Il touche la couverture du livre.
+narrateur|Le rayon de soleil a quitté le tapis.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -6252,7 +6227,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>La dînette est sur la couverture. Une petite casserole roule un peu. La casserole dans le sac, Amir. La casserole. Amir la rattrape, puis la met près de la pomme. Bravo. Tu as mis ce que maman a dit. Ça sonne tout petit, dans le sac. On fera un goûter de dînette plus tard. Oui.</t>
+          <t>La dînette est dans la caisse, sous le lit. Une petite assiette dépasse. Amir tire l'assiette. Un couvercle tombe sur le tapis. Toc. L'assiette dans le sac. L'assiette. Il la met près de la pomme. Le couvercle, on le laisse. D'accord.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -6392,19 +6367,18 @@
       <c r="AV30" s="2" t="inlineStr"/>
       <c r="AW30" t="inlineStr">
         <is>
-          <t>narrateur|La dînette est sur la couverture.
-narrateur|Une petite casserole roule un peu.
-maman|La casserole dans le sac, Amir.
-enfant-m|La casserole.
-narrateur|Amir la rattrape, puis la met près de la pomme.
-papa|Bravo.
-papa|Tu as mis ce que maman a dit.
-narrateur|Ça sonne tout petit, dans le sac.
-maman|On fera un goûter de dînette plus tard.
-enfant-m|Oui.</t>
-        </is>
-      </c>
-      <c r="AX30" t="inlineStr"/>
+          <t>narrateur|La dînette est dans la caisse, sous le lit.
+narrateur|Une petite assiette dépasse.
+narrateur|Amir tire l'assiette.
+narrateur|Un couvercle tombe sur le tapis.
+narrateur|Toc.
+maman|L'assiette dans le sac.
+enfant-m|L'assiette.
+narrateur|Il la met près de la pomme.
+maman|Le couvercle, on le laisse.
+enfant-m|D'accord.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -6429,7 +6403,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Amir s'assoit près du sac. Bravo, Amir. Tu as mis ce que l'adulte a dit. La pomme est dedans. Le tapis est doux sous les genoux. On reste un moment. L'histoire est finie.</t>
+          <t>Amir s'assoit sur le tapis. Le sac est sur ses genoux. Le sac est prêt. Merci. Il sort l'assiette. Il y pose la pomme, pour rire. On va vraiment jouer, maintenant. La couverture retombe sur le lit. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -6569,16 +6543,17 @@
       <c r="AV31" s="2" t="inlineStr"/>
       <c r="AW31" t="inlineStr">
         <is>
-          <t>narrateur|Amir s'assoit près du sac.
-maman|Bravo, Amir.
-papa|Tu as mis ce que l'adulte a dit.
-enfant-m|La pomme est dedans.
-narrateur|Le tapis est doux sous les genoux.
-maman|On reste un moment.
+          <t>narrateur|Amir s'assoit sur le tapis.
+narrateur|Le sac est sur ses genoux.
+papa|Le sac est prêt.
+enfant-m|Merci.
+narrateur|Il sort l'assiette.
+narrateur|Il y pose la pomme, pour rire.
+maman|On va vraiment jouer, maintenant.
+narrateur|La couverture retombe sur le lit.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -6603,7 +6578,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Papa ouvre le frigo. Un air frais sort. Un petit yaourt attend sur la tablette. Le yaourt dans le sac, Amir. Le yaourt. Le pot est frais sous les doigts. Amir le pose dans le sac. Le sac se creuse un peu. Bravo. Tu as mis ce que papa a dit. Tu as fini de mettre le yaourt ? Oui, papa. Amir referme un peu le sac.</t>
+          <t>Papa ouvre le frigo. Un air frais sort. Un petit yaourt attend sur la tablette. Papa le tend. Le couvercle glisse un peu. Amir le tient à deux mains. Tout doux. Dans le sac. Le yaourt. Amir le pose bien droit. Il tient ? Il tient. Le pot est froid contre le tissu.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -6746,19 +6721,17 @@
           <t>narrateur|Papa ouvre le frigo.
 narrateur|Un air frais sort.
 narrateur|Un petit yaourt attend sur la tablette.
-papa|Le yaourt dans le sac, Amir.
+narrateur|Papa le tend.
+narrateur|Le couvercle glisse un peu.
+narrateur|Amir le tient à deux mains.
+papa|Tout doux. Dans le sac.
 enfant-m|Le yaourt.
-narrateur|Le pot est frais sous les doigts.
-narrateur|Amir le pose dans le sac.
-narrateur|Le sac se creuse un peu.
-maman|Bravo.
-maman|Tu as mis ce que papa a dit.
-papa|Tu as fini de mettre le yaourt ?
-enfant-m|Oui, papa.
-narrateur|Amir referme un peu le sac.</t>
-        </is>
-      </c>
-      <c r="AX32" t="inlineStr"/>
+narrateur|Amir le pose bien droit.
+papa|Il tient ?
+enfant-m|Il tient.
+narrateur|Le pot est froid contre le tissu.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -6783,7 +6756,7 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Le sac : on met ce que l'adulte a dit ?</t>
+          <t>On met quoi dans le sac ?</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -6798,27 +6771,27 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>le sac</t>
+          <t>le yaourt</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>le sac | mettre | ce que l'adulte a dit</t>
+          <t>le yaourt | un yaourt | yaourt | le pot</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>Oui, c'est la bonne réponse.</t>
+          <t>Oui.</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Tu étais presque.</t>
+          <t>C'est dans le sac. Le yaourt.</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>Dis : le sac.</t>
+          <t>Dis : le yaourt.</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr"/>
@@ -6943,10 +6916,9 @@
       </c>
       <c r="AW33" t="inlineStr">
         <is>
-          <t>narrateur|Le sac : on met ce que l'adulte a dit ?</t>
-        </is>
-      </c>
-      <c r="AX33" t="inlineStr"/>
+          <t>narrateur|On met quoi dans le sac ?</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -6971,7 +6943,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Oui. On met dans le sac ce que papa a dit. Le yaourt reste au fond, bien droit. Bravo, Amir. Tu as écouté. C'est du bon travail. Le sac a ce que l'adulte a dit. Le yaourt est dedans. On continue ensemble ? Oui.</t>
+          <t>Le yaourt est au fond. Il est froid. Amir veut fermer le sac. On n'a pas fini. Il manque encore des choses. D'accord.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -7115,19 +7087,14 @@
       </c>
       <c r="AW34" t="inlineStr">
         <is>
-          <t>narrateur|Oui.
-narrateur|On met dans le sac ce que papa a dit.
-narrateur|Le yaourt reste au fond, bien droit.
-papa|Bravo, Amir.
-papa|Tu as écouté.
-maman|C'est du bon travail.
-maman|Le sac a ce que l'adulte a dit.
-enfant-m|Le yaourt est dedans.
-papa|On continue ensemble ?
-enfant-m|Oui.</t>
-        </is>
-      </c>
-      <c r="AX34" t="inlineStr"/>
+          <t>narrateur|Le yaourt est au fond.
+narrateur|Il est froid.
+narrateur|Amir veut fermer le sac.
+papa|On n'a pas fini.
+papa|Il manque encore des choses.
+enfant-m|D'accord.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -7152,7 +7119,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>On peut aller dans la cuisine, le jardin, ou la chambre.</t>
+          <t>On peut aller où ? La cuisine, le jardin, ou la chambre.</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -7316,10 +7283,10 @@
       <c r="AV35" s="2" t="inlineStr"/>
       <c r="AW35" t="inlineStr">
         <is>
-          <t>narrateur|On peut aller dans la cuisine, le jardin, ou la chambre.</t>
-        </is>
-      </c>
-      <c r="AX35" t="inlineStr"/>
+          <t>narrateur|On peut aller où ?
+narrateur|La cuisine, le jardin, ou la chambre.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -7344,7 +7311,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Amir pose le sac sur la table de la cuisine. Le yaourt reste bien droit. Le frigo ronronne tout bas. La cuillère, Amir. On la met dans le sac. La cuillère. Elle est lisse et froide. Amir la glisse à côté du yaourt. Bravo. Tu as mis ce que papa a dit. Ça sent encore la soupe. On goûtera plus tard.</t>
+          <t>Amir pose le sac sur la table. Le yaourt reste bien droit. Le frigo ronronne tout bas. Amir ouvre le tiroir du bas. Une petite cuillère brille. La cuillère, dans le sac. La cuillère. Elle est lisse et froide. Il la glisse à côté du yaourt. Elle est à côté ? Oui, papa. Ça sent encore la soupe.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -7484,21 +7451,20 @@
       <c r="AV36" s="2" t="inlineStr"/>
       <c r="AW36" t="inlineStr">
         <is>
-          <t>narrateur|Amir pose le sac sur la table de la cuisine.
+          <t>narrateur|Amir pose le sac sur la table.
 narrateur|Le yaourt reste bien droit.
 narrateur|Le frigo ronronne tout bas.
-papa|La cuillère, Amir.
-papa|On la met dans le sac.
+narrateur|Amir ouvre le tiroir du bas.
+narrateur|Une petite cuillère brille.
+papa|La cuillère, dans le sac.
 enfant-m|La cuillère.
 narrateur|Elle est lisse et froide.
-narrateur|Amir la glisse à côté du yaourt.
-maman|Bravo.
-maman|Tu as mis ce que papa a dit.
-narrateur|Ça sent encore la soupe.
-maman|On goûtera plus tard.</t>
-        </is>
-      </c>
-      <c r="AX36" t="inlineStr"/>
+narrateur|Il la glisse à côté du yaourt.
+papa|Elle est à côté ?
+enfant-m|Oui, papa.
+narrateur|Ça sent encore la soupe.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -7523,7 +7489,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre les cubes, le livre, ou la dînette.</t>
+          <t>On peut prendre quoi ? Les cubes, le livre, ou la dînette.</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -7687,10 +7653,10 @@
       <c r="AV37" s="2" t="inlineStr"/>
       <c r="AW37" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre les cubes, le livre, ou la dînette.</t>
-        </is>
-      </c>
-      <c r="AX37" t="inlineStr"/>
+          <t>narrateur|On peut prendre quoi ?
+narrateur|Les cubes, le livre, ou la dînette.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -7715,7 +7681,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Les cubes sont près du yaourt, sur la table. Le bois est lisse et un peu collant. Trois cubes dans le sac, Amir. Trois cubes. Amir les compte tout bas. Il les met près du yaourt. Bravo. Tu as mis ce que papa a dit. Le frigo ronronne encore. Tu as bien compté.</t>
+          <t>Les cubes sont près du saladier. Amir en prend trois. Il fait un petit pont. Le pont touche le yaourt. Les cubes, dans le sac. Pas le pont. Les cubes. Il les empile près du pot. Le pot est encore droit ? Droit.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -7855,19 +7821,17 @@
       <c r="AV38" s="2" t="inlineStr"/>
       <c r="AW38" t="inlineStr">
         <is>
-          <t>narrateur|Les cubes sont près du yaourt, sur la table.
-narrateur|Le bois est lisse et un peu collant.
-papa|Trois cubes dans le sac, Amir.
-enfant-m|Trois cubes.
-narrateur|Amir les compte tout bas.
-narrateur|Il les met près du yaourt.
-maman|Bravo.
-maman|Tu as mis ce que papa a dit.
-narrateur|Le frigo ronronne encore.
-papa|Tu as bien compté.</t>
-        </is>
-      </c>
-      <c r="AX38" t="inlineStr"/>
+          <t>narrateur|Les cubes sont près du saladier.
+narrateur|Amir en prend trois.
+narrateur|Il fait un petit pont.
+narrateur|Le pont touche le yaourt.
+maman|Les cubes, dans le sac. Pas le pont.
+enfant-m|Les cubes.
+narrateur|Il les empile près du pot.
+maman|Le pot est encore droit ?
+enfant-m|Droit.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -7892,7 +7856,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Amir ferme le sac près de l'évier. Bravo. Le yaourt et les cubes sont dedans. Merci, maman. Une cuillère brille encore sur la table. Elle aussi, on l'a mise. L'histoire est finie.</t>
+          <t>Amir ferme le sac près de l'évier. Le yaourt est encore droit ? Oui. On joue aux cubes ici. Amir sort deux cubes. Il les pose contre la cuillère. Toc, toc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -8033,15 +7997,15 @@
       <c r="AW39" t="inlineStr">
         <is>
           <t>narrateur|Amir ferme le sac près de l'évier.
-papa|Bravo.
-maman|Le yaourt et les cubes sont dedans.
-enfant-m|Merci, maman.
-narrateur|Une cuillère brille encore sur la table.
-papa|Elle aussi, on l'a mise.
+papa|Le yaourt est encore droit ?
+enfant-m|Oui.
+maman|On joue aux cubes ici.
+narrateur|Amir sort deux cubes.
+narrateur|Il les pose contre la cuillère.
+narrateur|Toc, toc.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -8066,7 +8030,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Le livre est contre le pot de farine. Une page est un peu cornée. Le livre dans le sac, Amir. Le livre. Amir le glisse à côté du yaourt. Bravo. Tu as mis ce que maman a dit. Ça sent le lait froid et le papier. On lira après le goûter. D'accord.</t>
+          <t>Le livre est sous un torchon. Le torchon sent le propre. Amir soulève le coin. Le livre dans le sac. Le livre. Il le sort du torchon. Il le glisse près du yaourt, à plat. Loin du pot froid. Loin.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -8206,19 +8170,17 @@
       <c r="AV40" s="2" t="inlineStr"/>
       <c r="AW40" t="inlineStr">
         <is>
-          <t>narrateur|Le livre est contre le pot de farine.
-narrateur|Une page est un peu cornée.
-maman|Le livre dans le sac, Amir.
+          <t>narrateur|Le livre est sous un torchon.
+narrateur|Le torchon sent le propre.
+narrateur|Amir soulève le coin.
+papa|Le livre dans le sac.
 enfant-m|Le livre.
-narrateur|Amir le glisse à côté du yaourt.
-papa|Bravo.
-papa|Tu as mis ce que maman a dit.
-narrateur|Ça sent le lait froid et le papier.
-maman|On lira après le goûter.
-enfant-m|D'accord.</t>
-        </is>
-      </c>
-      <c r="AX40" t="inlineStr"/>
+narrateur|Il le sort du torchon.
+narrateur|Il le glisse près du yaourt, à plat.
+papa|Loin du pot froid.
+enfant-m|Loin.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -8243,7 +8205,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Le sac est lourd d'un côté. Bravo, Amir. Tu as écouté. Le livre est dedans. La soupe ne fume plus. On peut jouer. L'histoire est finie.</t>
+          <t>Le sac est posé contre la chaise. On lit ? Une page. Puis on range. Amir ouvre le sac. Il montre la couverture à papa. On y va. Ça sent encore un peu le four. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -8383,16 +8345,16 @@
       <c r="AV41" s="2" t="inlineStr"/>
       <c r="AW41" t="inlineStr">
         <is>
-          <t>narrateur|Le sac est lourd d'un côté.
-maman|Bravo, Amir.
-papa|Tu as écouté.
-enfant-m|Le livre est dedans.
-narrateur|La soupe ne fume plus.
-maman|On peut jouer.
+          <t>narrateur|Le sac est posé contre la chaise.
+enfant-m|On lit ?
+maman|Une page. Puis on range.
+narrateur|Amir ouvre le sac.
+narrateur|Il montre la couverture à papa.
+papa|On y va.
+narrateur|Ça sent encore un peu le four.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -8417,7 +8379,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Une petite cuillère de dînette attend près de l'évier. Elle est jaune et légère. La petite cuillère dans le sac, Amir. La cuillère. Amir la pose près du vrai yaourt. Bravo. Tu as mis ce que papa a dit. Deux cuillères, une grande, une petite. On les a mises toutes les deux. Oui.</t>
+          <t>La dînette est dans le tiroir du haut. Une casserole minuscule brille. Amir ouvre le tiroir tout doux. La casserole dans le sac. La casserole. Il la met près du yaourt. Elle fait un tout petit cling. On fera la soupe pour de faux. Oui.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -8557,19 +8519,17 @@
       <c r="AV42" s="2" t="inlineStr"/>
       <c r="AW42" t="inlineStr">
         <is>
-          <t>narrateur|Une petite cuillère de dînette attend près de l'évier.
-narrateur|Elle est jaune et légère.
-papa|La petite cuillère dans le sac, Amir.
-enfant-m|La cuillère.
-narrateur|Amir la pose près du vrai yaourt.
-maman|Bravo.
-maman|Tu as mis ce que papa a dit.
-narrateur|Deux cuillères, une grande, une petite.
-papa|On les a mises toutes les deux.
+          <t>narrateur|La dînette est dans le tiroir du haut.
+narrateur|Une casserole minuscule brille.
+narrateur|Amir ouvre le tiroir tout doux.
+maman|La casserole dans le sac.
+enfant-m|La casserole.
+narrateur|Il la met près du yaourt.
+narrateur|Elle fait un tout petit cling.
+maman|On fera la soupe pour de faux.
 enfant-m|Oui.</t>
         </is>
       </c>
-      <c r="AX42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -8594,7 +8554,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Amir appuie sur la fermeture. Le sac est prêt. Bravo. Merci, papa. Le carrelage n'est plus si froid. On a bien travaillé. L'histoire est finie.</t>
+          <t>Amir tient la sangle du sac. Le sac est prêt. La casserole aussi. Il sort la casserole. Il fait semblant de remuer. La soupe de yaourt, c'est nouveau. Amir rit. La cuisine est calme. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -8734,16 +8694,17 @@
       <c r="AV43" s="2" t="inlineStr"/>
       <c r="AW43" t="inlineStr">
         <is>
-          <t>narrateur|Amir appuie sur la fermeture.
+          <t>narrateur|Amir tient la sangle du sac.
 papa|Le sac est prêt.
-maman|Bravo.
-enfant-m|Merci, papa.
-narrateur|Le carrelage n'est plus si froid.
-maman|On a bien travaillé.
+enfant-m|La casserole aussi.
+narrateur|Il sort la casserole.
+narrateur|Il fait semblant de remuer.
+maman|La soupe de yaourt, c'est nouveau.
+narrateur|Amir rit.
+narrateur|La cuisine est calme.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -8768,7 +8729,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Amir marche dans le jardin avec le sac. Le yaourt reste au fond, au frais. Un galet est encore chaud au soleil. Le petit gant, Amir. On le met dans le sac. Le gant. Le gant est un peu rêche. Amir le pose près du yaourt. Bravo. Tu as mis ce que maman a dit. Une goutte tombe de la gouttière. Plic ploc, tu as entendu ? Oui.</t>
+          <t>Amir marche dans le jardin avec le sac. Le yaourt reste au fond, au frais. Un galet est encore chaud au soleil. Un petit gant est posé dessus. Le petit gant, dans le sac. Le gant. Le gant est un peu rêche. Amir le pose près du yaourt. Une goutte tombe de la gouttière. Plic ploc. Tu as entendu ? Oui.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -8911,19 +8872,16 @@
           <t>narrateur|Amir marche dans le jardin avec le sac.
 narrateur|Le yaourt reste au fond, au frais.
 narrateur|Un galet est encore chaud au soleil.
-maman|Le petit gant, Amir.
-maman|On le met dans le sac.
+narrateur|Un petit gant est posé dessus.
+maman|Le petit gant, dans le sac.
 enfant-m|Le gant.
 narrateur|Le gant est un peu rêche.
 narrateur|Amir le pose près du yaourt.
-papa|Bravo.
-papa|Tu as mis ce que maman a dit.
 narrateur|Une goutte tombe de la gouttière.
-papa|Plic ploc, tu as entendu ?
+papa|Plic ploc. Tu as entendu ?
 enfant-m|Oui.</t>
         </is>
       </c>
-      <c r="AX44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -8948,7 +8906,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre les cubes, le livre, ou la dînette.</t>
+          <t>On peut prendre quoi ? Les cubes, le livre, ou la dînette.</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -9112,10 +9070,10 @@
       <c r="AV45" s="2" t="inlineStr"/>
       <c r="AW45" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre les cubes, le livre, ou la dînette.</t>
-        </is>
-      </c>
-      <c r="AX45" t="inlineStr"/>
+          <t>narrateur|On peut prendre quoi ?
+narrateur|Les cubes, le livre, ou la dînette.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -9140,7 +9098,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Les cubes sont dans l'herbe, près du galet. Un cube vert est un peu humide. Les cubes secs dans le sac, Amir. Les cubes secs. Amir choisit deux cubes secs. Il les met près du yaourt. Bravo. Tu as mis ce que maman a dit. Le galet reste au jardin. Le galet n'est pas pour le sac.</t>
+          <t>Les cubes sont dans l'herbe rase. Un cube a un peu d'herbe. Amir souffle dessus. Le cube propre, dans le sac. Le cube propre. Il le frotte, puis le met près du yaourt. On laisse l'herbe au jardin.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -9280,19 +9238,15 @@
       <c r="AV46" s="2" t="inlineStr"/>
       <c r="AW46" t="inlineStr">
         <is>
-          <t>narrateur|Les cubes sont dans l'herbe, près du galet.
-narrateur|Un cube vert est un peu humide.
-maman|Les cubes secs dans le sac, Amir.
-enfant-m|Les cubes secs.
-narrateur|Amir choisit deux cubes secs.
-narrateur|Il les met près du yaourt.
-papa|Bravo.
-papa|Tu as mis ce que maman a dit.
-narrateur|Le galet reste au jardin.
-maman|Le galet n'est pas pour le sac.</t>
-        </is>
-      </c>
-      <c r="AX46" t="inlineStr"/>
+          <t>narrateur|Les cubes sont dans l'herbe rase.
+narrateur|Un cube a un peu d'herbe.
+narrateur|Amir souffle dessus.
+papa|Le cube propre, dans le sac.
+enfant-m|Le cube propre.
+narrateur|Il le frotte, puis le met près du yaourt.
+papa|On laisse l'herbe au jardin.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -9317,7 +9271,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Amir essuie ses mains sur le linge. Bravo, Amir. Le sac a ce que l'adulte a dit. Merci. La gouttière fait encore plic ploc. On rentre. L'histoire est finie.</t>
+          <t>Amir referme le sac près du galet. Le yaourt est encore au frais ? Oui. Il sort le cube. Il le pose sur le galet chaud. On rentre. Le jardin sent l'herbe mouillée. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -9457,16 +9411,16 @@
       <c r="AV47" s="2" t="inlineStr"/>
       <c r="AW47" t="inlineStr">
         <is>
-          <t>narrateur|Amir essuie ses mains sur le linge.
-maman|Bravo, Amir.
-papa|Le sac a ce que l'adulte a dit.
-enfant-m|Merci.
-narrateur|La gouttière fait encore plic ploc.
+          <t>narrateur|Amir referme le sac près du galet.
+maman|Le yaourt est encore au frais ?
+enfant-m|Oui.
+narrateur|Il sort le cube.
+narrateur|Il le pose sur le galet chaud.
 papa|On rentre.
+narrateur|Le jardin sent l'herbe mouillée.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -9491,7 +9445,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Le livre est sur le muret, au soleil. La couverture est un peu chaude. Le livre dans le sac, Amir. Le livre. Amir le souffle, puis le glisse près du yaourt. Bravo. Tu as mis ce que papa a dit. Une fourmi passe sur le muret. On laisse la fourmi. Oui, papa.</t>
+          <t>Le livre est sur le muret, au soleil. La couverture est un peu chaude. Amir le souffle. Le livre dans le sac. Le livre. Il le glisse près du yaourt. Pas collé au pot froid. Pas collé.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -9633,17 +9587,14 @@
         <is>
           <t>narrateur|Le livre est sur le muret, au soleil.
 narrateur|La couverture est un peu chaude.
-papa|Le livre dans le sac, Amir.
+narrateur|Amir le souffle.
+maman|Le livre dans le sac.
 enfant-m|Le livre.
-narrateur|Amir le souffle, puis le glisse près du yaourt.
-maman|Bravo.
-maman|Tu as mis ce que papa a dit.
-narrateur|Une fourmi passe sur le muret.
-papa|On laisse la fourmi.
-enfant-m|Oui, papa.</t>
-        </is>
-      </c>
-      <c r="AX48" t="inlineStr"/>
+narrateur|Il le glisse près du yaourt.
+maman|Pas collé au pot froid.
+enfant-m|Pas collé.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -9668,7 +9619,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Le sac est posé sur le muret. Bravo. Tu as fait du bon travail. Le livre est dedans. Le vent est doux dans les cheveux. On rentre avec le sac. L'histoire est finie.</t>
+          <t>Le sac est posé sur le muret. Une page ? Une page. Le vent est doux. Amir ouvre le livre. Une page tremble. Il referme, puis le sac. On rentre avec le sac. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -9809,15 +9760,15 @@
       <c r="AW49" t="inlineStr">
         <is>
           <t>narrateur|Le sac est posé sur le muret.
-papa|Bravo.
-maman|Tu as fait du bon travail.
-enfant-m|Le livre est dedans.
-narrateur|Le vent est doux dans les cheveux.
-maman|On rentre avec le sac.
+enfant-m|Une page ?
+papa|Une page. Le vent est doux.
+narrateur|Amir ouvre le livre.
+narrateur|Une page tremble.
+narrateur|Il referme, puis le sac.
+narrateur|On rentre avec le sac.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -9842,7 +9793,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Une tasse de dînette est retournée dans l'herbe. Une goutte d'eau brille dedans. La tasse dans le sac, Amir. La tasse. Amir la vide, puis la met près du yaourt. Bravo. Tu as mis ce que maman a dit. L'herbe reste collée un instant. On l'enlève d'un doigt. C'est fait.</t>
+          <t>Une tasse de dînette est retournée dans l'herbe. Une goutte d'eau brille dedans. Amir la vide sur l'herbe. La tasse dans le sac. La tasse. Il la met près du yaourt. Elle est vide ? Vide.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -9984,17 +9935,14 @@
         <is>
           <t>narrateur|Une tasse de dînette est retournée dans l'herbe.
 narrateur|Une goutte d'eau brille dedans.
-maman|La tasse dans le sac, Amir.
+narrateur|Amir la vide sur l'herbe.
+papa|La tasse dans le sac.
 enfant-m|La tasse.
-narrateur|Amir la vide, puis la met près du yaourt.
-papa|Bravo.
-papa|Tu as mis ce que maman a dit.
-narrateur|L'herbe reste collée un instant.
-maman|On l'enlève d'un doigt.
-enfant-m|C'est fait.</t>
-        </is>
-      </c>
-      <c r="AX50" t="inlineStr"/>
+narrateur|Il la met près du yaourt.
+papa|Elle est vide ?
+enfant-m|Vide.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -10019,7 +9967,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Amir tient le sac à deux mains. Bravo, Amir. Tu as écouté. Merci. Le jardin sent l'herbe mouillée. On rentre. L'histoire est finie.</t>
+          <t>Amir tient le sac à deux mains. On rentre. La tasse aussi. Il fait un tout petit clin. Tasse contre yaourt. Santé, tout doux. Le jardin sent l'herbe mouillée. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -10160,15 +10108,15 @@
       <c r="AW51" t="inlineStr">
         <is>
           <t>narrateur|Amir tient le sac à deux mains.
-maman|Bravo, Amir.
-papa|Tu as écouté.
-enfant-m|Merci.
+maman|On rentre.
+enfant-m|La tasse aussi.
+narrateur|Il fait un tout petit clin.
+narrateur|Tasse contre yaourt.
+papa|Santé, tout doux.
 narrateur|Le jardin sent l'herbe mouillée.
-papa|On rentre.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -10193,7 +10141,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Amir s'assoit sur le tapis de la chambre. Le yaourt fait un petit rond dans le sac. La couverture est douce contre le genou. Les chaussons, Amir. On les met dans le sac. Les chaussons. Ils sont chauds et mous. Amir les glisse près du yaourt. Bravo. Tu as mis ce que papa a dit. Le rayon de soleil a bougé. Il touche maintenant le sac.</t>
+          <t>Amir s'assoit sur le tapis de la chambre. Le yaourt fait un petit rond dans le sac. La couverture est douce contre le genou. Un chausson dépasse sous le lit. Amir tire les deux chaussons. Les chaussons, dans le sac. Les chaussons. Ils sont chauds et mous. Il les glisse près du yaourt. Le rayon de soleil a bougé. Il touche maintenant le sac.</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -10336,18 +10284,16 @@
           <t>narrateur|Amir s'assoit sur le tapis de la chambre.
 narrateur|Le yaourt fait un petit rond dans le sac.
 narrateur|La couverture est douce contre le genou.
-papa|Les chaussons, Amir.
-papa|On les met dans le sac.
+narrateur|Un chausson dépasse sous le lit.
+narrateur|Amir tire les deux chaussons.
+papa|Les chaussons, dans le sac.
 enfant-m|Les chaussons.
 narrateur|Ils sont chauds et mous.
-narrateur|Amir les glisse près du yaourt.
-maman|Bravo.
-maman|Tu as mis ce que papa a dit.
+narrateur|Il les glisse près du yaourt.
 narrateur|Le rayon de soleil a bougé.
-maman|Il touche maintenant le sac.</t>
-        </is>
-      </c>
-      <c r="AX52" t="inlineStr"/>
+narrateur|Il touche maintenant le sac.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -10372,7 +10318,7 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre les cubes, le livre, ou la dînette.</t>
+          <t>On peut prendre quoi ? Les cubes, le livre, ou la dînette.</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -10536,10 +10482,10 @@
       <c r="AV53" s="2" t="inlineStr"/>
       <c r="AW53" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre les cubes, le livre, ou la dînette.</t>
-        </is>
-      </c>
-      <c r="AX53" t="inlineStr"/>
+          <t>narrateur|On peut prendre quoi ?
+narrateur|Les cubes, le livre, ou la dînette.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -10564,7 +10510,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Les cubes sont sous la chaise, dans la chambre. Un cube rouge a roulé loin. Les cubes dans le sac, Amir. Les cubes. Amir ramasse le cube rouge. Il les met près du yaourt. Bravo. Tu as mis ce que papa a dit. La chaise ne bouge plus. Tu as tout retrouvé.</t>
+          <t>Les cubes sont derrière le coffre. Amir pousse le coffre d'un doigt. Deux cubes apparaissent. Les cubes dans le sac. Les cubes. Il les met près du yaourt. Loin du pot, un peu. Loin.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -10704,19 +10650,16 @@
       <c r="AV54" s="2" t="inlineStr"/>
       <c r="AW54" t="inlineStr">
         <is>
-          <t>narrateur|Les cubes sont sous la chaise, dans la chambre.
-narrateur|Un cube rouge a roulé loin.
-papa|Les cubes dans le sac, Amir.
+          <t>narrateur|Les cubes sont derrière le coffre.
+narrateur|Amir pousse le coffre d'un doigt.
+narrateur|Deux cubes apparaissent.
+maman|Les cubes dans le sac.
 enfant-m|Les cubes.
-narrateur|Amir ramasse le cube rouge.
 narrateur|Il les met près du yaourt.
-maman|Bravo.
-maman|Tu as mis ce que papa a dit.
-narrateur|La chaise ne bouge plus.
-papa|Tu as tout retrouvé.</t>
-        </is>
-      </c>
-      <c r="AX54" t="inlineStr"/>
+maman|Loin du pot, un peu.
+enfant-m|Loin.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -10741,7 +10684,7 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Amir ferme le sac au pied du lit. Bravo. Les chaussons et les cubes sont dedans. Le sac est prêt. Le tapis rayé est calme. On peut jouer. L'histoire est finie.</t>
+          <t>Amir ferme le sac au pied du lit. Les chaussons et les cubes sont dedans. Le sac est prêt. Il sort un cube. Il le fait rouler sur une rayure bleue. On peut jouer. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -10882,15 +10825,14 @@
       <c r="AW55" t="inlineStr">
         <is>
           <t>narrateur|Amir ferme le sac au pied du lit.
-papa|Bravo.
-maman|Les chaussons et les cubes sont dedans.
+papa|Les chaussons et les cubes sont dedans.
 enfant-m|Le sac est prêt.
-narrateur|Le tapis rayé est calme.
+narrateur|Il sort un cube.
+narrateur|Il le fait rouler sur une rayure bleue.
 maman|On peut jouer.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -10915,7 +10857,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Le livre est ouvert sur la commode. Une image montre un bateau. Le livre dans le sac, Amir. Le livre. Amir le ferme tout doux. Il le glisse près du yaourt. Bravo. Tu as mis ce que maman a dit. Le bateau disparaît entre les pages. On le reverra plus tard.</t>
+          <t>Le livre est coincé entre deux peluches. Amir le tire tout doux. Le livre dans le sac. Le livre. Il le glisse près du yaourt. Les peluches restent au lit. D'accord.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -11055,19 +10997,15 @@
       <c r="AV56" s="2" t="inlineStr"/>
       <c r="AW56" t="inlineStr">
         <is>
-          <t>narrateur|Le livre est ouvert sur la commode.
-narrateur|Une image montre un bateau.
-maman|Le livre dans le sac, Amir.
+          <t>narrateur|Le livre est coincé entre deux peluches.
+narrateur|Amir le tire tout doux.
+papa|Le livre dans le sac.
 enfant-m|Le livre.
-narrateur|Amir le ferme tout doux.
 narrateur|Il le glisse près du yaourt.
-papa|Bravo.
-papa|Tu as mis ce que maman a dit.
-narrateur|Le bateau disparaît entre les pages.
-maman|On le reverra plus tard.</t>
-        </is>
-      </c>
-      <c r="AX56" t="inlineStr"/>
+papa|Les peluches restent au lit.
+enfant-m|D'accord.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -11092,7 +11030,7 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Le sac est sur la commode, une seconde. Bravo, Amir. C'est du bon travail. Merci, papa. Le rayon de soleil a quitté le tapis. On va jouer. L'histoire est finie.</t>
+          <t>Le sac attend près de la porte. Merci, papa. On lit sur le tapis ? Amir s'assoit. Il ouvre le livre sur ses genoux. Le rayon de soleil a quitté le tapis. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -11232,16 +11170,15 @@
       <c r="AV57" s="2" t="inlineStr"/>
       <c r="AW57" t="inlineStr">
         <is>
-          <t>narrateur|Le sac est sur la commode, une seconde.
-maman|Bravo, Amir.
-papa|C'est du bon travail.
+          <t>narrateur|Le sac attend près de la porte.
 enfant-m|Merci, papa.
+maman|On lit sur le tapis ?
+narrateur|Amir s'assoit.
+narrateur|Il ouvre le livre sur ses genoux.
 narrateur|Le rayon de soleil a quitté le tapis.
-maman|On va jouer.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -11266,7 +11203,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>La dînette est dans la caisse, sous le lit. Une petite assiette dépasse. L'assiette dans le sac, Amir. L'assiette. Amir la tire, puis la met près du yaourt. Bravo. Tu as mis ce que papa a dit. La caisse sent le bois. On laisse le reste dans la caisse. D'accord.</t>
+          <t>La dînette est dans le panier, près du lit. Une tasse et une assiette s'entrechoquent. La tasse seulement, Amir. La tasse. Amir prend la tasse. L'assiette reste dans le panier. Il met la tasse près du yaourt. Juste la tasse. Juste la tasse.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -11406,19 +11343,17 @@
       <c r="AV58" s="2" t="inlineStr"/>
       <c r="AW58" t="inlineStr">
         <is>
-          <t>narrateur|La dînette est dans la caisse, sous le lit.
-narrateur|Une petite assiette dépasse.
-papa|L'assiette dans le sac, Amir.
-enfant-m|L'assiette.
-narrateur|Amir la tire, puis la met près du yaourt.
-maman|Bravo.
-maman|Tu as mis ce que papa a dit.
-narrateur|La caisse sent le bois.
-papa|On laisse le reste dans la caisse.
-enfant-m|D'accord.</t>
-        </is>
-      </c>
-      <c r="AX58" t="inlineStr"/>
+          <t>narrateur|La dînette est dans le panier, près du lit.
+narrateur|Une tasse et une assiette s'entrechoquent.
+maman|La tasse seulement, Amir.
+enfant-m|La tasse.
+narrateur|Amir prend la tasse.
+narrateur|L'assiette reste dans le panier.
+narrateur|Il met la tasse près du yaourt.
+maman|Juste la tasse.
+enfant-m|Juste la tasse.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -11443,7 +11378,7 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Amir s'assoit sur le tapis. Le sac est prêt. Bravo. Merci, maman. La couverture retombe sur le lit. On a mis ce que l'adulte a dit. L'histoire est finie.</t>
+          <t>Amir s'assoit, le sac sur les genoux. Le sac est prêt. Merci, maman. Il sort la tasse. Il fait semblant de goûter le yaourt. Après, pour de vrai. La couverture retombe sur le lit. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -11583,16 +11518,16 @@
       <c r="AV59" s="2" t="inlineStr"/>
       <c r="AW59" t="inlineStr">
         <is>
-          <t>narrateur|Amir s'assoit sur le tapis.
+          <t>narrateur|Amir s'assoit, le sac sur les genoux.
 papa|Le sac est prêt.
-maman|Bravo.
 enfant-m|Merci, maman.
+narrateur|Il sort la tasse.
+narrateur|Il fait semblant de goûter le yaourt.
+maman|Après, pour de vrai.
 narrateur|La couverture retombe sur le lit.
-papa|On a mis ce que l'adulte a dit.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -11617,7 +11552,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Sur la planche, un morceau de pain attend. La croûte fait un petit bruit. Ça sent le four, encore un peu. Le pain dans le sac, Amir. Le pain. Amir le prend avec précaution. Il le glisse à côté de la paroi. Bravo. Tu as mis ce que maman a dit. Tu as fini de mettre le pain ? Oui, maman. Une miette reste sur le tapis. On la range après.</t>
+          <t>Sur la planche, un morceau de pain attend. La croûte fait un petit bruit. Ça sent encore le four. Une miette tombe sur le tapis. Le pain, dans le sac. Le pain. Amir le glisse contre la paroi. Une miette reste sur sa manche. Il souffle dessus. Il est dedans ? Oui, maman.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -11759,20 +11694,17 @@
         <is>
           <t>narrateur|Sur la planche, un morceau de pain attend.
 narrateur|La croûte fait un petit bruit.
-narrateur|Ça sent le four, encore un peu.
-maman|Le pain dans le sac, Amir.
+narrateur|Ça sent encore le four.
+narrateur|Une miette tombe sur le tapis.
+maman|Le pain, dans le sac.
 enfant-m|Le pain.
-narrateur|Amir le prend avec précaution.
-narrateur|Il le glisse à côté de la paroi.
-papa|Bravo.
-papa|Tu as mis ce que maman a dit.
-maman|Tu as fini de mettre le pain ?
-enfant-m|Oui, maman.
-narrateur|Une miette reste sur le tapis.
-papa|On la range après.</t>
-        </is>
-      </c>
-      <c r="AX60" t="inlineStr"/>
+narrateur|Amir le glisse contre la paroi.
+narrateur|Une miette reste sur sa manche.
+narrateur|Il souffle dessus.
+maman|Il est dedans ?
+enfant-m|Oui, maman.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -11797,7 +11729,7 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Qui dit ce qu'on met dans le sac ?</t>
+          <t>Qui a dit de mettre le pain ?</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -11812,27 +11744,27 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>le sac</t>
+          <t>maman</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>le sac | mettre | ce que l'adulte a dit</t>
+          <t>maman | ma maman</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>Oui, c'est la bonne réponse.</t>
+          <t>Oui.</t>
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>Tu étais presque.</t>
+          <t>C'est maman qui l'a dit.</t>
         </is>
       </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>Dis : le sac.</t>
+          <t>Dis : maman.</t>
         </is>
       </c>
       <c r="M61" s="2" t="inlineStr"/>
@@ -11957,10 +11889,9 @@
       </c>
       <c r="AW61" t="inlineStr">
         <is>
-          <t>narrateur|Qui dit ce qu'on met dans le sac ?</t>
-        </is>
-      </c>
-      <c r="AX61" t="inlineStr"/>
+          <t>narrateur|Qui a dit de mettre le pain ?</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -11985,7 +11916,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Oui. Papa ou maman dit ce qu'on met. On met dans le sac ce que l'adulte a dit. Bravo, Amir. Tu as écouté. C'est du bon travail. Le pain est dedans. On continue ensemble ? Oui.</t>
+          <t>Maman a dit le pain. Le pain est dans le sac. Ça sent encore le four. Amir tape sur le sac. Ce n'est pas fini. On cherche encore un peu.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -12129,18 +12060,14 @@
       </c>
       <c r="AW62" t="inlineStr">
         <is>
-          <t>narrateur|Oui.
-narrateur|Papa ou maman dit ce qu'on met.
-narrateur|On met dans le sac ce que l'adulte a dit.
-maman|Bravo, Amir.
-maman|Tu as écouté.
-papa|C'est du bon travail.
-enfant-m|Le pain est dedans.
-maman|On continue ensemble ?
-enfant-m|Oui.</t>
-        </is>
-      </c>
-      <c r="AX62" t="inlineStr"/>
+          <t>narrateur|Maman a dit le pain.
+narrateur|Le pain est dans le sac.
+narrateur|Ça sent encore le four.
+narrateur|Amir tape sur le sac.
+maman|Ce n'est pas fini.
+maman|On cherche encore un peu.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -12165,7 +12092,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>On peut aller dans la cuisine, le jardin, ou la chambre.</t>
+          <t>On peut aller où ? La cuisine, le jardin, ou la chambre.</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -12329,10 +12256,10 @@
       <c r="AV63" s="2" t="inlineStr"/>
       <c r="AW63" t="inlineStr">
         <is>
-          <t>narrateur|On peut aller dans la cuisine, le jardin, ou la chambre.</t>
-        </is>
-      </c>
-      <c r="AX63" t="inlineStr"/>
+          <t>narrateur|On peut aller où ?
+narrateur|La cuisine, le jardin, ou la chambre.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -12357,7 +12284,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Amir pose le sac près de l'évier. Le pain sent encore le four. L'eau fait un tout petit bruit. La boîte à goûter, Amir. On la met dans le sac. La boîte. La boîte est lisse et bleue. Amir y glisse le pain. Puis la boîte dans le sac. Bravo. Tu as mis ce que maman a dit. Tu as fini ? Oui, maman.</t>
+          <t>Amir pose le sac près de l'évier. Le pain sent encore le four. L'eau fait un tout petit bruit. Une boîte à goûter attend. Elle est lisse et bleue. La boîte, Amir. Le pain va dedans. La boîte. Amir sort le pain du sac. Il le glisse dans la boîte. Puis la boîte dans le sac. Tu as fini ? Oui, maman.</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -12500,19 +12427,18 @@
           <t>narrateur|Amir pose le sac près de l'évier.
 narrateur|Le pain sent encore le four.
 narrateur|L'eau fait un tout petit bruit.
-maman|La boîte à goûter, Amir.
-maman|On la met dans le sac.
+narrateur|Une boîte à goûter attend.
+narrateur|Elle est lisse et bleue.
+maman|La boîte, Amir.
+maman|Le pain va dedans.
 enfant-m|La boîte.
-narrateur|La boîte est lisse et bleue.
-narrateur|Amir y glisse le pain.
+narrateur|Amir sort le pain du sac.
+narrateur|Il le glisse dans la boîte.
 narrateur|Puis la boîte dans le sac.
-papa|Bravo.
-papa|Tu as mis ce que maman a dit.
 maman|Tu as fini ?
 enfant-m|Oui, maman.</t>
         </is>
       </c>
-      <c r="AX64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -12537,7 +12463,7 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre les cubes, le livre, ou la dînette.</t>
+          <t>On peut prendre quoi ? Les cubes, le livre, ou la dînette.</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -12701,10 +12627,10 @@
       <c r="AV65" s="2" t="inlineStr"/>
       <c r="AW65" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre les cubes, le livre, ou la dînette.</t>
-        </is>
-      </c>
-      <c r="AX65" t="inlineStr"/>
+          <t>narrateur|On peut prendre quoi ?
+narrateur|Les cubes, le livre, ou la dînette.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -12729,7 +12655,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Les cubes sont près de la boîte à goûter. Ils font une petite tour. La tour, non. Deux cubes dans le sac, Amir. Deux cubes. Amir défait la tour tout doux. Il met deux cubes près du pain. Bravo. Tu as mis ce que maman a dit. La tour n'est plus là. On en fera une autre plus tard.</t>
+          <t>Les cubes sont près de la boîte à goûter. Ils font une petite tour. Amir défait la tour tout doux. Deux cubes dans le sac. Deux cubes. Il les met à côté de la boîte. Pas dans la boîte. À côté.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -12871,18 +12797,14 @@
         <is>
           <t>narrateur|Les cubes sont près de la boîte à goûter.
 narrateur|Ils font une petite tour.
-maman|La tour, non.
-maman|Deux cubes dans le sac, Amir.
+narrateur|Amir défait la tour tout doux.
+papa|Deux cubes dans le sac.
 enfant-m|Deux cubes.
-narrateur|Amir défait la tour tout doux.
-narrateur|Il met deux cubes près du pain.
-papa|Bravo.
-papa|Tu as mis ce que maman a dit.
-narrateur|La tour n'est plus là.
-maman|On en fera une autre plus tard.</t>
-        </is>
-      </c>
-      <c r="AX66" t="inlineStr"/>
+narrateur|Il les met à côté de la boîte.
+papa|Pas dans la boîte.
+enfant-m|À côté.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -12907,7 +12829,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Amir ferme le sac près de l'évier. Bravo, Amir. Le pain est dans la boîte. Les cubes aussi. L'eau ne coule plus. On a fini le sac. L'histoire est finie.</t>
+          <t>Amir ferme le sac près de l'évier. Le pain est dans la boîte. Les cubes aussi, à côté. On a fini le sac. Il sort un cube. Il le pose sur le couvercle bleu. L'eau ne coule plus. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -13048,15 +12970,15 @@
       <c r="AW67" t="inlineStr">
         <is>
           <t>narrateur|Amir ferme le sac près de l'évier.
-maman|Bravo, Amir.
-papa|Le pain est dans la boîte.
-enfant-m|Les cubes aussi.
+maman|Le pain est dans la boîte.
+papa|Les cubes aussi, à côté.
+enfant-m|On a fini le sac.
+narrateur|Il sort un cube.
+narrateur|Il le pose sur le couvercle bleu.
 narrateur|L'eau ne coule plus.
-maman|On a fini le sac.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -13081,7 +13003,7 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Le livre est sous un torchon, dans la cuisine. Le torchon sent le propre. Le livre dans le sac, Amir. Le livre. Amir le sort du torchon. Il le glisse près du pain. Bravo. Tu as mis ce que papa a dit. Le torchon reste sur la table. Le torchon n'est pas pour le sac.</t>
+          <t>Le livre est debout entre deux bocaux. Amir le prend par le dos. Le livre dans le sac. Le livre. Il le glisse près de la boîte. Au-dessus du pain. Au-dessus.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -13221,19 +13143,15 @@
       <c r="AV68" s="2" t="inlineStr"/>
       <c r="AW68" t="inlineStr">
         <is>
-          <t>narrateur|Le livre est sous un torchon, dans la cuisine.
-narrateur|Le torchon sent le propre.
-papa|Le livre dans le sac, Amir.
+          <t>narrateur|Le livre est debout entre deux bocaux.
+narrateur|Amir le prend par le dos.
+papa|Le livre dans le sac.
 enfant-m|Le livre.
-narrateur|Amir le sort du torchon.
-narrateur|Il le glisse près du pain.
-maman|Bravo.
-maman|Tu as mis ce que papa a dit.
-narrateur|Le torchon reste sur la table.
-papa|Le torchon n'est pas pour le sac.</t>
-        </is>
-      </c>
-      <c r="AX68" t="inlineStr"/>
+narrateur|Il le glisse près de la boîte.
+papa|Au-dessus du pain.
+enfant-m|Au-dessus.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -13258,7 +13176,7 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Le sac est posé contre la chaise. Bravo. Tu as écouté. Merci. Ça sent encore un peu le four. On va jouer. L'histoire est finie.</t>
+          <t>Le sac est posé contre la chaise. On va jouer. On ouvre le livre d'abord ? Amir montre une page à maman. Ça sent encore un peu le four. On y va. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
@@ -13399,15 +13317,14 @@
       <c r="AW69" t="inlineStr">
         <is>
           <t>narrateur|Le sac est posé contre la chaise.
-papa|Bravo.
-maman|Tu as écouté.
-enfant-m|Merci.
+enfant-m|On va jouer.
+maman|On ouvre le livre d'abord ?
+narrateur|Amir montre une page à maman.
 narrateur|Ça sent encore un peu le four.
-papa|On va jouer.
+papa|On y va.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -13432,7 +13349,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>La dînette est dans le tiroir du bas. Une casserole minuscule brille. La casserole dans le sac, Amir. La casserole. Amir ouvre le tiroir tout doux. Il met la casserole près du pain. Bravo. Tu as mis ce que maman a dit. Le tiroir se referme sans bruit. Tu as bien fermé.</t>
+          <t>Une casserole de dînette est près du sel. Le couvercle est à l'envers. Amir le remet dessus. La casserole dans le sac. La casserole. Il la met près de la boîte. On fera le pain pour de faux. Oui.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -13572,19 +13489,16 @@
       <c r="AV70" s="2" t="inlineStr"/>
       <c r="AW70" t="inlineStr">
         <is>
-          <t>narrateur|La dînette est dans le tiroir du bas.
-narrateur|Une casserole minuscule brille.
-maman|La casserole dans le sac, Amir.
+          <t>narrateur|Une casserole de dînette est près du sel.
+narrateur|Le couvercle est à l'envers.
+narrateur|Amir le remet dessus.
+maman|La casserole dans le sac.
 enfant-m|La casserole.
-narrateur|Amir ouvre le tiroir tout doux.
-narrateur|Il met la casserole près du pain.
-papa|Bravo.
-papa|Tu as mis ce que maman a dit.
-narrateur|Le tiroir se referme sans bruit.
-maman|Tu as bien fermé.</t>
-        </is>
-      </c>
-      <c r="AX70" t="inlineStr"/>
+narrateur|Il la met près de la boîte.
+maman|On fera le pain pour de faux.
+enfant-m|Oui.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -13609,7 +13523,7 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Amir tient la sangle du sac. Bravo, Amir. C'est du bon travail. Le sac est prêt. La cuisine est calme. On a mis ce que l'adulte a dit. L'histoire est finie.</t>
+          <t>Amir tient la sangle du sac. Le sac est prêt. La casserole aussi. Il fait semblant de cuire le pain. Tout doux. C'est déjà cuit. Amir rit. La cuisine est calme. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -13750,15 +13664,15 @@
       <c r="AW71" t="inlineStr">
         <is>
           <t>narrateur|Amir tient la sangle du sac.
-maman|Bravo, Amir.
-papa|C'est du bon travail.
-enfant-m|Le sac est prêt.
+papa|Le sac est prêt.
+enfant-m|La casserole aussi.
+narrateur|Il fait semblant de cuire le pain.
+maman|Tout doux. C'est déjà cuit.
+narrateur|Amir rit.
 narrateur|La cuisine est calme.
-maman|On a mis ce que l'adulte a dit.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -13783,7 +13697,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Amir descend la marche du jardin. Le pain reste au fond du sac. Le vent est doux sur les joues. Le petit chapeau, Amir. On le met dans le sac. Le chapeau. Le chapeau est souple. Amir le tasse près du pain. Bravo. Tu as mis ce que papa a dit. Une feuille tourne au-dessus du bac. On la laisse au jardin.</t>
+          <t>Amir descend la marche du jardin. Le pain reste au fond du sac. Le vent est doux sur les joues. Un petit chapeau attend sur le banc. Le petit chapeau, dans le sac. Le chapeau. Le chapeau est souple. Amir le tasse près du pain. Une feuille tourne au-dessus du bac. On la laisse au jardin.</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -13926,18 +13840,15 @@
           <t>narrateur|Amir descend la marche du jardin.
 narrateur|Le pain reste au fond du sac.
 narrateur|Le vent est doux sur les joues.
-papa|Le petit chapeau, Amir.
-papa|On le met dans le sac.
+narrateur|Un petit chapeau attend sur le banc.
+papa|Le petit chapeau, dans le sac.
 enfant-m|Le chapeau.
 narrateur|Le chapeau est souple.
 narrateur|Amir le tasse près du pain.
-maman|Bravo.
-maman|Tu as mis ce que papa a dit.
 narrateur|Une feuille tourne au-dessus du bac.
 papa|On la laisse au jardin.</t>
         </is>
       </c>
-      <c r="AX72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -13962,7 +13873,7 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre les cubes, le livre, ou la dînette.</t>
+          <t>On peut prendre quoi ? Les cubes, le livre, ou la dînette.</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
@@ -14126,10 +14037,10 @@
       <c r="AV73" s="2" t="inlineStr"/>
       <c r="AW73" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre les cubes, le livre, ou la dînette.</t>
-        </is>
-      </c>
-      <c r="AX73" t="inlineStr"/>
+          <t>narrateur|On peut prendre quoi ?
+narrateur|Les cubes, le livre, ou la dînette.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -14154,7 +14065,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Les cubes sont dans le bac à sable, au jardin. Un cube a un peu de sable. Le cube propre dans le sac, Amir. Le cube propre. Amir le frotte, puis le met près du pain. Bravo. Tu as mis ce que papa a dit. Le chapeau bouge dans le sac. Le sable reste au jardin. Oui.</t>
+          <t>Les cubes sont dans le bac à sable. Un cube a un peu de sable. Amir le frotte. Le cube propre, dans le sac. Le cube propre. Il le met près du pain. Le sable reste au bac.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -14294,19 +14205,15 @@
       <c r="AV74" s="2" t="inlineStr"/>
       <c r="AW74" t="inlineStr">
         <is>
-          <t>narrateur|Les cubes sont dans le bac à sable, au jardin.
+          <t>narrateur|Les cubes sont dans le bac à sable.
 narrateur|Un cube a un peu de sable.
-papa|Le cube propre dans le sac, Amir.
+narrateur|Amir le frotte.
+papa|Le cube propre, dans le sac.
 enfant-m|Le cube propre.
-narrateur|Amir le frotte, puis le met près du pain.
-maman|Bravo.
-maman|Tu as mis ce que papa a dit.
-narrateur|Le chapeau bouge dans le sac.
-papa|Le sable reste au jardin.
-enfant-m|Oui.</t>
-        </is>
-      </c>
-      <c r="AX74" t="inlineStr"/>
+narrateur|Il le met près du pain.
+papa|Le sable reste au bac.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -14331,7 +14238,7 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Amir remonte la marche avec le sac. Bravo. Tu as fait du bon travail. Merci, papa. Une feuille reste sur le bac. On rentre. L'histoire est finie.</t>
+          <t>Amir remonte la marche avec le sac. Merci, papa. On joue au cube, une minute. Amir pose le cube sur la marche. Une feuille reste sur le bac. On rentre. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -14472,15 +14379,14 @@
       <c r="AW75" t="inlineStr">
         <is>
           <t>narrateur|Amir remonte la marche avec le sac.
-papa|Bravo.
-maman|Tu as fait du bon travail.
 enfant-m|Merci, papa.
+maman|On joue au cube, une minute.
+narrateur|Amir pose le cube sur la marche.
 narrateur|Une feuille reste sur le bac.
-maman|On rentre.
+papa|On rentre.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -14505,7 +14411,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Le livre est sous le chapeau, sur le banc. Une page tremble au vent. Le livre dans le sac, Amir. Le livre. Amir le met près du pain. Puis le chapeau par-dessus. Bravo. Tu as mis ce que maman a dit. Le vent n'attrape plus les pages. Le livre est à l'abri. Oui, maman.</t>
+          <t>Le livre est sous le chapeau, sur le banc. Une page tremble au vent. Le livre dans le sac. Le livre. Amir le met près du pain. Puis le chapeau par-dessus. Le chapeau garde le livre. Oui.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -14647,18 +14553,14 @@
         <is>
           <t>narrateur|Le livre est sous le chapeau, sur le banc.
 narrateur|Une page tremble au vent.
-maman|Le livre dans le sac, Amir.
+maman|Le livre dans le sac.
 enfant-m|Le livre.
 narrateur|Amir le met près du pain.
 narrateur|Puis le chapeau par-dessus.
-papa|Bravo.
-papa|Tu as mis ce que maman a dit.
-narrateur|Le vent n'attrape plus les pages.
-maman|Le livre est à l'abri.
-enfant-m|Oui, maman.</t>
-        </is>
-      </c>
-      <c r="AX76" t="inlineStr"/>
+maman|Le chapeau garde le livre.
+enfant-m|Oui.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -14683,7 +14585,7 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Le sac est lourd, un peu. Bravo, Amir. Tu as écouté. Merci. Le jardin sent la terre mouillée. On rentre avec le sac. L'histoire est finie.</t>
+          <t>Le sac est un peu lourd. Merci. On rentre avec le sac. Amir soulève le chapeau. Il touche le livre, juste un peu. Le jardin sent la terre mouillée. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -14823,16 +14725,15 @@
       <c r="AV77" s="2" t="inlineStr"/>
       <c r="AW77" t="inlineStr">
         <is>
-          <t>narrateur|Le sac est lourd, un peu.
-maman|Bravo, Amir.
-papa|Tu as écouté.
+          <t>narrateur|Le sac est un peu lourd.
 enfant-m|Merci.
+papa|On rentre avec le sac.
+narrateur|Amir soulève le chapeau.
+narrateur|Il touche le livre, juste un peu.
 narrateur|Le jardin sent la terre mouillée.
-papa|On rentre avec le sac.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -14857,7 +14758,7 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Une assiette de dînette est sur le muret. Une feuille sèche est posée dessus. L'assiette dans le sac, Amir. L'assiette. Amir enlève la feuille. Il met l'assiette près du pain. Bravo. Tu as mis ce que papa a dit. La feuille s'envole. Elle reste au jardin.</t>
+          <t>Une assiette de dînette est sur le muret. Un caillou rond est posé dessus. Amir pose le caillou à côté. L'assiette dans le sac. L'assiette. Il la met près du pain. On y mettra le pain, pour de faux. Pour de faux.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -14998,18 +14899,15 @@
       <c r="AW78" t="inlineStr">
         <is>
           <t>narrateur|Une assiette de dînette est sur le muret.
-narrateur|Une feuille sèche est posée dessus.
-papa|L'assiette dans le sac, Amir.
+narrateur|Un caillou rond est posé dessus.
+narrateur|Amir pose le caillou à côté.
+maman|L'assiette dans le sac.
 enfant-m|L'assiette.
-narrateur|Amir enlève la feuille.
-narrateur|Il met l'assiette près du pain.
-maman|Bravo.
-maman|Tu as mis ce que papa a dit.
-narrateur|La feuille s'envole.
-papa|Elle reste au jardin.</t>
-        </is>
-      </c>
-      <c r="AX78" t="inlineStr"/>
+narrateur|Il la met près du pain.
+maman|On y mettra le pain, pour de faux.
+enfant-m|Pour de faux.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -15034,7 +14932,7 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Amir serre le sac contre lui. Le sac est prêt. Bravo. Merci, maman. Le vent est plus calme. On a mis ce que l'adulte a dit. L'histoire est finie.</t>
+          <t>Amir serre le sac contre lui. Le sac est prêt. Merci, maman. Amir sort l'assiette. Il y pose le pain un instant. Puis tout rentre. Le vent est plus calme. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -15175,15 +15073,15 @@
       <c r="AW79" t="inlineStr">
         <is>
           <t>narrateur|Amir serre le sac contre lui.
-papa|Le sac est prêt.
-maman|Bravo.
-enfant-m|Merci, maman.
+enfant-m|Le sac est prêt.
+papa|Merci, maman.
+narrateur|Amir sort l'assiette.
+narrateur|Il y pose le pain un instant.
+narrateur|Puis tout rentre.
 narrateur|Le vent est plus calme.
-papa|On a mis ce que l'adulte a dit.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -15208,7 +15106,7 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Amir repose le sac sur le tapis rayé. Le pain fait un petit bruit de croûte. Le volet jaune claque une fois. Le doudou du sac, Amir. On le met dans le sac. Le doudou. Le doudou est chaud et un peu plat. Amir le glisse près du pain. Bravo. Tu as mis ce que maman a dit. Le sac se remplit bien. Il est presque prêt.</t>
+          <t>Amir repose le sac sur le tapis rayé. Le pain fait un petit bruit de croûte. Le volet jaune claque une fois. Le doudou attend près de l'oreiller. Le doudou du sac, Amir. Le doudou. Le doudou est chaud et un peu plat. Amir le glisse près du pain. Il est bien dedans ? Oui. Le sac se remplit.</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -15351,18 +15249,16 @@
           <t>narrateur|Amir repose le sac sur le tapis rayé.
 narrateur|Le pain fait un petit bruit de croûte.
 narrateur|Le volet jaune claque une fois.
+narrateur|Le doudou attend près de l'oreiller.
 maman|Le doudou du sac, Amir.
-maman|On le met dans le sac.
 enfant-m|Le doudou.
 narrateur|Le doudou est chaud et un peu plat.
 narrateur|Amir le glisse près du pain.
-papa|Bravo.
-papa|Tu as mis ce que maman a dit.
-maman|Le sac se remplit bien.
-enfant-m|Il est presque prêt.</t>
-        </is>
-      </c>
-      <c r="AX80" t="inlineStr"/>
+maman|Il est bien dedans ?
+enfant-m|Oui.
+narrateur|Le sac se remplit.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -15387,7 +15283,7 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre les cubes, le livre, ou la dînette.</t>
+          <t>On peut prendre quoi ? Les cubes, le livre, ou la dînette.</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
@@ -15551,10 +15447,10 @@
       <c r="AV81" s="2" t="inlineStr"/>
       <c r="AW81" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre les cubes, le livre, ou la dînette.</t>
-        </is>
-      </c>
-      <c r="AX81" t="inlineStr"/>
+          <t>narrateur|On peut prendre quoi ?
+narrateur|Les cubes, le livre, ou la dînette.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -15579,7 +15475,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Les cubes sont près du doudou, sur le tapis. Un cube touche la patte du doudou. Les cubes dans le sac, Amir. Les cubes. Amir les met près du pain et du doudou. Bravo. Tu as mis ce que maman a dit. Le doudou ne tombe pas. Tu as été doux. Oui.</t>
+          <t>Les cubes sont près du doudou, sur le tapis. Un cube touche la patte du doudou. Les cubes dans le sac. Les cubes. Amir les met près du pain et du doudou. La patte est libre. Libre.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -15721,17 +15617,13 @@
         <is>
           <t>narrateur|Les cubes sont près du doudou, sur le tapis.
 narrateur|Un cube touche la patte du doudou.
-maman|Les cubes dans le sac, Amir.
+papa|Les cubes dans le sac.
 enfant-m|Les cubes.
 narrateur|Amir les met près du pain et du doudou.
-papa|Bravo.
-papa|Tu as mis ce que maman a dit.
-narrateur|Le doudou ne tombe pas.
-maman|Tu as été doux.
-enfant-m|Oui.</t>
-        </is>
-      </c>
-      <c r="AX82" t="inlineStr"/>
+papa|La patte est libre.
+enfant-m|Libre.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -15756,7 +15648,7 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Amir ferme le sac sur le tapis rayé. Bravo, Amir. Tu as fait du bon travail. Le sac est prêt. Le volet jaune est calme. On peut jouer maintenant. L'histoire est finie.</t>
+          <t>Amir ferme le sac sur le tapis rayé. On peut jouer maintenant. Oui. Il sort un cube. Il le pose sur le doudou, pour rire. Le volet jaune est calme. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -15897,15 +15789,14 @@
       <c r="AW83" t="inlineStr">
         <is>
           <t>narrateur|Amir ferme le sac sur le tapis rayé.
-maman|Bravo, Amir.
-papa|Tu as fait du bon travail.
-enfant-m|Le sac est prêt.
-narrateur|Le volet jaune est calme.
-maman|On peut jouer maintenant.
+enfant-m|On peut jouer maintenant.
+maman|Oui.
+narrateur|Il sort un cube.
+narrateur|Il le pose sur le doudou, pour rire.
+papa|Le volet jaune est calme.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -15930,7 +15821,7 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Le livre est coincé entre deux peluches. Amir le tire tout doux. Le livre dans le sac, Amir. Le livre. Il le glisse près du pain. Bravo. Tu as mis ce que papa a dit. Les peluches restent sur le lit. Elles ne vont pas dans le sac. D'accord.</t>
+          <t>Le livre est sous l'oreiller. Amir soulève l'oreiller d'une main. Le livre dans le sac. Le livre. Il le glisse près du pain. Sous le doudou, tout doux. Tout doux.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -16070,19 +15961,15 @@
       <c r="AV84" s="2" t="inlineStr"/>
       <c r="AW84" t="inlineStr">
         <is>
-          <t>narrateur|Le livre est coincé entre deux peluches.
-narrateur|Amir le tire tout doux.
-papa|Le livre dans le sac, Amir.
+          <t>narrateur|Le livre est sous l'oreiller.
+narrateur|Amir soulève l'oreiller d'une main.
+papa|Le livre dans le sac.
 enfant-m|Le livre.
 narrateur|Il le glisse près du pain.
-maman|Bravo.
-maman|Tu as mis ce que papa a dit.
-narrateur|Les peluches restent sur le lit.
-papa|Elles ne vont pas dans le sac.
-enfant-m|D'accord.</t>
-        </is>
-      </c>
-      <c r="AX84" t="inlineStr"/>
+papa|Sous le doudou, tout doux.
+enfant-m|Tout doux.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -16107,7 +15994,7 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Le sac attend près de la porte de la chambre. Bravo. Tu as écouté. Merci, papa. Le tapis n'a plus de cubes. On a mis ce que l'adulte a dit. L'histoire est finie.</t>
+          <t>Le sac attend près de la porte de la chambre. Merci, papa. On lit une page ? Amir ouvre le livre contre le doudou. Le tapis n'a plus de cubes. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -16248,15 +16135,13 @@
       <c r="AW85" t="inlineStr">
         <is>
           <t>narrateur|Le sac attend près de la porte de la chambre.
-papa|Bravo.
-maman|Tu as écouté.
 enfant-m|Merci, papa.
+maman|On lit une page ?
+narrateur|Amir ouvre le livre contre le doudou.
 narrateur|Le tapis n'a plus de cubes.
-maman|On a mis ce que l'adulte a dit.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -16281,7 +16166,7 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>La dînette est dans le panier, près du lit. Une tasse et une assiette s'entrechoquent. La tasse seulement, Amir. On la met dans le sac. La tasse. Amir prend la tasse, pas l'assiette. Il la met près du pain. Bravo. Tu as mis ce que maman a dit. L'assiette reste dans le panier. C'est ça.</t>
+          <t>La dînette est dans le panier, près du lit. Une tasse et une assiette s'entrechoquent. La tasse seulement. La tasse. Amir prend la tasse. Il la met près du pain. L'assiette reste. Elle reste.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -16423,18 +16308,14 @@
         <is>
           <t>narrateur|La dînette est dans le panier, près du lit.
 narrateur|Une tasse et une assiette s'entrechoquent.
-maman|La tasse seulement, Amir.
-maman|On la met dans le sac.
+maman|La tasse seulement.
 enfant-m|La tasse.
-narrateur|Amir prend la tasse, pas l'assiette.
+narrateur|Amir prend la tasse.
 narrateur|Il la met près du pain.
-papa|Bravo.
-papa|Tu as mis ce que maman a dit.
-narrateur|L'assiette reste dans le panier.
-maman|C'est ça.</t>
-        </is>
-      </c>
-      <c r="AX86" t="inlineStr"/>
+maman|L'assiette reste.
+enfant-m|Elle reste.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -16459,7 +16340,7 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Amir s'assoit, le sac sur les genoux. Bravo, Amir. C'est du bon travail. Merci. La chambre sent encore la soupe, un peu. Le sac est prêt. L'histoire est finie.</t>
+          <t>Amir s'assoit, le sac sur les genoux. Le sac est prêt. Merci. Il sort la tasse. Il y glisse un tout petit bout de pain. Pour de faux. Puis on range. La chambre sent encore la soupe, un peu. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
@@ -16600,15 +16481,15 @@
       <c r="AW87" t="inlineStr">
         <is>
           <t>narrateur|Amir s'assoit, le sac sur les genoux.
-maman|Bravo, Amir.
-papa|C'est du bon travail.
+papa|Le sac est prêt.
 enfant-m|Merci.
+narrateur|Il sort la tasse.
+narrateur|Il y glisse un tout petit bout de pain.
+maman|Pour de faux. Puis on range.
 narrateur|La chambre sent encore la soupe, un peu.
-maman|Le sac est prêt.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX87" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:AV87"/>
@@ -16627,7 +16508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16679,6 +16560,20 @@
       <c r="A7" t="inlineStr">
         <is>
           <t>F-NAR-009 ouverture du monde, fusion agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-010…015 texte : désir jouer, sac vide, branches à conséquences, chaîne Q pomme/yaourt/maman, personnages Amir papa maman</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F-NAR-017): watchdog SSD+inotify ; bateau/flaque et voyage des pommes
Veille worktree et clone SSD (inotify libc). exemple2 + avis paquet :
TREE-AUT-001 projet bateau/flaque ; TREE-COL-001 voyage mené par les
enfants, T3 = qui pousse. Pas d'audio.
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-AUT-001.xlsx
+++ b/stories/arbres/TREE-AUT-001.xlsx
@@ -552,7 +552,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le sac d'Amir sur le tapis rayé</t>
+          <t>Le bateau d'Amir et la flaque</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>dans la chambre</t>
+          <t>dans la chambre, puis le jardin</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amir veut aller jouer. Son sac est vide sur le tapis rayé. Il demande à papa et maman. Il met la pomme, le yaourt ou le pain, puis ce qu'ils nomment. Quand le sac est fermé, il joue enfin.</t>
+          <t>Amir veut faire flotter son bateau en papier dans la flaque. Le sac doit être prêt. Il y met le bateau, puis le manteau, les bottes ou le linge. À la flaque, le bateau part. Il le remet dans le sac.</t>
         </is>
       </c>
     </row>
@@ -1197,17 +1197,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Sur le toit, la gouttière fait encore plic ploc. La pluie vient de s'arrêter. La maison a un volet jaune. Le volet claque tout doux. Dans la rue, les pavés brillent. Ils sont encore mouillés. Une odeur de soupe entre par la fenêtre. Le tapis de la chambre est rayé. Il est bleu et crème. Un rayon de soleil touche le plancher. Papa pose un pull sur le lit. Il est encore un peu chaud. Maman ouvre un peu la fenêtre. Tu as senti la soupe ? Oui, maman. En ce moment, Amir veut aller jouer. Son sac attend sur le tapis. Amir tire la fermeture. Ça fait zzz. Le sac est vide. Je veux jouer ! D'accord. On prépare ton sac d'abord. Tu mets quoi, Amir ? Je ne sais pas. Demande. On t'aide. Amir pose la main sur le sac.</t>
+          <t>Sur le toit, la gouttière fait encore plic ploc. La pluie vient de s'arrêter. Le volet jaune claque tout doux. Dans la rue, les pavés brillent. En ce moment, Amir a un bateau en papier. Une voile pliée. Un peu froissée. Papa, la flaque est là, dans le jardin. Oui. On y va quand le sac est prêt. Le sac attend sur le tapis rayé. Amir tire la fermeture. Zzz. Le sac est vide. Le bateau est sur la commode.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Lina est dans la chambre, avec maman. Papa plie un pull. Lina prépare son &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. Maman parle, tout doux. On met dans le sac ce que l'adulte a dit.&lt;/prosody&gt;&lt;break time="400ms"/&gt;&lt;/speak&gt;</t>
+          <t>Sur le toit, la gouttière fait encore plic ploc. La pluie vient de s'arrêter. Le volet jaune claque tout doux. Dans la rue, les pavés brillent. En ce moment, Amir a un bateau en papier. Une voile pliée. Un peu froissée. Papa, la flaque est là, dans le jardin. Oui. On y va quand le sac est prêt. Le sac attend sur le tapis rayé. Amir tire la fermeture. Zzz. Le sac est vide. Le bateau est sur la commode.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lina est dans la chambre, avec maman. Papa plie un pull. Lina prépare son &lt;emphasis&gt;sac&lt;/emphasis&gt;. Maman parle, tout doux. On met dans le sac ce que l'adulte a dit.&lt;/slow&gt; [pause]</t>
+          <t>Sur le toit, la gouttière fait encore plic ploc. La pluie vient de s'arrêter. Le volet jaune claque tout doux. Dans la rue, les pavés brillent. En ce moment, Amir a un bateau en papier. Une voile pliée. Un peu froissée. Papa, la flaque est là, dans le jardin. Oui. On y va quand le sac est prêt. Le sac attend sur le tapis rayé. Amir tire la fermeture. Zzz. Le sac est vide. Le bateau est sur la commode.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1339,31 +1339,16 @@
         <is>
           <t>narrateur|Sur le toit, la gouttière fait encore plic ploc.
 narrateur|La pluie vient de s'arrêter.
-narrateur|La maison a un volet jaune.
-narrateur|Le volet claque tout doux.
+narrateur|Le volet jaune claque tout doux.
 narrateur|Dans la rue, les pavés brillent.
-narrateur|Ils sont encore mouillés.
-narrateur|Une odeur de soupe entre par la fenêtre.
-narrateur|Le tapis de la chambre est rayé.
-narrateur|Il est bleu et crème.
-narrateur|Un rayon de soleil touche le plancher.
-narrateur|Papa pose un pull sur le lit.
-papa|Il est encore un peu chaud.
-narrateur|Maman ouvre un peu la fenêtre.
-maman|Tu as senti la soupe ?
-enfant-m|Oui, maman.
-narrateur|En ce moment, Amir veut aller jouer.
-narrateur|Son sac attend sur le tapis.
-narrateur|Amir tire la fermeture.
-narrateur|Ça fait zzz.
+narrateur|En ce moment, Amir a un bateau en papier.
+narrateur|Une voile pliée. Un peu froissée.
+enfant-m|Papa, la flaque est là, dans le jardin.
+papa|Oui. On y va quand le sac est prêt.
+narrateur|Le sac attend sur le tapis rayé.
+narrateur|Amir tire la fermeture. Zzz.
 narrateur|Le sac est vide.
-enfant-m|Je veux jouer !
-maman|D'accord.
-maman|On prépare ton sac d'abord.
-papa|Tu mets quoi, Amir ?
-enfant-m|Je ne sais pas.
-maman|Demande. On t'aide.
-narrateur|Amir pose la main sur le sac.</t>
+narrateur|Le bateau est sur la commode.</t>
         </is>
       </c>
     </row>
@@ -1390,17 +1375,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Pour le goûter, on peut choisir. Une pomme, un yaourt, ou un morceau de pain.</t>
+          <t>Pour aller à la flaque, on prend aussi… Le manteau, les bottes, ou un linge.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;On peut prendre une pomme, un yaourt, ou un mor&lt;emphasis level="moderate"&gt;ce&lt;/emphasis&gt;au de pain.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>Pour aller à la flaque, on prend aussi… Le manteau, les bottes, ou un linge.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;On peut prendre une pomme, un yaourt, ou un mor&lt;emphasis&gt;ce&lt;/emphasis&gt;au de pain.&lt;/slow&gt; [pause]</t>
+          <t>Pour aller à la flaque, on prend aussi… Le manteau, les bottes, ou un linge.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
@@ -1418,7 +1403,7 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>une pomme</t>
+          <t>le manteau</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -1428,7 +1413,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>un yaourt</t>
+          <t>les bottes</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -1438,7 +1423,7 @@
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>un morceau de pain</t>
+          <t>un linge</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -1558,8 +1543,8 @@
       <c r="AV3" s="2" t="inlineStr"/>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Pour le goûter, on peut choisir.
-narrateur|Une pomme, un yaourt, ou un morceau de pain.</t>
+          <t>narrateur|Pour aller à la flaque, on prend aussi…
+narrateur|Le manteau, les bottes, ou un linge.</t>
         </is>
       </c>
     </row>
@@ -1586,17 +1571,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Dans la coupe, une pomme rouge brille. Elle sent le fruit. Amir tend la main. La pomme roule sur la table. Il la rattrape contre son ventre. La peau est lisse et froide. Celle-là, dans le sac. La pomme. Amir la glisse au fond. Le sac fait un petit toc. Elle est bien au fond ? Oui. Ça sent encore le fruit.</t>
+          <t>Amir prend le bateau sur la commode. Le bateau, dans le sac d'abord. Il le glisse au fond. Toc. La voile dépasse un tout petit peu. Il la rentre avec le doigt. Le manteau est sur la chaise. Il est encore un peu chaud. Pour la flaque. Il est encore frais dehors. Amir le plie. Il le met à côté du bateau.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Lina met une pomme dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. Maman a dit : la pomme. On met dans le sac ce que l'adulte a dit. Lina appuie un peu. Ça sent le fruit. Papa dit : c'est ça.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir prend le bateau sur la commode. Le bateau, dans le sac d'abord. Il le glisse au fond. Toc. La voile dépasse un tout petit peu. Il la rentre avec le doigt. Le manteau est sur la chaise. Il est encore un peu chaud. Pour la flaque. Il est encore frais dehors. Amir le plie. Il le met à côté du bateau.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lina met une pomme dans le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Maman a dit : la pomme. On met dans le sac ce que l'adulte a dit. Lina appuie un peu. Ça sent le fruit. Papa dit : c'est ça.&lt;/slow&gt; [pause]</t>
+          <t>Amir prend le bateau sur la commode. Le bateau, dans le sac d'abord. Il le glisse au fond. Toc. La voile dépasse un tout petit peu. Il la rentre avec le doigt. Le manteau est sur la chaise. Il est encore un peu chaud. Pour la flaque. Il est encore frais dehors. Amir le plie. Il le met à côté du bateau.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1726,19 +1711,17 @@
       <c r="AV4" s="2" t="inlineStr"/>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Dans la coupe, une pomme rouge brille.
-narrateur|Elle sent le fruit.
-narrateur|Amir tend la main.
-narrateur|La pomme roule sur la table.
-narrateur|Il la rattrape contre son ventre.
-narrateur|La peau est lisse et froide.
-maman|Celle-là, dans le sac.
-enfant-m|La pomme.
-narrateur|Amir la glisse au fond.
-narrateur|Le sac fait un petit toc.
-maman|Elle est bien au fond ?
-enfant-m|Oui.
-narrateur|Ça sent encore le fruit.</t>
+          <t>narrateur|Amir prend le bateau sur la commode.
+maman|Le bateau, dans le sac d'abord.
+narrateur|Il le glisse au fond.
+narrateur|Toc.
+narrateur|La voile dépasse un tout petit peu.
+narrateur|Il la rentre avec le doigt.
+narrateur|Le manteau est sur la chaise.
+narrateur|Il est encore un peu chaud.
+papa|Pour la flaque. Il est encore frais dehors.
+narrateur|Amir le plie.
+narrateur|Il le met à côté du bateau.</t>
         </is>
       </c>
     </row>
@@ -1765,27 +1748,27 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On met quoi dans le sac ?</t>
+          <t>Où Amir met-il le bateau ?</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;On met quoi dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ?&lt;/prosody&gt;&lt;break time="250ms"/&gt;&lt;/speak&gt;</t>
+          <t>Où Amir met-il le bateau ?</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;On met quoi dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ?&lt;/slow&gt;</t>
+          <t>Où Amir met-il le bateau ?</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>la pomme</t>
+          <t>le sac</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>la pomme | une pomme | pomme | le fruit</t>
+          <t>le sac | dans le sac | au fond</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -1795,12 +1778,12 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>C'est dans le sac. La pomme.</t>
+          <t>Dans le sac.</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Dis : la pomme.</t>
+          <t>Le bateau va dans le sac.</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr"/>
@@ -1925,7 +1908,7 @@
       </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|On met quoi dans le sac ?</t>
+          <t>narrateur|Où Amir met-il le bateau ?</t>
         </is>
       </c>
     </row>
@@ -1952,17 +1935,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>La pomme est dans le sac. Elle fait un petit rond. Amir touche la fermeture. Pas encore. Il manque encore des choses. Quoi ? On va voir ensemble.</t>
+          <t>Le bateau est dans le sac. La voile est rentrée. Le manteau est à côté. C'est bon ? Presque. On va à la flaque.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Oui. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. Lina respire. Maman est là. On met dans le sac ce que l'adulte a dit.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le bateau est dans le sac. La voile est rentrée. Le manteau est à côté. C'est bon ? Presque. On va à la flaque.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Oui. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. Lina respire. Maman est là. On met dans le sac ce que l'adulte a dit.&lt;/slow&gt; [pause]</t>
+          <t>Le bateau est dans le sac. La voile est rentrée. Le manteau est à côté. C'est bon ? Presque. On va à la flaque.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2096,13 +2079,11 @@
       </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|La pomme est dans le sac.
-narrateur|Elle fait un petit rond.
-narrateur|Amir touche la fermeture.
-maman|Pas encore.
-maman|Il manque encore des choses.
-enfant-m|Quoi ?
-maman|On va voir ensemble.</t>
+          <t>narrateur|Le bateau est dans le sac.
+narrateur|La voile est rentrée.
+narrateur|Le manteau est à côté.
+enfant-m|C'est bon ?
+papa|Presque. On va à la flaque.</t>
         </is>
       </c>
     </row>
@@ -2129,17 +2110,17 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>On peut aller où ? La cuisine, le jardin, ou la chambre.</t>
+          <t>Quelle flaque ? Sous la gouttière, près du potager, ou près du bac.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;On peut prendre la cuisine, le jardin, ou la chambre.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>Quelle flaque ? Sous la gouttière, près du potager, ou près du bac.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;On peut prendre la cuisine, le jardin, ou la chambre.&lt;/slow&gt; [pause]</t>
+          <t>Quelle flaque ? Sous la gouttière, près du potager, ou près du bac.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
@@ -2157,7 +2138,7 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>la cuisine</t>
+          <t>sous la gouttière</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -2167,7 +2148,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>le jardin</t>
+          <t>près du potager</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -2177,7 +2158,7 @@
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>la chambre</t>
+          <t>près du bac</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
@@ -2293,8 +2274,8 @@
       <c r="AV7" s="2" t="inlineStr"/>
       <c r="AW7" t="inlineStr">
         <is>
-          <t>narrateur|On peut aller où ?
-narrateur|La cuisine, le jardin, ou la chambre.</t>
+          <t>narrateur|Quelle flaque ?
+narrateur|Sous la gouttière, près du potager, ou près du bac.</t>
         </is>
       </c>
     </row>
@@ -2321,17 +2302,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Amir emporte le sac vers la cuisine. Le carrelage est un peu froid. La soupe fume encore dans la casserole. Une serviette dépasse sous une cuillère. Amir tire le coin tout doux. La petite serviette, dans le sac. La serviette. Elle est douce et pliée. Il la glisse près de la pomme. Tu as fini de la mettre ? Oui, maman. Une miette reste sur la table.</t>
+          <t>Amir met le manteau. Il est tiède. Ils sortent. Le sac tape contre sa hanche. Sous la gouttière, une flaque ronde. Une goutte tombe. Plic. L'eau tremble. Le bateau, maintenant.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Ensuite Lina va dans la cuisine. Elle met les cubes près du &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. On met dans le sac ce que l'adulte a dit. Maman dit : les cubes, oui. Maman montre le geste, lentement. On met dans le sac ce que l'adulte a dit.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir met le manteau. Il est tiède. Ils sortent. Le sac tape contre sa hanche. Sous la gouttière, une flaque ronde. Une goutte tombe. Plic. L'eau tremble. Le bateau, maintenant.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Ensuite Lina va dans la cuisine. Elle met les cubes près du &lt;emphasis&gt;sac&lt;/emphasis&gt;. On met dans le sac ce que l'adulte a dit. Maman dit : les cubes, oui. Maman montre le geste, lentement. On met dans le sac ce que l'adulte a dit.&lt;/slow&gt; [pause]</t>
+          <t>Amir met le manteau. Il est tiède. Ils sortent. Le sac tape contre sa hanche. Sous la gouttière, une flaque ronde. Une goutte tombe. Plic. L'eau tremble. Le bateau, maintenant.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -2461,18 +2442,12 @@
       <c r="AV8" s="2" t="inlineStr"/>
       <c r="AW8" t="inlineStr">
         <is>
-          <t>narrateur|Amir emporte le sac vers la cuisine.
-narrateur|Le carrelage est un peu froid.
-narrateur|La soupe fume encore dans la casserole.
-narrateur|Une serviette dépasse sous une cuillère.
-narrateur|Amir tire le coin tout doux.
-maman|La petite serviette, dans le sac.
-enfant-m|La serviette.
-narrateur|Elle est douce et pliée.
-narrateur|Il la glisse près de la pomme.
-maman|Tu as fini de la mettre ?
-enfant-m|Oui, maman.
-narrateur|Une miette reste sur la table.</t>
+          <t>narrateur|Amir met le manteau. Il est tiède.
+narrateur|Ils sortent. Le sac tape contre sa hanche.
+narrateur|Sous la gouttière, une flaque ronde.
+narrateur|Une goutte tombe. Plic.
+narrateur|L'eau tremble.
+papa|Le bateau, maintenant.</t>
         </is>
       </c>
     </row>
@@ -2499,17 +2474,17 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre quoi ? Les cubes, le livre, ou la dînette.</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;On peut prendre les cubes, le livre, ou la dînette.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;On peut prendre les cubes, le livre, ou la dînette.&lt;/slow&gt; [pause]</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -2527,7 +2502,7 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>les cubes</t>
+          <t>au milieu</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -2537,7 +2512,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>le livre</t>
+          <t>près du bord</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -2547,7 +2522,7 @@
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>la dînette</t>
+          <t>sur le sac</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
@@ -2663,8 +2638,8 @@
       <c r="AV9" s="2" t="inlineStr"/>
       <c r="AW9" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre quoi ?
-narrateur|Les cubes, le livre, ou la dînette.</t>
+          <t>narrateur|On pose le bateau…
+narrateur|Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
     </row>
@@ -2691,17 +2666,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Les cubes bleus attendent près de l'assiette. Ils tapent un peu sur le bois. Amir en empile deux. La tour penche vers la pomme. Deux cubes dans le sac. Deux cubes. Il défait la tour tout doux. Il les glisse près de la pomme. Ils tiennent ? Ils tiennent.</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Lina a choisi une pomme. Puis la cuisine. Puis les cubes. Un vélo passe au loin. Lina prend la main de maman. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lina a choisi une pomme. Puis la cuisine. Puis les cubes. Un vélo passe au loin. Lina prend la main de maman. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -2831,16 +2806,13 @@
       <c r="AV10" s="2" t="inlineStr"/>
       <c r="AW10" t="inlineStr">
         <is>
-          <t>narrateur|Les cubes bleus attendent près de l'assiette.
-narrateur|Ils tapent un peu sur le bois.
-narrateur|Amir en empile deux.
-narrateur|La tour penche vers la pomme.
-maman|Deux cubes dans le sac.
-enfant-m|Deux cubes.
-narrateur|Il défait la tour tout doux.
-narrateur|Il les glisse près de la pomme.
-papa|Ils tiennent ?
-enfant-m|Ils tiennent.</t>
+          <t>narrateur|Amir sort le bateau du sac.
+narrateur|Il le pose au milieu de l'eau.
+narrateur|La voile se tient.
+narrateur|Un peu d'eau touche le papier.
+papa|Il avance.
+narrateur|Amir souffle. Ffff.
+narrateur|Le bateau part tout doux.</t>
         </is>
       </c>
     </row>
@@ -2867,17 +2839,17 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Amir ferme le sac près de la table. Ça fait zzz. Le sac est prêt. On peut jouer ? Oui. Les cubes, après. Amir sort un cube. Il le pose sur la table. Toc. La cuisine sent encore la soupe. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -3007,15 +2979,12 @@
       <c r="AV11" s="2" t="inlineStr"/>
       <c r="AW11" t="inlineStr">
         <is>
-          <t>narrateur|Amir ferme le sac près de la table.
-narrateur|Ça fait zzz.
-papa|Le sac est prêt.
-enfant-m|On peut jouer ?
-maman|Oui. Les cubes, après.
-narrateur|Amir sort un cube.
-narrateur|Il le pose sur la table.
-narrateur|Toc.
-narrateur|La cuisine sent encore la soupe.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir reprend le bateau.
+narrateur|Il le remet dans le sac.
+narrateur|Le manteau rentre aussi.
+narrateur|On referme. Zzz.
+narrateur|La gouttière fait un dernier plic.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -3043,17 +3012,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Un petit livre est posé près du sel. Les pages sentent le papier. Une page colle un peu. Amir souffle dessus. Le livre, à plat dans le sac. Le livre. Il le glisse près de la pomme. Il est à plat ? À plat.</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Lina s'arrête près de le livre. la cuisine est rangé. On entend un oiseau. Papa n'est pas loin. Lina les rejoint. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lina s'arrête près de le livre. la cuisine est rangé. On entend un oiseau. Papa n'est pas loin. Lina les rejoint. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -3183,15 +3152,13 @@
       <c r="AV12" s="2" t="inlineStr"/>
       <c r="AW12" t="inlineStr">
         <is>
-          <t>narrateur|Un petit livre est posé près du sel.
-narrateur|Les pages sentent le papier.
-narrateur|Une page colle un peu.
-narrateur|Amir souffle dessus.
-papa|Le livre, à plat dans le sac.
-enfant-m|Le livre.
-narrateur|Il le glisse près de la pomme.
-papa|Il est à plat ?
-enfant-m|À plat.</t>
+          <t>narrateur|Amir sort le bateau.
+narrateur|Il le donne à papa.
+papa|Près du bord, ensemble.
+narrateur|Papa le pose. Amir tient le sac.
+narrateur|Le bateau part.
+narrateur|Amir marche le long de l'eau.
+narrateur|Le sac est à l'épaule.</t>
         </is>
       </c>
     </row>
@@ -3218,17 +3185,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Amir appuie sur la fermeture. Tu as mis le livre. Et la pomme. Le sac est prêt. On ouvre juste la couverture ? Oui. Amir montre un bateau sur la page. Puis il referme le sac. Ils restent un moment près de la table. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -3358,15 +3325,12 @@
       <c r="AV13" s="2" t="inlineStr"/>
       <c r="AW13" t="inlineStr">
         <is>
-          <t>narrateur|Amir appuie sur la fermeture.
-maman|Tu as mis le livre.
-papa|Et la pomme.
-enfant-m|Le sac est prêt.
-maman|On ouvre juste la couverture ?
-enfant-m|Oui.
-narrateur|Amir montre un bateau sur la page.
-narrateur|Puis il referme le sac.
-narrateur|Ils restent un moment près de la table.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir reprend le bateau.
+narrateur|Il le remet dans le sac.
+narrateur|Le manteau rentre aussi.
+narrateur|On referme. Zzz.
+narrateur|La gouttière fait un dernier plic.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -3394,17 +3358,17 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>La petite tasse de dînette cliquette. Elle est rouge, près de l'évier. Une goutte brille au fond. Amir la verse dans l'évier. La tasse, dans le sac. La tasse. Il la pose tout doux près de la pomme. Ça sonne comme un tout petit verre. On fera la dînette après. Oui, maman.</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Lina se souvient de une pomme. Et de la cuisine. Et de la dînette. La couverture est douce. Lina enfile ses chaussons. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lina se souvient de une pomme. Et de la cuisine. Et de la dînette. La couverture est douce. Lina enfile ses chaussons. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -3534,16 +3498,11 @@
       <c r="AV14" s="2" t="inlineStr"/>
       <c r="AW14" t="inlineStr">
         <is>
-          <t>narrateur|La petite tasse de dînette cliquette.
-narrateur|Elle est rouge, près de l'évier.
-narrateur|Une goutte brille au fond.
-narrateur|Amir la verse dans l'évier.
-maman|La tasse, dans le sac.
-enfant-m|La tasse.
-narrateur|Il la pose tout doux près de la pomme.
-narrateur|Ça sonne comme un tout petit verre.
-maman|On fera la dînette après.
-enfant-m|Oui, maman.</t>
+          <t>narrateur|Amir pose d'abord le sac.
+narrateur|Il pose le bateau sur le sac.
+narrateur|Il regarde la flaque.
+narrateur|Puis il met le bateau dans l'eau.
+papa|Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
     </row>
@@ -3570,17 +3529,17 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Le sac a la pomme et la tasse. Amir le serre contre lui. On va jouer ? Oui. Il sort la tasse. Il fait semblant de boire. À plus tard, petite tasse. Une goutte tombe dans l'évier. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr"/>
@@ -3710,14 +3669,12 @@
       <c r="AV15" s="2" t="inlineStr"/>
       <c r="AW15" t="inlineStr">
         <is>
-          <t>narrateur|Le sac a la pomme et la tasse.
-narrateur|Amir le serre contre lui.
-papa|On va jouer ?
-enfant-m|Oui.
-narrateur|Il sort la tasse.
-narrateur|Il fait semblant de boire.
-maman|À plus tard, petite tasse.
-narrateur|Une goutte tombe dans l'évier.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir reprend le bateau.
+narrateur|Il le remet dans le sac.
+narrateur|Le manteau rentre aussi.
+narrateur|On referme. Zzz.
+narrateur|La gouttière fait un dernier plic.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -3745,17 +3702,17 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Amir pousse la porte du jardin. L'herbe est encore mouillée. Une feuille colle à sa chaussette. Un petit linge sèche sur le banc. Le petit linge, Amir. On le met dans le sac. Le linge. Le linge sent l'air frais. Amir le pose près de la pomme. Un oiseau chante sur le mur. Tu as entendu l'oiseau ? Oui, papa.</t>
+          <t>Amir met le manteau. Ils vont près du potager. La flaque est ronde, entre deux choux. Une feuille y trempe le bout. L'eau tremble un peu. Le bateau, Amir.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Ensuite Lina va dans la cuisine. Elle met le livre près du &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. On met dans le sac ce que l'adulte a dit. Maman dit : le livre, oui. Maman dit : je suis là. On met dans le sac ce que l'adulte a dit.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir met le manteau. Ils vont près du potager. La flaque est ronde, entre deux choux. Une feuille y trempe le bout. L'eau tremble un peu. Le bateau, Amir.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Ensuite Lina va dans la cuisine. Elle met le livre près du &lt;emphasis&gt;sac&lt;/emphasis&gt;. On met dans le sac ce que l'adulte a dit. Maman dit : le livre, oui. Maman dit : je suis là. On met dans le sac ce que l'adulte a dit.&lt;/slow&gt; [pause]</t>
+          <t>Amir met le manteau. Ils vont près du potager. La flaque est ronde, entre deux choux. Une feuille y trempe le bout. L'eau tremble un peu. Le bateau, Amir.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -3885,18 +3842,12 @@
       <c r="AV16" s="2" t="inlineStr"/>
       <c r="AW16" t="inlineStr">
         <is>
-          <t>narrateur|Amir pousse la porte du jardin.
-narrateur|L'herbe est encore mouillée.
-narrateur|Une feuille colle à sa chaussette.
-narrateur|Un petit linge sèche sur le banc.
-papa|Le petit linge, Amir.
-papa|On le met dans le sac.
-enfant-m|Le linge.
-narrateur|Le linge sent l'air frais.
-narrateur|Amir le pose près de la pomme.
-narrateur|Un oiseau chante sur le mur.
-papa|Tu as entendu l'oiseau ?
-enfant-m|Oui, papa.</t>
+          <t>narrateur|Amir met le manteau.
+narrateur|Ils vont près du potager.
+narrateur|La flaque est ronde, entre deux choux.
+narrateur|Une feuille y trempe le bout.
+narrateur|L'eau tremble un peu.
+maman|Le bateau, Amir.</t>
         </is>
       </c>
     </row>
@@ -3923,17 +3874,17 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre quoi ? Les cubes, le livre, ou la dînette.</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;On peut prendre les cubes, le livre, ou la dînette.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;On peut prendre les cubes, le livre, ou la dînette.&lt;/slow&gt; [pause]</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr"/>
@@ -3951,7 +3902,7 @@
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>les cubes</t>
+          <t>au milieu</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
@@ -3961,7 +3912,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>le livre</t>
+          <t>près du bord</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -3971,7 +3922,7 @@
       </c>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>la dînette</t>
+          <t>sur le sac</t>
         </is>
       </c>
       <c r="R17" s="2" t="inlineStr">
@@ -4087,8 +4038,8 @@
       <c r="AV17" s="2" t="inlineStr"/>
       <c r="AW17" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre quoi ?
-narrateur|Les cubes, le livre, ou la dînette.</t>
+          <t>narrateur|On pose le bateau…
+narrateur|Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
     </row>
@@ -4115,17 +4066,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Les cubes sont sur la pierre chaude. Ils sentent un peu le soleil. Un cube a une goutte dessus. Amir l'essuie sur son pantalon. Un cube dans le sac. Un cube. Il le met près de la pomme. Une abeille passe, tout loin. On laisse l'abeille au jardin.</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Avec les cubes. Après le jardin. Près de une pomme. Lina s'arrête. Il y a des miettes sur la table. Lina tend les cubes à papa. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Avec les cubes. Après le jardin. Près de une pomme. Lina s'arrête. Il y a des miettes sur la table. Lina tend les cubes à papa. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -4255,15 +4206,13 @@
       <c r="AV18" s="2" t="inlineStr"/>
       <c r="AW18" t="inlineStr">
         <is>
-          <t>narrateur|Les cubes sont sur la pierre chaude.
-narrateur|Ils sentent un peu le soleil.
-narrateur|Un cube a une goutte dessus.
-narrateur|Amir l'essuie sur son pantalon.
-papa|Un cube dans le sac.
-enfant-m|Un cube.
-narrateur|Il le met près de la pomme.
-narrateur|Une abeille passe, tout loin.
-papa|On laisse l'abeille au jardin.</t>
+          <t>narrateur|Amir sort le bateau du sac.
+narrateur|Il le pose au milieu de l'eau.
+narrateur|La voile se tient.
+narrateur|Un peu d'eau touche le papier.
+papa|Il avance.
+narrateur|Amir souffle. Ffff.
+narrateur|Le bateau part tout doux.</t>
         </is>
       </c>
     </row>
@@ -4290,17 +4239,17 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Amir referme le sac sur l'herbe. C'est prêt. On enlève la feuille, d'abord. Amir ôte la feuille de sa chaussette. Il sort le cube. Il le pose sur la pierre. On rentre quand tu veux. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -4430,13 +4379,12 @@
       <c r="AV19" s="2" t="inlineStr"/>
       <c r="AW19" t="inlineStr">
         <is>
-          <t>narrateur|Amir referme le sac sur l'herbe.
-enfant-m|C'est prêt.
-papa|On enlève la feuille, d'abord.
-narrateur|Amir ôte la feuille de sa chaussette.
-narrateur|Il sort le cube.
-narrateur|Il le pose sur la pierre.
-maman|On rentre quand tu veux.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir reprend le bateau.
+narrateur|Il le remet dans le sac.
+narrateur|Le manteau rentre aussi.
+narrateur|On referme. Zzz.
+narrateur|Une feuille lâche la flaque.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -4464,17 +4412,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Le livre est à l'ombre, sous le banc. L'herbe chatouille les chevilles. Amir se penche. Les pages sont un peu fraîches. Le livre dans le sac, Amir. Le livre. Il le glisse près de la pomme. On lira plus tard, au calme. D'accord.</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Lina range le jardin. le livre reste près de une pomme. La lumière est claire. Lina s'assoit près de maman. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lina range le jardin. le livre reste près de une pomme. La lumière est claire. Lina s'assoit près de maman. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -4604,15 +4552,13 @@
       <c r="AV20" s="2" t="inlineStr"/>
       <c r="AW20" t="inlineStr">
         <is>
-          <t>narrateur|Le livre est à l'ombre, sous le banc.
-narrateur|L'herbe chatouille les chevilles.
-narrateur|Amir se penche.
-narrateur|Les pages sont un peu fraîches.
-maman|Le livre dans le sac, Amir.
-enfant-m|Le livre.
-narrateur|Il le glisse près de la pomme.
-maman|On lira plus tard, au calme.
-enfant-m|D'accord.</t>
+          <t>narrateur|Amir sort le bateau.
+narrateur|Il le donne à papa.
+papa|Près du bord, ensemble.
+narrateur|Papa le pose. Amir tient le sac.
+narrateur|Le bateau part.
+narrateur|Amir marche le long de l'eau.
+narrateur|Le sac est à l'épaule.</t>
         </is>
       </c>
     </row>
@@ -4639,17 +4585,17 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Le sac est posé sur le banc. Amir ouvre un tout petit coin. Il regarde une page. On rentre avec le sac. Oui. Un oiseau s'envole du mur. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -4779,12 +4725,12 @@
       <c r="AV21" s="2" t="inlineStr"/>
       <c r="AW21" t="inlineStr">
         <is>
-          <t>narrateur|Le sac est posé sur le banc.
-narrateur|Amir ouvre un tout petit coin.
-narrateur|Il regarde une page.
-papa|On rentre avec le sac.
-enfant-m|Oui.
-narrateur|Un oiseau s'envole du mur.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir reprend le bateau.
+narrateur|Il le remet dans le sac.
+narrateur|Le manteau rentre aussi.
+narrateur|On referme. Zzz.
+narrateur|Une feuille lâche la flaque.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -4812,17 +4758,17 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>La dînette est sur un linge, dans l'herbe. Une assiette minuscule brille. Une feuille sèche est posée dessus. Amir enlève la feuille. L'assiette dans le sac, Amir. L'assiette. Il la pose à plat près de la pomme. Elle est à plat ? Oui.</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;la dînette est là. le jardin aussi. une pomme reste dans le souvenir. On attend son tour. Lina ferme la porte, tout doux. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;la dînette est là. le jardin aussi. une pomme reste dans le souvenir. On attend son tour. Lina ferme la porte, tout doux. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -4952,15 +4898,11 @@
       <c r="AV22" s="2" t="inlineStr"/>
       <c r="AW22" t="inlineStr">
         <is>
-          <t>narrateur|La dînette est sur un linge, dans l'herbe.
-narrateur|Une assiette minuscule brille.
-narrateur|Une feuille sèche est posée dessus.
-narrateur|Amir enlève la feuille.
-maman|L'assiette dans le sac, Amir.
-enfant-m|L'assiette.
-narrateur|Il la pose à plat près de la pomme.
-papa|Elle est à plat ?
-enfant-m|Oui.</t>
+          <t>narrateur|Amir pose d'abord le sac.
+narrateur|Il pose le bateau sur le sac.
+narrateur|Il regarde la flaque.
+narrateur|Puis il met le bateau dans l'eau.
+papa|Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
     </row>
@@ -4987,17 +4929,17 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Amir tient le sac contre lui. Le sac est prêt. On goûte la pomme dehors ? Après. Il sort l'assiette. Il pose la pomme dessus, un instant. Puis tout rentre dans le sac. Une goutte tombe de la gouttière. Plic ploc. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -5127,15 +5069,12 @@
       <c r="AV23" s="2" t="inlineStr"/>
       <c r="AW23" t="inlineStr">
         <is>
-          <t>narrateur|Amir tient le sac contre lui.
-enfant-m|Le sac est prêt.
-maman|On goûte la pomme dehors ?
-enfant-m|Après.
-narrateur|Il sort l'assiette.
-narrateur|Il pose la pomme dessus, un instant.
-narrateur|Puis tout rentre dans le sac.
-narrateur|Une goutte tombe de la gouttière.
-narrateur|Plic ploc.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir reprend le bateau.
+narrateur|Il le remet dans le sac.
+narrateur|Le manteau rentre aussi.
+narrateur|On referme. Zzz.
+narrateur|Une feuille lâche la flaque.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -5163,17 +5102,17 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Amir revient dans la chambre. Le tapis rayé est tiède. Le pull marine attend sur le lit. Amir essaie de le plier. Une manche dépasse. Le pull, dans le sac. Le pull. Il le tasse près de la pomme. La manche est rentrée ? Presque. Le volet claque encore un peu.</t>
+          <t>Amir met le manteau. Ils vont près du bac à sable. Une flaque borde le bois du bac. Un peu de sable brille au fond. Le bateau, Amir.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Ensuite Lina va dans la cuisine. Elle met la dînette près du &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. On met dans le sac ce que l'adulte a dit. Maman dit : une tasse seulement. Maman reste tout près. On met dans le sac ce que l'adulte a dit.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir met le manteau. Ils vont près du bac à sable. Une flaque borde le bois du bac. Un peu de sable brille au fond. Le bateau, Amir.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Ensuite Lina va dans la cuisine. Elle met la dînette près du &lt;emphasis&gt;sac&lt;/emphasis&gt;. On met dans le sac ce que l'adulte a dit. Maman dit : une tasse seulement. Maman reste tout près. On met dans le sac ce que l'adulte a dit.&lt;/slow&gt; [pause]</t>
+          <t>Amir met le manteau. Ils vont près du bac à sable. Une flaque borde le bois du bac. Un peu de sable brille au fond. Le bateau, Amir.</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -5303,17 +5242,11 @@
       <c r="AV24" s="2" t="inlineStr"/>
       <c r="AW24" t="inlineStr">
         <is>
-          <t>narrateur|Amir revient dans la chambre.
-narrateur|Le tapis rayé est tiède.
-narrateur|Le pull marine attend sur le lit.
-narrateur|Amir essaie de le plier.
-narrateur|Une manche dépasse.
-papa|Le pull, dans le sac.
-enfant-m|Le pull.
-narrateur|Il le tasse près de la pomme.
-papa|La manche est rentrée ?
-enfant-m|Presque.
-narrateur|Le volet claque encore un peu.</t>
+          <t>narrateur|Amir met le manteau.
+narrateur|Ils vont près du bac à sable.
+narrateur|Une flaque borde le bois du bac.
+narrateur|Un peu de sable brille au fond.
+papa|Le bateau, Amir.</t>
         </is>
       </c>
     </row>
@@ -5340,17 +5273,17 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre quoi ? Les cubes, le livre, ou la dînette.</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;On peut prendre les cubes, le livre, ou la dînette.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;On peut prendre les cubes, le livre, ou la dînette.&lt;/slow&gt; [pause]</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr"/>
@@ -5368,7 +5301,7 @@
       <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>les cubes</t>
+          <t>au milieu</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
@@ -5378,7 +5311,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>le livre</t>
+          <t>près du bord</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -5388,7 +5321,7 @@
       </c>
       <c r="Q25" s="2" t="inlineStr">
         <is>
-          <t>la dînette</t>
+          <t>sur le sac</t>
         </is>
       </c>
       <c r="R25" s="2" t="inlineStr">
@@ -5504,8 +5437,8 @@
       <c r="AV25" s="2" t="inlineStr"/>
       <c r="AW25" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre quoi ?
-narrateur|Les cubes, le livre, ou la dînette.</t>
+          <t>narrateur|On pose le bateau…
+narrateur|Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
     </row>
@@ -5532,17 +5465,17 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Les cubes sont sous la chaise. Un cube rouge a roulé loin. Amir rampe sur le tapis. Il rattrape le cube rouge. Les cubes dans le sac. Les cubes. Il les met près de la pomme. Tu as le rouge ? Oui.</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Lina rejoint les cubes. la chambre est rangé. une pomme est fini. Une cloche tinte, tout loin. Lina chuchote : c'est fini. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lina rejoint les cubes. la chambre est rangé. une pomme est fini. Une cloche tinte, tout loin. Lina chuchote : c'est fini. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -5672,15 +5605,13 @@
       <c r="AV26" s="2" t="inlineStr"/>
       <c r="AW26" t="inlineStr">
         <is>
-          <t>narrateur|Les cubes sont sous la chaise.
-narrateur|Un cube rouge a roulé loin.
-narrateur|Amir rampe sur le tapis.
-narrateur|Il rattrape le cube rouge.
-maman|Les cubes dans le sac.
-enfant-m|Les cubes.
-narrateur|Il les met près de la pomme.
-maman|Tu as le rouge ?
-enfant-m|Oui.</t>
+          <t>narrateur|Amir sort le bateau du sac.
+narrateur|Il le pose au milieu de l'eau.
+narrateur|La voile se tient.
+narrateur|Un peu d'eau touche le papier.
+papa|Il avance.
+narrateur|Amir souffle. Ffff.
+narrateur|Le bateau part tout doux.</t>
         </is>
       </c>
     </row>
@@ -5707,17 +5638,17 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Amir ferme le sac au pied du lit. On peut jouer ? Oui. Sur le tapis. Amir sort deux cubes. Il les pose sur une rayure crème. Le tapis rayé est calme. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -5847,12 +5778,12 @@
       <c r="AV27" s="2" t="inlineStr"/>
       <c r="AW27" t="inlineStr">
         <is>
-          <t>narrateur|Amir ferme le sac au pied du lit.
-enfant-m|On peut jouer ?
-papa|Oui. Sur le tapis.
-narrateur|Amir sort deux cubes.
-narrateur|Il les pose sur une rayure crème.
-narrateur|Le tapis rayé est calme.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir reprend le bateau.
+narrateur|Il le remet dans le sac.
+narrateur|Le manteau rentre aussi.
+narrateur|On referme. Zzz.
+narrateur|Un grain de sable reste sur le bois.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -5880,17 +5811,17 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Le livre est ouvert sur la commode. Une image montre un bateau. Amir le ferme tout doux. Le livre dans le sac, Amir. Le livre. Il le glisse près de la pomme. Le bateau est dedans aussi. Oui.</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Près de le livre. Lina pose la chambre. une pomme est derrière. On écoute jusqu'au bout. Lina dit merci à maman. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Près de le livre. Lina pose la chambre. une pomme est derrière. On écoute jusqu'au bout. Lina dit merci à maman. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -6020,14 +5951,13 @@
       <c r="AV28" s="2" t="inlineStr"/>
       <c r="AW28" t="inlineStr">
         <is>
-          <t>narrateur|Le livre est ouvert sur la commode.
-narrateur|Une image montre un bateau.
-narrateur|Amir le ferme tout doux.
-papa|Le livre dans le sac, Amir.
-enfant-m|Le livre.
-narrateur|Il le glisse près de la pomme.
-papa|Le bateau est dedans aussi.
-enfant-m|Oui.</t>
+          <t>narrateur|Amir sort le bateau.
+narrateur|Il le donne à papa.
+papa|Près du bord, ensemble.
+narrateur|Papa le pose. Amir tient le sac.
+narrateur|Le bateau part.
+narrateur|Amir marche le long de l'eau.
+narrateur|Le sac est à l'épaule.</t>
         </is>
       </c>
     </row>
@@ -6054,17 +5984,17 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Le sac est sur la commode, une seconde. On va jouer ? Oui. Amir ouvre le sac. Il touche la couverture du livre. Le rayon de soleil a quitté le tapis. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -6194,12 +6124,12 @@
       <c r="AV29" s="2" t="inlineStr"/>
       <c r="AW29" t="inlineStr">
         <is>
-          <t>narrateur|Le sac est sur la commode, une seconde.
-maman|On va jouer ?
-enfant-m|Oui.
-narrateur|Amir ouvre le sac.
-narrateur|Il touche la couverture du livre.
-narrateur|Le rayon de soleil a quitté le tapis.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir reprend le bateau.
+narrateur|Il le remet dans le sac.
+narrateur|Le manteau rentre aussi.
+narrateur|On referme. Zzz.
+narrateur|Un grain de sable reste sur le bois.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -6227,17 +6157,17 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>La dînette est dans la caisse, sous le lit. Une petite assiette dépasse. Amir tire l'assiette. Un couvercle tombe sur le tapis. Toc. L'assiette dans le sac. L'assiette. Il la met près de la pomme. Le couvercle, on le laisse. D'accord.</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Lina montre la dînette. Maman a vu une pomme. Et la chambre. Un crochet tient bien le manteau. Lina ferme le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lina montre la dînette. Maman a vu une pomme. Et la chambre. Un crochet tient bien le manteau. Lina ferme le &lt;emphasis&gt;sac&lt;/emphasis&gt;. On met dans le sac ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -6367,16 +6297,11 @@
       <c r="AV30" s="2" t="inlineStr"/>
       <c r="AW30" t="inlineStr">
         <is>
-          <t>narrateur|La dînette est dans la caisse, sous le lit.
-narrateur|Une petite assiette dépasse.
-narrateur|Amir tire l'assiette.
-narrateur|Un couvercle tombe sur le tapis.
-narrateur|Toc.
-maman|L'assiette dans le sac.
-enfant-m|L'assiette.
-narrateur|Il la met près de la pomme.
-maman|Le couvercle, on le laisse.
-enfant-m|D'accord.</t>
+          <t>narrateur|Amir pose d'abord le sac.
+narrateur|Il pose le bateau sur le sac.
+narrateur|Il regarde la flaque.
+narrateur|Puis il met le bateau dans l'eau.
+papa|Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
     </row>
@@ -6403,17 +6328,17 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Amir s'assoit sur le tapis. Le sac est sur ses genoux. Le sac est prêt. Merci. Il sort l'assiette. Il y pose la pomme, pour rire. On va vraiment jouer, maintenant. La couverture retombe sur le lit. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -6543,14 +6468,12 @@
       <c r="AV31" s="2" t="inlineStr"/>
       <c r="AW31" t="inlineStr">
         <is>
-          <t>narrateur|Amir s'assoit sur le tapis.
-narrateur|Le sac est sur ses genoux.
-papa|Le sac est prêt.
-enfant-m|Merci.
-narrateur|Il sort l'assiette.
-narrateur|Il y pose la pomme, pour rire.
-maman|On va vraiment jouer, maintenant.
-narrateur|La couverture retombe sur le lit.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir reprend le bateau.
+narrateur|Il le remet dans le sac.
+narrateur|Le manteau rentre aussi.
+narrateur|On referme. Zzz.
+narrateur|Un grain de sable reste sur le bois.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -6578,17 +6501,17 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Papa ouvre le frigo. Un air frais sort. Un petit yaourt attend sur la tablette. Papa le tend. Le couvercle glisse un peu. Amir le tient à deux mains. Tout doux. Dans le sac. Le yaourt. Amir le pose bien droit. Il tient ? Il tient. Le pot est froid contre le tissu.</t>
+          <t>Amir glisse le bateau au fond du sac. Toc. La voile dépasse. Il la rentre. Les bottes sont près de la porte. Elles sont encore mouillées dehors. Attends. Je les essuie. Maman frotte le bout, tout doux. Merci, maman. Amir les pose à côté du sac. Au pied, juste avant de sortir.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Lina met un yaourt dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. Maman a dit : le yaourt. On met dans le sac ce que l'adulte a dit. Le pot est frais. Lina le cale. Papa ferme un coin du sac.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir glisse le bateau au fond du sac. Toc. La voile dépasse. Il la rentre. Les bottes sont près de la porte. Elles sont encore mouillées dehors. Attends. Je les essuie. Maman frotte le bout, tout doux. Merci, maman. Amir les pose à côté du sac. Au pied, juste avant de sortir.</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lina met un yaourt dans le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Maman a dit : le yaourt. On met dans le sac ce que l'adulte a dit. Le pot est frais. Lina le cale. Papa ferme un coin du sac.&lt;/slow&gt; [pause]</t>
+          <t>Amir glisse le bateau au fond du sac. Toc. La voile dépasse. Il la rentre. Les bottes sont près de la porte. Elles sont encore mouillées dehors. Attends. Je les essuie. Maman frotte le bout, tout doux. Merci, maman. Amir les pose à côté du sac. Au pied, juste avant de sortir.</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -6718,18 +6641,16 @@
       <c r="AV32" s="2" t="inlineStr"/>
       <c r="AW32" t="inlineStr">
         <is>
-          <t>narrateur|Papa ouvre le frigo.
-narrateur|Un air frais sort.
-narrateur|Un petit yaourt attend sur la tablette.
-narrateur|Papa le tend.
-narrateur|Le couvercle glisse un peu.
-narrateur|Amir le tient à deux mains.
-papa|Tout doux. Dans le sac.
-enfant-m|Le yaourt.
-narrateur|Amir le pose bien droit.
-papa|Il tient ?
-enfant-m|Il tient.
-narrateur|Le pot est froid contre le tissu.</t>
+          <t>narrateur|Amir glisse le bateau au fond du sac.
+narrateur|Toc.
+narrateur|La voile dépasse. Il la rentre.
+narrateur|Les bottes sont près de la porte.
+narrateur|Elles sont encore mouillées dehors.
+maman|Attends. Je les essuie.
+narrateur|Maman frotte le bout, tout doux.
+enfant-m|Merci, maman.
+narrateur|Amir les pose à côté du sac.
+maman|Au pied, juste avant de sortir.</t>
         </is>
       </c>
     </row>
@@ -6756,27 +6677,27 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>On met quoi dans le sac ?</t>
+          <t>Qui essuie les bottes ?</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; : on met ce que l'adulte a dit ?&lt;/prosody&gt;&lt;break time="250ms"/&gt;&lt;/speak&gt;</t>
+          <t>Qui essuie les bottes ?</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le &lt;emphasis&gt;sac&lt;/emphasis&gt; : on met ce que l'adulte a dit ?&lt;/slow&gt;</t>
+          <t>Qui essuie les bottes ?</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>le yaourt</t>
+          <t>maman</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>le yaourt | un yaourt | yaourt | le pot</t>
+          <t>maman | ma maman</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -6786,12 +6707,12 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>C'est dans le sac. Le yaourt.</t>
+          <t>Maman essuie les bottes.</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>Dis : le yaourt.</t>
+          <t>C'est maman qui essuie.</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr"/>
@@ -6916,7 +6837,7 @@
       </c>
       <c r="AW33" t="inlineStr">
         <is>
-          <t>narrateur|On met quoi dans le sac ?</t>
+          <t>narrateur|Qui essuie les bottes ?</t>
         </is>
       </c>
     </row>
@@ -6943,17 +6864,17 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Le yaourt est au fond. Il est froid. Amir veut fermer le sac. On n'a pas fini. Il manque encore des choses. D'accord.</t>
+          <t>Maman a essuyé les bottes. Le bateau est dans le sac. Les bottes attendent près de la porte. On va à la flaque.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Oui. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. Lina retient le geste. Maman sourit. On met dans le sac ce que l'adulte a dit.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Maman a essuyé les bottes. Le bateau est dans le sac. Les bottes attendent près de la porte. On va à la flaque.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Oui. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. Lina retient le geste. Maman sourit. On met dans le sac ce que l'adulte a dit.&lt;/slow&gt; [pause]</t>
+          <t>Maman a essuyé les bottes. Le bateau est dans le sac. Les bottes attendent près de la porte. On va à la flaque.</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
@@ -7087,12 +7008,10 @@
       </c>
       <c r="AW34" t="inlineStr">
         <is>
-          <t>narrateur|Le yaourt est au fond.
-narrateur|Il est froid.
-narrateur|Amir veut fermer le sac.
-papa|On n'a pas fini.
-papa|Il manque encore des choses.
-enfant-m|D'accord.</t>
+          <t>narrateur|Maman a essuyé les bottes.
+narrateur|Le bateau est dans le sac.
+narrateur|Les bottes attendent près de la porte.
+papa|On va à la flaque.</t>
         </is>
       </c>
     </row>
@@ -7119,17 +7038,17 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>On peut aller où ? La cuisine, le jardin, ou la chambre.</t>
+          <t>Quelle flaque ? Sous la gouttière, près du potager, ou près du bac.</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;On peut prendre la cuisine, le jardin, ou la chambre.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>Quelle flaque ? Sous la gouttière, près du potager, ou près du bac.</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;On peut prendre la cuisine, le jardin, ou la chambre.&lt;/slow&gt; [pause]</t>
+          <t>Quelle flaque ? Sous la gouttière, près du potager, ou près du bac.</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr"/>
@@ -7147,7 +7066,7 @@
       <c r="L35" s="2" t="inlineStr"/>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>la cuisine</t>
+          <t>sous la gouttière</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr">
@@ -7157,7 +7076,7 @@
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>le jardin</t>
+          <t>près du potager</t>
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr">
@@ -7167,7 +7086,7 @@
       </c>
       <c r="Q35" s="2" t="inlineStr">
         <is>
-          <t>la chambre</t>
+          <t>près du bac</t>
         </is>
       </c>
       <c r="R35" s="2" t="inlineStr">
@@ -7283,8 +7202,8 @@
       <c r="AV35" s="2" t="inlineStr"/>
       <c r="AW35" t="inlineStr">
         <is>
-          <t>narrateur|On peut aller où ?
-narrateur|La cuisine, le jardin, ou la chambre.</t>
+          <t>narrateur|Quelle flaque ?
+narrateur|Sous la gouttière, près du potager, ou près du bac.</t>
         </is>
       </c>
     </row>
@@ -7311,17 +7230,17 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Amir pose le sac sur la table. Le yaourt reste bien droit. Le frigo ronronne tout bas. Amir ouvre le tiroir du bas. Une petite cuillère brille. La cuillère, dans le sac. La cuillère. Elle est lisse et froide. Il la glisse à côté du yaourt. Elle est à côté ? Oui, papa. Ça sent encore la soupe.</t>
+          <t>Amir enfile les bottes près de la porte. Elles sont un peu froides, plus mouillées. Sous la gouttière, une flaque ronde. Ses bottes font un petit clap dans l'herbe. Une goutte tombe. Plic. Le bateau, maintenant.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Ensuite Lina va dans le jardin. Elle met les cubes au soleil, puis dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. On met dans le sac ce que l'adulte a dit. Maman dit : je suis là. On met dans le sac ce que l'adulte a dit.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir enfile les bottes près de la porte. Elles sont un peu froides, plus mouillées. Sous la gouttière, une flaque ronde. Ses bottes font un petit clap dans l'herbe. Une goutte tombe. Plic. Le bateau, maintenant.</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Ensuite Lina va dans le jardin. Elle met les cubes au soleil, puis dans le &lt;emphasis&gt;sac&lt;/emphasis&gt;. On met dans le sac ce que l'adulte a dit. Maman dit : je suis là. On met dans le sac ce que l'adulte a dit.&lt;/slow&gt; [pause]</t>
+          <t>Amir enfile les bottes près de la porte. Elles sont un peu froides, plus mouillées. Sous la gouttière, une flaque ronde. Ses bottes font un petit clap dans l'herbe. Une goutte tombe. Plic. Le bateau, maintenant.</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
@@ -7451,18 +7370,12 @@
       <c r="AV36" s="2" t="inlineStr"/>
       <c r="AW36" t="inlineStr">
         <is>
-          <t>narrateur|Amir pose le sac sur la table.
-narrateur|Le yaourt reste bien droit.
-narrateur|Le frigo ronronne tout bas.
-narrateur|Amir ouvre le tiroir du bas.
-narrateur|Une petite cuillère brille.
-papa|La cuillère, dans le sac.
-enfant-m|La cuillère.
-narrateur|Elle est lisse et froide.
-narrateur|Il la glisse à côté du yaourt.
-papa|Elle est à côté ?
-enfant-m|Oui, papa.
-narrateur|Ça sent encore la soupe.</t>
+          <t>narrateur|Amir enfile les bottes près de la porte.
+narrateur|Elles sont un peu froides, plus mouillées.
+narrateur|Sous la gouttière, une flaque ronde.
+narrateur|Ses bottes font un petit clap dans l'herbe.
+narrateur|Une goutte tombe. Plic.
+papa|Le bateau, maintenant.</t>
         </is>
       </c>
     </row>
@@ -7489,17 +7402,17 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre quoi ? Les cubes, le livre, ou la dînette.</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;On peut prendre les cubes, le livre, ou la dînette.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;On peut prendre les cubes, le livre, ou la dînette.&lt;/slow&gt; [pause]</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr"/>
@@ -7517,7 +7430,7 @@
       <c r="L37" s="2" t="inlineStr"/>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>les cubes</t>
+          <t>au milieu</t>
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr">
@@ -7527,7 +7440,7 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>le livre</t>
+          <t>près du bord</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
@@ -7537,7 +7450,7 @@
       </c>
       <c r="Q37" s="2" t="inlineStr">
         <is>
-          <t>la dînette</t>
+          <t>sur le sac</t>
         </is>
       </c>
       <c r="R37" s="2" t="inlineStr">
@@ -7653,8 +7566,8 @@
       <c r="AV37" s="2" t="inlineStr"/>
       <c r="AW37" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre quoi ?
-narrateur|Les cubes, le livre, ou la dînette.</t>
+          <t>narrateur|On pose le bateau…
+narrateur|Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
     </row>
@@ -7681,17 +7594,17 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Les cubes sont près du saladier. Amir en prend trois. Il fait un petit pont. Le pont touche le yaourt. Les cubes, dans le sac. Pas le pont. Les cubes. Il les empile près du pot. Le pot est encore droit ? Droit.</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Lina a choisi un yaourt. Puis la cuisine. Puis les cubes. Un galet est encore chaud. Lina plie un pull. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lina a choisi un yaourt. Puis la cuisine. Puis les cubes. Un galet est encore chaud. Lina plie un pull. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -7821,15 +7734,13 @@
       <c r="AV38" s="2" t="inlineStr"/>
       <c r="AW38" t="inlineStr">
         <is>
-          <t>narrateur|Les cubes sont près du saladier.
-narrateur|Amir en prend trois.
-narrateur|Il fait un petit pont.
-narrateur|Le pont touche le yaourt.
-maman|Les cubes, dans le sac. Pas le pont.
-enfant-m|Les cubes.
-narrateur|Il les empile près du pot.
-maman|Le pot est encore droit ?
-enfant-m|Droit.</t>
+          <t>narrateur|Amir sort le bateau du sac.
+narrateur|Il le pose au milieu de l'eau.
+narrateur|La voile se tient.
+narrateur|Un peu d'eau touche le papier.
+papa|Il avance.
+narrateur|Amir souffle. Ffff.
+narrateur|Le bateau part tout doux.</t>
         </is>
       </c>
     </row>
@@ -7856,17 +7767,17 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Amir ferme le sac près de l'évier. Le yaourt est encore droit ? Oui. On joue aux cubes ici. Amir sort deux cubes. Il les pose contre la cuillère. Toc, toc. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
@@ -7996,13 +7907,12 @@
       <c r="AV39" s="2" t="inlineStr"/>
       <c r="AW39" t="inlineStr">
         <is>
-          <t>narrateur|Amir ferme le sac près de l'évier.
-papa|Le yaourt est encore droit ?
-enfant-m|Oui.
-maman|On joue aux cubes ici.
-narrateur|Amir sort deux cubes.
-narrateur|Il les pose contre la cuillère.
-narrateur|Toc, toc.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir reprend le bateau.
+narrateur|Il le remet dans le sac.
+narrateur|Les bottes restent aux pieds, jusqu'à la porte.
+narrateur|On referme. Zzz.
+narrateur|La gouttière fait un dernier plic.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -8030,17 +7940,17 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Le livre est sous un torchon. Le torchon sent le propre. Amir soulève le coin. Le livre dans le sac. Le livre. Il le sort du torchon. Il le glisse près du yaourt, à plat. Loin du pot froid. Loin.</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Lina s'arrête près de le livre. la cuisine est rangé. On rit un peu. Lina raccroche un linge. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lina s'arrête près de le livre. la cuisine est rangé. On rit un peu. Lina raccroche un linge. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -8170,15 +8080,13 @@
       <c r="AV40" s="2" t="inlineStr"/>
       <c r="AW40" t="inlineStr">
         <is>
-          <t>narrateur|Le livre est sous un torchon.
-narrateur|Le torchon sent le propre.
-narrateur|Amir soulève le coin.
-papa|Le livre dans le sac.
-enfant-m|Le livre.
-narrateur|Il le sort du torchon.
-narrateur|Il le glisse près du yaourt, à plat.
-papa|Loin du pot froid.
-enfant-m|Loin.</t>
+          <t>narrateur|Amir sort le bateau.
+narrateur|Il le donne à papa.
+papa|Près du bord, ensemble.
+narrateur|Papa le pose. Amir tient le sac.
+narrateur|Le bateau part.
+narrateur|Amir marche le long de l'eau.
+narrateur|Le sac est à l'épaule.</t>
         </is>
       </c>
     </row>
@@ -8205,17 +8113,17 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Le sac est posé contre la chaise. On lit ? Une page. Puis on range. Amir ouvre le sac. Il montre la couverture à papa. On y va. Ça sent encore un peu le four. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
@@ -8345,13 +8253,12 @@
       <c r="AV41" s="2" t="inlineStr"/>
       <c r="AW41" t="inlineStr">
         <is>
-          <t>narrateur|Le sac est posé contre la chaise.
-enfant-m|On lit ?
-maman|Une page. Puis on range.
-narrateur|Amir ouvre le sac.
-narrateur|Il montre la couverture à papa.
-papa|On y va.
-narrateur|Ça sent encore un peu le four.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir reprend le bateau.
+narrateur|Il le remet dans le sac.
+narrateur|Les bottes restent aux pieds, jusqu'à la porte.
+narrateur|On referme. Zzz.
+narrateur|La gouttière fait un dernier plic.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -8379,17 +8286,17 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>La dînette est dans le tiroir du haut. Une casserole minuscule brille. Amir ouvre le tiroir tout doux. La casserole dans le sac. La casserole. Il la met près du yaourt. Elle fait un tout petit cling. On fera la soupe pour de faux. Oui.</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Lina se souvient de un yaourt. Et de la cuisine. Et de la dînette. On souffle doucement. Lina écoute maman encore une fois. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lina se souvient de un yaourt. Et de la cuisine. Et de la dînette. On souffle doucement. Lina écoute maman encore une fois. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -8519,15 +8426,11 @@
       <c r="AV42" s="2" t="inlineStr"/>
       <c r="AW42" t="inlineStr">
         <is>
-          <t>narrateur|La dînette est dans le tiroir du haut.
-narrateur|Une casserole minuscule brille.
-narrateur|Amir ouvre le tiroir tout doux.
-maman|La casserole dans le sac.
-enfant-m|La casserole.
-narrateur|Il la met près du yaourt.
-narrateur|Elle fait un tout petit cling.
-maman|On fera la soupe pour de faux.
-enfant-m|Oui.</t>
+          <t>narrateur|Amir pose d'abord le sac.
+narrateur|Il pose le bateau sur le sac.
+narrateur|Il regarde la flaque.
+narrateur|Puis il met le bateau dans l'eau.
+papa|Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
     </row>
@@ -8554,17 +8457,17 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Amir tient la sangle du sac. Le sac est prêt. La casserole aussi. Il sort la casserole. Il fait semblant de remuer. La soupe de yaourt, c'est nouveau. Amir rit. La cuisine est calme. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -8694,14 +8597,12 @@
       <c r="AV43" s="2" t="inlineStr"/>
       <c r="AW43" t="inlineStr">
         <is>
-          <t>narrateur|Amir tient la sangle du sac.
-papa|Le sac est prêt.
-enfant-m|La casserole aussi.
-narrateur|Il sort la casserole.
-narrateur|Il fait semblant de remuer.
-maman|La soupe de yaourt, c'est nouveau.
-narrateur|Amir rit.
-narrateur|La cuisine est calme.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir reprend le bateau.
+narrateur|Il le remet dans le sac.
+narrateur|Les bottes restent aux pieds, jusqu'à la porte.
+narrateur|On referme. Zzz.
+narrateur|La gouttière fait un dernier plic.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -8729,17 +8630,17 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Amir marche dans le jardin avec le sac. Le yaourt reste au fond, au frais. Un galet est encore chaud au soleil. Un petit gant est posé dessus. Le petit gant, dans le sac. Le gant. Le gant est un peu rêche. Amir le pose près du yaourt. Une goutte tombe de la gouttière. Plic ploc. Tu as entendu ? Oui.</t>
+          <t>Amir enfile les bottes. Ils vont près du potager. La terre est molle. Les bottes tiennent. La flaque est ronde, entre deux choux. Le bateau, Amir.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Ensuite Lina va dans le jardin. Elle met le livre à l'ombre, puis dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. On met dans le sac ce que l'adulte a dit. Maman reste tout près. On met dans le sac ce que l'adulte a dit.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir enfile les bottes. Ils vont près du potager. La terre est molle. Les bottes tiennent. La flaque est ronde, entre deux choux. Le bateau, Amir.</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Ensuite Lina va dans le jardin. Elle met le livre à l'ombre, puis dans le &lt;emphasis&gt;sac&lt;/emphasis&gt;. On met dans le sac ce que l'adulte a dit. Maman reste tout près. On met dans le sac ce que l'adulte a dit.&lt;/slow&gt; [pause]</t>
+          <t>Amir enfile les bottes. Ils vont près du potager. La terre est molle. Les bottes tiennent. La flaque est ronde, entre deux choux. Le bateau, Amir.</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
@@ -8869,17 +8770,11 @@
       <c r="AV44" s="2" t="inlineStr"/>
       <c r="AW44" t="inlineStr">
         <is>
-          <t>narrateur|Amir marche dans le jardin avec le sac.
-narrateur|Le yaourt reste au fond, au frais.
-narrateur|Un galet est encore chaud au soleil.
-narrateur|Un petit gant est posé dessus.
-maman|Le petit gant, dans le sac.
-enfant-m|Le gant.
-narrateur|Le gant est un peu rêche.
-narrateur|Amir le pose près du yaourt.
-narrateur|Une goutte tombe de la gouttière.
-papa|Plic ploc. Tu as entendu ?
-enfant-m|Oui.</t>
+          <t>narrateur|Amir enfile les bottes.
+narrateur|Ils vont près du potager.
+narrateur|La terre est molle. Les bottes tiennent.
+narrateur|La flaque est ronde, entre deux choux.
+maman|Le bateau, Amir.</t>
         </is>
       </c>
     </row>
@@ -8906,17 +8801,17 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre quoi ? Les cubes, le livre, ou la dînette.</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;On peut prendre les cubes, le livre, ou la dînette.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;On peut prendre les cubes, le livre, ou la dînette.&lt;/slow&gt; [pause]</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr"/>
@@ -8934,7 +8829,7 @@
       <c r="L45" s="2" t="inlineStr"/>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>les cubes</t>
+          <t>au milieu</t>
         </is>
       </c>
       <c r="N45" s="2" t="inlineStr">
@@ -8944,7 +8839,7 @@
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>le livre</t>
+          <t>près du bord</t>
         </is>
       </c>
       <c r="P45" s="2" t="inlineStr">
@@ -8954,7 +8849,7 @@
       </c>
       <c r="Q45" s="2" t="inlineStr">
         <is>
-          <t>la dînette</t>
+          <t>sur le sac</t>
         </is>
       </c>
       <c r="R45" s="2" t="inlineStr">
@@ -9070,8 +8965,8 @@
       <c r="AV45" s="2" t="inlineStr"/>
       <c r="AW45" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre quoi ?
-narrateur|Les cubes, le livre, ou la dînette.</t>
+          <t>narrateur|On pose le bateau…
+narrateur|Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
     </row>
@@ -9098,17 +8993,17 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Les cubes sont dans l'herbe rase. Un cube a un peu d'herbe. Amir souffle dessus. Le cube propre, dans le sac. Le cube propre. Il le frotte, puis le met près du yaourt. On laisse l'herbe au jardin.</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Avec les cubes. Après le jardin. Près de un yaourt. Lina s'arrête. On range un objet. Lina montre les cubes à maman. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Avec les cubes. Après le jardin. Près de un yaourt. Lina s'arrête. On range un objet. Lina montre les cubes à maman. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -9238,13 +9133,13 @@
       <c r="AV46" s="2" t="inlineStr"/>
       <c r="AW46" t="inlineStr">
         <is>
-          <t>narrateur|Les cubes sont dans l'herbe rase.
-narrateur|Un cube a un peu d'herbe.
-narrateur|Amir souffle dessus.
-papa|Le cube propre, dans le sac.
-enfant-m|Le cube propre.
-narrateur|Il le frotte, puis le met près du yaourt.
-papa|On laisse l'herbe au jardin.</t>
+          <t>narrateur|Amir sort le bateau du sac.
+narrateur|Il le pose au milieu de l'eau.
+narrateur|La voile se tient.
+narrateur|Un peu d'eau touche le papier.
+papa|Il avance.
+narrateur|Amir souffle. Ffff.
+narrateur|Le bateau part tout doux.</t>
         </is>
       </c>
     </row>
@@ -9271,17 +9166,17 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Amir referme le sac près du galet. Le yaourt est encore au frais ? Oui. Il sort le cube. Il le pose sur le galet chaud. On rentre. Le jardin sent l'herbe mouillée. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -9411,13 +9306,12 @@
       <c r="AV47" s="2" t="inlineStr"/>
       <c r="AW47" t="inlineStr">
         <is>
-          <t>narrateur|Amir referme le sac près du galet.
-maman|Le yaourt est encore au frais ?
-enfant-m|Oui.
-narrateur|Il sort le cube.
-narrateur|Il le pose sur le galet chaud.
-papa|On rentre.
-narrateur|Le jardin sent l'herbe mouillée.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir reprend le bateau.
+narrateur|Il le remet dans le sac.
+narrateur|Les bottes restent aux pieds, jusqu'à la porte.
+narrateur|On referme. Zzz.
+narrateur|Une feuille lâche la flaque.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -9445,17 +9339,17 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Le livre est sur le muret, au soleil. La couverture est un peu chaude. Amir le souffle. Le livre dans le sac. Le livre. Il le glisse près du yaourt. Pas collé au pot froid. Pas collé.</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Lina range le jardin. le livre reste près de un yaourt. On dit merci. Lina souffle, puis sourit à maman. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lina range le jardin. le livre reste près de un yaourt. On dit merci. Lina souffle, puis sourit à maman. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -9585,14 +9479,13 @@
       <c r="AV48" s="2" t="inlineStr"/>
       <c r="AW48" t="inlineStr">
         <is>
-          <t>narrateur|Le livre est sur le muret, au soleil.
-narrateur|La couverture est un peu chaude.
-narrateur|Amir le souffle.
-maman|Le livre dans le sac.
-enfant-m|Le livre.
-narrateur|Il le glisse près du yaourt.
-maman|Pas collé au pot froid.
-enfant-m|Pas collé.</t>
+          <t>narrateur|Amir sort le bateau.
+narrateur|Il le donne à papa.
+papa|Près du bord, ensemble.
+narrateur|Papa le pose. Amir tient le sac.
+narrateur|Le bateau part.
+narrateur|Amir marche le long de l'eau.
+narrateur|Le sac est à l'épaule.</t>
         </is>
       </c>
     </row>
@@ -9619,17 +9512,17 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Le sac est posé sur le muret. Une page ? Une page. Le vent est doux. Amir ouvre le livre. Une page tremble. Il referme, puis le sac. On rentre avec le sac. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -9759,13 +9652,12 @@
       <c r="AV49" s="2" t="inlineStr"/>
       <c r="AW49" t="inlineStr">
         <is>
-          <t>narrateur|Le sac est posé sur le muret.
-enfant-m|Une page ?
-papa|Une page. Le vent est doux.
-narrateur|Amir ouvre le livre.
-narrateur|Une page tremble.
-narrateur|Il referme, puis le sac.
-narrateur|On rentre avec le sac.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir reprend le bateau.
+narrateur|Il le remet dans le sac.
+narrateur|Les bottes restent aux pieds, jusqu'à la porte.
+narrateur|On referme. Zzz.
+narrateur|Une feuille lâche la flaque.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -9793,17 +9685,17 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Une tasse de dînette est retournée dans l'herbe. Une goutte d'eau brille dedans. Amir la vide sur l'herbe. La tasse dans le sac. La tasse. Il la met près du yaourt. Elle est vide ? Vide.</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;la dînette est là. le jardin aussi. un yaourt reste dans le souvenir. Un ballon s'immobilise. Lina essuie ses mains. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;la dînette est là. le jardin aussi. un yaourt reste dans le souvenir. Un ballon s'immobilise. Lina essuie ses mains. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -9933,14 +9825,11 @@
       <c r="AV50" s="2" t="inlineStr"/>
       <c r="AW50" t="inlineStr">
         <is>
-          <t>narrateur|Une tasse de dînette est retournée dans l'herbe.
-narrateur|Une goutte d'eau brille dedans.
-narrateur|Amir la vide sur l'herbe.
-papa|La tasse dans le sac.
-enfant-m|La tasse.
-narrateur|Il la met près du yaourt.
-papa|Elle est vide ?
-enfant-m|Vide.</t>
+          <t>narrateur|Amir pose d'abord le sac.
+narrateur|Il pose le bateau sur le sac.
+narrateur|Il regarde la flaque.
+narrateur|Puis il met le bateau dans l'eau.
+papa|Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
     </row>
@@ -9967,17 +9856,17 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Amir tient le sac à deux mains. On rentre. La tasse aussi. Il fait un tout petit clin. Tasse contre yaourt. Santé, tout doux. Le jardin sent l'herbe mouillée. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
@@ -10107,13 +9996,12 @@
       <c r="AV51" s="2" t="inlineStr"/>
       <c r="AW51" t="inlineStr">
         <is>
-          <t>narrateur|Amir tient le sac à deux mains.
-maman|On rentre.
-enfant-m|La tasse aussi.
-narrateur|Il fait un tout petit clin.
-narrateur|Tasse contre yaourt.
-papa|Santé, tout doux.
-narrateur|Le jardin sent l'herbe mouillée.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir reprend le bateau.
+narrateur|Il le remet dans le sac.
+narrateur|Les bottes restent aux pieds, jusqu'à la porte.
+narrateur|On referme. Zzz.
+narrateur|Une feuille lâche la flaque.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -10141,17 +10029,17 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Amir s'assoit sur le tapis de la chambre. Le yaourt fait un petit rond dans le sac. La couverture est douce contre le genou. Un chausson dépasse sous le lit. Amir tire les deux chaussons. Les chaussons, dans le sac. Les chaussons. Ils sont chauds et mous. Il les glisse près du yaourt. Le rayon de soleil a bougé. Il touche maintenant le sac.</t>
+          <t>Amir enfile les bottes. Ils vont près du bac à sable. Une flaque borde le bois du bac. Les bottes s'arrêtent au bord, pile. Le bateau, Amir.</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Ensuite Lina va dans le jardin. Elle met une tasse de dînette, puis dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. On met dans le sac ce que l'adulte a dit. Maman montre le geste, lentement. On met dans le sac ce que l'adulte a dit.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir enfile les bottes. Ils vont près du bac à sable. Une flaque borde le bois du bac. Les bottes s'arrêtent au bord, pile. Le bateau, Amir.</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Ensuite Lina va dans le jardin. Elle met une tasse de dînette, puis dans le &lt;emphasis&gt;sac&lt;/emphasis&gt;. On met dans le sac ce que l'adulte a dit. Maman montre le geste, lentement. On met dans le sac ce que l'adulte a dit.&lt;/slow&gt; [pause]</t>
+          <t>Amir enfile les bottes. Ils vont près du bac à sable. Une flaque borde le bois du bac. Les bottes s'arrêtent au bord, pile. Le bateau, Amir.</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
@@ -10281,17 +10169,11 @@
       <c r="AV52" s="2" t="inlineStr"/>
       <c r="AW52" t="inlineStr">
         <is>
-          <t>narrateur|Amir s'assoit sur le tapis de la chambre.
-narrateur|Le yaourt fait un petit rond dans le sac.
-narrateur|La couverture est douce contre le genou.
-narrateur|Un chausson dépasse sous le lit.
-narrateur|Amir tire les deux chaussons.
-papa|Les chaussons, dans le sac.
-enfant-m|Les chaussons.
-narrateur|Ils sont chauds et mous.
-narrateur|Il les glisse près du yaourt.
-narrateur|Le rayon de soleil a bougé.
-narrateur|Il touche maintenant le sac.</t>
+          <t>narrateur|Amir enfile les bottes.
+narrateur|Ils vont près du bac à sable.
+narrateur|Une flaque borde le bois du bac.
+narrateur|Les bottes s'arrêtent au bord, pile.
+papa|Le bateau, Amir.</t>
         </is>
       </c>
     </row>
@@ -10318,17 +10200,17 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre quoi ? Les cubes, le livre, ou la dînette.</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;On peut prendre les cubes, le livre, ou la dînette.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;On peut prendre les cubes, le livre, ou la dînette.&lt;/slow&gt; [pause]</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr"/>
@@ -10346,7 +10228,7 @@
       <c r="L53" s="2" t="inlineStr"/>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>les cubes</t>
+          <t>au milieu</t>
         </is>
       </c>
       <c r="N53" s="2" t="inlineStr">
@@ -10356,7 +10238,7 @@
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>le livre</t>
+          <t>près du bord</t>
         </is>
       </c>
       <c r="P53" s="2" t="inlineStr">
@@ -10366,7 +10248,7 @@
       </c>
       <c r="Q53" s="2" t="inlineStr">
         <is>
-          <t>la dînette</t>
+          <t>sur le sac</t>
         </is>
       </c>
       <c r="R53" s="2" t="inlineStr">
@@ -10482,8 +10364,8 @@
       <c r="AV53" s="2" t="inlineStr"/>
       <c r="AW53" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre quoi ?
-narrateur|Les cubes, le livre, ou la dînette.</t>
+          <t>narrateur|On pose le bateau…
+narrateur|Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
     </row>
@@ -10510,17 +10392,17 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Les cubes sont derrière le coffre. Amir pousse le coffre d'un doigt. Deux cubes apparaissent. Les cubes dans le sac. Les cubes. Il les met près du yaourt. Loin du pot, un peu. Loin.</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Lina rejoint les cubes. la chambre est rangé. un yaourt est fini. Une tasse cliquette. Lina dit : j'ai appris. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lina rejoint les cubes. la chambre est rangé. un yaourt est fini. Une tasse cliquette. Lina dit : j'ai appris. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -10650,14 +10532,13 @@
       <c r="AV54" s="2" t="inlineStr"/>
       <c r="AW54" t="inlineStr">
         <is>
-          <t>narrateur|Les cubes sont derrière le coffre.
-narrateur|Amir pousse le coffre d'un doigt.
-narrateur|Deux cubes apparaissent.
-maman|Les cubes dans le sac.
-enfant-m|Les cubes.
-narrateur|Il les met près du yaourt.
-maman|Loin du pot, un peu.
-enfant-m|Loin.</t>
+          <t>narrateur|Amir sort le bateau du sac.
+narrateur|Il le pose au milieu de l'eau.
+narrateur|La voile se tient.
+narrateur|Un peu d'eau touche le papier.
+papa|Il avance.
+narrateur|Amir souffle. Ffff.
+narrateur|Le bateau part tout doux.</t>
         </is>
       </c>
     </row>
@@ -10684,17 +10565,17 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Amir ferme le sac au pied du lit. Les chaussons et les cubes sont dedans. Le sac est prêt. Il sort un cube. Il le fait rouler sur une rayure bleue. On peut jouer. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -10824,12 +10705,12 @@
       <c r="AV55" s="2" t="inlineStr"/>
       <c r="AW55" t="inlineStr">
         <is>
-          <t>narrateur|Amir ferme le sac au pied du lit.
-papa|Les chaussons et les cubes sont dedans.
-enfant-m|Le sac est prêt.
-narrateur|Il sort un cube.
-narrateur|Il le fait rouler sur une rayure bleue.
-maman|On peut jouer.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir reprend le bateau.
+narrateur|Il le remet dans le sac.
+narrateur|Les bottes restent aux pieds, jusqu'à la porte.
+narrateur|On referme. Zzz.
+narrateur|Un grain de sable reste sur le bois.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -10857,17 +10738,17 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Le livre est coincé entre deux peluches. Amir le tire tout doux. Le livre dans le sac. Le livre. Il le glisse près du yaourt. Les peluches restent au lit. D'accord.</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Près de le livre. Lina pose la chambre. un yaourt est derrière. Un chat miaule une fois. Lina range encore un peu, près de maman. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Près de le livre. Lina pose la chambre. un yaourt est derrière. Un chat miaule une fois. Lina range encore un peu, près de maman. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -10997,13 +10878,13 @@
       <c r="AV56" s="2" t="inlineStr"/>
       <c r="AW56" t="inlineStr">
         <is>
-          <t>narrateur|Le livre est coincé entre deux peluches.
-narrateur|Amir le tire tout doux.
-papa|Le livre dans le sac.
-enfant-m|Le livre.
-narrateur|Il le glisse près du yaourt.
-papa|Les peluches restent au lit.
-enfant-m|D'accord.</t>
+          <t>narrateur|Amir sort le bateau.
+narrateur|Il le donne à papa.
+papa|Près du bord, ensemble.
+narrateur|Papa le pose. Amir tient le sac.
+narrateur|Le bateau part.
+narrateur|Amir marche le long de l'eau.
+narrateur|Le sac est à l'épaule.</t>
         </is>
       </c>
     </row>
@@ -11030,17 +10911,17 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Le sac attend près de la porte. Merci, papa. On lit sur le tapis ? Amir s'assoit. Il ouvre le livre sur ses genoux. Le rayon de soleil a quitté le tapis. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
@@ -11170,12 +11051,12 @@
       <c r="AV57" s="2" t="inlineStr"/>
       <c r="AW57" t="inlineStr">
         <is>
-          <t>narrateur|Le sac attend près de la porte.
-enfant-m|Merci, papa.
-maman|On lit sur le tapis ?
-narrateur|Amir s'assoit.
-narrateur|Il ouvre le livre sur ses genoux.
-narrateur|Le rayon de soleil a quitté le tapis.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir reprend le bateau.
+narrateur|Il le remet dans le sac.
+narrateur|Les bottes restent aux pieds, jusqu'à la porte.
+narrateur|On referme. Zzz.
+narrateur|Un grain de sable reste sur le bois.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -11203,17 +11084,17 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>La dînette est dans le panier, près du lit. Une tasse et une assiette s'entrechoquent. La tasse seulement, Amir. La tasse. Amir prend la tasse. L'assiette reste dans le panier. Il met la tasse près du yaourt. Juste la tasse. Juste la tasse.</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Lina montre la dînette. Maman a vu un yaourt. Et la chambre. Le sol est un peu froid. Lina caresse le doudou. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lina montre la dînette. Maman a vu un yaourt. Et la chambre. Le sol est un peu froid. Lina caresse le doudou. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -11343,15 +11224,11 @@
       <c r="AV58" s="2" t="inlineStr"/>
       <c r="AW58" t="inlineStr">
         <is>
-          <t>narrateur|La dînette est dans le panier, près du lit.
-narrateur|Une tasse et une assiette s'entrechoquent.
-maman|La tasse seulement, Amir.
-enfant-m|La tasse.
-narrateur|Amir prend la tasse.
-narrateur|L'assiette reste dans le panier.
-narrateur|Il met la tasse près du yaourt.
-maman|Juste la tasse.
-enfant-m|Juste la tasse.</t>
+          <t>narrateur|Amir pose d'abord le sac.
+narrateur|Il pose le bateau sur le sac.
+narrateur|Il regarde la flaque.
+narrateur|Puis il met le bateau dans l'eau.
+papa|Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
     </row>
@@ -11378,17 +11255,17 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Amir s'assoit, le sac sur les genoux. Le sac est prêt. Merci, maman. Il sort la tasse. Il fait semblant de goûter le yaourt. Après, pour de vrai. La couverture retombe sur le lit. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -11518,13 +11395,12 @@
       <c r="AV59" s="2" t="inlineStr"/>
       <c r="AW59" t="inlineStr">
         <is>
-          <t>narrateur|Amir s'assoit, le sac sur les genoux.
-papa|Le sac est prêt.
-enfant-m|Merci, maman.
-narrateur|Il sort la tasse.
-narrateur|Il fait semblant de goûter le yaourt.
-maman|Après, pour de vrai.
-narrateur|La couverture retombe sur le lit.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir reprend le bateau.
+narrateur|Il le remet dans le sac.
+narrateur|Les bottes restent aux pieds, jusqu'à la porte.
+narrateur|On referme. Zzz.
+narrateur|Un grain de sable reste sur le bois.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -11552,17 +11428,17 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Sur la planche, un morceau de pain attend. La croûte fait un petit bruit. Ça sent encore le four. Une miette tombe sur le tapis. Le pain, dans le sac. Le pain. Amir le glisse contre la paroi. Une miette reste sur sa manche. Il souffle dessus. Il est dedans ? Oui, maman.</t>
+          <t>Amir met le bateau dans le sac. Toc. La voile rentre sous son doigt. Le linge est sur le radiateur. Il sent le propre. Pour tes mains, après la flaque. Amir le roule. Il le glisse près du bateau.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Lina met un morceau de pain dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. Maman a dit : le pain. On met dans le sac ce que l'adulte a dit. Le pain est un peu dur. Lina le glisse sur le côté.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir met le bateau dans le sac. Toc. La voile rentre sous son doigt. Le linge est sur le radiateur. Il sent le propre. Pour tes mains, après la flaque. Amir le roule. Il le glisse près du bateau.</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lina met un morceau de pain dans le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Maman a dit : le pain. On met dans le sac ce que l'adulte a dit. Le pain est un peu dur. Lina le glisse sur le côté.&lt;/slow&gt; [pause]</t>
+          <t>Amir met le bateau dans le sac. Toc. La voile rentre sous son doigt. Le linge est sur le radiateur. Il sent le propre. Pour tes mains, après la flaque. Amir le roule. Il le glisse près du bateau.</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr"/>
@@ -11692,17 +11568,13 @@
       <c r="AV60" s="2" t="inlineStr"/>
       <c r="AW60" t="inlineStr">
         <is>
-          <t>narrateur|Sur la planche, un morceau de pain attend.
-narrateur|La croûte fait un petit bruit.
-narrateur|Ça sent encore le four.
-narrateur|Une miette tombe sur le tapis.
-maman|Le pain, dans le sac.
-enfant-m|Le pain.
-narrateur|Amir le glisse contre la paroi.
-narrateur|Une miette reste sur sa manche.
-narrateur|Il souffle dessus.
-maman|Il est dedans ?
-enfant-m|Oui, maman.</t>
+          <t>narrateur|Amir met le bateau dans le sac.
+narrateur|Toc. La voile rentre sous son doigt.
+narrateur|Le linge est sur le radiateur.
+narrateur|Il sent le propre.
+maman|Pour tes mains, après la flaque.
+narrateur|Amir le roule.
+narrateur|Il le glisse près du bateau.</t>
         </is>
       </c>
     </row>
@@ -11729,27 +11601,27 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Qui a dit de mettre le pain ?</t>
+          <t>On met le linge où ?</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Qui dit ce qu'on met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ?&lt;/prosody&gt;&lt;break time="250ms"/&gt;&lt;/speak&gt;</t>
+          <t>On met le linge où ?</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Qui dit ce qu'on met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ?&lt;/slow&gt;</t>
+          <t>On met le linge où ?</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>maman</t>
+          <t>le sac</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>maman | ma maman</t>
+          <t>le sac | dans le sac</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
@@ -11759,12 +11631,12 @@
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>C'est maman qui l'a dit.</t>
+          <t>Dans le sac.</t>
         </is>
       </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>Dis : maman.</t>
+          <t>Le linge va dans le sac.</t>
         </is>
       </c>
       <c r="M61" s="2" t="inlineStr"/>
@@ -11889,7 +11761,7 @@
       </c>
       <c r="AW61" t="inlineStr">
         <is>
-          <t>narrateur|Qui a dit de mettre le pain ?</t>
+          <t>narrateur|On met le linge où ?</t>
         </is>
       </c>
     </row>
@@ -11916,17 +11788,17 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Maman a dit le pain. Le pain est dans le sac. Ça sent encore le four. Amir tape sur le sac. Ce n'est pas fini. On cherche encore un peu.</t>
+          <t>Le linge est dans le sac. Le bateau aussi. On y va ? Oui. Vers la flaque.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Oui. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. Lina hoche la tête. On continue, avec maman. On met dans le sac ce que l'adulte a dit.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le linge est dans le sac. Le bateau aussi. On y va ? Oui. Vers la flaque.</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Oui. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. Lina hoche la tête. On continue, avec maman. On met dans le sac ce que l'adulte a dit.&lt;/slow&gt; [pause]</t>
+          <t>Le linge est dans le sac. Le bateau aussi. On y va ? Oui. Vers la flaque.</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr"/>
@@ -12060,12 +11932,10 @@
       </c>
       <c r="AW62" t="inlineStr">
         <is>
-          <t>narrateur|Maman a dit le pain.
-narrateur|Le pain est dans le sac.
-narrateur|Ça sent encore le four.
-narrateur|Amir tape sur le sac.
-maman|Ce n'est pas fini.
-maman|On cherche encore un peu.</t>
+          <t>narrateur|Le linge est dans le sac.
+narrateur|Le bateau aussi.
+enfant-m|On y va ?
+papa|Oui. Vers la flaque.</t>
         </is>
       </c>
     </row>
@@ -12092,17 +11962,17 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>On peut aller où ? La cuisine, le jardin, ou la chambre.</t>
+          <t>Quelle flaque ? Sous la gouttière, près du potager, ou près du bac.</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;On peut prendre la cuisine, le jardin, ou la chambre.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>Quelle flaque ? Sous la gouttière, près du potager, ou près du bac.</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;On peut prendre la cuisine, le jardin, ou la chambre.&lt;/slow&gt; [pause]</t>
+          <t>Quelle flaque ? Sous la gouttière, près du potager, ou près du bac.</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr"/>
@@ -12120,7 +11990,7 @@
       <c r="L63" s="2" t="inlineStr"/>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>la cuisine</t>
+          <t>sous la gouttière</t>
         </is>
       </c>
       <c r="N63" s="2" t="inlineStr">
@@ -12130,7 +12000,7 @@
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>le jardin</t>
+          <t>près du potager</t>
         </is>
       </c>
       <c r="P63" s="2" t="inlineStr">
@@ -12140,7 +12010,7 @@
       </c>
       <c r="Q63" s="2" t="inlineStr">
         <is>
-          <t>la chambre</t>
+          <t>près du bac</t>
         </is>
       </c>
       <c r="R63" s="2" t="inlineStr">
@@ -12256,8 +12126,8 @@
       <c r="AV63" s="2" t="inlineStr"/>
       <c r="AW63" t="inlineStr">
         <is>
-          <t>narrateur|On peut aller où ?
-narrateur|La cuisine, le jardin, ou la chambre.</t>
+          <t>narrateur|Quelle flaque ?
+narrateur|Sous la gouttière, près du potager, ou près du bac.</t>
         </is>
       </c>
     </row>
@@ -12284,17 +12154,17 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Amir pose le sac près de l'évier. Le pain sent encore le four. L'eau fait un tout petit bruit. Une boîte à goûter attend. Elle est lisse et bleue. La boîte, Amir. Le pain va dedans. La boîte. Amir sort le pain du sac. Il le glisse dans la boîte. Puis la boîte dans le sac. Tu as fini ? Oui, maman.</t>
+          <t>Amir porte le sac. Le linge est dedans. Sous la gouttière, une flaque ronde. Une goutte tombe. Plic. L'eau tremble. Le bateau, maintenant.</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Ensuite Lina reste dans la chambre. Elle met les cubes dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. On met dans le sac ce que l'adulte a dit. Papa tient le sac. Maman reste tout près. On met dans le sac ce que l'adulte a dit.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir porte le sac. Le linge est dedans. Sous la gouttière, une flaque ronde. Une goutte tombe. Plic. L'eau tremble. Le bateau, maintenant.</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Ensuite Lina reste dans la chambre. Elle met les cubes dans le &lt;emphasis&gt;sac&lt;/emphasis&gt;. On met dans le sac ce que l'adulte a dit. Papa tient le sac. Maman reste tout près. On met dans le sac ce que l'adulte a dit.&lt;/slow&gt; [pause]</t>
+          <t>Amir porte le sac. Le linge est dedans. Sous la gouttière, une flaque ronde. Une goutte tombe. Plic. L'eau tremble. Le bateau, maintenant.</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr"/>
@@ -12424,19 +12294,11 @@
       <c r="AV64" s="2" t="inlineStr"/>
       <c r="AW64" t="inlineStr">
         <is>
-          <t>narrateur|Amir pose le sac près de l'évier.
-narrateur|Le pain sent encore le four.
-narrateur|L'eau fait un tout petit bruit.
-narrateur|Une boîte à goûter attend.
-narrateur|Elle est lisse et bleue.
-maman|La boîte, Amir.
-maman|Le pain va dedans.
-enfant-m|La boîte.
-narrateur|Amir sort le pain du sac.
-narrateur|Il le glisse dans la boîte.
-narrateur|Puis la boîte dans le sac.
-maman|Tu as fini ?
-enfant-m|Oui, maman.</t>
+          <t>narrateur|Amir porte le sac. Le linge est dedans.
+narrateur|Sous la gouttière, une flaque ronde.
+narrateur|Une goutte tombe. Plic.
+narrateur|L'eau tremble.
+papa|Le bateau, maintenant.</t>
         </is>
       </c>
     </row>
@@ -12463,17 +12325,17 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre quoi ? Les cubes, le livre, ou la dînette.</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;On peut prendre les cubes, le livre, ou la dînette.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;On peut prendre les cubes, le livre, ou la dînette.&lt;/slow&gt; [pause]</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr"/>
@@ -12491,7 +12353,7 @@
       <c r="L65" s="2" t="inlineStr"/>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>les cubes</t>
+          <t>au milieu</t>
         </is>
       </c>
       <c r="N65" s="2" t="inlineStr">
@@ -12501,7 +12363,7 @@
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>le livre</t>
+          <t>près du bord</t>
         </is>
       </c>
       <c r="P65" s="2" t="inlineStr">
@@ -12511,7 +12373,7 @@
       </c>
       <c r="Q65" s="2" t="inlineStr">
         <is>
-          <t>la dînette</t>
+          <t>sur le sac</t>
         </is>
       </c>
       <c r="R65" s="2" t="inlineStr">
@@ -12627,8 +12489,8 @@
       <c r="AV65" s="2" t="inlineStr"/>
       <c r="AW65" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre quoi ?
-narrateur|Les cubes, le livre, ou la dînette.</t>
+          <t>narrateur|On pose le bateau…
+narrateur|Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
     </row>
@@ -12655,17 +12517,17 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Les cubes sont près de la boîte à goûter. Ils font une petite tour. Amir défait la tour tout doux. Deux cubes dans le sac. Deux cubes. Il les met à côté de la boîte. Pas dans la boîte. À côté.</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Lina a choisi un morceau de pain. Puis la cuisine. Puis les cubes. L'eau coule, tout petit bruit. Lina répète tout bas le geste. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lina a choisi un morceau de pain. Puis la cuisine. Puis les cubes. L'eau coule, tout petit bruit. Lina répète tout bas le geste. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -12795,14 +12657,13 @@
       <c r="AV66" s="2" t="inlineStr"/>
       <c r="AW66" t="inlineStr">
         <is>
-          <t>narrateur|Les cubes sont près de la boîte à goûter.
-narrateur|Ils font une petite tour.
-narrateur|Amir défait la tour tout doux.
-papa|Deux cubes dans le sac.
-enfant-m|Deux cubes.
-narrateur|Il les met à côté de la boîte.
-papa|Pas dans la boîte.
-enfant-m|À côté.</t>
+          <t>narrateur|Amir sort le bateau du sac.
+narrateur|Il le pose au milieu de l'eau.
+narrateur|La voile se tient.
+narrateur|Un peu d'eau touche le papier.
+papa|Il avance.
+narrateur|Amir souffle. Ffff.
+narrateur|Le bateau part tout doux.</t>
         </is>
       </c>
     </row>
@@ -12829,17 +12690,17 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Amir ferme le sac près de l'évier. Le pain est dans la boîte. Les cubes aussi, à côté. On a fini le sac. Il sort un cube. Il le pose sur le couvercle bleu. L'eau ne coule plus. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
@@ -12969,13 +12830,12 @@
       <c r="AV67" s="2" t="inlineStr"/>
       <c r="AW67" t="inlineStr">
         <is>
-          <t>narrateur|Amir ferme le sac près de l'évier.
-maman|Le pain est dans la boîte.
-papa|Les cubes aussi, à côté.
-enfant-m|On a fini le sac.
-narrateur|Il sort un cube.
-narrateur|Il le pose sur le couvercle bleu.
-narrateur|L'eau ne coule plus.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir sèche ses doigts avec le linge.
+narrateur|Il remet le bateau dans le sac.
+narrateur|Le linge rentre aussi.
+narrateur|On referme. Zzz.
+narrateur|La gouttière fait un dernier plic.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -13003,17 +12863,17 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Le livre est debout entre deux bocaux. Amir le prend par le dos. Le livre dans le sac. Le livre. Il le glisse près de la boîte. Au-dessus du pain. Au-dessus.</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Lina s'arrête près de le livre. la cuisine est rangé. Une feuille tombe. Lina range un morceau de pain dans sa tête, comme un souvenir. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lina s'arrête près de le livre. la cuisine est rangé. Une feuille tombe. Lina range un morceau de pain dans sa tête, comme un souvenir. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -13143,13 +13003,13 @@
       <c r="AV68" s="2" t="inlineStr"/>
       <c r="AW68" t="inlineStr">
         <is>
-          <t>narrateur|Le livre est debout entre deux bocaux.
-narrateur|Amir le prend par le dos.
-papa|Le livre dans le sac.
-enfant-m|Le livre.
-narrateur|Il le glisse près de la boîte.
-papa|Au-dessus du pain.
-enfant-m|Au-dessus.</t>
+          <t>narrateur|Amir sort le bateau.
+narrateur|Il le donne à papa.
+papa|Près du bord, ensemble.
+narrateur|Papa le pose. Amir tient le sac.
+narrateur|Le bateau part.
+narrateur|Amir marche le long de l'eau.
+narrateur|Le sac est à l'épaule.</t>
         </is>
       </c>
     </row>
@@ -13176,17 +13036,17 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Le sac est posé contre la chaise. On va jouer. On ouvre le livre d'abord ? Amir montre une page à maman. Ça sent encore un peu le four. On y va. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -13316,12 +13176,12 @@
       <c r="AV69" s="2" t="inlineStr"/>
       <c r="AW69" t="inlineStr">
         <is>
-          <t>narrateur|Le sac est posé contre la chaise.
-enfant-m|On va jouer.
-maman|On ouvre le livre d'abord ?
-narrateur|Amir montre une page à maman.
-narrateur|Ça sent encore un peu le four.
-papa|On y va.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir sèche ses doigts avec le linge.
+narrateur|Il remet le bateau dans le sac.
+narrateur|Le linge rentre aussi.
+narrateur|On referme. Zzz.
+narrateur|La gouttière fait un dernier plic.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -13349,17 +13209,17 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Une casserole de dînette est près du sel. Le couvercle est à l'envers. Amir le remet dessus. La casserole dans le sac. La casserole. Il la met près de la boîte. On fera le pain pour de faux. Oui.</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Lina se souvient de un morceau de pain. Et de la cuisine. Et de la dînette. Le vent est doux. Lina boit une gorgée d'eau. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lina se souvient de un morceau de pain. Et de la cuisine. Et de la dînette. Le vent est doux. Lina boit une gorgée d'eau. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
@@ -13489,14 +13349,11 @@
       <c r="AV70" s="2" t="inlineStr"/>
       <c r="AW70" t="inlineStr">
         <is>
-          <t>narrateur|Une casserole de dînette est près du sel.
-narrateur|Le couvercle est à l'envers.
-narrateur|Amir le remet dessus.
-maman|La casserole dans le sac.
-enfant-m|La casserole.
-narrateur|Il la met près de la boîte.
-maman|On fera le pain pour de faux.
-enfant-m|Oui.</t>
+          <t>narrateur|Amir pose d'abord le sac.
+narrateur|Il pose le bateau sur le sac.
+narrateur|Il regarde la flaque.
+narrateur|Puis il met le bateau dans l'eau.
+papa|Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
     </row>
@@ -13523,17 +13380,17 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Amir tient la sangle du sac. Le sac est prêt. La casserole aussi. Il fait semblant de cuire le pain. Tout doux. C'est déjà cuit. Amir rit. La cuisine est calme. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr"/>
@@ -13663,13 +13520,12 @@
       <c r="AV71" s="2" t="inlineStr"/>
       <c r="AW71" t="inlineStr">
         <is>
-          <t>narrateur|Amir tient la sangle du sac.
-papa|Le sac est prêt.
-enfant-m|La casserole aussi.
-narrateur|Il fait semblant de cuire le pain.
-maman|Tout doux. C'est déjà cuit.
-narrateur|Amir rit.
-narrateur|La cuisine est calme.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir sèche ses doigts avec le linge.
+narrateur|Il remet le bateau dans le sac.
+narrateur|Le linge rentre aussi.
+narrateur|On referme. Zzz.
+narrateur|La gouttière fait un dernier plic.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -13697,17 +13553,17 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Amir descend la marche du jardin. Le pain reste au fond du sac. Le vent est doux sur les joues. Un petit chapeau attend sur le banc. Le petit chapeau, dans le sac. Le chapeau. Le chapeau est souple. Amir le tasse près du pain. Une feuille tourne au-dessus du bac. On la laisse au jardin.</t>
+          <t>Amir porte le sac avec le linge. Ils vont près du potager. La flaque est ronde, entre deux choux. L'eau tremble un peu. Le bateau, Amir.</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Ensuite Lina reste dans la chambre. Elle met le livre dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. On met dans le sac ce que l'adulte a dit. Papa tient le sac. Maman montre le geste, lentement. On met dans le sac ce que l'adulte a dit.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir porte le sac avec le linge. Ils vont près du potager. La flaque est ronde, entre deux choux. L'eau tremble un peu. Le bateau, Amir.</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Ensuite Lina reste dans la chambre. Elle met le livre dans le &lt;emphasis&gt;sac&lt;/emphasis&gt;. On met dans le sac ce que l'adulte a dit. Papa tient le sac. Maman montre le geste, lentement. On met dans le sac ce que l'adulte a dit.&lt;/slow&gt; [pause]</t>
+          <t>Amir porte le sac avec le linge. Ils vont près du potager. La flaque est ronde, entre deux choux. L'eau tremble un peu. Le bateau, Amir.</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
@@ -13837,16 +13693,11 @@
       <c r="AV72" s="2" t="inlineStr"/>
       <c r="AW72" t="inlineStr">
         <is>
-          <t>narrateur|Amir descend la marche du jardin.
-narrateur|Le pain reste au fond du sac.
-narrateur|Le vent est doux sur les joues.
-narrateur|Un petit chapeau attend sur le banc.
-papa|Le petit chapeau, dans le sac.
-enfant-m|Le chapeau.
-narrateur|Le chapeau est souple.
-narrateur|Amir le tasse près du pain.
-narrateur|Une feuille tourne au-dessus du bac.
-papa|On la laisse au jardin.</t>
+          <t>narrateur|Amir porte le sac avec le linge.
+narrateur|Ils vont près du potager.
+narrateur|La flaque est ronde, entre deux choux.
+narrateur|L'eau tremble un peu.
+maman|Le bateau, Amir.</t>
         </is>
       </c>
     </row>
@@ -13873,17 +13724,17 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre quoi ? Les cubes, le livre, ou la dînette.</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;On peut prendre les cubes, le livre, ou la dînette.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;On peut prendre les cubes, le livre, ou la dînette.&lt;/slow&gt; [pause]</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr"/>
@@ -13901,7 +13752,7 @@
       <c r="L73" s="2" t="inlineStr"/>
       <c r="M73" s="2" t="inlineStr">
         <is>
-          <t>les cubes</t>
+          <t>au milieu</t>
         </is>
       </c>
       <c r="N73" s="2" t="inlineStr">
@@ -13911,7 +13762,7 @@
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>le livre</t>
+          <t>près du bord</t>
         </is>
       </c>
       <c r="P73" s="2" t="inlineStr">
@@ -13921,7 +13772,7 @@
       </c>
       <c r="Q73" s="2" t="inlineStr">
         <is>
-          <t>la dînette</t>
+          <t>sur le sac</t>
         </is>
       </c>
       <c r="R73" s="2" t="inlineStr">
@@ -14037,8 +13888,8 @@
       <c r="AV73" s="2" t="inlineStr"/>
       <c r="AW73" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre quoi ?
-narrateur|Les cubes, le livre, ou la dînette.</t>
+          <t>narrateur|On pose le bateau…
+narrateur|Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
     </row>
@@ -14065,17 +13916,17 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Les cubes sont dans le bac à sable. Un cube a un peu de sable. Amir le frotte. Le cube propre, dans le sac. Le cube propre. Il le met près du pain. Le sable reste au bac.</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Avec les cubes. Après le jardin. Près de un morceau de pain. Lina s'arrête. Le savon sent bon. Lina pose sa tête un moment. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Avec les cubes. Après le jardin. Près de un morceau de pain. Lina s'arrête. Le savon sent bon. Lina pose sa tête un moment. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
@@ -14205,13 +14056,13 @@
       <c r="AV74" s="2" t="inlineStr"/>
       <c r="AW74" t="inlineStr">
         <is>
-          <t>narrateur|Les cubes sont dans le bac à sable.
-narrateur|Un cube a un peu de sable.
-narrateur|Amir le frotte.
-papa|Le cube propre, dans le sac.
-enfant-m|Le cube propre.
-narrateur|Il le met près du pain.
-papa|Le sable reste au bac.</t>
+          <t>narrateur|Amir sort le bateau du sac.
+narrateur|Il le pose au milieu de l'eau.
+narrateur|La voile se tient.
+narrateur|Un peu d'eau touche le papier.
+papa|Il avance.
+narrateur|Amir souffle. Ffff.
+narrateur|Le bateau part tout doux.</t>
         </is>
       </c>
     </row>
@@ -14238,17 +14089,17 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Amir remonte la marche avec le sac. Merci, papa. On joue au cube, une minute. Amir pose le cube sur la marche. Une feuille reste sur le bac. On rentre. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
@@ -14378,12 +14229,12 @@
       <c r="AV75" s="2" t="inlineStr"/>
       <c r="AW75" t="inlineStr">
         <is>
-          <t>narrateur|Amir remonte la marche avec le sac.
-enfant-m|Merci, papa.
-maman|On joue au cube, une minute.
-narrateur|Amir pose le cube sur la marche.
-narrateur|Une feuille reste sur le bac.
-papa|On rentre.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir sèche ses doigts avec le linge.
+narrateur|Il remet le bateau dans le sac.
+narrateur|Le linge rentre aussi.
+narrateur|On referme. Zzz.
+narrateur|Une feuille lâche la flaque.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -14411,17 +14262,17 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Le livre est sous le chapeau, sur le banc. Une page tremble au vent. Le livre dans le sac. Le livre. Amir le met près du pain. Puis le chapeau par-dessus. Le chapeau garde le livre. Oui.</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Lina range le jardin. le livre reste près de un morceau de pain. Un panier est posé sur le banc. Lina sourit. Maman sourit aussi. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lina range le jardin. le livre reste près de un morceau de pain. Un panier est posé sur le banc. Lina sourit. Maman sourit aussi. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -14551,14 +14402,13 @@
       <c r="AV76" s="2" t="inlineStr"/>
       <c r="AW76" t="inlineStr">
         <is>
-          <t>narrateur|Le livre est sous le chapeau, sur le banc.
-narrateur|Une page tremble au vent.
-maman|Le livre dans le sac.
-enfant-m|Le livre.
-narrateur|Amir le met près du pain.
-narrateur|Puis le chapeau par-dessus.
-maman|Le chapeau garde le livre.
-enfant-m|Oui.</t>
+          <t>narrateur|Amir sort le bateau.
+narrateur|Il le donne à papa.
+papa|Près du bord, ensemble.
+narrateur|Papa le pose. Amir tient le sac.
+narrateur|Le bateau part.
+narrateur|Amir marche le long de l'eau.
+narrateur|Le sac est à l'épaule.</t>
         </is>
       </c>
     </row>
@@ -14585,17 +14435,17 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Le sac est un peu lourd. Merci. On rentre avec le sac. Amir soulève le chapeau. Il touche le livre, juste un peu. Le jardin sent la terre mouillée. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr"/>
@@ -14725,12 +14575,12 @@
       <c r="AV77" s="2" t="inlineStr"/>
       <c r="AW77" t="inlineStr">
         <is>
-          <t>narrateur|Le sac est un peu lourd.
-enfant-m|Merci.
-papa|On rentre avec le sac.
-narrateur|Amir soulève le chapeau.
-narrateur|Il touche le livre, juste un peu.
-narrateur|Le jardin sent la terre mouillée.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir sèche ses doigts avec le linge.
+narrateur|Il remet le bateau dans le sac.
+narrateur|Le linge rentre aussi.
+narrateur|On referme. Zzz.
+narrateur|Une feuille lâche la flaque.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -14758,17 +14608,17 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Une assiette de dînette est sur le muret. Un caillou rond est posé dessus. Amir pose le caillou à côté. L'assiette dans le sac. L'assiette. Il la met près du pain. On y mettra le pain, pour de faux. Pour de faux.</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;la dînette est là. le jardin aussi. un morceau de pain reste dans le souvenir. Un linge sèche à l'air. Lina range la tasse. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;la dînette est là. le jardin aussi. un morceau de pain reste dans le souvenir. Un linge sèche à l'air. Lina range la tasse. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
@@ -14898,14 +14748,11 @@
       <c r="AV78" s="2" t="inlineStr"/>
       <c r="AW78" t="inlineStr">
         <is>
-          <t>narrateur|Une assiette de dînette est sur le muret.
-narrateur|Un caillou rond est posé dessus.
-narrateur|Amir pose le caillou à côté.
-maman|L'assiette dans le sac.
-enfant-m|L'assiette.
-narrateur|Il la met près du pain.
-maman|On y mettra le pain, pour de faux.
-enfant-m|Pour de faux.</t>
+          <t>narrateur|Amir pose d'abord le sac.
+narrateur|Il pose le bateau sur le sac.
+narrateur|Il regarde la flaque.
+narrateur|Puis il met le bateau dans l'eau.
+papa|Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
     </row>
@@ -14932,17 +14779,17 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Amir serre le sac contre lui. Le sac est prêt. Merci, maman. Amir sort l'assiette. Il y pose le pain un instant. Puis tout rentre. Le vent est plus calme. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr"/>
@@ -15072,13 +14919,12 @@
       <c r="AV79" s="2" t="inlineStr"/>
       <c r="AW79" t="inlineStr">
         <is>
-          <t>narrateur|Amir serre le sac contre lui.
-enfant-m|Le sac est prêt.
-papa|Merci, maman.
-narrateur|Amir sort l'assiette.
-narrateur|Il y pose le pain un instant.
-narrateur|Puis tout rentre.
-narrateur|Le vent est plus calme.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir sèche ses doigts avec le linge.
+narrateur|Il remet le bateau dans le sac.
+narrateur|Le linge rentre aussi.
+narrateur|On referme. Zzz.
+narrateur|Une feuille lâche la flaque.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -15106,17 +14952,17 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Amir repose le sac sur le tapis rayé. Le pain fait un petit bruit de croûte. Le volet jaune claque une fois. Le doudou attend près de l'oreiller. Le doudou du sac, Amir. Le doudou. Le doudou est chaud et un peu plat. Amir le glisse près du pain. Il est bien dedans ? Oui. Le sac se remplit.</t>
+          <t>Amir porte le sac avec le linge. Ils vont près du bac à sable. Une flaque borde le bois du bac. Un peu de sable brille au fond. Le bateau, Amir.</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Ensuite Lina reste dans la chambre. Elle met une tasse de dînette dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. On met dans le sac ce que l'adulte a dit. Maman dit : je suis là. On met dans le sac ce que l'adulte a dit.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir porte le sac avec le linge. Ils vont près du bac à sable. Une flaque borde le bois du bac. Un peu de sable brille au fond. Le bateau, Amir.</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Ensuite Lina reste dans la chambre. Elle met une tasse de dînette dans le &lt;emphasis&gt;sac&lt;/emphasis&gt;. On met dans le sac ce que l'adulte a dit. Maman dit : je suis là. On met dans le sac ce que l'adulte a dit.&lt;/slow&gt; [pause]</t>
+          <t>Amir porte le sac avec le linge. Ils vont près du bac à sable. Une flaque borde le bois du bac. Un peu de sable brille au fond. Le bateau, Amir.</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr"/>
@@ -15246,17 +15092,11 @@
       <c r="AV80" s="2" t="inlineStr"/>
       <c r="AW80" t="inlineStr">
         <is>
-          <t>narrateur|Amir repose le sac sur le tapis rayé.
-narrateur|Le pain fait un petit bruit de croûte.
-narrateur|Le volet jaune claque une fois.
-narrateur|Le doudou attend près de l'oreiller.
-maman|Le doudou du sac, Amir.
-enfant-m|Le doudou.
-narrateur|Le doudou est chaud et un peu plat.
-narrateur|Amir le glisse près du pain.
-maman|Il est bien dedans ?
-enfant-m|Oui.
-narrateur|Le sac se remplit.</t>
+          <t>narrateur|Amir porte le sac avec le linge.
+narrateur|Ils vont près du bac à sable.
+narrateur|Une flaque borde le bois du bac.
+narrateur|Un peu de sable brille au fond.
+papa|Le bateau, Amir.</t>
         </is>
       </c>
     </row>
@@ -15283,17 +15123,17 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre quoi ? Les cubes, le livre, ou la dînette.</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;On peut prendre les cubes, le livre, ou la dînette.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;On peut prendre les cubes, le livre, ou la dînette.&lt;/slow&gt; [pause]</t>
+          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr"/>
@@ -15311,7 +15151,7 @@
       <c r="L81" s="2" t="inlineStr"/>
       <c r="M81" s="2" t="inlineStr">
         <is>
-          <t>les cubes</t>
+          <t>au milieu</t>
         </is>
       </c>
       <c r="N81" s="2" t="inlineStr">
@@ -15321,7 +15161,7 @@
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>le livre</t>
+          <t>près du bord</t>
         </is>
       </c>
       <c r="P81" s="2" t="inlineStr">
@@ -15331,7 +15171,7 @@
       </c>
       <c r="Q81" s="2" t="inlineStr">
         <is>
-          <t>la dînette</t>
+          <t>sur le sac</t>
         </is>
       </c>
       <c r="R81" s="2" t="inlineStr">
@@ -15447,8 +15287,8 @@
       <c r="AV81" s="2" t="inlineStr"/>
       <c r="AW81" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre quoi ?
-narrateur|Les cubes, le livre, ou la dînette.</t>
+          <t>narrateur|On pose le bateau…
+narrateur|Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
         </is>
       </c>
     </row>
@@ -15475,17 +15315,17 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Les cubes sont près du doudou, sur le tapis. Un cube touche la patte du doudou. Les cubes dans le sac. Les cubes. Amir les met près du pain et du doudou. La patte est libre. Libre.</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Lina rejoint les cubes. la chambre est rangé. un morceau de pain est fini. Les chaussures font toc toc. Lina serre la main de maman. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lina rejoint les cubes. la chambre est rangé. un morceau de pain est fini. Les chaussures font toc toc. Lina serre la main de maman. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr"/>
@@ -15615,13 +15455,13 @@
       <c r="AV82" s="2" t="inlineStr"/>
       <c r="AW82" t="inlineStr">
         <is>
-          <t>narrateur|Les cubes sont près du doudou, sur le tapis.
-narrateur|Un cube touche la patte du doudou.
-papa|Les cubes dans le sac.
-enfant-m|Les cubes.
-narrateur|Amir les met près du pain et du doudou.
-papa|La patte est libre.
-enfant-m|Libre.</t>
+          <t>narrateur|Amir sort le bateau du sac.
+narrateur|Il le pose au milieu de l'eau.
+narrateur|La voile se tient.
+narrateur|Un peu d'eau touche le papier.
+papa|Il avance.
+narrateur|Amir souffle. Ffff.
+narrateur|Le bateau part tout doux.</t>
         </is>
       </c>
     </row>
@@ -15648,17 +15488,17 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Amir ferme le sac sur le tapis rayé. On peut jouer maintenant. Oui. Il sort un cube. Il le pose sur le doudou, pour rire. Le volet jaune est calme. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -15788,12 +15628,12 @@
       <c r="AV83" s="2" t="inlineStr"/>
       <c r="AW83" t="inlineStr">
         <is>
-          <t>narrateur|Amir ferme le sac sur le tapis rayé.
-enfant-m|On peut jouer maintenant.
-maman|Oui.
-narrateur|Il sort un cube.
-narrateur|Il le pose sur le doudou, pour rire.
-papa|Le volet jaune est calme.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir sèche ses doigts avec le linge.
+narrateur|Il remet le bateau dans le sac.
+narrateur|Le linge rentre aussi.
+narrateur|On referme. Zzz.
+narrateur|Un grain de sable reste sur le bois.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -15821,17 +15661,17 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Le livre est sous l'oreiller. Amir soulève l'oreiller d'une main. Le livre dans le sac. Le livre. Il le glisse près du pain. Sous le doudou, tout doux. Tout doux.</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Près de le livre. Lina pose la chambre. un morceau de pain est derrière. Une pomme brille un peu. Lina marche près de maman. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Près de le livre. Lina pose la chambre. un morceau de pain est derrière. Une pomme brille un peu. Lina marche près de maman. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
@@ -15961,13 +15801,13 @@
       <c r="AV84" s="2" t="inlineStr"/>
       <c r="AW84" t="inlineStr">
         <is>
-          <t>narrateur|Le livre est sous l'oreiller.
-narrateur|Amir soulève l'oreiller d'une main.
-papa|Le livre dans le sac.
-enfant-m|Le livre.
-narrateur|Il le glisse près du pain.
-papa|Sous le doudou, tout doux.
-enfant-m|Tout doux.</t>
+          <t>narrateur|Amir sort le bateau.
+narrateur|Il le donne à papa.
+papa|Près du bord, ensemble.
+narrateur|Papa le pose. Amir tient le sac.
+narrateur|Le bateau part.
+narrateur|Amir marche le long de l'eau.
+narrateur|Le sac est à l'épaule.</t>
         </is>
       </c>
     </row>
@@ -15994,17 +15834,17 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Le sac attend près de la porte de la chambre. Merci, papa. On lit une page ? Amir ouvre le livre contre le doudou. Le tapis n'a plus de cubes. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr"/>
@@ -16134,11 +15974,12 @@
       <c r="AV85" s="2" t="inlineStr"/>
       <c r="AW85" t="inlineStr">
         <is>
-          <t>narrateur|Le sac attend près de la porte de la chambre.
-enfant-m|Merci, papa.
-maman|On lit une page ?
-narrateur|Amir ouvre le livre contre le doudou.
-narrateur|Le tapis n'a plus de cubes.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir sèche ses doigts avec le linge.
+narrateur|Il remet le bateau dans le sac.
+narrateur|Le linge rentre aussi.
+narrateur|On referme. Zzz.
+narrateur|Un grain de sable reste sur le bois.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -16166,17 +16007,17 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>La dînette est dans le panier, près du lit. Une tasse et une assiette s'entrechoquent. La tasse seulement. La tasse. Amir prend la tasse. Il la met près du pain. L'assiette reste. Elle reste.</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Lina montre la dînette. Maman a vu un morceau de pain. Et la chambre. On se tient la main. Lina pose la chambre à sa place. On met dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lina montre la dînette. Maman a vu un morceau de pain. Et la chambre. On se tient la main. Lina pose la chambre à sa place. On met dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ce que l'adulte a dit. On met dans le sac ce que papa ou maman a dit. Lina dit merci à maman.&lt;/slow&gt; [pause]</t>
+          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -16306,14 +16147,11 @@
       <c r="AV86" s="2" t="inlineStr"/>
       <c r="AW86" t="inlineStr">
         <is>
-          <t>narrateur|La dînette est dans le panier, près du lit.
-narrateur|Une tasse et une assiette s'entrechoquent.
-maman|La tasse seulement.
-enfant-m|La tasse.
-narrateur|Amir prend la tasse.
-narrateur|Il la met près du pain.
-maman|L'assiette reste.
-enfant-m|Elle reste.</t>
+          <t>narrateur|Amir pose d'abord le sac.
+narrateur|Il pose le bateau sur le sac.
+narrateur|Il regarde la flaque.
+narrateur|Puis il met le bateau dans l'eau.
+papa|Tu as préparé. Maintenant il flotte.</t>
         </is>
       </c>
     </row>
@@ -16340,17 +16178,17 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Amir s'assoit, le sac sur les genoux. Le sac est prêt. Merci. Il sort la tasse. Il y glisse un tout petit bout de pain. Pour de faux. Puis on range. La chambre sent encore la soupe, un peu. L'histoire est finie.</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr"/>
@@ -16480,13 +16318,12 @@
       <c r="AV87" s="2" t="inlineStr"/>
       <c r="AW87" t="inlineStr">
         <is>
-          <t>narrateur|Amir s'assoit, le sac sur les genoux.
-papa|Le sac est prêt.
-enfant-m|Merci.
-narrateur|Il sort la tasse.
-narrateur|Il y glisse un tout petit bout de pain.
-maman|Pour de faux. Puis on range.
-narrateur|La chambre sent encore la soupe, un peu.
+          <t>narrateur|Le papier est un peu mouillé.
+narrateur|Amir sèche ses doigts avec le linge.
+narrateur|Il remet le bateau dans le sac.
+narrateur|Le linge rentre aussi.
+narrateur|On referme. Zzz.
+narrateur|Un grain de sable reste sur le bois.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -16508,7 +16345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16574,6 +16411,20 @@
       <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-010…015 texte : désir jouer, sac vide, branches à conséquences, chaîne Q pomme/yaourt/maman, personnages Amir papa maman</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>exemple2 + avis 88534be : bateau/flaque, labels manteau/bottes/linge, fins qui flottent, SSML = texte</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F-NAR-017): avis1 — TREE-AUT-001, chemins vraiment différents
Le bateau voyage : gouttière, choux, bac. Chaque issue a sa fin. Pas d'audio. COL inchangé.
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-AUT-001.xlsx
+++ b/stories/arbres/TREE-AUT-001.xlsx
@@ -552,7 +552,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le bateau d'Amir et la flaque</t>
+          <t>Le bateau d'Amir et la rivière du jardin</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>dans la chambre, puis le jardin</t>
+          <t>dans la maison, puis le jardin</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amir veut faire flotter son bateau en papier dans la flaque. Le sac doit être prêt. Il y met le bateau, puis le manteau, les bottes ou le linge. À la flaque, le bateau part. Il le remet dans le sac.</t>
+          <t>Amir veut faire voyager son bateau en papier dans le jardin après la pluie. Il prépare le sac (manteau, bottes ou linge). Puis il choisit un vrai chemin : rivière de la gouttière, port des choux, ou île du bac. Chaque chemin a un obstacle et une fin différente. Il rentre. Le bateau attend le prochain voyage.</t>
         </is>
       </c>
     </row>
@@ -1197,17 +1197,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Sur le toit, la gouttière fait encore plic ploc. La pluie vient de s'arrêter. Le volet jaune claque tout doux. Dans la rue, les pavés brillent. En ce moment, Amir a un bateau en papier. Une voile pliée. Un peu froissée. Papa, la flaque est là, dans le jardin. Oui. On y va quand le sac est prêt. Le sac attend sur le tapis rayé. Amir tire la fermeture. Zzz. Le sac est vide. Le bateau est sur la commode.</t>
+          <t>Le volet jaune bouge encore un peu. Dans la rue, les pavés brillent. Dans la maison, ça sent la soupe. Maman est dans la cuisine. Papa est à la grande table. Son ordinateur fait un petit vent. Sur le tapis, Amir plie un coin de papier. Celle-ci, la coque. Il plie encore. Une voile un peu froissée. Et ça, la cheminée. C'est un bateau en papier. Assez petit pour ses deux mains. Il le fait glisser. Le bateau s'arrête contre la pantoufle de papa. Votre bateau s'est échoué, capitaine Amir. Il lui faut de l'eau. Dehors, la pluie s'arrête. Une dernière goutte. Ploc. Amir court à la fenêtre. L'eau a dessiné un chemin. La gouttière. Le potager. Le bac à sable. Papa ! Mon bateau peut faire un vrai voyage ! Jusqu'où ? Je ne sais pas encore. C'est le bateau qui choisira. Maman arrive avec le petit sac. Le jardin est encore mouillé. De quoi auras-tu besoin ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Sur le toit, la gouttière fait encore plic ploc. La pluie vient de s'arrêter. Le volet jaune claque tout doux. Dans la rue, les pavés brillent. En ce moment, Amir a un bateau en papier. Une voile pliée. Un peu froissée. Papa, la flaque est là, dans le jardin. Oui. On y va quand le sac est prêt. Le sac attend sur le tapis rayé. Amir tire la fermeture. Zzz. Le sac est vide. Le bateau est sur la commode.</t>
+          <t>Le volet jaune bouge encore un peu. Dans la rue, les pavés brillent. Dans la maison, ça sent la soupe. Maman est dans la cuisine. Papa est à la grande table. Son ordinateur fait un petit vent. Sur le tapis, Amir plie un coin de papier. Celle-ci, la coque. Il plie encore. Une voile un peu froissée. Et ça, la cheminée. C'est un bateau en papier. Assez petit pour ses deux mains. Il le fait glisser. Le bateau s'arrête contre la pantoufle de papa. Votre bateau s'est échoué, capitaine Amir. Il lui faut de l'eau. Dehors, la pluie s'arrête. Une dernière goutte. Ploc. Amir court à la fenêtre. L'eau a dessiné un chemin. La gouttière. Le potager. Le bac à sable. Papa ! Mon bateau peut faire un vrai voyage ! Jusqu'où ? Je ne sais pas encore. C'est le bateau qui choisira. Maman arrive avec le petit sac. Le jardin est encore mouillé. De quoi auras-tu besoin ?</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Sur le toit, la gouttière fait encore plic ploc. La pluie vient de s'arrêter. Le volet jaune claque tout doux. Dans la rue, les pavés brillent. En ce moment, Amir a un bateau en papier. Une voile pliée. Un peu froissée. Papa, la flaque est là, dans le jardin. Oui. On y va quand le sac est prêt. Le sac attend sur le tapis rayé. Amir tire la fermeture. Zzz. Le sac est vide. Le bateau est sur la commode.</t>
+          <t>Le volet jaune bouge encore un peu. Dans la rue, les pavés brillent. Dans la maison, ça sent la soupe. Maman est dans la cuisine. Papa est à la grande table. Son ordinateur fait un petit vent. Sur le tapis, Amir plie un coin de papier. Celle-ci, la coque. Il plie encore. Une voile un peu froissée. Et ça, la cheminée. C'est un bateau en papier. Assez petit pour ses deux mains. Il le fait glisser. Le bateau s'arrête contre la pantoufle de papa. Votre bateau s'est échoué, capitaine Amir. Il lui faut de l'eau. Dehors, la pluie s'arrête. Une dernière goutte. Ploc. Amir court à la fenêtre. L'eau a dessiné un chemin. La gouttière. Le potager. Le bac à sable. Papa ! Mon bateau peut faire un vrai voyage ! Jusqu'où ? Je ne sais pas encore. C'est le bateau qui choisira. Maman arrive avec le petit sac. Le jardin est encore mouillé. De quoi auras-tu besoin ?</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1337,18 +1337,27 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Sur le toit, la gouttière fait encore plic ploc.
-narrateur|La pluie vient de s'arrêter.
-narrateur|Le volet jaune claque tout doux.
+          <t>narrateur|Le volet jaune bouge encore un peu.
 narrateur|Dans la rue, les pavés brillent.
-narrateur|En ce moment, Amir a un bateau en papier.
-narrateur|Une voile pliée. Un peu froissée.
-enfant-m|Papa, la flaque est là, dans le jardin.
-papa|Oui. On y va quand le sac est prêt.
-narrateur|Le sac attend sur le tapis rayé.
-narrateur|Amir tire la fermeture. Zzz.
-narrateur|Le sac est vide.
-narrateur|Le bateau est sur la commode.</t>
+narrateur|Dans la maison, ça sent la soupe.
+narrateur|Maman est dans la cuisine.
+narrateur|Papa est à la grande table. Son ordinateur fait un petit vent.
+narrateur|Sur le tapis, Amir plie un coin de papier.
+enfant-m|Celle-ci, la coque.
+narrateur|Il plie encore. Une voile un peu froissée.
+enfant-m|Et ça, la cheminée.
+narrateur|C'est un bateau en papier. Assez petit pour ses deux mains.
+narrateur|Il le fait glisser. Le bateau s'arrête contre la pantoufle de papa.
+papa|Votre bateau s'est échoué, capitaine Amir.
+enfant-m|Il lui faut de l'eau.
+narrateur|Dehors, la pluie s'arrête. Une dernière goutte. Ploc.
+narrateur|Amir court à la fenêtre.
+narrateur|L'eau a dessiné un chemin. La gouttière. Le potager. Le bac à sable.
+enfant-m|Papa ! Mon bateau peut faire un vrai voyage !
+papa|Jusqu'où ?
+enfant-m|Je ne sais pas encore. C'est le bateau qui choisira.
+narrateur|Maman arrive avec le petit sac.
+maman|Le jardin est encore mouillé. De quoi auras-tu besoin ?</t>
         </is>
       </c>
     </row>
@@ -1375,17 +1384,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Pour aller à la flaque, on prend aussi… Le manteau, les bottes, ou un linge.</t>
+          <t>Avant de partir, un capitaine prépare ses affaires. Le manteau, les bottes, ou un linge. Qu'est-ce que tu prends, Amir ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Pour aller à la flaque, on prend aussi… Le manteau, les bottes, ou un linge.</t>
+          <t>Avant de partir, un capitaine prépare ses affaires. Le manteau, les bottes, ou un linge. Qu'est-ce que tu prends, Amir ?</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Pour aller à la flaque, on prend aussi… Le manteau, les bottes, ou un linge.</t>
+          <t>Avant de partir, un capitaine prépare ses affaires. Le manteau, les bottes, ou un linge. Qu'est-ce que tu prends, Amir ?</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
@@ -1543,8 +1552,9 @@
       <c r="AV3" s="2" t="inlineStr"/>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Pour aller à la flaque, on prend aussi…
-narrateur|Le manteau, les bottes, ou un linge.</t>
+          <t>narrateur|Avant de partir, un capitaine prépare ses affaires.
+narrateur|Le manteau, les bottes, ou un linge.
+maman|Qu'est-ce que tu prends, Amir ?</t>
         </is>
       </c>
     </row>
@@ -1571,17 +1581,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Amir prend le bateau sur la commode. Le bateau, dans le sac d'abord. Il le glisse au fond. Toc. La voile dépasse un tout petit peu. Il la rentre avec le doigt. Le manteau est sur la chaise. Il est encore un peu chaud. Pour la flaque. Il est encore frais dehors. Amir le plie. Il le met à côté du bateau.</t>
+          <t>Amir prend le bateau en papier sur la commode. Il le glisse au fond du sac. Toc. La voile dépasse. Il la rentre du doigt. Le manteau est sur la chaise. Il est tiède. Le jardin est encore mouillé. Le manteau, Amir. Oui. Pour le voyage.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Amir prend le bateau sur la commode. Le bateau, dans le sac d'abord. Il le glisse au fond. Toc. La voile dépasse un tout petit peu. Il la rentre avec le doigt. Le manteau est sur la chaise. Il est encore un peu chaud. Pour la flaque. Il est encore frais dehors. Amir le plie. Il le met à côté du bateau.</t>
+          <t>Amir prend le bateau en papier sur la commode. Il le glisse au fond du sac. Toc. La voile dépasse. Il la rentre du doigt. Le manteau est sur la chaise. Il est tiède. Le jardin est encore mouillé. Le manteau, Amir. Oui. Pour le voyage.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Amir prend le bateau sur la commode. Le bateau, dans le sac d'abord. Il le glisse au fond. Toc. La voile dépasse un tout petit peu. Il la rentre avec le doigt. Le manteau est sur la chaise. Il est encore un peu chaud. Pour la flaque. Il est encore frais dehors. Amir le plie. Il le met à côté du bateau.</t>
+          <t>Amir prend le bateau en papier sur la commode. Il le glisse au fond du sac. Toc. La voile dépasse. Il la rentre du doigt. Le manteau est sur la chaise. Il est tiède. Le jardin est encore mouillé. Le manteau, Amir. Oui. Pour le voyage.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1711,17 +1721,13 @@
       <c r="AV4" s="2" t="inlineStr"/>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Amir prend le bateau sur la commode.
-maman|Le bateau, dans le sac d'abord.
-narrateur|Il le glisse au fond.
-narrateur|Toc.
-narrateur|La voile dépasse un tout petit peu.
-narrateur|Il la rentre avec le doigt.
-narrateur|Le manteau est sur la chaise.
-narrateur|Il est encore un peu chaud.
-papa|Pour la flaque. Il est encore frais dehors.
-narrateur|Amir le plie.
-narrateur|Il le met à côté du bateau.</t>
+          <t>narrateur|Amir prend le bateau en papier sur la commode.
+narrateur|Il le glisse au fond du sac. Toc.
+narrateur|La voile dépasse. Il la rentre du doigt.
+narrateur|Le manteau est sur la chaise. Il est tiède.
+maman|Le jardin est encore mouillé.
+maman|Le manteau, Amir.
+enfant-m|Oui. Pour le voyage.</t>
         </is>
       </c>
     </row>
@@ -1763,12 +1769,12 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>le sac</t>
+          <t>dans le sac</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>le sac | dans le sac | au fond</t>
+          <t>sac|le sac|dans le sac|au fond du sac</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -1935,17 +1941,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le bateau est dans le sac. La voile est rentrée. Le manteau est à côté. C'est bon ? Presque. On va à la flaque.</t>
+          <t>Le bateau est dans le sac. La voile est rentrée. Le manteau attend à côté. On y va, capitaine ? Oui. Le bateau va choisir.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le bateau est dans le sac. La voile est rentrée. Le manteau est à côté. C'est bon ? Presque. On va à la flaque.</t>
+          <t>Le bateau est dans le sac. La voile est rentrée. Le manteau attend à côté. On y va, capitaine ? Oui. Le bateau va choisir.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Le bateau est dans le sac. La voile est rentrée. Le manteau est à côté. C'est bon ? Presque. On va à la flaque.</t>
+          <t>Le bateau est dans le sac. La voile est rentrée. Le manteau attend à côté. On y va, capitaine ? Oui. Le bateau va choisir.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2079,11 +2085,10 @@
       </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le bateau est dans le sac.
-narrateur|La voile est rentrée.
-narrateur|Le manteau est à côté.
-enfant-m|C'est bon ?
-papa|Presque. On va à la flaque.</t>
+          <t>narrateur|Le bateau est dans le sac. La voile est rentrée.
+narrateur|Le manteau attend à côté.
+papa|On y va, capitaine ?
+enfant-m|Oui. Le bateau va choisir.</t>
         </is>
       </c>
     </row>
@@ -2110,17 +2115,17 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Quelle flaque ? Sous la gouttière, près du potager, ou près du bac.</t>
+          <t>Dehors, l'eau a fait trois chemins. La rivière de la gouttière. Le port des choux. L'île du bac. Où commence le voyage, capitaine ?</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Quelle flaque ? Sous la gouttière, près du potager, ou près du bac.</t>
+          <t>Dehors, l'eau a fait trois chemins. La rivière de la gouttière. Le port des choux. L'île du bac. Où commence le voyage, capitaine ?</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Quelle flaque ? Sous la gouttière, près du potager, ou près du bac.</t>
+          <t>Dehors, l'eau a fait trois chemins. La rivière de la gouttière. Le port des choux. L'île du bac. Où commence le voyage, capitaine ?</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
@@ -2138,7 +2143,7 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>sous la gouttière</t>
+          <t>la rivière de la gouttière</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -2148,7 +2153,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>près du potager</t>
+          <t>le port des choux</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -2158,7 +2163,7 @@
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>près du bac</t>
+          <t>l'île du bac</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
@@ -2274,8 +2279,9 @@
       <c r="AV7" s="2" t="inlineStr"/>
       <c r="AW7" t="inlineStr">
         <is>
-          <t>narrateur|Quelle flaque ?
-narrateur|Sous la gouttière, près du potager, ou près du bac.</t>
+          <t>narrateur|Dehors, l'eau a fait trois chemins.
+narrateur|La rivière de la gouttière. Le port des choux. L'île du bac.
+papa|Où commence le voyage, capitaine ?</t>
         </is>
       </c>
     </row>
@@ -2302,17 +2308,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Amir met le manteau. Il est tiède. Ils sortent. Le sac tape contre sa hanche. Sous la gouttière, une flaque ronde. Une goutte tombe. Plic. L'eau tremble. Le bateau, maintenant.</t>
+          <t>Amir enfile le manteau. Il est tiède contre ses bras. Sous la gouttière, l'eau tremble. Plic. Ploc. Une grosse feuille barre le passage. La rivière est fermée. Le bateau ne peut pas passer. Amir s'accroupit. La feuille ne bouge presque pas.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Amir met le manteau. Il est tiède. Ils sortent. Le sac tape contre sa hanche. Sous la gouttière, une flaque ronde. Une goutte tombe. Plic. L'eau tremble. Le bateau, maintenant.</t>
+          <t>Amir enfile le manteau. Il est tiède contre ses bras. Sous la gouttière, l'eau tremble. Plic. Ploc. Une grosse feuille barre le passage. La rivière est fermée. Le bateau ne peut pas passer. Amir s'accroupit. La feuille ne bouge presque pas.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Amir met le manteau. Il est tiède. Ils sortent. Le sac tape contre sa hanche. Sous la gouttière, une flaque ronde. Une goutte tombe. Plic. L'eau tremble. Le bateau, maintenant.</t>
+          <t>Amir enfile le manteau. Il est tiède contre ses bras. Sous la gouttière, l'eau tremble. Plic. Ploc. Une grosse feuille barre le passage. La rivière est fermée. Le bateau ne peut pas passer. Amir s'accroupit. La feuille ne bouge presque pas.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -2442,12 +2448,12 @@
       <c r="AV8" s="2" t="inlineStr"/>
       <c r="AW8" t="inlineStr">
         <is>
-          <t>narrateur|Amir met le manteau. Il est tiède.
-narrateur|Ils sortent. Le sac tape contre sa hanche.
-narrateur|Sous la gouttière, une flaque ronde.
-narrateur|Une goutte tombe. Plic.
-narrateur|L'eau tremble.
-papa|Le bateau, maintenant.</t>
+          <t>narrateur|Amir enfile le manteau. Il est tiède contre ses bras.
+narrateur|Sous la gouttière, l'eau tremble. Plic. Ploc.
+narrateur|Une grosse feuille barre le passage.
+enfant-m|La rivière est fermée.
+papa|Le bateau ne peut pas passer.
+narrateur|Amir s'accroupit. La feuille ne bouge presque pas.</t>
         </is>
       </c>
     </row>
@@ -2474,17 +2480,17 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -2502,7 +2508,7 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>au milieu</t>
+          <t>attendre les gouttes</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -2512,7 +2518,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>près du bord</t>
+          <t>appeler papa</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -2522,7 +2528,7 @@
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>sur le sac</t>
+          <t>changer de départ</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
@@ -2638,8 +2644,8 @@
       <c r="AV9" s="2" t="inlineStr"/>
       <c r="AW9" t="inlineStr">
         <is>
-          <t>narrateur|On pose le bateau…
-narrateur|Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>narrateur|Amir regarde.
+papa|Comment on fait, capitaine ?</t>
         </is>
       </c>
     </row>
@@ -2666,17 +2672,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Amir s'accroupit près de la feuille. J'attends encore un peu. Une goutte. Plic. La feuille bouge à peine. Une deuxième. Ploc. La feuille tourne. Une troisième. Plouf. La feuille ouvre un passage. La rivière est libre !</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Amir s'accroupit près de la feuille. J'attends encore un peu. Une goutte. Plic. La feuille bouge à peine. Une deuxième. Ploc. La feuille tourne. Une troisième. Plouf. La feuille ouvre un passage. La rivière est libre !</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Amir s'accroupit près de la feuille. J'attends encore un peu. Une goutte. Plic. La feuille bouge à peine. Une deuxième. Ploc. La feuille tourne. Une troisième. Plouf. La feuille ouvre un passage. La rivière est libre !</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -2806,13 +2812,12 @@
       <c r="AV10" s="2" t="inlineStr"/>
       <c r="AW10" t="inlineStr">
         <is>
-          <t>narrateur|Amir sort le bateau du sac.
-narrateur|Il le pose au milieu de l'eau.
-narrateur|La voile se tient.
-narrateur|Un peu d'eau touche le papier.
-papa|Il avance.
-narrateur|Amir souffle. Ffff.
-narrateur|Le bateau part tout doux.</t>
+          <t>narrateur|Amir s'accroupit près de la feuille.
+enfant-m|J'attends encore un peu.
+narrateur|Une goutte. Plic. La feuille bouge à peine.
+narrateur|Une deuxième. Ploc. La feuille tourne.
+narrateur|Une troisième. Plouf. La feuille ouvre un passage.
+enfant-m|La rivière est libre !</t>
         </is>
       </c>
     </row>
@@ -2839,17 +2844,17 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>De retour, Amir pose le bateau sur le petit linge. Alors, capitaine, jusqu'où es-tu allé ? Très loin. J'ai attendu trois gouttes. C'est vraiment loin. Une dernière goutte, dehors. Plic. Sur le linge, le bateau attend déjà le prochain voyage. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>De retour, Amir pose le bateau sur le petit linge. Alors, capitaine, jusqu'où es-tu allé ? Très loin. J'ai attendu trois gouttes. C'est vraiment loin. Une dernière goutte, dehors. Plic. Sur le linge, le bateau attend déjà le prochain voyage. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>De retour, Amir pose le bateau sur le petit linge. Alors, capitaine, jusqu'où es-tu allé ? Très loin. J'ai attendu trois gouttes. C'est vraiment loin. Une dernière goutte, dehors. Plic. Sur le linge, le bateau attend déjà le prochain voyage. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -2979,13 +2984,13 @@
       <c r="AV11" s="2" t="inlineStr"/>
       <c r="AW11" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir reprend le bateau.
-narrateur|Il le remet dans le sac.
-narrateur|Le manteau rentre aussi.
-narrateur|On referme. Zzz.
-narrateur|La gouttière fait un dernier plic.
-narrateur|L'histoire est finie.</t>
+          <t>narrateur|De retour, Amir pose le bateau sur le petit linge.
+papa|Alors, capitaine, jusqu'où es-tu allé ?
+enfant-m|Très loin. J'ai attendu trois gouttes.
+papa|C'est vraiment loin.
+narrateur|Une dernière goutte, dehors. Plic.
+narrateur|Sur le linge, le bateau attend déjà le prochain voyage.
+narrateur|Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -3012,17 +3017,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Papa, tu peux bouger la feuille ? On la pousse ensemble. Tout doux. Papa soulève le bord. Amir tient le bateau. La feuille glisse. L'eau circule. À toi, capitaine.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Papa, tu peux bouger la feuille ? On la pousse ensemble. Tout doux. Papa soulève le bord. Amir tient le bateau. La feuille glisse. L'eau circule. À toi, capitaine.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Papa, tu peux bouger la feuille ? On la pousse ensemble. Tout doux. Papa soulève le bord. Amir tient le bateau. La feuille glisse. L'eau circule. À toi, capitaine.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -3152,13 +3157,11 @@
       <c r="AV12" s="2" t="inlineStr"/>
       <c r="AW12" t="inlineStr">
         <is>
-          <t>narrateur|Amir sort le bateau.
-narrateur|Il le donne à papa.
-papa|Près du bord, ensemble.
-narrateur|Papa le pose. Amir tient le sac.
-narrateur|Le bateau part.
-narrateur|Amir marche le long de l'eau.
-narrateur|Le sac est à l'épaule.</t>
+          <t>enfant-m|Papa, tu peux bouger la feuille ?
+papa|On la pousse ensemble. Tout doux.
+narrateur|Papa soulève le bord. Amir tient le bateau.
+narrateur|La feuille glisse. L'eau circule.
+papa|À toi, capitaine.</t>
         </is>
       </c>
     </row>
@@ -3185,17 +3188,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>Dans la maison, Amir pose le bateau près de la fenêtre. On a poussé la feuille ensemble. Oui. La rivière a dit oui. Papa reprend sa table. Amir regarde le jardin. La gouttière fait encore un tout petit plic. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>Dans la maison, Amir pose le bateau près de la fenêtre. On a poussé la feuille ensemble. Oui. La rivière a dit oui. Papa reprend sa table. Amir regarde le jardin. La gouttière fait encore un tout petit plic. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>Dans la maison, Amir pose le bateau près de la fenêtre. On a poussé la feuille ensemble. Oui. La rivière a dit oui. Papa reprend sa table. Amir regarde le jardin. La gouttière fait encore un tout petit plic. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -3325,13 +3328,12 @@
       <c r="AV13" s="2" t="inlineStr"/>
       <c r="AW13" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir reprend le bateau.
-narrateur|Il le remet dans le sac.
-narrateur|Le manteau rentre aussi.
-narrateur|On referme. Zzz.
-narrateur|La gouttière fait un dernier plic.
-narrateur|L'histoire est finie.</t>
+          <t>narrateur|Dans la maison, Amir pose le bateau près de la fenêtre.
+papa|On a poussé la feuille ensemble.
+enfant-m|Oui. La rivière a dit oui.
+narrateur|Papa reprend sa table. Amir regarde le jardin.
+narrateur|La gouttière fait encore un tout petit plic.
+narrateur|Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -3358,17 +3360,17 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>On part d'ici, plus loin. Amir pose le bateau après la feuille, là où l'eau court déjà. Un petit courant emmène le papier sous une brindille. Une autre rivière !</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>On part d'ici, plus loin. Amir pose le bateau après la feuille, là où l'eau court déjà. Un petit courant emmène le papier sous une brindille. Une autre rivière !</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>On part d'ici, plus loin. Amir pose le bateau après la feuille, là où l'eau court déjà. Un petit courant emmène le papier sous une brindille. Une autre rivière !</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -3498,11 +3500,10 @@
       <c r="AV14" s="2" t="inlineStr"/>
       <c r="AW14" t="inlineStr">
         <is>
-          <t>narrateur|Amir pose d'abord le sac.
-narrateur|Il pose le bateau sur le sac.
-narrateur|Il regarde la flaque.
-narrateur|Puis il met le bateau dans l'eau.
-papa|Tu as préparé. Maintenant il flotte.</t>
+          <t>enfant-m|On part d'ici, plus loin.
+narrateur|Amir pose le bateau après la feuille, là où l'eau court déjà.
+narrateur|Un petit courant emmène le papier sous une brindille.
+enfant-m|Une autre rivière !</t>
         </is>
       </c>
     </row>
@@ -3529,17 +3530,17 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>Amir rentre. Le bateau a une brindille collée à la voile. On a trouvé un autre courant. Le bateau a choisi. Amir sourit. Le sac attend près de la porte. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>Amir rentre. Le bateau a une brindille collée à la voile. On a trouvé un autre courant. Le bateau a choisi. Amir sourit. Le sac attend près de la porte. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>Amir rentre. Le bateau a une brindille collée à la voile. On a trouvé un autre courant. Le bateau a choisi. Amir sourit. Le sac attend près de la porte. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr"/>
@@ -3669,13 +3670,11 @@
       <c r="AV15" s="2" t="inlineStr"/>
       <c r="AW15" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir reprend le bateau.
-narrateur|Il le remet dans le sac.
-narrateur|Le manteau rentre aussi.
-narrateur|On referme. Zzz.
-narrateur|La gouttière fait un dernier plic.
-narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir rentre. Le bateau a une brindille collée à la voile.
+enfant-m|On a trouvé un autre courant.
+papa|Le bateau a choisi.
+narrateur|Amir sourit. Le sac attend près de la porte.
+narrateur|Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -3702,17 +3701,17 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Amir met le manteau. Ils vont près du potager. La flaque est ronde, entre deux choux. Une feuille y trempe le bout. L'eau tremble un peu. Le bateau, Amir.</t>
+          <t>Amir enfile le manteau. Une odeur de soupe reste dans le col. Entre deux choux, une flaque ronde. Comme un port. Trois petites feuilles flottent devant l'entrée. Les bateaux n'arrivent pas à accoster. Il y a trois feuilles. Amir compte. Une. Deux. Trois.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Amir met le manteau. Ils vont près du potager. La flaque est ronde, entre deux choux. Une feuille y trempe le bout. L'eau tremble un peu. Le bateau, Amir.</t>
+          <t>Amir enfile le manteau. Une odeur de soupe reste dans le col. Entre deux choux, une flaque ronde. Comme un port. Trois petites feuilles flottent devant l'entrée. Les bateaux n'arrivent pas à accoster. Il y a trois feuilles. Amir compte. Une. Deux. Trois.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Amir met le manteau. Ils vont près du potager. La flaque est ronde, entre deux choux. Une feuille y trempe le bout. L'eau tremble un peu. Le bateau, Amir.</t>
+          <t>Amir enfile le manteau. Une odeur de soupe reste dans le col. Entre deux choux, une flaque ronde. Comme un port. Trois petites feuilles flottent devant l'entrée. Les bateaux n'arrivent pas à accoster. Il y a trois feuilles. Amir compte. Une. Deux. Trois.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -3842,12 +3841,12 @@
       <c r="AV16" s="2" t="inlineStr"/>
       <c r="AW16" t="inlineStr">
         <is>
-          <t>narrateur|Amir met le manteau.
-narrateur|Ils vont près du potager.
-narrateur|La flaque est ronde, entre deux choux.
-narrateur|Une feuille y trempe le bout.
-narrateur|L'eau tremble un peu.
-maman|Le bateau, Amir.</t>
+          <t>narrateur|Amir enfile le manteau. Une odeur de soupe reste dans le col.
+narrateur|Entre deux choux, une flaque ronde. Comme un port.
+narrateur|Trois petites feuilles flottent devant l'entrée.
+enfant-m|Les bateaux n'arrivent pas à accoster.
+papa|Il y a trois feuilles.
+narrateur|Amir compte. Une. Deux. Trois.</t>
         </is>
       </c>
     </row>
@@ -3874,17 +3873,17 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr"/>
@@ -3902,7 +3901,7 @@
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>au milieu</t>
+          <t>compter les feuilles</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
@@ -3912,7 +3911,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>près du bord</t>
+          <t>attendre le courant</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -3922,7 +3921,7 @@
       </c>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>sur le sac</t>
+          <t>demander à maman</t>
         </is>
       </c>
       <c r="R17" s="2" t="inlineStr">
@@ -4038,8 +4037,8 @@
       <c r="AV17" s="2" t="inlineStr"/>
       <c r="AW17" t="inlineStr">
         <is>
-          <t>narrateur|On pose le bateau…
-narrateur|Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>narrateur|Amir regarde.
+papa|Comment on fait, capitaine ?</t>
         </is>
       </c>
     </row>
@@ -4066,17 +4065,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Amir compte encore. Une. Deux. Trois. Là. Un espace libre. Il glisse le bateau entre la deuxième et la troisième feuille. Le papier touche un quai de terre. Toc. Quai Deux.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Amir compte encore. Une. Deux. Trois. Là. Un espace libre. Il glisse le bateau entre la deuxième et la troisième feuille. Le papier touche un quai de terre. Toc. Quai Deux.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Amir compte encore. Une. Deux. Trois. Là. Un espace libre. Il glisse le bateau entre la deuxième et la troisième feuille. Le papier touche un quai de terre. Toc. Quai Deux.</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -4206,13 +4205,11 @@
       <c r="AV18" s="2" t="inlineStr"/>
       <c r="AW18" t="inlineStr">
         <is>
-          <t>narrateur|Amir sort le bateau du sac.
-narrateur|Il le pose au milieu de l'eau.
-narrateur|La voile se tient.
-narrateur|Un peu d'eau touche le papier.
-papa|Il avance.
-narrateur|Amir souffle. Ffff.
-narrateur|Le bateau part tout doux.</t>
+          <t>narrateur|Amir compte encore. Une. Deux. Trois.
+enfant-m|Là. Un espace libre.
+narrateur|Il glisse le bateau entre la deuxième et la troisième feuille.
+narrateur|Le papier touche un quai de terre. Toc.
+enfant-m|Quai Deux.</t>
         </is>
       </c>
     </row>
@@ -4239,17 +4236,17 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>À table, Amir dit : Quai Un. Quai Deux. Quai Trois. Ton bateau a visité le port. Sans déranger les choux. Le bateau sèche. Les choux, dehors, restent droits. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>À table, Amir dit : Quai Un. Quai Deux. Quai Trois. Ton bateau a visité le port. Sans déranger les choux. Le bateau sèche. Les choux, dehors, restent droits. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>À table, Amir dit : Quai Un. Quai Deux. Quai Trois. Ton bateau a visité le port. Sans déranger les choux. Le bateau sèche. Les choux, dehors, restent droits. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -4379,13 +4376,12 @@
       <c r="AV19" s="2" t="inlineStr"/>
       <c r="AW19" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir reprend le bateau.
-narrateur|Il le remet dans le sac.
-narrateur|Le manteau rentre aussi.
-narrateur|On referme. Zzz.
-narrateur|Une feuille lâche la flaque.
-narrateur|L'histoire est finie.</t>
+          <t>narrateur|À table, Amir dit :
+enfant-m|Quai Un. Quai Deux. Quai Trois.
+maman|Ton bateau a visité le port.
+enfant-m|Sans déranger les choux.
+narrateur|Le bateau sèche. Les choux, dehors, restent droits.
+narrateur|Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -4412,17 +4408,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Amir attend. L'eau pousse tout doux. Une feuille s'écarte. Puis une autre. Le port s'ouvre. Le bateau avance tout seul jusqu'au chou.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Amir attend. L'eau pousse tout doux. Une feuille s'écarte. Puis une autre. Le port s'ouvre. Le bateau avance tout seul jusqu'au chou.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Amir attend. L'eau pousse tout doux. Une feuille s'écarte. Puis une autre. Le port s'ouvre. Le bateau avance tout seul jusqu'au chou.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -4552,13 +4548,10 @@
       <c r="AV20" s="2" t="inlineStr"/>
       <c r="AW20" t="inlineStr">
         <is>
-          <t>narrateur|Amir sort le bateau.
-narrateur|Il le donne à papa.
-papa|Près du bord, ensemble.
-narrateur|Papa le pose. Amir tient le sac.
-narrateur|Le bateau part.
-narrateur|Amir marche le long de l'eau.
-narrateur|Le sac est à l'épaule.</t>
+          <t>narrateur|Amir attend. L'eau pousse tout doux.
+narrateur|Une feuille s'écarte. Puis une autre.
+enfant-m|Le port s'ouvre.
+narrateur|Le bateau avance tout seul jusqu'au chou.</t>
         </is>
       </c>
     </row>
@@ -4585,17 +4578,17 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>Amir raconte : J'ai attendu. Les feuilles ont ouvert le port. Le courant a aidé. Le bateau sent encore un peu le chou. Amir rit. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>Amir raconte : J'ai attendu. Les feuilles ont ouvert le port. Le courant a aidé. Le bateau sent encore un peu le chou. Amir rit. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>Amir raconte : J'ai attendu. Les feuilles ont ouvert le port. Le courant a aidé. Le bateau sent encore un peu le chou. Amir rit. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -4725,13 +4718,11 @@
       <c r="AV21" s="2" t="inlineStr"/>
       <c r="AW21" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir reprend le bateau.
-narrateur|Il le remet dans le sac.
-narrateur|Le manteau rentre aussi.
-narrateur|On referme. Zzz.
-narrateur|Une feuille lâche la flaque.
-narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir raconte :
+enfant-m|J'ai attendu. Les feuilles ont ouvert le port.
+papa|Le courant a aidé.
+narrateur|Le bateau sent encore un peu le chou. Amir rit.
+narrateur|Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -4758,17 +4749,17 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>Maman est venue jusqu'au potager. Maman, je veux jouer sans abîmer les choux. Passe entre les feuilles. Pas dessus. Amir pose le bateau dans l'espace libre. Les plants ne bougent pas. Ton port est gentil avec le jardin.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>Maman est venue jusqu'au potager. Maman, je veux jouer sans abîmer les choux. Passe entre les feuilles. Pas dessus. Amir pose le bateau dans l'espace libre. Les plants ne bougent pas. Ton port est gentil avec le jardin.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>Maman est venue jusqu'au potager. Maman, je veux jouer sans abîmer les choux. Passe entre les feuilles. Pas dessus. Amir pose le bateau dans l'espace libre. Les plants ne bougent pas. Ton port est gentil avec le jardin.</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -4898,11 +4889,11 @@
       <c r="AV22" s="2" t="inlineStr"/>
       <c r="AW22" t="inlineStr">
         <is>
-          <t>narrateur|Amir pose d'abord le sac.
-narrateur|Il pose le bateau sur le sac.
-narrateur|Il regarde la flaque.
-narrateur|Puis il met le bateau dans l'eau.
-papa|Tu as préparé. Maintenant il flotte.</t>
+          <t>narrateur|Maman est venue jusqu'au potager.
+enfant-m|Maman, je veux jouer sans abîmer les choux.
+maman|Passe entre les feuilles. Pas dessus.
+narrateur|Amir pose le bateau dans l'espace libre. Les plants ne bougent pas.
+maman|Ton port est gentil avec le jardin.</t>
         </is>
       </c>
     </row>
@@ -4929,17 +4920,17 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>Merci d'avoir demandé. Le port est dans le jardin. On le garde. Amir pose le bateau. Maman pose la soupe. Deux voyages : l'eau, et la maison. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>Merci d'avoir demandé. Le port est dans le jardin. On le garde. Amir pose le bateau. Maman pose la soupe. Deux voyages : l'eau, et la maison. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>Merci d'avoir demandé. Le port est dans le jardin. On le garde. Amir pose le bateau. Maman pose la soupe. Deux voyages : l'eau, et la maison. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -5069,13 +5060,11 @@
       <c r="AV23" s="2" t="inlineStr"/>
       <c r="AW23" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir reprend le bateau.
-narrateur|Il le remet dans le sac.
-narrateur|Le manteau rentre aussi.
-narrateur|On referme. Zzz.
-narrateur|Une feuille lâche la flaque.
-narrateur|L'histoire est finie.</t>
+          <t>maman|Merci d'avoir demandé.
+enfant-m|Le port est dans le jardin. On le garde.
+narrateur|Amir pose le bateau. Maman pose la soupe.
+narrateur|Deux voyages : l'eau, et la maison.
+narrateur|Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -5102,17 +5091,17 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Amir met le manteau. Ils vont près du bac à sable. Une flaque borde le bois du bac. Un peu de sable brille au fond. Le bateau, Amir.</t>
+          <t>Amir enfile le manteau. Le sac tape contre le tissu. Près du bac à sable, l'eau devient de plus en plus petite. Elle rentre dans le sol. Le bateau n'aurait plus assez d'eau. Mon chemin disparaît. Le sable boit la flaque. Amir serre le bateau. Il avait imaginé cette île.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Amir met le manteau. Ils vont près du bac à sable. Une flaque borde le bois du bac. Un peu de sable brille au fond. Le bateau, Amir.</t>
+          <t>Amir enfile le manteau. Le sac tape contre le tissu. Près du bac à sable, l'eau devient de plus en plus petite. Elle rentre dans le sol. Le bateau n'aurait plus assez d'eau. Mon chemin disparaît. Le sable boit la flaque. Amir serre le bateau. Il avait imaginé cette île.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Amir met le manteau. Ils vont près du bac à sable. Une flaque borde le bois du bac. Un peu de sable brille au fond. Le bateau, Amir.</t>
+          <t>Amir enfile le manteau. Le sac tape contre le tissu. Près du bac à sable, l'eau devient de plus en plus petite. Elle rentre dans le sol. Le bateau n'aurait plus assez d'eau. Mon chemin disparaît. Le sable boit la flaque. Amir serre le bateau. Il avait imaginé cette île.</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -5242,11 +5231,12 @@
       <c r="AV24" s="2" t="inlineStr"/>
       <c r="AW24" t="inlineStr">
         <is>
-          <t>narrateur|Amir met le manteau.
-narrateur|Ils vont près du bac à sable.
-narrateur|Une flaque borde le bois du bac.
-narrateur|Un peu de sable brille au fond.
-papa|Le bateau, Amir.</t>
+          <t>narrateur|Amir enfile le manteau. Le sac tape contre le tissu.
+narrateur|Près du bac à sable, l'eau devient de plus en plus petite.
+narrateur|Elle rentre dans le sol. Le bateau n'aurait plus assez d'eau.
+enfant-m|Mon chemin disparaît.
+papa|Le sable boit la flaque.
+narrateur|Amir serre le bateau. Il avait imaginé cette île.</t>
         </is>
       </c>
     </row>
@@ -5273,17 +5263,17 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr"/>
@@ -5301,7 +5291,7 @@
       <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>au milieu</t>
+          <t>une autre flaque</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
@@ -5311,7 +5301,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>près du bord</t>
+          <t>sur le sable</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -5321,7 +5311,7 @@
       </c>
       <c r="Q25" s="2" t="inlineStr">
         <is>
-          <t>sur le sac</t>
+          <t>un autre bateau</t>
         </is>
       </c>
       <c r="R25" s="2" t="inlineStr">
@@ -5437,8 +5427,8 @@
       <c r="AV25" s="2" t="inlineStr"/>
       <c r="AW25" t="inlineStr">
         <is>
-          <t>narrateur|On pose le bateau…
-narrateur|Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>narrateur|Amir regarde.
+papa|Comment on fait, capitaine ?</t>
         </is>
       </c>
     </row>
@@ -5465,17 +5455,17 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Celle-ci s'en va. On prend l'autre. À côté, une flaque plus ronde tient encore. Amir y pose le bateau. Il avance. Ffff. Nouveau départ.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Celle-ci s'en va. On prend l'autre. À côté, une flaque plus ronde tient encore. Amir y pose le bateau. Il avance. Ffff. Nouveau départ.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Celle-ci s'en va. On prend l'autre. À côté, une flaque plus ronde tient encore. Amir y pose le bateau. Il avance. Ffff. Nouveau départ.</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -5605,13 +5595,10 @@
       <c r="AV26" s="2" t="inlineStr"/>
       <c r="AW26" t="inlineStr">
         <is>
-          <t>narrateur|Amir sort le bateau du sac.
-narrateur|Il le pose au milieu de l'eau.
-narrateur|La voile se tient.
-narrateur|Un peu d'eau touche le papier.
-papa|Il avance.
-narrateur|Amir souffle. Ffff.
-narrateur|Le bateau part tout doux.</t>
+          <t>enfant-m|Celle-ci s'en va. On prend l'autre.
+narrateur|À côté, une flaque plus ronde tient encore.
+narrateur|Amir y pose le bateau. Il avance. Ffff.
+papa|Nouveau départ.</t>
         </is>
       </c>
     </row>
@@ -5638,17 +5625,17 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>La première flaque est partie. L'autre m'a emmené. Changer de chemin, ce n'est pas perdre. Amir hoche la tête. Le bateau sèche près du volet jaune. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>La première flaque est partie. L'autre m'a emmené. Changer de chemin, ce n'est pas perdre. Amir hoche la tête. Le bateau sèche près du volet jaune. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>La première flaque est partie. L'autre m'a emmené. Changer de chemin, ce n'est pas perdre. Amir hoche la tête. Le bateau sèche près du volet jaune. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -5778,13 +5765,10 @@
       <c r="AV27" s="2" t="inlineStr"/>
       <c r="AW27" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir reprend le bateau.
-narrateur|Il le remet dans le sac.
-narrateur|Le manteau rentre aussi.
-narrateur|On referme. Zzz.
-narrateur|Un grain de sable reste sur le bois.
-narrateur|L'histoire est finie.</t>
+          <t>enfant-m|La première flaque est partie. L'autre m'a emmené.
+papa|Changer de chemin, ce n'est pas perdre.
+narrateur|Amir hoche la tête. Le bateau sèche près du volet jaune.
+narrateur|Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -5811,17 +5795,17 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Plus d'eau. Alors il marche. Amir pousse le bateau sur le sable humide. Une piste. Le papier glisse. Grain. Grain. Un bateau de terre, aujourd'hui.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Plus d'eau. Alors il marche. Amir pousse le bateau sur le sable humide. Une piste. Le papier glisse. Grain. Grain. Un bateau de terre, aujourd'hui.</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Plus d'eau. Alors il marche. Amir pousse le bateau sur le sable humide. Une piste. Le papier glisse. Grain. Grain. Un bateau de terre, aujourd'hui.</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -5951,13 +5935,10 @@
       <c r="AV28" s="2" t="inlineStr"/>
       <c r="AW28" t="inlineStr">
         <is>
-          <t>narrateur|Amir sort le bateau.
-narrateur|Il le donne à papa.
-papa|Près du bord, ensemble.
-narrateur|Papa le pose. Amir tient le sac.
-narrateur|Le bateau part.
-narrateur|Amir marche le long de l'eau.
-narrateur|Le sac est à l'épaule.</t>
+          <t>enfant-m|Plus d'eau. Alors il marche.
+narrateur|Amir pousse le bateau sur le sable humide. Une piste.
+narrateur|Le papier glisse. Grain. Grain.
+papa|Un bateau de terre, aujourd'hui.</t>
         </is>
       </c>
     </row>
@@ -5984,17 +5965,17 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>Aujourd'hui, mon bateau a marché. Un capitaine de sable. Un grain reste sur la cheminée rouge. Amir le souffle. Ffff. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>Aujourd'hui, mon bateau a marché. Un capitaine de sable. Un grain reste sur la cheminée rouge. Amir le souffle. Ffff. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>Aujourd'hui, mon bateau a marché. Un capitaine de sable. Un grain reste sur la cheminée rouge. Amir le souffle. Ffff. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -6124,13 +6105,10 @@
       <c r="AV29" s="2" t="inlineStr"/>
       <c r="AW29" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir reprend le bateau.
-narrateur|Il le remet dans le sac.
-narrateur|Le manteau rentre aussi.
-narrateur|On referme. Zzz.
-narrateur|Un grain de sable reste sur le bois.
-narrateur|L'histoire est finie.</t>
+          <t>enfant-m|Aujourd'hui, mon bateau a marché.
+papa|Un capitaine de sable.
+narrateur|Un grain reste sur la cheminée rouge. Amir le souffle. Ffff.
+narrateur|Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -6157,17 +6135,17 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>Celui-là est trop fragile. Amir pose le bateau en papier dans le sac. On en fabrique un autre, plus solide. Avec une feuille plus épaisse, ils plient une nouvelle coque. Celui-ci, pour le sable.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>Celui-là est trop fragile. Amir pose le bateau en papier dans le sac. On en fabrique un autre, plus solide. Avec une feuille plus épaisse, ils plient une nouvelle coque. Celui-ci, pour le sable.</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>Celui-là est trop fragile. Amir pose le bateau en papier dans le sac. On en fabrique un autre, plus solide. Avec une feuille plus épaisse, ils plient une nouvelle coque. Celui-ci, pour le sable.</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -6297,11 +6275,11 @@
       <c r="AV30" s="2" t="inlineStr"/>
       <c r="AW30" t="inlineStr">
         <is>
-          <t>narrateur|Amir pose d'abord le sac.
-narrateur|Il pose le bateau sur le sac.
-narrateur|Il regarde la flaque.
-narrateur|Puis il met le bateau dans l'eau.
-papa|Tu as préparé. Maintenant il flotte.</t>
+          <t>enfant-m|Celui-là est trop fragile.
+narrateur|Amir pose le bateau en papier dans le sac.
+papa|On en fabrique un autre, plus solide.
+narrateur|Avec une feuille plus épaisse, ils plient une nouvelle coque.
+enfant-m|Celui-ci, pour le sable.</t>
         </is>
       </c>
     </row>
@@ -6328,17 +6306,17 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>Deux bateaux maintenant. L'ancien dans le sac. Le nouveau sur la table. Celui-là, pour demain. On a bien fait. Le papier fragile se repose. L'autre attend le jardin. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>Deux bateaux maintenant. L'ancien dans le sac. Le nouveau sur la table. Celui-là, pour demain. On a bien fait. Le papier fragile se repose. L'autre attend le jardin. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Le manteau rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>Deux bateaux maintenant. L'ancien dans le sac. Le nouveau sur la table. Celui-là, pour demain. On a bien fait. Le papier fragile se repose. L'autre attend le jardin. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -6468,13 +6446,11 @@
       <c r="AV31" s="2" t="inlineStr"/>
       <c r="AW31" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir reprend le bateau.
-narrateur|Il le remet dans le sac.
-narrateur|Le manteau rentre aussi.
-narrateur|On referme. Zzz.
-narrateur|Un grain de sable reste sur le bois.
-narrateur|L'histoire est finie.</t>
+          <t>narrateur|Deux bateaux maintenant. L'ancien dans le sac. Le nouveau sur la table.
+enfant-m|Celui-là, pour demain.
+papa|On a bien fait.
+narrateur|Le papier fragile se repose. L'autre attend le jardin.
+narrateur|Il raccroche le manteau. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -6501,17 +6477,17 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Amir glisse le bateau au fond du sac. Toc. La voile dépasse. Il la rentre. Les bottes sont près de la porte. Elles sont encore mouillées dehors. Attends. Je les essuie. Maman frotte le bout, tout doux. Merci, maman. Amir les pose à côté du sac. Au pied, juste avant de sortir.</t>
+          <t>Amir glisse le bateau au fond du sac. Toc. La voile dépasse. Il la rentre. Les bottes sont près de la porte. Un peu mouillées dehors. Attends. Je les essuie. Maman passe le linge sur chaque botte. Voilà. Tes pieds resteront au sec.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Amir glisse le bateau au fond du sac. Toc. La voile dépasse. Il la rentre. Les bottes sont près de la porte. Elles sont encore mouillées dehors. Attends. Je les essuie. Maman frotte le bout, tout doux. Merci, maman. Amir les pose à côté du sac. Au pied, juste avant de sortir.</t>
+          <t>Amir glisse le bateau au fond du sac. Toc. La voile dépasse. Il la rentre. Les bottes sont près de la porte. Un peu mouillées dehors. Attends. Je les essuie. Maman passe le linge sur chaque botte. Voilà. Tes pieds resteront au sec.</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Amir glisse le bateau au fond du sac. Toc. La voile dépasse. Il la rentre. Les bottes sont près de la porte. Elles sont encore mouillées dehors. Attends. Je les essuie. Maman frotte le bout, tout doux. Merci, maman. Amir les pose à côté du sac. Au pied, juste avant de sortir.</t>
+          <t>Amir glisse le bateau au fond du sac. Toc. La voile dépasse. Il la rentre. Les bottes sont près de la porte. Un peu mouillées dehors. Attends. Je les essuie. Maman passe le linge sur chaque botte. Voilà. Tes pieds resteront au sec.</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -6641,16 +6617,12 @@
       <c r="AV32" s="2" t="inlineStr"/>
       <c r="AW32" t="inlineStr">
         <is>
-          <t>narrateur|Amir glisse le bateau au fond du sac.
-narrateur|Toc.
+          <t>narrateur|Amir glisse le bateau au fond du sac. Toc.
 narrateur|La voile dépasse. Il la rentre.
-narrateur|Les bottes sont près de la porte.
-narrateur|Elles sont encore mouillées dehors.
+narrateur|Les bottes sont près de la porte. Un peu mouillées dehors.
 maman|Attends. Je les essuie.
-narrateur|Maman frotte le bout, tout doux.
-enfant-m|Merci, maman.
-narrateur|Amir les pose à côté du sac.
-maman|Au pied, juste avant de sortir.</t>
+narrateur|Maman passe le linge sur chaque botte.
+maman|Voilà. Tes pieds resteront au sec.</t>
         </is>
       </c>
     </row>
@@ -6697,7 +6669,7 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>maman | ma maman</t>
+          <t>maman|ma maman|maman essuie</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -6712,7 +6684,7 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>C'est maman qui essuie.</t>
+          <t>Maman essuie les bottes.</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr"/>
@@ -6864,17 +6836,17 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Maman a essuyé les bottes. Le bateau est dans le sac. Les bottes attendent près de la porte. On va à la flaque.</t>
+          <t>Les bottes sont sèches. Elles attendent près de la porte. Le bateau est dans le sac. Capitaine, tes bottes sont prêtes. On va au jardin.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Maman a essuyé les bottes. Le bateau est dans le sac. Les bottes attendent près de la porte. On va à la flaque.</t>
+          <t>Les bottes sont sèches. Elles attendent près de la porte. Le bateau est dans le sac. Capitaine, tes bottes sont prêtes. On va au jardin.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Maman a essuyé les bottes. Le bateau est dans le sac. Les bottes attendent près de la porte. On va à la flaque.</t>
+          <t>Les bottes sont sèches. Elles attendent près de la porte. Le bateau est dans le sac. Capitaine, tes bottes sont prêtes. On va au jardin.</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
@@ -7008,10 +6980,10 @@
       </c>
       <c r="AW34" t="inlineStr">
         <is>
-          <t>narrateur|Maman a essuyé les bottes.
+          <t>narrateur|Les bottes sont sèches. Elles attendent près de la porte.
 narrateur|Le bateau est dans le sac.
-narrateur|Les bottes attendent près de la porte.
-papa|On va à la flaque.</t>
+papa|Capitaine, tes bottes sont prêtes.
+enfant-m|On va au jardin.</t>
         </is>
       </c>
     </row>
@@ -7038,17 +7010,17 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Quelle flaque ? Sous la gouttière, près du potager, ou près du bac.</t>
+          <t>Dehors, l'eau a fait trois chemins. La rivière de la gouttière. Le port des choux. L'île du bac. Où commence le voyage, capitaine ?</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Quelle flaque ? Sous la gouttière, près du potager, ou près du bac.</t>
+          <t>Dehors, l'eau a fait trois chemins. La rivière de la gouttière. Le port des choux. L'île du bac. Où commence le voyage, capitaine ?</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Quelle flaque ? Sous la gouttière, près du potager, ou près du bac.</t>
+          <t>Dehors, l'eau a fait trois chemins. La rivière de la gouttière. Le port des choux. L'île du bac. Où commence le voyage, capitaine ?</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr"/>
@@ -7066,7 +7038,7 @@
       <c r="L35" s="2" t="inlineStr"/>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>sous la gouttière</t>
+          <t>la rivière de la gouttière</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr">
@@ -7076,7 +7048,7 @@
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>près du potager</t>
+          <t>le port des choux</t>
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr">
@@ -7086,7 +7058,7 @@
       </c>
       <c r="Q35" s="2" t="inlineStr">
         <is>
-          <t>près du bac</t>
+          <t>l'île du bac</t>
         </is>
       </c>
       <c r="R35" s="2" t="inlineStr">
@@ -7202,8 +7174,9 @@
       <c r="AV35" s="2" t="inlineStr"/>
       <c r="AW35" t="inlineStr">
         <is>
-          <t>narrateur|Quelle flaque ?
-narrateur|Sous la gouttière, près du potager, ou près du bac.</t>
+          <t>narrateur|Dehors, l'eau a fait trois chemins.
+narrateur|La rivière de la gouttière. Le port des choux. L'île du bac.
+papa|Où commence le voyage, capitaine ?</t>
         </is>
       </c>
     </row>
@@ -7230,17 +7203,17 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Amir enfile les bottes près de la porte. Elles sont un peu froides, plus mouillées. Sous la gouttière, une flaque ronde. Ses bottes font un petit clap dans l'herbe. Une goutte tombe. Plic. Le bateau, maintenant.</t>
+          <t>Amir enfile les bottes. Elles sont un peu froides. Clap. Sous la gouttière, l'eau tremble. Plic. Ploc. Une grosse feuille barre le passage. La rivière est fermée. Le bateau ne peut pas passer. Amir s'accroupit. La feuille ne bouge presque pas.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Amir enfile les bottes près de la porte. Elles sont un peu froides, plus mouillées. Sous la gouttière, une flaque ronde. Ses bottes font un petit clap dans l'herbe. Une goutte tombe. Plic. Le bateau, maintenant.</t>
+          <t>Amir enfile les bottes. Elles sont un peu froides. Clap. Sous la gouttière, l'eau tremble. Plic. Ploc. Une grosse feuille barre le passage. La rivière est fermée. Le bateau ne peut pas passer. Amir s'accroupit. La feuille ne bouge presque pas.</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Amir enfile les bottes près de la porte. Elles sont un peu froides, plus mouillées. Sous la gouttière, une flaque ronde. Ses bottes font un petit clap dans l'herbe. Une goutte tombe. Plic. Le bateau, maintenant.</t>
+          <t>Amir enfile les bottes. Elles sont un peu froides. Clap. Sous la gouttière, l'eau tremble. Plic. Ploc. Une grosse feuille barre le passage. La rivière est fermée. Le bateau ne peut pas passer. Amir s'accroupit. La feuille ne bouge presque pas.</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
@@ -7370,12 +7343,12 @@
       <c r="AV36" s="2" t="inlineStr"/>
       <c r="AW36" t="inlineStr">
         <is>
-          <t>narrateur|Amir enfile les bottes près de la porte.
-narrateur|Elles sont un peu froides, plus mouillées.
-narrateur|Sous la gouttière, une flaque ronde.
-narrateur|Ses bottes font un petit clap dans l'herbe.
-narrateur|Une goutte tombe. Plic.
-papa|Le bateau, maintenant.</t>
+          <t>narrateur|Amir enfile les bottes. Elles sont un peu froides. Clap.
+narrateur|Sous la gouttière, l'eau tremble. Plic. Ploc.
+narrateur|Une grosse feuille barre le passage.
+enfant-m|La rivière est fermée.
+papa|Le bateau ne peut pas passer.
+narrateur|Amir s'accroupit. La feuille ne bouge presque pas.</t>
         </is>
       </c>
     </row>
@@ -7402,17 +7375,17 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr"/>
@@ -7430,7 +7403,7 @@
       <c r="L37" s="2" t="inlineStr"/>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>au milieu</t>
+          <t>attendre les gouttes</t>
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr">
@@ -7440,7 +7413,7 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>près du bord</t>
+          <t>appeler papa</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
@@ -7450,7 +7423,7 @@
       </c>
       <c r="Q37" s="2" t="inlineStr">
         <is>
-          <t>sur le sac</t>
+          <t>changer de départ</t>
         </is>
       </c>
       <c r="R37" s="2" t="inlineStr">
@@ -7566,8 +7539,8 @@
       <c r="AV37" s="2" t="inlineStr"/>
       <c r="AW37" t="inlineStr">
         <is>
-          <t>narrateur|On pose le bateau…
-narrateur|Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>narrateur|Amir regarde.
+papa|Comment on fait, capitaine ?</t>
         </is>
       </c>
     </row>
@@ -7594,17 +7567,17 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Amir s'accroupit près de la feuille. J'attends encore un peu. Une goutte. Plic. La feuille bouge à peine. Une deuxième. Ploc. La feuille tourne. Une troisième. Plouf. La feuille ouvre un passage. La rivière est libre !</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Amir s'accroupit près de la feuille. J'attends encore un peu. Une goutte. Plic. La feuille bouge à peine. Une deuxième. Ploc. La feuille tourne. Une troisième. Plouf. La feuille ouvre un passage. La rivière est libre !</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Amir s'accroupit près de la feuille. J'attends encore un peu. Une goutte. Plic. La feuille bouge à peine. Une deuxième. Ploc. La feuille tourne. Une troisième. Plouf. La feuille ouvre un passage. La rivière est libre !</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -7734,13 +7707,12 @@
       <c r="AV38" s="2" t="inlineStr"/>
       <c r="AW38" t="inlineStr">
         <is>
-          <t>narrateur|Amir sort le bateau du sac.
-narrateur|Il le pose au milieu de l'eau.
-narrateur|La voile se tient.
-narrateur|Un peu d'eau touche le papier.
-papa|Il avance.
-narrateur|Amir souffle. Ffff.
-narrateur|Le bateau part tout doux.</t>
+          <t>narrateur|Amir s'accroupit près de la feuille.
+enfant-m|J'attends encore un peu.
+narrateur|Une goutte. Plic. La feuille bouge à peine.
+narrateur|Une deuxième. Ploc. La feuille tourne.
+narrateur|Une troisième. Plouf. La feuille ouvre un passage.
+enfant-m|La rivière est libre !</t>
         </is>
       </c>
     </row>
@@ -7767,17 +7739,17 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>De retour, Amir pose le bateau sur le petit linge. Alors, capitaine, jusqu'où es-tu allé ? Très loin. J'ai attendu trois gouttes. C'est vraiment loin. Une dernière goutte, dehors. Plic. Sur le linge, le bateau attend déjà le prochain voyage. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>De retour, Amir pose le bateau sur le petit linge. Alors, capitaine, jusqu'où es-tu allé ? Très loin. J'ai attendu trois gouttes. C'est vraiment loin. Une dernière goutte, dehors. Plic. Sur le linge, le bateau attend déjà le prochain voyage. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>De retour, Amir pose le bateau sur le petit linge. Alors, capitaine, jusqu'où es-tu allé ? Très loin. J'ai attendu trois gouttes. C'est vraiment loin. Une dernière goutte, dehors. Plic. Sur le linge, le bateau attend déjà le prochain voyage. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
@@ -7907,13 +7879,13 @@
       <c r="AV39" s="2" t="inlineStr"/>
       <c r="AW39" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir reprend le bateau.
-narrateur|Il le remet dans le sac.
-narrateur|Les bottes restent aux pieds, jusqu'à la porte.
-narrateur|On referme. Zzz.
-narrateur|La gouttière fait un dernier plic.
-narrateur|L'histoire est finie.</t>
+          <t>narrateur|De retour, Amir pose le bateau sur le petit linge.
+papa|Alors, capitaine, jusqu'où es-tu allé ?
+enfant-m|Très loin. J'ai attendu trois gouttes.
+papa|C'est vraiment loin.
+narrateur|Une dernière goutte, dehors. Plic.
+narrateur|Sur le linge, le bateau attend déjà le prochain voyage.
+narrateur|À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -7940,17 +7912,17 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Papa, tu peux bouger la feuille ? On la pousse ensemble. Tout doux. Papa soulève le bord. Amir tient le bateau. La feuille glisse. L'eau circule. À toi, capitaine.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Papa, tu peux bouger la feuille ? On la pousse ensemble. Tout doux. Papa soulève le bord. Amir tient le bateau. La feuille glisse. L'eau circule. À toi, capitaine.</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Papa, tu peux bouger la feuille ? On la pousse ensemble. Tout doux. Papa soulève le bord. Amir tient le bateau. La feuille glisse. L'eau circule. À toi, capitaine.</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -8080,13 +8052,11 @@
       <c r="AV40" s="2" t="inlineStr"/>
       <c r="AW40" t="inlineStr">
         <is>
-          <t>narrateur|Amir sort le bateau.
-narrateur|Il le donne à papa.
-papa|Près du bord, ensemble.
-narrateur|Papa le pose. Amir tient le sac.
-narrateur|Le bateau part.
-narrateur|Amir marche le long de l'eau.
-narrateur|Le sac est à l'épaule.</t>
+          <t>enfant-m|Papa, tu peux bouger la feuille ?
+papa|On la pousse ensemble. Tout doux.
+narrateur|Papa soulève le bord. Amir tient le bateau.
+narrateur|La feuille glisse. L'eau circule.
+papa|À toi, capitaine.</t>
         </is>
       </c>
     </row>
@@ -8113,17 +8083,17 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>Dans la maison, Amir pose le bateau près de la fenêtre. On a poussé la feuille ensemble. Oui. La rivière a dit oui. Papa reprend sa table. Amir regarde le jardin. La gouttière fait encore un tout petit plic. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>Dans la maison, Amir pose le bateau près de la fenêtre. On a poussé la feuille ensemble. Oui. La rivière a dit oui. Papa reprend sa table. Amir regarde le jardin. La gouttière fait encore un tout petit plic. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>Dans la maison, Amir pose le bateau près de la fenêtre. On a poussé la feuille ensemble. Oui. La rivière a dit oui. Papa reprend sa table. Amir regarde le jardin. La gouttière fait encore un tout petit plic. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
@@ -8253,13 +8223,12 @@
       <c r="AV41" s="2" t="inlineStr"/>
       <c r="AW41" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir reprend le bateau.
-narrateur|Il le remet dans le sac.
-narrateur|Les bottes restent aux pieds, jusqu'à la porte.
-narrateur|On referme. Zzz.
-narrateur|La gouttière fait un dernier plic.
-narrateur|L'histoire est finie.</t>
+          <t>narrateur|Dans la maison, Amir pose le bateau près de la fenêtre.
+papa|On a poussé la feuille ensemble.
+enfant-m|Oui. La rivière a dit oui.
+narrateur|Papa reprend sa table. Amir regarde le jardin.
+narrateur|La gouttière fait encore un tout petit plic.
+narrateur|À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -8286,17 +8255,17 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>On part d'ici, plus loin. Amir pose le bateau après la feuille, là où l'eau court déjà. Un petit courant emmène le papier sous une brindille. Une autre rivière !</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>On part d'ici, plus loin. Amir pose le bateau après la feuille, là où l'eau court déjà. Un petit courant emmène le papier sous une brindille. Une autre rivière !</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>On part d'ici, plus loin. Amir pose le bateau après la feuille, là où l'eau court déjà. Un petit courant emmène le papier sous une brindille. Une autre rivière !</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -8426,11 +8395,10 @@
       <c r="AV42" s="2" t="inlineStr"/>
       <c r="AW42" t="inlineStr">
         <is>
-          <t>narrateur|Amir pose d'abord le sac.
-narrateur|Il pose le bateau sur le sac.
-narrateur|Il regarde la flaque.
-narrateur|Puis il met le bateau dans l'eau.
-papa|Tu as préparé. Maintenant il flotte.</t>
+          <t>enfant-m|On part d'ici, plus loin.
+narrateur|Amir pose le bateau après la feuille, là où l'eau court déjà.
+narrateur|Un petit courant emmène le papier sous une brindille.
+enfant-m|Une autre rivière !</t>
         </is>
       </c>
     </row>
@@ -8457,17 +8425,17 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>Amir rentre. Le bateau a une brindille collée à la voile. On a trouvé un autre courant. Le bateau a choisi. Amir sourit. Le sac attend près de la porte. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>Amir rentre. Le bateau a une brindille collée à la voile. On a trouvé un autre courant. Le bateau a choisi. Amir sourit. Le sac attend près de la porte. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>Amir rentre. Le bateau a une brindille collée à la voile. On a trouvé un autre courant. Le bateau a choisi. Amir sourit. Le sac attend près de la porte. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -8597,13 +8565,11 @@
       <c r="AV43" s="2" t="inlineStr"/>
       <c r="AW43" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir reprend le bateau.
-narrateur|Il le remet dans le sac.
-narrateur|Les bottes restent aux pieds, jusqu'à la porte.
-narrateur|On referme. Zzz.
-narrateur|La gouttière fait un dernier plic.
-narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir rentre. Le bateau a une brindille collée à la voile.
+enfant-m|On a trouvé un autre courant.
+papa|Le bateau a choisi.
+narrateur|Amir sourit. Le sac attend près de la porte.
+narrateur|À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -8630,17 +8596,17 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Amir enfile les bottes. Ils vont près du potager. La terre est molle. Les bottes tiennent. La flaque est ronde, entre deux choux. Le bateau, Amir.</t>
+          <t>Amir enfile les bottes. Elles font clap-clap vers les choux. Entre deux choux, une flaque ronde. Comme un port. Trois petites feuilles flottent devant l'entrée. Les bateaux n'arrivent pas à accoster. Il y a trois feuilles. Amir compte. Une. Deux. Trois.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Amir enfile les bottes. Ils vont près du potager. La terre est molle. Les bottes tiennent. La flaque est ronde, entre deux choux. Le bateau, Amir.</t>
+          <t>Amir enfile les bottes. Elles font clap-clap vers les choux. Entre deux choux, une flaque ronde. Comme un port. Trois petites feuilles flottent devant l'entrée. Les bateaux n'arrivent pas à accoster. Il y a trois feuilles. Amir compte. Une. Deux. Trois.</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Amir enfile les bottes. Ils vont près du potager. La terre est molle. Les bottes tiennent. La flaque est ronde, entre deux choux. Le bateau, Amir.</t>
+          <t>Amir enfile les bottes. Elles font clap-clap vers les choux. Entre deux choux, une flaque ronde. Comme un port. Trois petites feuilles flottent devant l'entrée. Les bateaux n'arrivent pas à accoster. Il y a trois feuilles. Amir compte. Une. Deux. Trois.</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
@@ -8770,11 +8736,12 @@
       <c r="AV44" s="2" t="inlineStr"/>
       <c r="AW44" t="inlineStr">
         <is>
-          <t>narrateur|Amir enfile les bottes.
-narrateur|Ils vont près du potager.
-narrateur|La terre est molle. Les bottes tiennent.
-narrateur|La flaque est ronde, entre deux choux.
-maman|Le bateau, Amir.</t>
+          <t>narrateur|Amir enfile les bottes. Elles font clap-clap vers les choux.
+narrateur|Entre deux choux, une flaque ronde. Comme un port.
+narrateur|Trois petites feuilles flottent devant l'entrée.
+enfant-m|Les bateaux n'arrivent pas à accoster.
+papa|Il y a trois feuilles.
+narrateur|Amir compte. Une. Deux. Trois.</t>
         </is>
       </c>
     </row>
@@ -8801,17 +8768,17 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr"/>
@@ -8829,7 +8796,7 @@
       <c r="L45" s="2" t="inlineStr"/>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>au milieu</t>
+          <t>compter les feuilles</t>
         </is>
       </c>
       <c r="N45" s="2" t="inlineStr">
@@ -8839,7 +8806,7 @@
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>près du bord</t>
+          <t>attendre le courant</t>
         </is>
       </c>
       <c r="P45" s="2" t="inlineStr">
@@ -8849,7 +8816,7 @@
       </c>
       <c r="Q45" s="2" t="inlineStr">
         <is>
-          <t>sur le sac</t>
+          <t>demander à maman</t>
         </is>
       </c>
       <c r="R45" s="2" t="inlineStr">
@@ -8965,8 +8932,8 @@
       <c r="AV45" s="2" t="inlineStr"/>
       <c r="AW45" t="inlineStr">
         <is>
-          <t>narrateur|On pose le bateau…
-narrateur|Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>narrateur|Amir regarde.
+papa|Comment on fait, capitaine ?</t>
         </is>
       </c>
     </row>
@@ -8993,17 +8960,17 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Amir compte encore. Une. Deux. Trois. Là. Un espace libre. Il glisse le bateau entre la deuxième et la troisième feuille. Le papier touche un quai de terre. Toc. Quai Deux.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Amir compte encore. Une. Deux. Trois. Là. Un espace libre. Il glisse le bateau entre la deuxième et la troisième feuille. Le papier touche un quai de terre. Toc. Quai Deux.</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Amir compte encore. Une. Deux. Trois. Là. Un espace libre. Il glisse le bateau entre la deuxième et la troisième feuille. Le papier touche un quai de terre. Toc. Quai Deux.</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -9133,13 +9100,11 @@
       <c r="AV46" s="2" t="inlineStr"/>
       <c r="AW46" t="inlineStr">
         <is>
-          <t>narrateur|Amir sort le bateau du sac.
-narrateur|Il le pose au milieu de l'eau.
-narrateur|La voile se tient.
-narrateur|Un peu d'eau touche le papier.
-papa|Il avance.
-narrateur|Amir souffle. Ffff.
-narrateur|Le bateau part tout doux.</t>
+          <t>narrateur|Amir compte encore. Une. Deux. Trois.
+enfant-m|Là. Un espace libre.
+narrateur|Il glisse le bateau entre la deuxième et la troisième feuille.
+narrateur|Le papier touche un quai de terre. Toc.
+enfant-m|Quai Deux.</t>
         </is>
       </c>
     </row>
@@ -9166,17 +9131,17 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>À table, Amir dit : Quai Un. Quai Deux. Quai Trois. Ton bateau a visité le port. Sans déranger les choux. Le bateau sèche. Les choux, dehors, restent droits. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>À table, Amir dit : Quai Un. Quai Deux. Quai Trois. Ton bateau a visité le port. Sans déranger les choux. Le bateau sèche. Les choux, dehors, restent droits. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>À table, Amir dit : Quai Un. Quai Deux. Quai Trois. Ton bateau a visité le port. Sans déranger les choux. Le bateau sèche. Les choux, dehors, restent droits. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -9306,13 +9271,12 @@
       <c r="AV47" s="2" t="inlineStr"/>
       <c r="AW47" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir reprend le bateau.
-narrateur|Il le remet dans le sac.
-narrateur|Les bottes restent aux pieds, jusqu'à la porte.
-narrateur|On referme. Zzz.
-narrateur|Une feuille lâche la flaque.
-narrateur|L'histoire est finie.</t>
+          <t>narrateur|À table, Amir dit :
+enfant-m|Quai Un. Quai Deux. Quai Trois.
+maman|Ton bateau a visité le port.
+enfant-m|Sans déranger les choux.
+narrateur|Le bateau sèche. Les choux, dehors, restent droits.
+narrateur|À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -9339,17 +9303,17 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Amir attend. L'eau pousse tout doux. Une feuille s'écarte. Puis une autre. Le port s'ouvre. Le bateau avance tout seul jusqu'au chou.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Amir attend. L'eau pousse tout doux. Une feuille s'écarte. Puis une autre. Le port s'ouvre. Le bateau avance tout seul jusqu'au chou.</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Amir attend. L'eau pousse tout doux. Une feuille s'écarte. Puis une autre. Le port s'ouvre. Le bateau avance tout seul jusqu'au chou.</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -9479,13 +9443,10 @@
       <c r="AV48" s="2" t="inlineStr"/>
       <c r="AW48" t="inlineStr">
         <is>
-          <t>narrateur|Amir sort le bateau.
-narrateur|Il le donne à papa.
-papa|Près du bord, ensemble.
-narrateur|Papa le pose. Amir tient le sac.
-narrateur|Le bateau part.
-narrateur|Amir marche le long de l'eau.
-narrateur|Le sac est à l'épaule.</t>
+          <t>narrateur|Amir attend. L'eau pousse tout doux.
+narrateur|Une feuille s'écarte. Puis une autre.
+enfant-m|Le port s'ouvre.
+narrateur|Le bateau avance tout seul jusqu'au chou.</t>
         </is>
       </c>
     </row>
@@ -9512,17 +9473,17 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>Amir raconte : J'ai attendu. Les feuilles ont ouvert le port. Le courant a aidé. Le bateau sent encore un peu le chou. Amir rit. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>Amir raconte : J'ai attendu. Les feuilles ont ouvert le port. Le courant a aidé. Le bateau sent encore un peu le chou. Amir rit. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>Amir raconte : J'ai attendu. Les feuilles ont ouvert le port. Le courant a aidé. Le bateau sent encore un peu le chou. Amir rit. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -9652,13 +9613,11 @@
       <c r="AV49" s="2" t="inlineStr"/>
       <c r="AW49" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir reprend le bateau.
-narrateur|Il le remet dans le sac.
-narrateur|Les bottes restent aux pieds, jusqu'à la porte.
-narrateur|On referme. Zzz.
-narrateur|Une feuille lâche la flaque.
-narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir raconte :
+enfant-m|J'ai attendu. Les feuilles ont ouvert le port.
+papa|Le courant a aidé.
+narrateur|Le bateau sent encore un peu le chou. Amir rit.
+narrateur|À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -9685,17 +9644,17 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>Maman est venue jusqu'au potager. Maman, je veux jouer sans abîmer les choux. Passe entre les feuilles. Pas dessus. Amir pose le bateau dans l'espace libre. Les plants ne bougent pas. Ton port est gentil avec le jardin.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>Maman est venue jusqu'au potager. Maman, je veux jouer sans abîmer les choux. Passe entre les feuilles. Pas dessus. Amir pose le bateau dans l'espace libre. Les plants ne bougent pas. Ton port est gentil avec le jardin.</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>Maman est venue jusqu'au potager. Maman, je veux jouer sans abîmer les choux. Passe entre les feuilles. Pas dessus. Amir pose le bateau dans l'espace libre. Les plants ne bougent pas. Ton port est gentil avec le jardin.</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -9825,11 +9784,11 @@
       <c r="AV50" s="2" t="inlineStr"/>
       <c r="AW50" t="inlineStr">
         <is>
-          <t>narrateur|Amir pose d'abord le sac.
-narrateur|Il pose le bateau sur le sac.
-narrateur|Il regarde la flaque.
-narrateur|Puis il met le bateau dans l'eau.
-papa|Tu as préparé. Maintenant il flotte.</t>
+          <t>narrateur|Maman est venue jusqu'au potager.
+enfant-m|Maman, je veux jouer sans abîmer les choux.
+maman|Passe entre les feuilles. Pas dessus.
+narrateur|Amir pose le bateau dans l'espace libre. Les plants ne bougent pas.
+maman|Ton port est gentil avec le jardin.</t>
         </is>
       </c>
     </row>
@@ -9856,17 +9815,17 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>Merci d'avoir demandé. Le port est dans le jardin. On le garde. Amir pose le bateau. Maman pose la soupe. Deux voyages : l'eau, et la maison. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>Merci d'avoir demandé. Le port est dans le jardin. On le garde. Amir pose le bateau. Maman pose la soupe. Deux voyages : l'eau, et la maison. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>Merci d'avoir demandé. Le port est dans le jardin. On le garde. Amir pose le bateau. Maman pose la soupe. Deux voyages : l'eau, et la maison. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
@@ -9996,13 +9955,11 @@
       <c r="AV51" s="2" t="inlineStr"/>
       <c r="AW51" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir reprend le bateau.
-narrateur|Il le remet dans le sac.
-narrateur|Les bottes restent aux pieds, jusqu'à la porte.
-narrateur|On referme. Zzz.
-narrateur|Une feuille lâche la flaque.
-narrateur|L'histoire est finie.</t>
+          <t>maman|Merci d'avoir demandé.
+enfant-m|Le port est dans le jardin. On le garde.
+narrateur|Amir pose le bateau. Maman pose la soupe.
+narrateur|Deux voyages : l'eau, et la maison.
+narrateur|À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -10029,17 +9986,17 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Amir enfile les bottes. Ils vont près du bac à sable. Une flaque borde le bois du bac. Les bottes s'arrêtent au bord, pile. Le bateau, Amir.</t>
+          <t>Amir enfile les bottes. Elles s'arrêtent pile au bord du bac. Près du bac à sable, l'eau devient de plus en plus petite. Elle rentre dans le sol. Le bateau n'aurait plus assez d'eau. Mon chemin disparaît. Le sable boit la flaque. Amir serre le bateau. Il avait imaginé cette île.</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Amir enfile les bottes. Ils vont près du bac à sable. Une flaque borde le bois du bac. Les bottes s'arrêtent au bord, pile. Le bateau, Amir.</t>
+          <t>Amir enfile les bottes. Elles s'arrêtent pile au bord du bac. Près du bac à sable, l'eau devient de plus en plus petite. Elle rentre dans le sol. Le bateau n'aurait plus assez d'eau. Mon chemin disparaît. Le sable boit la flaque. Amir serre le bateau. Il avait imaginé cette île.</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Amir enfile les bottes. Ils vont près du bac à sable. Une flaque borde le bois du bac. Les bottes s'arrêtent au bord, pile. Le bateau, Amir.</t>
+          <t>Amir enfile les bottes. Elles s'arrêtent pile au bord du bac. Près du bac à sable, l'eau devient de plus en plus petite. Elle rentre dans le sol. Le bateau n'aurait plus assez d'eau. Mon chemin disparaît. Le sable boit la flaque. Amir serre le bateau. Il avait imaginé cette île.</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
@@ -10169,11 +10126,12 @@
       <c r="AV52" s="2" t="inlineStr"/>
       <c r="AW52" t="inlineStr">
         <is>
-          <t>narrateur|Amir enfile les bottes.
-narrateur|Ils vont près du bac à sable.
-narrateur|Une flaque borde le bois du bac.
-narrateur|Les bottes s'arrêtent au bord, pile.
-papa|Le bateau, Amir.</t>
+          <t>narrateur|Amir enfile les bottes. Elles s'arrêtent pile au bord du bac.
+narrateur|Près du bac à sable, l'eau devient de plus en plus petite.
+narrateur|Elle rentre dans le sol. Le bateau n'aurait plus assez d'eau.
+enfant-m|Mon chemin disparaît.
+papa|Le sable boit la flaque.
+narrateur|Amir serre le bateau. Il avait imaginé cette île.</t>
         </is>
       </c>
     </row>
@@ -10200,17 +10158,17 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr"/>
@@ -10228,7 +10186,7 @@
       <c r="L53" s="2" t="inlineStr"/>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>au milieu</t>
+          <t>une autre flaque</t>
         </is>
       </c>
       <c r="N53" s="2" t="inlineStr">
@@ -10238,7 +10196,7 @@
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>près du bord</t>
+          <t>sur le sable</t>
         </is>
       </c>
       <c r="P53" s="2" t="inlineStr">
@@ -10248,7 +10206,7 @@
       </c>
       <c r="Q53" s="2" t="inlineStr">
         <is>
-          <t>sur le sac</t>
+          <t>un autre bateau</t>
         </is>
       </c>
       <c r="R53" s="2" t="inlineStr">
@@ -10364,8 +10322,8 @@
       <c r="AV53" s="2" t="inlineStr"/>
       <c r="AW53" t="inlineStr">
         <is>
-          <t>narrateur|On pose le bateau…
-narrateur|Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>narrateur|Amir regarde.
+papa|Comment on fait, capitaine ?</t>
         </is>
       </c>
     </row>
@@ -10392,17 +10350,17 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Celle-ci s'en va. On prend l'autre. À côté, une flaque plus ronde tient encore. Amir y pose le bateau. Il avance. Ffff. Nouveau départ.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Celle-ci s'en va. On prend l'autre. À côté, une flaque plus ronde tient encore. Amir y pose le bateau. Il avance. Ffff. Nouveau départ.</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Celle-ci s'en va. On prend l'autre. À côté, une flaque plus ronde tient encore. Amir y pose le bateau. Il avance. Ffff. Nouveau départ.</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -10532,13 +10490,10 @@
       <c r="AV54" s="2" t="inlineStr"/>
       <c r="AW54" t="inlineStr">
         <is>
-          <t>narrateur|Amir sort le bateau du sac.
-narrateur|Il le pose au milieu de l'eau.
-narrateur|La voile se tient.
-narrateur|Un peu d'eau touche le papier.
-papa|Il avance.
-narrateur|Amir souffle. Ffff.
-narrateur|Le bateau part tout doux.</t>
+          <t>enfant-m|Celle-ci s'en va. On prend l'autre.
+narrateur|À côté, une flaque plus ronde tient encore.
+narrateur|Amir y pose le bateau. Il avance. Ffff.
+papa|Nouveau départ.</t>
         </is>
       </c>
     </row>
@@ -10565,17 +10520,17 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>La première flaque est partie. L'autre m'a emmené. Changer de chemin, ce n'est pas perdre. Amir hoche la tête. Le bateau sèche près du volet jaune. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>La première flaque est partie. L'autre m'a emmené. Changer de chemin, ce n'est pas perdre. Amir hoche la tête. Le bateau sèche près du volet jaune. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>La première flaque est partie. L'autre m'a emmené. Changer de chemin, ce n'est pas perdre. Amir hoche la tête. Le bateau sèche près du volet jaune. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -10705,13 +10660,10 @@
       <c r="AV55" s="2" t="inlineStr"/>
       <c r="AW55" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir reprend le bateau.
-narrateur|Il le remet dans le sac.
-narrateur|Les bottes restent aux pieds, jusqu'à la porte.
-narrateur|On referme. Zzz.
-narrateur|Un grain de sable reste sur le bois.
-narrateur|L'histoire est finie.</t>
+          <t>enfant-m|La première flaque est partie. L'autre m'a emmené.
+papa|Changer de chemin, ce n'est pas perdre.
+narrateur|Amir hoche la tête. Le bateau sèche près du volet jaune.
+narrateur|À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -10738,17 +10690,17 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Plus d'eau. Alors il marche. Amir pousse le bateau sur le sable humide. Une piste. Le papier glisse. Grain. Grain. Un bateau de terre, aujourd'hui.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Plus d'eau. Alors il marche. Amir pousse le bateau sur le sable humide. Une piste. Le papier glisse. Grain. Grain. Un bateau de terre, aujourd'hui.</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Plus d'eau. Alors il marche. Amir pousse le bateau sur le sable humide. Une piste. Le papier glisse. Grain. Grain. Un bateau de terre, aujourd'hui.</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -10878,13 +10830,10 @@
       <c r="AV56" s="2" t="inlineStr"/>
       <c r="AW56" t="inlineStr">
         <is>
-          <t>narrateur|Amir sort le bateau.
-narrateur|Il le donne à papa.
-papa|Près du bord, ensemble.
-narrateur|Papa le pose. Amir tient le sac.
-narrateur|Le bateau part.
-narrateur|Amir marche le long de l'eau.
-narrateur|Le sac est à l'épaule.</t>
+          <t>enfant-m|Plus d'eau. Alors il marche.
+narrateur|Amir pousse le bateau sur le sable humide. Une piste.
+narrateur|Le papier glisse. Grain. Grain.
+papa|Un bateau de terre, aujourd'hui.</t>
         </is>
       </c>
     </row>
@@ -10911,17 +10860,17 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>Aujourd'hui, mon bateau a marché. Un capitaine de sable. Un grain reste sur la cheminée rouge. Amir le souffle. Ffff. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>Aujourd'hui, mon bateau a marché. Un capitaine de sable. Un grain reste sur la cheminée rouge. Amir le souffle. Ffff. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>Aujourd'hui, mon bateau a marché. Un capitaine de sable. Un grain reste sur la cheminée rouge. Amir le souffle. Ffff. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
@@ -11051,13 +11000,10 @@
       <c r="AV57" s="2" t="inlineStr"/>
       <c r="AW57" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir reprend le bateau.
-narrateur|Il le remet dans le sac.
-narrateur|Les bottes restent aux pieds, jusqu'à la porte.
-narrateur|On referme. Zzz.
-narrateur|Un grain de sable reste sur le bois.
-narrateur|L'histoire est finie.</t>
+          <t>enfant-m|Aujourd'hui, mon bateau a marché.
+papa|Un capitaine de sable.
+narrateur|Un grain reste sur la cheminée rouge. Amir le souffle. Ffff.
+narrateur|À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -11084,17 +11030,17 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>Celui-là est trop fragile. Amir pose le bateau en papier dans le sac. On en fabrique un autre, plus solide. Avec une feuille plus épaisse, ils plient une nouvelle coque. Celui-ci, pour le sable.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>Celui-là est trop fragile. Amir pose le bateau en papier dans le sac. On en fabrique un autre, plus solide. Avec une feuille plus épaisse, ils plient une nouvelle coque. Celui-ci, pour le sable.</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>Celui-là est trop fragile. Amir pose le bateau en papier dans le sac. On en fabrique un autre, plus solide. Avec une feuille plus épaisse, ils plient une nouvelle coque. Celui-ci, pour le sable.</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -11224,11 +11170,11 @@
       <c r="AV58" s="2" t="inlineStr"/>
       <c r="AW58" t="inlineStr">
         <is>
-          <t>narrateur|Amir pose d'abord le sac.
-narrateur|Il pose le bateau sur le sac.
-narrateur|Il regarde la flaque.
-narrateur|Puis il met le bateau dans l'eau.
-papa|Tu as préparé. Maintenant il flotte.</t>
+          <t>enfant-m|Celui-là est trop fragile.
+narrateur|Amir pose le bateau en papier dans le sac.
+papa|On en fabrique un autre, plus solide.
+narrateur|Avec une feuille plus épaisse, ils plient une nouvelle coque.
+enfant-m|Celui-ci, pour le sable.</t>
         </is>
       </c>
     </row>
@@ -11255,17 +11201,17 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>Deux bateaux maintenant. L'ancien dans le sac. Le nouveau sur la table. Celui-là, pour demain. On a bien fait. Le papier fragile se repose. L'autre attend le jardin. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>Deux bateaux maintenant. L'ancien dans le sac. Le nouveau sur la table. Celui-là, pour demain. On a bien fait. Le papier fragile se repose. L'autre attend le jardin. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir reprend le bateau. Il le remet dans le sac. Les bottes restent aux pieds, jusqu'à la porte. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>Deux bateaux maintenant. L'ancien dans le sac. Le nouveau sur la table. Celui-là, pour demain. On a bien fait. Le papier fragile se repose. L'autre attend le jardin. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -11395,13 +11341,11 @@
       <c r="AV59" s="2" t="inlineStr"/>
       <c r="AW59" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir reprend le bateau.
-narrateur|Il le remet dans le sac.
-narrateur|Les bottes restent aux pieds, jusqu'à la porte.
-narrateur|On referme. Zzz.
-narrateur|Un grain de sable reste sur le bois.
-narrateur|L'histoire est finie.</t>
+          <t>narrateur|Deux bateaux maintenant. L'ancien dans le sac. Le nouveau sur la table.
+enfant-m|Celui-là, pour demain.
+papa|On a bien fait.
+narrateur|Le papier fragile se repose. L'autre attend le jardin.
+narrateur|À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -11428,17 +11372,17 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Amir met le bateau dans le sac. Toc. La voile rentre sous son doigt. Le linge est sur le radiateur. Il sent le propre. Pour tes mains, après la flaque. Amir le roule. Il le glisse près du bateau.</t>
+          <t>Amir met le bateau dans le sac. Toc. La voile rentre sous son doigt. Le linge est sur le radiateur. Il sent le propre. Pour tes mains, après l'eau. Je le prends. Le linge rejoint le bateau dans le sac.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Amir met le bateau dans le sac. Toc. La voile rentre sous son doigt. Le linge est sur le radiateur. Il sent le propre. Pour tes mains, après la flaque. Amir le roule. Il le glisse près du bateau.</t>
+          <t>Amir met le bateau dans le sac. Toc. La voile rentre sous son doigt. Le linge est sur le radiateur. Il sent le propre. Pour tes mains, après l'eau. Je le prends. Le linge rejoint le bateau dans le sac.</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Amir met le bateau dans le sac. Toc. La voile rentre sous son doigt. Le linge est sur le radiateur. Il sent le propre. Pour tes mains, après la flaque. Amir le roule. Il le glisse près du bateau.</t>
+          <t>Amir met le bateau dans le sac. Toc. La voile rentre sous son doigt. Le linge est sur le radiateur. Il sent le propre. Pour tes mains, après l'eau. Je le prends. Le linge rejoint le bateau dans le sac.</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr"/>
@@ -11568,13 +11512,12 @@
       <c r="AV60" s="2" t="inlineStr"/>
       <c r="AW60" t="inlineStr">
         <is>
-          <t>narrateur|Amir met le bateau dans le sac.
-narrateur|Toc. La voile rentre sous son doigt.
-narrateur|Le linge est sur le radiateur.
-narrateur|Il sent le propre.
-maman|Pour tes mains, après la flaque.
-narrateur|Amir le roule.
-narrateur|Il le glisse près du bateau.</t>
+          <t>narrateur|Amir met le bateau dans le sac. Toc.
+narrateur|La voile rentre sous son doigt.
+narrateur|Le linge est sur le radiateur. Il sent le propre.
+maman|Pour tes mains, après l'eau.
+enfant-m|Je le prends.
+narrateur|Le linge rejoint le bateau dans le sac.</t>
         </is>
       </c>
     </row>
@@ -11616,12 +11559,12 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>le sac</t>
+          <t>dans le sac</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>le sac | dans le sac</t>
+          <t>sac|le sac|dans le sac</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
@@ -11788,17 +11731,17 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Le linge est dans le sac. Le bateau aussi. On y va ? Oui. Vers la flaque.</t>
+          <t>Le linge est dans le sac. Le bateau aussi. On ouvre la porte ? Oui. Le voyage commence.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Le linge est dans le sac. Le bateau aussi. On y va ? Oui. Vers la flaque.</t>
+          <t>Le linge est dans le sac. Le bateau aussi. On ouvre la porte ? Oui. Le voyage commence.</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Le linge est dans le sac. Le bateau aussi. On y va ? Oui. Vers la flaque.</t>
+          <t>Le linge est dans le sac. Le bateau aussi. On ouvre la porte ? Oui. Le voyage commence.</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr"/>
@@ -11932,10 +11875,9 @@
       </c>
       <c r="AW62" t="inlineStr">
         <is>
-          <t>narrateur|Le linge est dans le sac.
-narrateur|Le bateau aussi.
-enfant-m|On y va ?
-papa|Oui. Vers la flaque.</t>
+          <t>narrateur|Le linge est dans le sac. Le bateau aussi.
+papa|On ouvre la porte ?
+enfant-m|Oui. Le voyage commence.</t>
         </is>
       </c>
     </row>
@@ -11962,17 +11904,17 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Quelle flaque ? Sous la gouttière, près du potager, ou près du bac.</t>
+          <t>Dehors, l'eau a fait trois chemins. La rivière de la gouttière. Le port des choux. L'île du bac. Où commence le voyage, capitaine ?</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Quelle flaque ? Sous la gouttière, près du potager, ou près du bac.</t>
+          <t>Dehors, l'eau a fait trois chemins. La rivière de la gouttière. Le port des choux. L'île du bac. Où commence le voyage, capitaine ?</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Quelle flaque ? Sous la gouttière, près du potager, ou près du bac.</t>
+          <t>Dehors, l'eau a fait trois chemins. La rivière de la gouttière. Le port des choux. L'île du bac. Où commence le voyage, capitaine ?</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr"/>
@@ -11990,7 +11932,7 @@
       <c r="L63" s="2" t="inlineStr"/>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>sous la gouttière</t>
+          <t>la rivière de la gouttière</t>
         </is>
       </c>
       <c r="N63" s="2" t="inlineStr">
@@ -12000,7 +11942,7 @@
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>près du potager</t>
+          <t>le port des choux</t>
         </is>
       </c>
       <c r="P63" s="2" t="inlineStr">
@@ -12010,7 +11952,7 @@
       </c>
       <c r="Q63" s="2" t="inlineStr">
         <is>
-          <t>près du bac</t>
+          <t>l'île du bac</t>
         </is>
       </c>
       <c r="R63" s="2" t="inlineStr">
@@ -12126,8 +12068,9 @@
       <c r="AV63" s="2" t="inlineStr"/>
       <c r="AW63" t="inlineStr">
         <is>
-          <t>narrateur|Quelle flaque ?
-narrateur|Sous la gouttière, près du potager, ou près du bac.</t>
+          <t>narrateur|Dehors, l'eau a fait trois chemins.
+narrateur|La rivière de la gouttière. Le port des choux. L'île du bac.
+papa|Où commence le voyage, capitaine ?</t>
         </is>
       </c>
     </row>
@@ -12154,17 +12097,17 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Amir porte le sac. Le linge est dedans. Sous la gouttière, une flaque ronde. Une goutte tombe. Plic. L'eau tremble. Le bateau, maintenant.</t>
+          <t>Amir porte le sac. Le linge est dedans, au chaud. Sous la gouttière, l'eau tremble. Plic. Ploc. Une grosse feuille barre le passage. La rivière est fermée. Le bateau ne peut pas passer. Amir s'accroupit. La feuille ne bouge presque pas.</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Amir porte le sac. Le linge est dedans. Sous la gouttière, une flaque ronde. Une goutte tombe. Plic. L'eau tremble. Le bateau, maintenant.</t>
+          <t>Amir porte le sac. Le linge est dedans, au chaud. Sous la gouttière, l'eau tremble. Plic. Ploc. Une grosse feuille barre le passage. La rivière est fermée. Le bateau ne peut pas passer. Amir s'accroupit. La feuille ne bouge presque pas.</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Amir porte le sac. Le linge est dedans. Sous la gouttière, une flaque ronde. Une goutte tombe. Plic. L'eau tremble. Le bateau, maintenant.</t>
+          <t>Amir porte le sac. Le linge est dedans, au chaud. Sous la gouttière, l'eau tremble. Plic. Ploc. Une grosse feuille barre le passage. La rivière est fermée. Le bateau ne peut pas passer. Amir s'accroupit. La feuille ne bouge presque pas.</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr"/>
@@ -12294,11 +12237,12 @@
       <c r="AV64" s="2" t="inlineStr"/>
       <c r="AW64" t="inlineStr">
         <is>
-          <t>narrateur|Amir porte le sac. Le linge est dedans.
-narrateur|Sous la gouttière, une flaque ronde.
-narrateur|Une goutte tombe. Plic.
-narrateur|L'eau tremble.
-papa|Le bateau, maintenant.</t>
+          <t>narrateur|Amir porte le sac. Le linge est dedans, au chaud.
+narrateur|Sous la gouttière, l'eau tremble. Plic. Ploc.
+narrateur|Une grosse feuille barre le passage.
+enfant-m|La rivière est fermée.
+papa|Le bateau ne peut pas passer.
+narrateur|Amir s'accroupit. La feuille ne bouge presque pas.</t>
         </is>
       </c>
     </row>
@@ -12325,17 +12269,17 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr"/>
@@ -12353,7 +12297,7 @@
       <c r="L65" s="2" t="inlineStr"/>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>au milieu</t>
+          <t>attendre les gouttes</t>
         </is>
       </c>
       <c r="N65" s="2" t="inlineStr">
@@ -12363,7 +12307,7 @@
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>près du bord</t>
+          <t>appeler papa</t>
         </is>
       </c>
       <c r="P65" s="2" t="inlineStr">
@@ -12373,7 +12317,7 @@
       </c>
       <c r="Q65" s="2" t="inlineStr">
         <is>
-          <t>sur le sac</t>
+          <t>changer de départ</t>
         </is>
       </c>
       <c r="R65" s="2" t="inlineStr">
@@ -12489,8 +12433,8 @@
       <c r="AV65" s="2" t="inlineStr"/>
       <c r="AW65" t="inlineStr">
         <is>
-          <t>narrateur|On pose le bateau…
-narrateur|Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>narrateur|Amir regarde.
+papa|Comment on fait, capitaine ?</t>
         </is>
       </c>
     </row>
@@ -12517,17 +12461,17 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Amir s'accroupit près de la feuille. J'attends encore un peu. Une goutte. Plic. La feuille bouge à peine. Une deuxième. Ploc. La feuille tourne. Une troisième. Plouf. La feuille ouvre un passage. La rivière est libre !</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Amir s'accroupit près de la feuille. J'attends encore un peu. Une goutte. Plic. La feuille bouge à peine. Une deuxième. Ploc. La feuille tourne. Une troisième. Plouf. La feuille ouvre un passage. La rivière est libre !</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Amir s'accroupit près de la feuille. J'attends encore un peu. Une goutte. Plic. La feuille bouge à peine. Une deuxième. Ploc. La feuille tourne. Une troisième. Plouf. La feuille ouvre un passage. La rivière est libre !</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -12657,13 +12601,12 @@
       <c r="AV66" s="2" t="inlineStr"/>
       <c r="AW66" t="inlineStr">
         <is>
-          <t>narrateur|Amir sort le bateau du sac.
-narrateur|Il le pose au milieu de l'eau.
-narrateur|La voile se tient.
-narrateur|Un peu d'eau touche le papier.
-papa|Il avance.
-narrateur|Amir souffle. Ffff.
-narrateur|Le bateau part tout doux.</t>
+          <t>narrateur|Amir s'accroupit près de la feuille.
+enfant-m|J'attends encore un peu.
+narrateur|Une goutte. Plic. La feuille bouge à peine.
+narrateur|Une deuxième. Ploc. La feuille tourne.
+narrateur|Une troisième. Plouf. La feuille ouvre un passage.
+enfant-m|La rivière est libre !</t>
         </is>
       </c>
     </row>
@@ -12690,17 +12633,17 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>De retour, Amir pose le bateau sur le petit linge. Alors, capitaine, jusqu'où es-tu allé ? Très loin. J'ai attendu trois gouttes. C'est vraiment loin. Une dernière goutte, dehors. Plic. Sur le linge, le bateau attend déjà le prochain voyage. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>De retour, Amir pose le bateau sur le petit linge. Alors, capitaine, jusqu'où es-tu allé ? Très loin. J'ai attendu trois gouttes. C'est vraiment loin. Une dernière goutte, dehors. Plic. Sur le linge, le bateau attend déjà le prochain voyage. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>De retour, Amir pose le bateau sur le petit linge. Alors, capitaine, jusqu'où es-tu allé ? Très loin. J'ai attendu trois gouttes. C'est vraiment loin. Une dernière goutte, dehors. Plic. Sur le linge, le bateau attend déjà le prochain voyage. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
@@ -12830,13 +12773,13 @@
       <c r="AV67" s="2" t="inlineStr"/>
       <c r="AW67" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir sèche ses doigts avec le linge.
-narrateur|Il remet le bateau dans le sac.
-narrateur|Le linge rentre aussi.
-narrateur|On referme. Zzz.
-narrateur|La gouttière fait un dernier plic.
-narrateur|L'histoire est finie.</t>
+          <t>narrateur|De retour, Amir pose le bateau sur le petit linge.
+papa|Alors, capitaine, jusqu'où es-tu allé ?
+enfant-m|Très loin. J'ai attendu trois gouttes.
+papa|C'est vraiment loin.
+narrateur|Une dernière goutte, dehors. Plic.
+narrateur|Sur le linge, le bateau attend déjà le prochain voyage.
+narrateur|Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -12863,17 +12806,17 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Papa, tu peux bouger la feuille ? On la pousse ensemble. Tout doux. Papa soulève le bord. Amir tient le bateau. La feuille glisse. L'eau circule. À toi, capitaine.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Papa, tu peux bouger la feuille ? On la pousse ensemble. Tout doux. Papa soulève le bord. Amir tient le bateau. La feuille glisse. L'eau circule. À toi, capitaine.</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Papa, tu peux bouger la feuille ? On la pousse ensemble. Tout doux. Papa soulève le bord. Amir tient le bateau. La feuille glisse. L'eau circule. À toi, capitaine.</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -13003,13 +12946,11 @@
       <c r="AV68" s="2" t="inlineStr"/>
       <c r="AW68" t="inlineStr">
         <is>
-          <t>narrateur|Amir sort le bateau.
-narrateur|Il le donne à papa.
-papa|Près du bord, ensemble.
-narrateur|Papa le pose. Amir tient le sac.
-narrateur|Le bateau part.
-narrateur|Amir marche le long de l'eau.
-narrateur|Le sac est à l'épaule.</t>
+          <t>enfant-m|Papa, tu peux bouger la feuille ?
+papa|On la pousse ensemble. Tout doux.
+narrateur|Papa soulève le bord. Amir tient le bateau.
+narrateur|La feuille glisse. L'eau circule.
+papa|À toi, capitaine.</t>
         </is>
       </c>
     </row>
@@ -13036,17 +12977,17 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>Dans la maison, Amir pose le bateau près de la fenêtre. On a poussé la feuille ensemble. Oui. La rivière a dit oui. Papa reprend sa table. Amir regarde le jardin. La gouttière fait encore un tout petit plic. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>Dans la maison, Amir pose le bateau près de la fenêtre. On a poussé la feuille ensemble. Oui. La rivière a dit oui. Papa reprend sa table. Amir regarde le jardin. La gouttière fait encore un tout petit plic. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>Dans la maison, Amir pose le bateau près de la fenêtre. On a poussé la feuille ensemble. Oui. La rivière a dit oui. Papa reprend sa table. Amir regarde le jardin. La gouttière fait encore un tout petit plic. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -13176,13 +13117,12 @@
       <c r="AV69" s="2" t="inlineStr"/>
       <c r="AW69" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir sèche ses doigts avec le linge.
-narrateur|Il remet le bateau dans le sac.
-narrateur|Le linge rentre aussi.
-narrateur|On referme. Zzz.
-narrateur|La gouttière fait un dernier plic.
-narrateur|L'histoire est finie.</t>
+          <t>narrateur|Dans la maison, Amir pose le bateau près de la fenêtre.
+papa|On a poussé la feuille ensemble.
+enfant-m|Oui. La rivière a dit oui.
+narrateur|Papa reprend sa table. Amir regarde le jardin.
+narrateur|La gouttière fait encore un tout petit plic.
+narrateur|Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -13209,17 +13149,17 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>On part d'ici, plus loin. Amir pose le bateau après la feuille, là où l'eau court déjà. Un petit courant emmène le papier sous une brindille. Une autre rivière !</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>On part d'ici, plus loin. Amir pose le bateau après la feuille, là où l'eau court déjà. Un petit courant emmène le papier sous une brindille. Une autre rivière !</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>On part d'ici, plus loin. Amir pose le bateau après la feuille, là où l'eau court déjà. Un petit courant emmène le papier sous une brindille. Une autre rivière !</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
@@ -13349,11 +13289,10 @@
       <c r="AV70" s="2" t="inlineStr"/>
       <c r="AW70" t="inlineStr">
         <is>
-          <t>narrateur|Amir pose d'abord le sac.
-narrateur|Il pose le bateau sur le sac.
-narrateur|Il regarde la flaque.
-narrateur|Puis il met le bateau dans l'eau.
-papa|Tu as préparé. Maintenant il flotte.</t>
+          <t>enfant-m|On part d'ici, plus loin.
+narrateur|Amir pose le bateau après la feuille, là où l'eau court déjà.
+narrateur|Un petit courant emmène le papier sous une brindille.
+enfant-m|Une autre rivière !</t>
         </is>
       </c>
     </row>
@@ -13380,17 +13319,17 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>Amir rentre. Le bateau a une brindille collée à la voile. On a trouvé un autre courant. Le bateau a choisi. Amir sourit. Le sac attend près de la porte. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>Amir rentre. Le bateau a une brindille collée à la voile. On a trouvé un autre courant. Le bateau a choisi. Amir sourit. Le sac attend près de la porte. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. La gouttière fait un dernier plic. L'histoire est finie.</t>
+          <t>Amir rentre. Le bateau a une brindille collée à la voile. On a trouvé un autre courant. Le bateau a choisi. Amir sourit. Le sac attend près de la porte. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr"/>
@@ -13520,13 +13459,11 @@
       <c r="AV71" s="2" t="inlineStr"/>
       <c r="AW71" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir sèche ses doigts avec le linge.
-narrateur|Il remet le bateau dans le sac.
-narrateur|Le linge rentre aussi.
-narrateur|On referme. Zzz.
-narrateur|La gouttière fait un dernier plic.
-narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir rentre. Le bateau a une brindille collée à la voile.
+enfant-m|On a trouvé un autre courant.
+papa|Le bateau a choisi.
+narrateur|Amir sourit. Le sac attend près de la porte.
+narrateur|Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -13553,17 +13490,17 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Amir porte le sac avec le linge. Ils vont près du potager. La flaque est ronde, entre deux choux. L'eau tremble un peu. Le bateau, Amir.</t>
+          <t>Amir porte le sac. Le linge sent encore le radiateur. Entre deux choux, une flaque ronde. Comme un port. Trois petites feuilles flottent devant l'entrée. Les bateaux n'arrivent pas à accoster. Il y a trois feuilles. Amir compte. Une. Deux. Trois.</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Amir porte le sac avec le linge. Ils vont près du potager. La flaque est ronde, entre deux choux. L'eau tremble un peu. Le bateau, Amir.</t>
+          <t>Amir porte le sac. Le linge sent encore le radiateur. Entre deux choux, une flaque ronde. Comme un port. Trois petites feuilles flottent devant l'entrée. Les bateaux n'arrivent pas à accoster. Il y a trois feuilles. Amir compte. Une. Deux. Trois.</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Amir porte le sac avec le linge. Ils vont près du potager. La flaque est ronde, entre deux choux. L'eau tremble un peu. Le bateau, Amir.</t>
+          <t>Amir porte le sac. Le linge sent encore le radiateur. Entre deux choux, une flaque ronde. Comme un port. Trois petites feuilles flottent devant l'entrée. Les bateaux n'arrivent pas à accoster. Il y a trois feuilles. Amir compte. Une. Deux. Trois.</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
@@ -13693,11 +13630,12 @@
       <c r="AV72" s="2" t="inlineStr"/>
       <c r="AW72" t="inlineStr">
         <is>
-          <t>narrateur|Amir porte le sac avec le linge.
-narrateur|Ils vont près du potager.
-narrateur|La flaque est ronde, entre deux choux.
-narrateur|L'eau tremble un peu.
-maman|Le bateau, Amir.</t>
+          <t>narrateur|Amir porte le sac. Le linge sent encore le radiateur.
+narrateur|Entre deux choux, une flaque ronde. Comme un port.
+narrateur|Trois petites feuilles flottent devant l'entrée.
+enfant-m|Les bateaux n'arrivent pas à accoster.
+papa|Il y a trois feuilles.
+narrateur|Amir compte. Une. Deux. Trois.</t>
         </is>
       </c>
     </row>
@@ -13724,17 +13662,17 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr"/>
@@ -13752,7 +13690,7 @@
       <c r="L73" s="2" t="inlineStr"/>
       <c r="M73" s="2" t="inlineStr">
         <is>
-          <t>au milieu</t>
+          <t>compter les feuilles</t>
         </is>
       </c>
       <c r="N73" s="2" t="inlineStr">
@@ -13762,7 +13700,7 @@
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>près du bord</t>
+          <t>attendre le courant</t>
         </is>
       </c>
       <c r="P73" s="2" t="inlineStr">
@@ -13772,7 +13710,7 @@
       </c>
       <c r="Q73" s="2" t="inlineStr">
         <is>
-          <t>sur le sac</t>
+          <t>demander à maman</t>
         </is>
       </c>
       <c r="R73" s="2" t="inlineStr">
@@ -13888,8 +13826,8 @@
       <c r="AV73" s="2" t="inlineStr"/>
       <c r="AW73" t="inlineStr">
         <is>
-          <t>narrateur|On pose le bateau…
-narrateur|Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>narrateur|Amir regarde.
+papa|Comment on fait, capitaine ?</t>
         </is>
       </c>
     </row>
@@ -13916,17 +13854,17 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Amir compte encore. Une. Deux. Trois. Là. Un espace libre. Il glisse le bateau entre la deuxième et la troisième feuille. Le papier touche un quai de terre. Toc. Quai Deux.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Amir compte encore. Une. Deux. Trois. Là. Un espace libre. Il glisse le bateau entre la deuxième et la troisième feuille. Le papier touche un quai de terre. Toc. Quai Deux.</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Amir compte encore. Une. Deux. Trois. Là. Un espace libre. Il glisse le bateau entre la deuxième et la troisième feuille. Le papier touche un quai de terre. Toc. Quai Deux.</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
@@ -14056,13 +13994,11 @@
       <c r="AV74" s="2" t="inlineStr"/>
       <c r="AW74" t="inlineStr">
         <is>
-          <t>narrateur|Amir sort le bateau du sac.
-narrateur|Il le pose au milieu de l'eau.
-narrateur|La voile se tient.
-narrateur|Un peu d'eau touche le papier.
-papa|Il avance.
-narrateur|Amir souffle. Ffff.
-narrateur|Le bateau part tout doux.</t>
+          <t>narrateur|Amir compte encore. Une. Deux. Trois.
+enfant-m|Là. Un espace libre.
+narrateur|Il glisse le bateau entre la deuxième et la troisième feuille.
+narrateur|Le papier touche un quai de terre. Toc.
+enfant-m|Quai Deux.</t>
         </is>
       </c>
     </row>
@@ -14089,17 +14025,17 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>À table, Amir dit : Quai Un. Quai Deux. Quai Trois. Ton bateau a visité le port. Sans déranger les choux. Le bateau sèche. Les choux, dehors, restent droits. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>À table, Amir dit : Quai Un. Quai Deux. Quai Trois. Ton bateau a visité le port. Sans déranger les choux. Le bateau sèche. Les choux, dehors, restent droits. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>À table, Amir dit : Quai Un. Quai Deux. Quai Trois. Ton bateau a visité le port. Sans déranger les choux. Le bateau sèche. Les choux, dehors, restent droits. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
@@ -14229,13 +14165,12 @@
       <c r="AV75" s="2" t="inlineStr"/>
       <c r="AW75" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir sèche ses doigts avec le linge.
-narrateur|Il remet le bateau dans le sac.
-narrateur|Le linge rentre aussi.
-narrateur|On referme. Zzz.
-narrateur|Une feuille lâche la flaque.
-narrateur|L'histoire est finie.</t>
+          <t>narrateur|À table, Amir dit :
+enfant-m|Quai Un. Quai Deux. Quai Trois.
+maman|Ton bateau a visité le port.
+enfant-m|Sans déranger les choux.
+narrateur|Le bateau sèche. Les choux, dehors, restent droits.
+narrateur|Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -14262,17 +14197,17 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Amir attend. L'eau pousse tout doux. Une feuille s'écarte. Puis une autre. Le port s'ouvre. Le bateau avance tout seul jusqu'au chou.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Amir attend. L'eau pousse tout doux. Une feuille s'écarte. Puis une autre. Le port s'ouvre. Le bateau avance tout seul jusqu'au chou.</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Amir attend. L'eau pousse tout doux. Une feuille s'écarte. Puis une autre. Le port s'ouvre. Le bateau avance tout seul jusqu'au chou.</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -14402,13 +14337,10 @@
       <c r="AV76" s="2" t="inlineStr"/>
       <c r="AW76" t="inlineStr">
         <is>
-          <t>narrateur|Amir sort le bateau.
-narrateur|Il le donne à papa.
-papa|Près du bord, ensemble.
-narrateur|Papa le pose. Amir tient le sac.
-narrateur|Le bateau part.
-narrateur|Amir marche le long de l'eau.
-narrateur|Le sac est à l'épaule.</t>
+          <t>narrateur|Amir attend. L'eau pousse tout doux.
+narrateur|Une feuille s'écarte. Puis une autre.
+enfant-m|Le port s'ouvre.
+narrateur|Le bateau avance tout seul jusqu'au chou.</t>
         </is>
       </c>
     </row>
@@ -14435,17 +14367,17 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>Amir raconte : J'ai attendu. Les feuilles ont ouvert le port. Le courant a aidé. Le bateau sent encore un peu le chou. Amir rit. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>Amir raconte : J'ai attendu. Les feuilles ont ouvert le port. Le courant a aidé. Le bateau sent encore un peu le chou. Amir rit. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>Amir raconte : J'ai attendu. Les feuilles ont ouvert le port. Le courant a aidé. Le bateau sent encore un peu le chou. Amir rit. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr"/>
@@ -14575,13 +14507,11 @@
       <c r="AV77" s="2" t="inlineStr"/>
       <c r="AW77" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir sèche ses doigts avec le linge.
-narrateur|Il remet le bateau dans le sac.
-narrateur|Le linge rentre aussi.
-narrateur|On referme. Zzz.
-narrateur|Une feuille lâche la flaque.
-narrateur|L'histoire est finie.</t>
+          <t>narrateur|Amir raconte :
+enfant-m|J'ai attendu. Les feuilles ont ouvert le port.
+papa|Le courant a aidé.
+narrateur|Le bateau sent encore un peu le chou. Amir rit.
+narrateur|Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -14608,17 +14538,17 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>Maman est venue jusqu'au potager. Maman, je veux jouer sans abîmer les choux. Passe entre les feuilles. Pas dessus. Amir pose le bateau dans l'espace libre. Les plants ne bougent pas. Ton port est gentil avec le jardin.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>Maman est venue jusqu'au potager. Maman, je veux jouer sans abîmer les choux. Passe entre les feuilles. Pas dessus. Amir pose le bateau dans l'espace libre. Les plants ne bougent pas. Ton port est gentil avec le jardin.</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>Maman est venue jusqu'au potager. Maman, je veux jouer sans abîmer les choux. Passe entre les feuilles. Pas dessus. Amir pose le bateau dans l'espace libre. Les plants ne bougent pas. Ton port est gentil avec le jardin.</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
@@ -14748,11 +14678,11 @@
       <c r="AV78" s="2" t="inlineStr"/>
       <c r="AW78" t="inlineStr">
         <is>
-          <t>narrateur|Amir pose d'abord le sac.
-narrateur|Il pose le bateau sur le sac.
-narrateur|Il regarde la flaque.
-narrateur|Puis il met le bateau dans l'eau.
-papa|Tu as préparé. Maintenant il flotte.</t>
+          <t>narrateur|Maman est venue jusqu'au potager.
+enfant-m|Maman, je veux jouer sans abîmer les choux.
+maman|Passe entre les feuilles. Pas dessus.
+narrateur|Amir pose le bateau dans l'espace libre. Les plants ne bougent pas.
+maman|Ton port est gentil avec le jardin.</t>
         </is>
       </c>
     </row>
@@ -14779,17 +14709,17 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>Merci d'avoir demandé. Le port est dans le jardin. On le garde. Amir pose le bateau. Maman pose la soupe. Deux voyages : l'eau, et la maison. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>Merci d'avoir demandé. Le port est dans le jardin. On le garde. Amir pose le bateau. Maman pose la soupe. Deux voyages : l'eau, et la maison. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Une feuille lâche la flaque. L'histoire est finie.</t>
+          <t>Merci d'avoir demandé. Le port est dans le jardin. On le garde. Amir pose le bateau. Maman pose la soupe. Deux voyages : l'eau, et la maison. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr"/>
@@ -14919,13 +14849,11 @@
       <c r="AV79" s="2" t="inlineStr"/>
       <c r="AW79" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir sèche ses doigts avec le linge.
-narrateur|Il remet le bateau dans le sac.
-narrateur|Le linge rentre aussi.
-narrateur|On referme. Zzz.
-narrateur|Une feuille lâche la flaque.
-narrateur|L'histoire est finie.</t>
+          <t>maman|Merci d'avoir demandé.
+enfant-m|Le port est dans le jardin. On le garde.
+narrateur|Amir pose le bateau. Maman pose la soupe.
+narrateur|Deux voyages : l'eau, et la maison.
+narrateur|Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -14952,17 +14880,17 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Amir porte le sac avec le linge. Ils vont près du bac à sable. Une flaque borde le bois du bac. Un peu de sable brille au fond. Le bateau, Amir.</t>
+          <t>Amir porte le sac. Le linge attend les mains mouillées. Près du bac à sable, l'eau devient de plus en plus petite. Elle rentre dans le sol. Le bateau n'aurait plus assez d'eau. Mon chemin disparaît. Le sable boit la flaque. Amir serre le bateau. Il avait imaginé cette île.</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Amir porte le sac avec le linge. Ils vont près du bac à sable. Une flaque borde le bois du bac. Un peu de sable brille au fond. Le bateau, Amir.</t>
+          <t>Amir porte le sac. Le linge attend les mains mouillées. Près du bac à sable, l'eau devient de plus en plus petite. Elle rentre dans le sol. Le bateau n'aurait plus assez d'eau. Mon chemin disparaît. Le sable boit la flaque. Amir serre le bateau. Il avait imaginé cette île.</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Amir porte le sac avec le linge. Ils vont près du bac à sable. Une flaque borde le bois du bac. Un peu de sable brille au fond. Le bateau, Amir.</t>
+          <t>Amir porte le sac. Le linge attend les mains mouillées. Près du bac à sable, l'eau devient de plus en plus petite. Elle rentre dans le sol. Le bateau n'aurait plus assez d'eau. Mon chemin disparaît. Le sable boit la flaque. Amir serre le bateau. Il avait imaginé cette île.</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr"/>
@@ -15092,11 +15020,12 @@
       <c r="AV80" s="2" t="inlineStr"/>
       <c r="AW80" t="inlineStr">
         <is>
-          <t>narrateur|Amir porte le sac avec le linge.
-narrateur|Ils vont près du bac à sable.
-narrateur|Une flaque borde le bois du bac.
-narrateur|Un peu de sable brille au fond.
-papa|Le bateau, Amir.</t>
+          <t>narrateur|Amir porte le sac. Le linge attend les mains mouillées.
+narrateur|Près du bac à sable, l'eau devient de plus en plus petite.
+narrateur|Elle rentre dans le sol. Le bateau n'aurait plus assez d'eau.
+enfant-m|Mon chemin disparaît.
+papa|Le sable boit la flaque.
+narrateur|Amir serre le bateau. Il avait imaginé cette île.</t>
         </is>
       </c>
     </row>
@@ -15123,17 +15052,17 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>On pose le bateau… Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>Amir regarde. Comment on fait, capitaine ?</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr"/>
@@ -15151,7 +15080,7 @@
       <c r="L81" s="2" t="inlineStr"/>
       <c r="M81" s="2" t="inlineStr">
         <is>
-          <t>au milieu</t>
+          <t>une autre flaque</t>
         </is>
       </c>
       <c r="N81" s="2" t="inlineStr">
@@ -15161,7 +15090,7 @@
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>près du bord</t>
+          <t>sur le sable</t>
         </is>
       </c>
       <c r="P81" s="2" t="inlineStr">
@@ -15171,7 +15100,7 @@
       </c>
       <c r="Q81" s="2" t="inlineStr">
         <is>
-          <t>sur le sac</t>
+          <t>un autre bateau</t>
         </is>
       </c>
       <c r="R81" s="2" t="inlineStr">
@@ -15287,8 +15216,8 @@
       <c r="AV81" s="2" t="inlineStr"/>
       <c r="AW81" t="inlineStr">
         <is>
-          <t>narrateur|On pose le bateau…
-narrateur|Au milieu de l'eau, près du bord, ou d'abord sur le sac.</t>
+          <t>narrateur|Amir regarde.
+papa|Comment on fait, capitaine ?</t>
         </is>
       </c>
     </row>
@@ -15315,17 +15244,17 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Celle-ci s'en va. On prend l'autre. À côté, une flaque plus ronde tient encore. Amir y pose le bateau. Il avance. Ffff. Nouveau départ.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Celle-ci s'en va. On prend l'autre. À côté, une flaque plus ronde tient encore. Amir y pose le bateau. Il avance. Ffff. Nouveau départ.</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau du sac. Il le pose au milieu de l'eau. La voile se tient. Un peu d'eau touche le papier. Il avance. Amir souffle. Ffff. Le bateau part tout doux.</t>
+          <t>Celle-ci s'en va. On prend l'autre. À côté, une flaque plus ronde tient encore. Amir y pose le bateau. Il avance. Ffff. Nouveau départ.</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr"/>
@@ -15455,13 +15384,10 @@
       <c r="AV82" s="2" t="inlineStr"/>
       <c r="AW82" t="inlineStr">
         <is>
-          <t>narrateur|Amir sort le bateau du sac.
-narrateur|Il le pose au milieu de l'eau.
-narrateur|La voile se tient.
-narrateur|Un peu d'eau touche le papier.
-papa|Il avance.
-narrateur|Amir souffle. Ffff.
-narrateur|Le bateau part tout doux.</t>
+          <t>enfant-m|Celle-ci s'en va. On prend l'autre.
+narrateur|À côté, une flaque plus ronde tient encore.
+narrateur|Amir y pose le bateau. Il avance. Ffff.
+papa|Nouveau départ.</t>
         </is>
       </c>
     </row>
@@ -15488,17 +15414,17 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>La première flaque est partie. L'autre m'a emmené. Changer de chemin, ce n'est pas perdre. Amir hoche la tête. Le bateau sèche près du volet jaune. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>La première flaque est partie. L'autre m'a emmené. Changer de chemin, ce n'est pas perdre. Amir hoche la tête. Le bateau sèche près du volet jaune. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>La première flaque est partie. L'autre m'a emmené. Changer de chemin, ce n'est pas perdre. Amir hoche la tête. Le bateau sèche près du volet jaune. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -15628,13 +15554,10 @@
       <c r="AV83" s="2" t="inlineStr"/>
       <c r="AW83" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir sèche ses doigts avec le linge.
-narrateur|Il remet le bateau dans le sac.
-narrateur|Le linge rentre aussi.
-narrateur|On referme. Zzz.
-narrateur|Un grain de sable reste sur le bois.
-narrateur|L'histoire est finie.</t>
+          <t>enfant-m|La première flaque est partie. L'autre m'a emmené.
+papa|Changer de chemin, ce n'est pas perdre.
+narrateur|Amir hoche la tête. Le bateau sèche près du volet jaune.
+narrateur|Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -15661,17 +15584,17 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Plus d'eau. Alors il marche. Amir pousse le bateau sur le sable humide. Une piste. Le papier glisse. Grain. Grain. Un bateau de terre, aujourd'hui.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Plus d'eau. Alors il marche. Amir pousse le bateau sur le sable humide. Une piste. Le papier glisse. Grain. Grain. Un bateau de terre, aujourd'hui.</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Amir sort le bateau. Il le donne à papa. Près du bord, ensemble. Papa le pose. Amir tient le sac. Le bateau part. Amir marche le long de l'eau. Le sac est à l'épaule.</t>
+          <t>Plus d'eau. Alors il marche. Amir pousse le bateau sur le sable humide. Une piste. Le papier glisse. Grain. Grain. Un bateau de terre, aujourd'hui.</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
@@ -15801,13 +15724,10 @@
       <c r="AV84" s="2" t="inlineStr"/>
       <c r="AW84" t="inlineStr">
         <is>
-          <t>narrateur|Amir sort le bateau.
-narrateur|Il le donne à papa.
-papa|Près du bord, ensemble.
-narrateur|Papa le pose. Amir tient le sac.
-narrateur|Le bateau part.
-narrateur|Amir marche le long de l'eau.
-narrateur|Le sac est à l'épaule.</t>
+          <t>enfant-m|Plus d'eau. Alors il marche.
+narrateur|Amir pousse le bateau sur le sable humide. Une piste.
+narrateur|Le papier glisse. Grain. Grain.
+papa|Un bateau de terre, aujourd'hui.</t>
         </is>
       </c>
     </row>
@@ -15834,17 +15754,17 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>Aujourd'hui, mon bateau a marché. Un capitaine de sable. Un grain reste sur la cheminée rouge. Amir le souffle. Ffff. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>Aujourd'hui, mon bateau a marché. Un capitaine de sable. Un grain reste sur la cheminée rouge. Amir le souffle. Ffff. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>Aujourd'hui, mon bateau a marché. Un capitaine de sable. Un grain reste sur la cheminée rouge. Amir le souffle. Ffff. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr"/>
@@ -15974,13 +15894,10 @@
       <c r="AV85" s="2" t="inlineStr"/>
       <c r="AW85" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir sèche ses doigts avec le linge.
-narrateur|Il remet le bateau dans le sac.
-narrateur|Le linge rentre aussi.
-narrateur|On referme. Zzz.
-narrateur|Un grain de sable reste sur le bois.
-narrateur|L'histoire est finie.</t>
+          <t>enfant-m|Aujourd'hui, mon bateau a marché.
+papa|Un capitaine de sable.
+narrateur|Un grain reste sur la cheminée rouge. Amir le souffle. Ffff.
+narrateur|Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -16007,17 +15924,17 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>Celui-là est trop fragile. Amir pose le bateau en papier dans le sac. On en fabrique un autre, plus solide. Avec une feuille plus épaisse, ils plient une nouvelle coque. Celui-ci, pour le sable.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>Celui-là est trop fragile. Amir pose le bateau en papier dans le sac. On en fabrique un autre, plus solide. Avec une feuille plus épaisse, ils plient une nouvelle coque. Celui-ci, pour le sable.</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Amir pose d'abord le sac. Il pose le bateau sur le sac. Il regarde la flaque. Puis il met le bateau dans l'eau. Tu as préparé. Maintenant il flotte.</t>
+          <t>Celui-là est trop fragile. Amir pose le bateau en papier dans le sac. On en fabrique un autre, plus solide. Avec une feuille plus épaisse, ils plient une nouvelle coque. Celui-ci, pour le sable.</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -16147,11 +16064,11 @@
       <c r="AV86" s="2" t="inlineStr"/>
       <c r="AW86" t="inlineStr">
         <is>
-          <t>narrateur|Amir pose d'abord le sac.
-narrateur|Il pose le bateau sur le sac.
-narrateur|Il regarde la flaque.
-narrateur|Puis il met le bateau dans l'eau.
-papa|Tu as préparé. Maintenant il flotte.</t>
+          <t>enfant-m|Celui-là est trop fragile.
+narrateur|Amir pose le bateau en papier dans le sac.
+papa|On en fabrique un autre, plus solide.
+narrateur|Avec une feuille plus épaisse, ils plient une nouvelle coque.
+enfant-m|Celui-ci, pour le sable.</t>
         </is>
       </c>
     </row>
@@ -16178,17 +16095,17 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>Deux bateaux maintenant. L'ancien dans le sac. Le nouveau sur la table. Celui-là, pour demain. On a bien fait. Le papier fragile se repose. L'autre attend le jardin. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>Deux bateaux maintenant. L'ancien dans le sac. Le nouveau sur la table. Celui-là, pour demain. On a bien fait. Le papier fragile se repose. L'autre attend le jardin. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Le papier est un peu mouillé. Amir sèche ses doigts avec le linge. Il remet le bateau dans le sac. Le linge rentre aussi. On referme. Zzz. Un grain de sable reste sur le bois. L'histoire est finie.</t>
+          <t>Deux bateaux maintenant. L'ancien dans le sac. Le nouveau sur la table. Celui-là, pour demain. On a bien fait. Le papier fragile se repose. L'autre attend le jardin. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr"/>
@@ -16318,13 +16235,11 @@
       <c r="AV87" s="2" t="inlineStr"/>
       <c r="AW87" t="inlineStr">
         <is>
-          <t>narrateur|Le papier est un peu mouillé.
-narrateur|Amir sèche ses doigts avec le linge.
-narrateur|Il remet le bateau dans le sac.
-narrateur|Le linge rentre aussi.
-narrateur|On referme. Zzz.
-narrateur|Un grain de sable reste sur le bois.
-narrateur|L'histoire est finie.</t>
+          <t>narrateur|Deux bateaux maintenant. L'ancien dans le sac. Le nouveau sur la table.
+enfant-m|Celui-là, pour demain.
+papa|On a bien fait.
+narrateur|Le papier fragile se repose. L'autre attend le jardin.
+narrateur|Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
         </is>
       </c>
     </row>
@@ -16345,7 +16260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16425,6 +16340,18 @@
       <c r="A11" t="inlineStr">
         <is>
           <t>exemple2 + avis 88534be : bateau/flaque, labels manteau/bottes/linge, fins qui flottent, SSML = texte</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>avis1.txt</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>fins distinctes gouttière / choux / bac ; ouverture monde ; pas d'audio</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F-NAR-018): example1 ChatGPT — AUT-001, T1 équipe complète
Intègre la proposition de feedback_chatgpt/examples/example1 dans
TREE-AUT-001 (graphe inchangé). T1 prépare d'abord un objet, les trois
partent. T3 bac : canal / piste, plus un autre bateau. Retouches N1 :
en ce moment, pas d'aujourd'hui, vocabulaire adouci. Titre étalon gardé.
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-AUT-001.xlsx
+++ b/stories/arbres/TREE-AUT-001.xlsx
@@ -684,7 +684,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>dans la maison, puis le jardin</t>
+          <t>une petite maison, puis le jardin après la pluie</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amir veut faire voyager son bateau dans les chemins d'eau du jardin. Chaque lieu a son obstacle. L'accessoire change le voyage.</t>
+          <t>Après la pluie, Amir veut offrir un vrai voyage à son bateau et rapporter une histoire à ses parents. Il prépare son expédition, choisit une route du jardin, affronte un obstacle réel, trouve sa propre solution puis rentre avec une trace de l'aventure.</t>
         </is>
       </c>
     </row>
@@ -1197,12 +1197,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le volet jaune bouge encore un peu. Dans la rue, les pavés brillent. Dans la maison, ça sent la soupe. Maman est dans la cuisine. Papa est à la grande table. Son ordinateur fait un petit vent. En ce moment, Amir plie un coin de papier. Celle-ci, c'est la coque. Il plie encore. Une voile un peu froissée. Et ça, c'est la cheminée. C'est un bateau en papier. Assez petit pour ses deux mains. Il le fait glisser. Le bateau s'arrête contre la pantoufle de papa. Votre bateau s'est échoué, capitaine Amir. Il lui faut de l'eau. Dehors, la pluie s'arrête. Une dernière goutte. Ploc. Amir court à la fenêtre. L'eau a dessiné un chemin. La gouttière. Le potager. Le bac à sable. Papa ! Mon bateau peut faire un vrai voyage ! Jusqu'où ? Je ne sais pas encore. C'est le bateau qui choisira. Maman arrive avec le petit sac. Le jardin est encore mouillé. De quoi auras-tu besoin ?</t>
+          <t>Au bout d'une petite rue vit Amir. Sa maison a un jardin minuscule. Ce matin-là, la pluie vient de partir. Les pavés brillent derrière la fenêtre. Maman prépare une soupe dans la cuisine. Papa travaille près du volet jaune. Son ordinateur souffle comme un petit vent. En ce moment, Amir plie une feuille. Un pli devient coque. Un autre pli devient voile. Capitaine Amir est prêt ! Il pousse le bateau vers papa. Le bateau heurte sa pantoufle. Votre navire cherche-t-il la mer ? Oui, mais la mer est très loin. Une goutte tombe dehors. Puis une deuxième rejoint la gouttière. Amir colle son nez contre la vitre. L'eau dessine des chemins dans le jardin. Papa, mon bateau peut voyager ici ! Alors rapporte-nous une grande histoire. Et peut-être un trésor ! Merci, on t'attendra. Maman pose le petit sac près d'Amir. Prépare-toi, avant que le soleil sèche tout.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le volet jaune bouge encore un peu. Dans la rue, les pavés brillent. Dans la maison, ça sent la soupe. Maman est dans la cuisine. Papa est à la grande table. Son ordinateur fait un petit vent. En ce moment, Amir plie un coin de papier. Celle-ci, c'est la coque. Il plie encore. Une voile un peu froissée. Et ça, c'est la cheminée. C'est un bateau en papier. Assez petit pour ses deux mains. Il le fait glisser. Le bateau s'arrête contre la pantoufle de papa. Votre bateau s'est échoué, capitaine Amir. Il lui faut de l'eau. Dehors, la pluie s'arrête. Une dernière goutte. Ploc. Amir court à la fenêtre. L'eau a dessiné un chemin. La gouttière. Le potager. Le bac à sable. Papa ! Mon bateau peut faire un vrai voyage ! Jusqu'où ? Je ne sais pas encore. C'est le bateau qui choisira. Maman arrive avec le petit sac. Le jardin est encore mouillé. De quoi auras-tu besoin ?</t>
+          <t>Au bout d'une petite rue vit Amir. Sa maison a un jardin minuscule. Ce matin-là, la pluie vient de partir. Les pavés brillent derrière la fenêtre. Maman prépare une soupe dans la cuisine. Papa travaille près du volet jaune. Son ordinateur souffle comme un petit vent. En ce moment, Amir plie une feuille. Un pli devient coque. Un autre pli devient voile. Capitaine Amir est prêt ! Il pousse le bateau vers papa. Le bateau heurte sa pantoufle. Votre navire cherche-t-il la mer ? Oui, mais la mer est très loin. Une goutte tombe dehors. Puis une deuxième rejoint la gouttière. Amir colle son nez contre la vitre. L'eau dessine des chemins dans le jardin. Papa, mon bateau peut voyager ici ! Alors rapporte-nous une grande histoire. Et peut-être un trésor ! Merci, on t'attendra. Maman pose le petit sac près d'Amir. Prépare-toi, avant que le soleil sèche tout.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1337,39 +1337,31 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le volet jaune bouge encore un peu.
-narrateur|Dans la rue, les pavés brillent.
-narrateur|Dans la maison, ça sent la soupe.
-narrateur|Maman est dans la cuisine.
-narrateur|Papa est à la grande table.
-narrateur|Son ordinateur fait un petit vent.
-narrateur|En ce moment, Amir plie un coin de papier.
-enfant-m|Celle-ci, c'est la coque.
-narrateur|Il plie encore.
-narrateur|Une voile un peu froissée.
-enfant-m|Et ça, c'est la cheminée.
-narrateur|C'est un bateau en papier.
-narrateur|Assez petit pour ses deux mains.
-narrateur|Il le fait glisser.
-narrateur|Le bateau s'arrête contre la pantoufle de papa.
-papa|Votre bateau s'est échoué, capitaine Amir.
-enfant-m|Il lui faut de l'eau.
-narrateur|Dehors, la pluie s'arrête.
-narrateur|Une dernière goutte.
-narrateur|Ploc.
-narrateur|Amir court à la fenêtre.
-narrateur|L'eau a dessiné un chemin.
-narrateur|La gouttière.
-narrateur|Le potager.
-narrateur|Le bac à sable.
-enfant-m|Papa !
-enfant-m|Mon bateau peut faire un vrai voyage !
-papa|Jusqu'où ?
-enfant-m|Je ne sais pas encore.
-enfant-m|C'est le bateau qui choisira.
-narrateur|Maman arrive avec le petit sac.
-maman|Le jardin est encore mouillé.
-maman|De quoi auras-tu besoin ?</t>
+          <t>narrateur|Au bout d'une petite rue vit Amir.
+narrateur|Sa maison a un jardin minuscule.
+narrateur|Ce matin-là, la pluie vient de partir.
+narrateur|Les pavés brillent derrière la fenêtre.
+narrateur|Maman prépare une soupe dans la cuisine.
+narrateur|Papa travaille près du volet jaune.
+narrateur|Son ordinateur souffle comme un petit vent.
+narrateur|En ce moment, Amir plie une feuille.
+narrateur|Un pli devient coque.
+narrateur|Un autre pli devient voile.
+enfant-m|Capitaine Amir est prêt !
+narrateur|Il pousse le bateau vers papa.
+narrateur|Le bateau heurte sa pantoufle.
+papa|Votre navire cherche-t-il la mer ?
+enfant-m|Oui, mais la mer est très loin.
+narrateur|Une goutte tombe dehors.
+narrateur|Puis une deuxième rejoint la gouttière.
+narrateur|Amir colle son nez contre la vitre.
+narrateur|L'eau dessine des chemins dans le jardin.
+enfant-m|Papa, mon bateau peut voyager ici !
+papa|Alors rapporte-nous une grande histoire.
+enfant-m|Et peut-être un trésor !
+papa|Merci, on t'attendra.
+narrateur|Maman pose le petit sac près d'Amir.
+maman|Prépare-toi, avant que le soleil sèche tout.</t>
         </is>
       </c>
     </row>
@@ -1396,12 +1388,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Avant de partir, un capitaine prépare ses affaires. Le manteau, les bottes, ou un linge. Qu'est-ce que tu prends, Amir ?</t>
+          <t>Amir doit préparer trois choses. Son manteau, ses bottes et un linge. Laquelle prépares-tu d'abord ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Avant de partir, un capitaine prépare ses affaires. Le manteau, les bottes, ou un linge. Qu'est-ce que tu prends, Amir ?</t>
+          <t>Amir doit préparer trois choses. Son manteau, ses bottes et un linge. Laquelle prépares-tu d'abord ?</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -1444,7 +1436,7 @@
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>un linge</t>
+          <t>le petit linge</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -1564,9 +1556,9 @@
       <c r="AV3" s="2" t="inlineStr"/>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Avant de partir, un capitaine prépare ses affaires.
-narrateur|Le manteau, les bottes, ou un linge.
-maman|Qu'est-ce que tu prends, Amir ?</t>
+          <t>narrateur|Amir doit préparer trois choses.
+narrateur|Son manteau, ses bottes et un linge.
+maman|Laquelle prépares-tu d'abord ?</t>
         </is>
       </c>
     </row>
@@ -1593,12 +1585,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Amir prend le bateau en papier sur la commode. Il le glisse au fond du sac. Toc. La voile dépasse. Il la rentre du doigt. Le manteau est sur la chaise. Il est tiède. Le jardin est encore mouillé. Prends le manteau, Amir. Oui. Pour le voyage.</t>
+          <t>Amir choisit d'abord son manteau jaune. Il cherche la manche retournée. Je l'ai trouvée ! Il remet la manche dans le bon sens. Ton manteau est prêt. Amir glisse ensuite le bateau dans le sac. Maman ajoute le petit linge. Les bottes attendent près de la porte.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Amir prend le bateau en papier sur la commode. Il le glisse au fond du sac. Toc. La voile dépasse. Il la rentre du doigt. Le manteau est sur la chaise. Il est tiède. Le jardin est encore mouillé. Prends le manteau, Amir. Oui. Pour le voyage.</t>
+          <t>Amir choisit d'abord son manteau jaune. Il cherche la manche retournée. Je l'ai trouvée ! Il remet la manche dans le bon sens. Ton manteau est prêt. Amir glisse ensuite le bateau dans le sac. Maman ajoute le petit linge. Les bottes attendent près de la porte.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1733,17 +1725,14 @@
       <c r="AV4" s="2" t="inlineStr"/>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Amir prend le bateau en papier sur la commode.
-narrateur|Il le glisse au fond du sac.
-narrateur|Toc.
-narrateur|La voile dépasse.
-narrateur|Il la rentre du doigt.
-narrateur|Le manteau est sur la chaise.
-narrateur|Il est tiède.
-maman|Le jardin est encore mouillé.
-maman|Prends le manteau, Amir.
-enfant-m|Oui.
-enfant-m|Pour le voyage.</t>
+          <t>narrateur|Amir choisit d'abord son manteau jaune.
+narrateur|Il cherche la manche retournée.
+enfant-m|Je l'ai trouvée !
+narrateur|Il remet la manche dans le bon sens.
+maman|Ton manteau est prêt.
+narrateur|Amir glisse ensuite le bateau dans le sac.
+narrateur|Maman ajoute le petit linge.
+narrateur|Les bottes attendent près de la porte.</t>
         </is>
       </c>
     </row>
@@ -1770,19 +1759,19 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
+          <t>Où Amir range-t-il son bateau ?</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Où Amir range-t-il son bateau ?</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
           <t>Où Amir met-il le bateau ?</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Où Amir met-il le bateau ?</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Où Amir met-il le bateau ?</t>
-        </is>
-      </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
           <t>dans le sac</t>
@@ -1805,7 +1794,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Le bateau va dans le sac.</t>
+          <t>Le bateau est dans le sac.</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr"/>
@@ -1930,7 +1919,7 @@
       </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Où Amir met-il le bateau ?</t>
+          <t>narrateur|Où Amir range-t-il son bateau ?</t>
         </is>
       </c>
     </row>
@@ -1957,12 +1946,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le bateau est dans le sac. La voile est rentrée. Le manteau attend à côté. On y va, capitaine ? Oui. Le bateau va choisir.</t>
+          <t>Le bateau repose au fond du sac. Le linge protège sa voile. Bottes aux pieds, capitaine ? Bottes aux pieds, manteau fermé !</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le bateau est dans le sac. La voile est rentrée. Le manteau attend à côté. On y va, capitaine ? Oui. Le bateau va choisir.</t>
+          <t>Le bateau repose au fond du sac. Le linge protège sa voile. Bottes aux pieds, capitaine ? Bottes aux pieds, manteau fermé !</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2101,12 +2090,10 @@
       </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le bateau est dans le sac.
-narrateur|La voile est rentrée.
-narrateur|Le manteau attend à côté.
-papa|On y va, capitaine ?
-enfant-m|Oui.
-enfant-m|Le bateau va choisir.</t>
+          <t>narrateur|Le bateau repose au fond du sac.
+narrateur|Le linge protège sa voile.
+papa|Bottes aux pieds, capitaine ?
+enfant-m|Bottes aux pieds, manteau fermé !</t>
         </is>
       </c>
     </row>
@@ -2133,12 +2120,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Dehors, l'eau a fait trois chemins. La rivière de la gouttière. Le port des choux. L'île du bac. Où commence le voyage, capitaine ?</t>
+          <t>Dehors, trois chemins brillent encore. La rivière de la gouttière. Le port caché entre les choux. Puis l'île devant le bac. Quelle route choisis-tu, capitaine ?</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Dehors, l'eau a fait trois chemins. La rivière de la gouttière. Le port des choux. L'île du bac. Où commence le voyage, capitaine ?</t>
+          <t>Dehors, trois chemins brillent encore. La rivière de la gouttière. Le port caché entre les choux. Puis l'île devant le bac. Quelle route choisis-tu, capitaine ?</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -2297,11 +2284,11 @@
       <c r="AV7" s="2" t="inlineStr"/>
       <c r="AW7" t="inlineStr">
         <is>
-          <t>narrateur|Dehors, l'eau a fait trois chemins.
+          <t>narrateur|Dehors, trois chemins brillent encore.
 narrateur|La rivière de la gouttière.
-narrateur|Le port des choux.
-narrateur|L'île du bac.
-papa|Où commence le voyage, capitaine ?</t>
+narrateur|Le port caché entre les choux.
+narrateur|Puis l'île devant le bac.
+papa|Quelle route choisis-tu, capitaine ?</t>
         </is>
       </c>
     </row>
@@ -2328,12 +2315,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Amir enfile le manteau. Il est tiède contre ses bras. Sous la gouttière, l'eau tremble. Plic. Ploc. Une grosse feuille barre le passage. La rivière est fermée. Le bateau ne peut pas passer. Amir s'accroupit. La feuille ne bouge presque pas. Le manteau tiède frotte le sac.</t>
+          <t>Le manteau jaune brille sous la gouttière. Une rigole court sous la gouttière. Amir pose le bateau sur l'eau. Le voyage commence enfin. Soudain, une grande feuille tourne. Elle bouche toute la rivière. Le bateau s'arrête derrière elle. Vite, le soleil revient ! L'eau baisse déjà.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Amir enfile le manteau. Il est tiède contre ses bras. Sous la gouttière, l'eau tremble. Plic. Ploc. Une grosse feuille barre le passage. La rivière est fermée. Le bateau ne peut pas passer. Amir s'accroupit. La feuille ne bouge presque pas. Le manteau tiède frotte le sac.</t>
+          <t>Le manteau jaune brille sous la gouttière. Une rigole court sous la gouttière. Amir pose le bateau sur l'eau. Le voyage commence enfin. Soudain, une grande feuille tourne. Elle bouche toute la rivière. Le bateau s'arrête derrière elle. Vite, le soleil revient ! L'eau baisse déjà.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -2468,17 +2455,15 @@
       <c r="AV8" s="2" t="inlineStr"/>
       <c r="AW8" t="inlineStr">
         <is>
-          <t>narrateur|Amir enfile le manteau.
-narrateur|Il est tiède contre ses bras.
-narrateur|Sous la gouttière, l'eau tremble.
-narrateur|Plic.
-narrateur|Ploc.
-narrateur|Une grosse feuille barre le passage.
-enfant-m|La rivière est fermée.
-papa|Le bateau ne peut pas passer.
-narrateur|Amir s'accroupit.
-narrateur|La feuille ne bouge presque pas.
-narrateur|Le manteau tiède frotte le sac.</t>
+          <t>narrateur|Le manteau jaune brille sous la gouttière.
+narrateur|Une rigole court sous la gouttière.
+narrateur|Amir pose le bateau sur l'eau.
+narrateur|Le voyage commence enfin.
+narrateur|Soudain, une grande feuille tourne.
+narrateur|Elle bouche toute la rivière.
+narrateur|Le bateau s'arrête derrière elle.
+enfant-m|Vite, le soleil revient !
+papa|L'eau baisse déjà.</t>
         </is>
       </c>
     </row>
@@ -2505,12 +2490,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit, et il regarde. Comment on fait, capitaine ?</t>
+          <t>La feuille tient bon. L'eau devient moins profonde. Que tente le capitaine ?</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit, et il regarde. Comment on fait, capitaine ?</t>
+          <t>La feuille tient bon. L'eau devient moins profonde. Que tente le capitaine ?</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -2533,7 +2518,7 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>attendre les gouttes</t>
+          <t>attendre trois gouttes</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -2543,7 +2528,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>appeler papa</t>
+          <t>demander l'aide de papa</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -2553,7 +2538,7 @@
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>changer de départ</t>
+          <t>chercher un autre départ</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
@@ -2669,8 +2654,9 @@
       <c r="AV9" s="2" t="inlineStr"/>
       <c r="AW9" t="inlineStr">
         <is>
-          <t>narrateur|Amir s'accroupit, et il regarde.
-papa|Comment on fait, capitaine ?</t>
+          <t>narrateur|La feuille tient bon.
+narrateur|L'eau devient moins profonde.
+papa|Que tente le capitaine ?</t>
         </is>
       </c>
     </row>
@@ -2697,12 +2683,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit près de la feuille. J'attends encore un peu. Une goutte. Plic. La feuille bouge à peine. Une deuxième. Ploc. La feuille tourne. Une troisième. Plouf. La feuille ouvre un passage. La rivière est libre !</t>
+          <t>J'attends trois gouttes. La première frappe la feuille. La deuxième soulève son bord. La troisième la fait pivoter. Un passage étroit apparaît. Maintenant, petit bateau ! Le bateau file sous une brindille.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit près de la feuille. J'attends encore un peu. Une goutte. Plic. La feuille bouge à peine. Une deuxième. Ploc. La feuille tourne. Une troisième. Plouf. La feuille ouvre un passage. La rivière est libre !</t>
+          <t>J'attends trois gouttes. La première frappe la feuille. La deuxième soulève son bord. La troisième la fait pivoter. Un passage étroit apparaît. Maintenant, petit bateau ! Le bateau file sous une brindille.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -2837,18 +2823,13 @@
       <c r="AV10" s="2" t="inlineStr"/>
       <c r="AW10" t="inlineStr">
         <is>
-          <t>narrateur|Amir s'accroupit près de la feuille.
-enfant-m|J'attends encore un peu.
-narrateur|Une goutte.
-narrateur|Plic.
-narrateur|La feuille bouge à peine.
-narrateur|Une deuxième.
-narrateur|Ploc.
-narrateur|La feuille tourne.
-narrateur|Une troisième.
-narrateur|Plouf.
-narrateur|La feuille ouvre un passage.
-enfant-m|La rivière est libre !</t>
+          <t>enfant-m|J'attends trois gouttes.
+narrateur|La première frappe la feuille.
+narrateur|La deuxième soulève son bord.
+narrateur|La troisième la fait pivoter.
+narrateur|Un passage étroit apparaît.
+enfant-m|Maintenant, petit bateau !
+narrateur|Le bateau file sous une brindille.</t>
         </is>
       </c>
     </row>
@@ -2875,12 +2856,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>De retour, Amir pose le bateau sur le petit linge. Alors, capitaine, jusqu'où es-tu allé ? Très loin. J'ai attendu trois gouttes. C'est vraiment loin. Une dernière goutte, dehors. Plic. Sur le linge, le bateau attend déjà le prochain voyage. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
+          <t>Le bateau atteint le pot violet. Une petite feuille colle devant. Amir la garde comme drapeau. Puis il rentre avant la dernière goutte. Quel trésor rapporte votre navire ? Un drapeau gagné après trois gouttes. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>De retour, Amir pose le bateau sur le petit linge. Alors, capitaine, jusqu'où es-tu allé ? Très loin. J'ai attendu trois gouttes. C'est vraiment loin. Une dernière goutte, dehors. Plic. Sur le linge, le bateau attend déjà le prochain voyage. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
+          <t>Le bateau atteint le pot violet. Une petite feuille colle devant. Amir la garde comme drapeau. Puis il rentre avant la dernière goutte. Quel trésor rapporte votre navire ? Un drapeau gagné après trois gouttes. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -3015,17 +2996,16 @@
       <c r="AV11" s="2" t="inlineStr"/>
       <c r="AW11" t="inlineStr">
         <is>
-          <t>narrateur|De retour, Amir pose le bateau sur le petit linge.
-papa|Alors, capitaine, jusqu'où es-tu allé ?
-enfant-m|Très loin.
-enfant-m|J'ai attendu trois gouttes.
-papa|C'est vraiment loin.
-narrateur|Une dernière goutte, dehors.
-narrateur|Plic.
-narrateur|Sur le linge, le bateau attend déjà le prochain voyage.
-narrateur|Il raccroche le manteau.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|Le bateau atteint le pot violet.
+narrateur|Une petite feuille colle devant.
+narrateur|Amir la garde comme drapeau.
+narrateur|Puis il rentre avant la dernière goutte.
+papa|Quel trésor rapporte votre navire ?
+enfant-m|Un drapeau gagné après trois gouttes.
+narrateur|Amir suspend son manteau jaune.
+narrateur|Une goutte tombe de sa capuche.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -3052,12 +3032,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu peux bouger la feuille ? On la pousse ensemble. Tout doux. Papa soulève le bord. Amir tient le bateau. La feuille glisse. L'eau circule. C'est à toi, capitaine.</t>
+          <t>Papa, j'ai besoin de toi. Tiens le bateau contre le courant. Papa soulève doucement la feuille. Amir maintient la coque bien droite. Maintenant, laisse-le partir. Le bateau bondit dans l'eau libre.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu peux bouger la feuille ? On la pousse ensemble. Tout doux. Papa soulève le bord. Amir tient le bateau. La feuille glisse. L'eau circule. C'est à toi, capitaine.</t>
+          <t>Papa, j'ai besoin de toi. Tiens le bateau contre le courant. Papa soulève doucement la feuille. Amir maintient la coque bien droite. Maintenant, laisse-le partir. Le bateau bondit dans l'eau libre.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -3192,14 +3172,12 @@
       <c r="AV12" s="2" t="inlineStr"/>
       <c r="AW12" t="inlineStr">
         <is>
-          <t>enfant-m|Papa, tu peux bouger la feuille ?
-papa|On la pousse ensemble.
-papa|Tout doux.
-narrateur|Papa soulève le bord.
-narrateur|Amir tient le bateau.
-narrateur|La feuille glisse.
-narrateur|L'eau circule.
-papa|C'est à toi, capitaine.</t>
+          <t>enfant-m|Papa, j'ai besoin de toi.
+papa|Tiens le bateau contre le courant.
+narrateur|Papa soulève doucement la feuille.
+narrateur|Amir maintient la coque bien droite.
+papa|Maintenant, laisse-le partir.
+narrateur|Le bateau bondit dans l'eau libre.</t>
         </is>
       </c>
     </row>
@@ -3226,12 +3204,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Dans la maison. Amir pose le bateau près de la fenêtre. On a poussé la feuille ensemble. Oui. La rivière a dit oui. Papa reprend sa table. Amir regarde le jardin. La gouttière fait encore un tout petit plic. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
+          <t>Le bateau traverse la rivière délivrée. Une ligne brillante marque sa coque. Amir la montre en rentrant. Nous avons formé un bon équipage. Moi devant, et toi derrière ! Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Dans la maison. Amir pose le bateau près de la fenêtre. On a poussé la feuille ensemble. Oui. La rivière a dit oui. Papa reprend sa table. Amir regarde le jardin. La gouttière fait encore un tout petit plic. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
+          <t>Le bateau traverse la rivière délivrée. Une ligne brillante marque sa coque. Amir la montre en rentrant. Nous avons formé un bon équipage. Moi devant, et toi derrière ! Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -3366,17 +3344,15 @@
       <c r="AV13" s="2" t="inlineStr"/>
       <c r="AW13" t="inlineStr">
         <is>
-          <t>narrateur|Dans la maison.
-narrateur|Amir pose le bateau près de la fenêtre.
-papa|On a poussé la feuille ensemble.
-enfant-m|Oui.
-enfant-m|La rivière a dit oui.
-narrateur|Papa reprend sa table.
-narrateur|Amir regarde le jardin.
-narrateur|La gouttière fait encore un tout petit plic.
-narrateur|Il raccroche le manteau.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|Le bateau traverse la rivière délivrée.
+narrateur|Une ligne brillante marque sa coque.
+narrateur|Amir la montre en rentrant.
+papa|Nous avons formé un bon équipage.
+enfant-m|Moi devant, et toi derrière !
+narrateur|Amir suspend son manteau jaune.
+narrateur|Une goutte tombe de sa capuche.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -3403,12 +3379,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>On part d'ici, plus loin. Amir pose le bateau après la feuille. Là où l'eau court déjà. Un petit courant emmène le papier sous une brindille. Une autre rivière !</t>
+          <t>Je cherche un autre départ. Amir longe la rivière sans courir. Derrière un pot, l'eau recommence. Il pose le bateau après la feuille. Le courant l'emporte vers les violettes. J'ai trouvé le passage secret !</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>On part d'ici, plus loin. Amir pose le bateau après la feuille. Là où l'eau court déjà. Un petit courant emmène le papier sous une brindille. Une autre rivière !</t>
+          <t>Je cherche un autre départ. Amir longe la rivière sans courir. Derrière un pot, l'eau recommence. Il pose le bateau après la feuille. Le courant l'emporte vers les violettes. J'ai trouvé le passage secret !</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -3543,11 +3519,12 @@
       <c r="AV14" s="2" t="inlineStr"/>
       <c r="AW14" t="inlineStr">
         <is>
-          <t>enfant-m|On part d'ici, plus loin.
-narrateur|Amir pose le bateau après la feuille.
-narrateur|Là où l'eau court déjà.
-narrateur|Un petit courant emmène le papier sous une brindille.
-enfant-m|Une autre rivière !</t>
+          <t>enfant-m|Je cherche un autre départ.
+narrateur|Amir longe la rivière sans courir.
+narrateur|Derrière un pot, l'eau recommence.
+narrateur|Il pose le bateau après la feuille.
+narrateur|Le courant l'emporte vers les violettes.
+enfant-m|J'ai trouvé le passage secret !</t>
         </is>
       </c>
     </row>
@@ -3574,12 +3551,12 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Amir rentre. Le bateau a une brindille collée à la voile. On a trouvé un autre courant. Le bateau a choisi. Amir sourit. Le sac attend près de la porte. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
+          <t>Le courant dépose une brindille sur la voile. Amir rapporte le bateau ainsi décoré. Je reconnais le passage secret. Il commence derrière le grand pot. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Amir rentre. Le bateau a une brindille collée à la voile. On a trouvé un autre courant. Le bateau a choisi. Amir sourit. Le sac attend près de la porte. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
+          <t>Le courant dépose une brindille sur la voile. Amir rapporte le bateau ainsi décoré. Je reconnais le passage secret. Il commence derrière le grand pot. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -3714,15 +3691,14 @@
       <c r="AV15" s="2" t="inlineStr"/>
       <c r="AW15" t="inlineStr">
         <is>
-          <t>narrateur|Amir rentre.
-narrateur|Le bateau a une brindille collée à la voile.
-enfant-m|On a trouvé un autre courant.
-papa|Le bateau a choisi.
-narrateur|Amir sourit.
-narrateur|Le sac attend près de la porte.
-narrateur|Il raccroche le manteau.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|Le courant dépose une brindille sur la voile.
+narrateur|Amir rapporte le bateau ainsi décoré.
+papa|Je reconnais le passage secret.
+enfant-m|Il commence derrière le grand pot.
+narrateur|Amir suspend son manteau jaune.
+narrateur|Une goutte tombe de sa capuche.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -3749,12 +3725,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Amir enfile le manteau. Une odeur de soupe reste dans le col. Entre deux choux, une flaque ronde. Comme un port. Trois petites feuilles flottent devant l'entrée. Les bateaux n'arrivent pas à accoster. Il y a trois feuilles. Amir compte. Une. Deux. Trois. Le manteau tiède frotte le sac.</t>
+          <t>Une odeur de soupe reste dans son col. Entre les choux se cache un port. Trois feuilles flottent devant l'entrée. Le bateau avance vers elles. La première touche sa voile. La deuxième ferme le passage. La troisième frôle un jeune chou. Je ne veux rien abîmer. Amir retient aussitôt son bateau.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Amir enfile le manteau. Une odeur de soupe reste dans le col. Entre deux choux, une flaque ronde. Comme un port. Trois petites feuilles flottent devant l'entrée. Les bateaux n'arrivent pas à accoster. Il y a trois feuilles. Amir compte. Une. Deux. Trois. Le manteau tiède frotte le sac.</t>
+          <t>Une odeur de soupe reste dans son col. Entre les choux se cache un port. Trois feuilles flottent devant l'entrée. Le bateau avance vers elles. La première touche sa voile. La deuxième ferme le passage. La troisième frôle un jeune chou. Je ne veux rien abîmer. Amir retient aussitôt son bateau.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -3889,18 +3865,15 @@
       <c r="AV16" s="2" t="inlineStr"/>
       <c r="AW16" t="inlineStr">
         <is>
-          <t>narrateur|Amir enfile le manteau.
-narrateur|Une odeur de soupe reste dans le col.
-narrateur|Entre deux choux, une flaque ronde.
-narrateur|Comme un port.
-narrateur|Trois petites feuilles flottent devant l'entrée.
-enfant-m|Les bateaux n'arrivent pas à accoster.
-papa|Il y a trois feuilles.
-narrateur|Amir compte.
-narrateur|Une.
-narrateur|Deux.
-narrateur|Trois.
-narrateur|Le manteau tiède frotte le sac.</t>
+          <t>narrateur|Une odeur de soupe reste dans son col.
+narrateur|Entre les choux se cache un port.
+narrateur|Trois feuilles flottent devant l'entrée.
+narrateur|Le bateau avance vers elles.
+narrateur|La première touche sa voile.
+narrateur|La deuxième ferme le passage.
+narrateur|La troisième frôle un jeune chou.
+enfant-m|Je ne veux rien abîmer.
+narrateur|Amir retient aussitôt son bateau.</t>
         </is>
       </c>
     </row>
@@ -3927,12 +3900,12 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit, et il regarde. Comment on fait, capitaine ?</t>
+          <t>Le port semble fermé. Derrière, la terre forme un petit quai. Comment entrera ton bateau ?</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit, et il regarde. Comment on fait, capitaine ?</t>
+          <t>Le port semble fermé. Derrière, la terre forme un petit quai. Comment entrera ton bateau ?</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -3955,7 +3928,7 @@
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>compter les feuilles</t>
+          <t>compter les passages</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
@@ -3975,7 +3948,7 @@
       </c>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>demander à maman</t>
+          <t>demander conseil à maman</t>
         </is>
       </c>
       <c r="R17" s="2" t="inlineStr">
@@ -4091,8 +4064,9 @@
       <c r="AV17" s="2" t="inlineStr"/>
       <c r="AW17" t="inlineStr">
         <is>
-          <t>narrateur|Amir s'accroupit, et il regarde.
-papa|Comment on fait, capitaine ?</t>
+          <t>narrateur|Le port semble fermé.
+narrateur|Derrière, la terre forme un petit quai.
+maman|Comment entrera ton bateau ?</t>
         </is>
       </c>
     </row>
@@ -4119,12 +4093,12 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Amir compte encore. Une. Deux. Trois. Là. Un espace libre. Il glisse le bateau entre la deuxième. La troisième feuille. Le papier touche un quai de terre. Toc. Celui-ci, c'est le quai Deux.</t>
+          <t>Amir observe les trois feuilles. Une, deux, trois. Entre deux et trois, l'eau brille. Il guide doucement le bateau. Le bateau traverse sans toucher les choux. Quai numéro deux !</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Amir compte encore. Une. Deux. Trois. Là. Un espace libre. Il glisse le bateau entre la deuxième. La troisième feuille. Le papier touche un quai de terre. Toc. Celui-ci, c'est le quai Deux.</t>
+          <t>Amir observe les trois feuilles. Une, deux, trois. Entre deux et trois, l'eau brille. Il guide doucement le bateau. Le bateau traverse sans toucher les choux. Quai numéro deux !</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -4259,17 +4233,12 @@
       <c r="AV18" s="2" t="inlineStr"/>
       <c r="AW18" t="inlineStr">
         <is>
-          <t>narrateur|Amir compte encore.
-narrateur|Une.
-narrateur|Deux.
-narrateur|Trois.
-enfant-m|Là.
-enfant-m|Un espace libre.
-narrateur|Il glisse le bateau entre la deuxième.
-narrateur|La troisième feuille.
-narrateur|Le papier touche un quai de terre.
-narrateur|Toc.
-enfant-m|Celui-ci, c'est le quai Deux.</t>
+          <t>narrateur|Amir observe les trois feuilles.
+enfant-m|Une, deux, trois.
+narrateur|Entre deux et trois, l'eau brille.
+narrateur|Il guide doucement le bateau.
+narrateur|Le bateau traverse sans toucher les choux.
+enfant-m|Quai numéro deux !</t>
         </is>
       </c>
     </row>
@@ -4296,12 +4265,12 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>À table, Amir dit :. Quai Un. Quai Deux. Quai Trois. Ton bateau a visité le port. Sans déranger les choux. Le bateau sèche. Les choux, dehors, restent droits. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
+          <t>Au quai, une feuille devient drapeau. Amir la plante dans le sable humide. Les trois choux restent bien droits. À table, Amir dessine son port. Quel passage as-tu choisi ? Celui entre deux et trois. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>À table, Amir dit :. Quai Un. Quai Deux. Quai Trois. Ton bateau a visité le port. Sans déranger les choux. Le bateau sèche. Les choux, dehors, restent droits. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
+          <t>Au quai, une feuille devient drapeau. Amir la plante dans le sable humide. Les trois choux restent bien droits. À table, Amir dessine son port. Quel passage as-tu choisi ? Celui entre deux et trois. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -4436,17 +4405,16 @@
       <c r="AV19" s="2" t="inlineStr"/>
       <c r="AW19" t="inlineStr">
         <is>
-          <t>narrateur|À table, Amir dit :.
-enfant-m|Quai Un.
-enfant-m|Quai Deux.
-enfant-m|Quai Trois.
-maman|Ton bateau a visité le port.
-enfant-m|Sans déranger les choux.
-narrateur|Le bateau sèche.
-narrateur|Les choux, dehors, restent droits.
-narrateur|Il raccroche le manteau.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|Au quai, une feuille devient drapeau.
+narrateur|Amir la plante dans le sable humide.
+narrateur|Les trois choux restent bien droits.
+narrateur|À table, Amir dessine son port.
+maman|Quel passage as-tu choisi ?
+enfant-m|Celui entre deux et trois.
+narrateur|Amir suspend son manteau jaune.
+narrateur|Une goutte tombe de sa capuche.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -4473,12 +4441,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Amir attend. L'eau pousse tout doux. Une feuille s'écarte. Puis une autre. Le port s'ouvre. Le bateau avance tout seul jusqu'au chou.</t>
+          <t>J'attends le prochain courant. Amir garde le bateau contre sa botte. L'eau pousse lentement la première feuille. Puis la seconde s'écarte aussi. Le port s'ouvre juste assez. Le bateau glisse jusqu'au quai.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Amir attend. L'eau pousse tout doux. Une feuille s'écarte. Puis une autre. Le port s'ouvre. Le bateau avance tout seul jusqu'au chou.</t>
+          <t>J'attends le prochain courant. Amir garde le bateau contre sa botte. L'eau pousse lentement la première feuille. Puis la seconde s'écarte aussi. Le port s'ouvre juste assez. Le bateau glisse jusqu'au quai.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -4613,12 +4581,12 @@
       <c r="AV20" s="2" t="inlineStr"/>
       <c r="AW20" t="inlineStr">
         <is>
-          <t>narrateur|Amir attend.
-narrateur|L'eau pousse tout doux.
-narrateur|Une feuille s'écarte.
-narrateur|Puis une autre.
-enfant-m|Le port s'ouvre.
-narrateur|Le bateau avance tout seul jusqu'au chou.</t>
+          <t>enfant-m|J'attends le prochain courant.
+narrateur|Amir garde le bateau contre sa botte.
+narrateur|L'eau pousse lentement la première feuille.
+narrateur|Puis la seconde s'écarte aussi.
+narrateur|Le port s'ouvre juste assez.
+narrateur|Le bateau glisse jusqu'au quai.</t>
         </is>
       </c>
     </row>
@@ -4645,12 +4613,12 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Amir raconte, tout doux. J'ai attendu. Les feuilles ont ouvert le port. Le courant a aidé. Le bateau sent encore un peu le chou. Amir rit. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
+          <t>Le bateau touche enfin le quai de terre. Une odeur de chou monte de sa coque. Amir éclate de rire en rentrant. Ton trésor sent vraiment le potager ! C'est le parfum de mon port. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Amir raconte, tout doux. J'ai attendu. Les feuilles ont ouvert le port. Le courant a aidé. Le bateau sent encore un peu le chou. Amir rit. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
+          <t>Le bateau touche enfin le quai de terre. Une odeur de chou monte de sa coque. Amir éclate de rire en rentrant. Ton trésor sent vraiment le potager ! C'est le parfum de mon port. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -4785,15 +4753,15 @@
       <c r="AV21" s="2" t="inlineStr"/>
       <c r="AW21" t="inlineStr">
         <is>
-          <t>narrateur|Amir raconte, tout doux.
-enfant-m|J'ai attendu.
-enfant-m|Les feuilles ont ouvert le port.
-papa|Le courant a aidé.
-narrateur|Le bateau sent encore un peu le chou.
-narrateur|Amir rit.
-narrateur|Il raccroche le manteau.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|Le bateau touche enfin le quai de terre.
+narrateur|Une odeur de chou monte de sa coque.
+narrateur|Amir éclate de rire en rentrant.
+papa|Ton trésor sent vraiment le potager !
+enfant-m|C'est le parfum de mon port.
+narrateur|Amir suspend son manteau jaune.
+narrateur|Une goutte tombe de sa capuche.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -4820,12 +4788,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Maman est venue jusqu'au potager. Maman, je veux jouer sans abîmer les choux. Passe entre les feuilles. Pas dessus. Amir pose le bateau dans l'espace libre. Les plants ne bougent pas. Ton port est gentil avec le jardin.</t>
+          <t>Maman, peux-tu regarder mon port ? Vois-tu cette rigole près du thym ? Amir suit la rigole avec son doigt. Elle contourne toutes les jeunes pousses. Voilà ma route ! Le bateau rejoint le quai sans rien plier.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Maman est venue jusqu'au potager. Maman, je veux jouer sans abîmer les choux. Passe entre les feuilles. Pas dessus. Amir pose le bateau dans l'espace libre. Les plants ne bougent pas. Ton port est gentil avec le jardin.</t>
+          <t>Maman, peux-tu regarder mon port ? Vois-tu cette rigole près du thym ? Amir suit la rigole avec son doigt. Elle contourne toutes les jeunes pousses. Voilà ma route ! Le bateau rejoint le quai sans rien plier.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -4960,13 +4928,12 @@
       <c r="AV22" s="2" t="inlineStr"/>
       <c r="AW22" t="inlineStr">
         <is>
-          <t>narrateur|Maman est venue jusqu'au potager.
-enfant-m|Maman, je veux jouer sans abîmer les choux.
-maman|Passe entre les feuilles.
-maman|Pas dessus.
-narrateur|Amir pose le bateau dans l'espace libre.
-narrateur|Les plants ne bougent pas.
-maman|Ton port est gentil avec le jardin.</t>
+          <t>enfant-m|Maman, peux-tu regarder mon port ?
+maman|Vois-tu cette rigole près du thym ?
+narrateur|Amir suit la rigole avec son doigt.
+narrateur|Elle contourne toutes les jeunes pousses.
+enfant-m|Voilà ma route !
+narrateur|Le bateau rejoint le quai sans rien plier.</t>
         </is>
       </c>
     </row>
@@ -4993,12 +4960,12 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Merci d'avoir demandé. Le port est dans le jardin. On le garde. Amir pose le bateau. Maman pose la soupe. Deux voyages : l'eau, et la maison. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
+          <t>La rigole conduit le bateau au thym. Une minuscule fleur touche sa voile. Amir rentre avec son bateau parfumé. Tu as trouvé sans écraser mes choux. La route passait près du thym. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Merci d'avoir demandé. Le port est dans le jardin. On le garde. Amir pose le bateau. Maman pose la soupe. Deux voyages : l'eau, et la maison. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
+          <t>La rigole conduit le bateau au thym. Une minuscule fleur touche sa voile. Amir rentre avec son bateau parfumé. Tu as trouvé sans écraser mes choux. La route passait près du thym. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -5133,15 +5100,15 @@
       <c r="AV23" s="2" t="inlineStr"/>
       <c r="AW23" t="inlineStr">
         <is>
-          <t>maman|Merci d'avoir demandé.
-enfant-m|Le port est dans le jardin.
-enfant-m|On le garde.
-narrateur|Amir pose le bateau.
-narrateur|Maman pose la soupe.
-narrateur|Deux voyages : l'eau, et la maison.
-narrateur|Il raccroche le manteau.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|La rigole conduit le bateau au thym.
+narrateur|Une minuscule fleur touche sa voile.
+narrateur|Amir rentre avec son bateau parfumé.
+maman|Tu as trouvé sans écraser mes choux.
+enfant-m|La route passait près du thym.
+narrateur|Amir suspend son manteau jaune.
+narrateur|Une goutte tombe de sa capuche.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -5168,12 +5135,12 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Amir enfile le manteau. Le sac tape contre le tissu. Près du bac à sable. L'eau devient de plus en plus petite. Elle rentre dans le sol. Le bateau n'aurait plus assez d'eau. Mon chemin s'en va dans le sable. Le sable boit la flaque. Amir serre le bateau. Il avait imaginé cette île. Le manteau tiède frotte le sac.</t>
+          <t>Le vent gonfle doucement son manteau jaune. Devant le bac brille une île ronde. Au milieu repose un caillou blanc. Voilà l'île au trésor ! Amir approche le bateau de l'eau. Mais la flaque devient soudain plus petite. Le sable boit ses derniers reflets. Mon île disparaît ! Il reste encore un peu de temps.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Amir enfile le manteau. Le sac tape contre le tissu. Près du bac à sable. L'eau devient de plus en plus petite. Elle rentre dans le sol. Le bateau n'aurait plus assez d'eau. Mon chemin s'en va dans le sable. Le sable boit la flaque. Amir serre le bateau. Il avait imaginé cette île. Le manteau tiède frotte le sac.</t>
+          <t>Le vent gonfle doucement son manteau jaune. Devant le bac brille une île ronde. Au milieu repose un caillou blanc. Voilà l'île au trésor ! Amir approche le bateau de l'eau. Mais la flaque devient soudain plus petite. Le sable boit ses derniers reflets. Mon île disparaît ! Il reste encore un peu de temps.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -5308,17 +5275,15 @@
       <c r="AV24" s="2" t="inlineStr"/>
       <c r="AW24" t="inlineStr">
         <is>
-          <t>narrateur|Amir enfile le manteau.
-narrateur|Le sac tape contre le tissu.
-narrateur|Près du bac à sable.
-narrateur|L'eau devient de plus en plus petite.
-narrateur|Elle rentre dans le sol.
-narrateur|Le bateau n'aurait plus assez d'eau.
-enfant-m|Mon chemin s'en va dans le sable.
-papa|Le sable boit la flaque.
-narrateur|Amir serre le bateau.
-narrateur|Il avait imaginé cette île.
-narrateur|Le manteau tiède frotte le sac.</t>
+          <t>narrateur|Le vent gonfle doucement son manteau jaune.
+narrateur|Devant le bac brille une île ronde.
+narrateur|Au milieu repose un caillou blanc.
+enfant-m|Voilà l'île au trésor !
+narrateur|Amir approche le bateau de l'eau.
+narrateur|Mais la flaque devient soudain plus petite.
+narrateur|Le sable boit ses derniers reflets.
+enfant-m|Mon île disparaît !
+papa|Il reste encore un peu de temps.</t>
         </is>
       </c>
     </row>
@@ -5345,12 +5310,12 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit, et il regarde. Comment on fait, capitaine ?</t>
+          <t>Le bateau attend dans les mains d'Amir. Le caillou blanc reste hors d'atteinte. Comment sauver ce voyage ?</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit, et il regarde. Comment on fait, capitaine ?</t>
+          <t>Le bateau attend dans les mains d'Amir. Le caillou blanc reste hors d'atteinte. Comment sauver ce voyage ?</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -5373,7 +5338,7 @@
       <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>une autre flaque</t>
+          <t>chercher une autre flaque</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
@@ -5383,7 +5348,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>sur le sable</t>
+          <t>creuser un petit canal</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -5393,7 +5358,7 @@
       </c>
       <c r="Q25" s="2" t="inlineStr">
         <is>
-          <t>un autre bateau</t>
+          <t>faire une piste de sable</t>
         </is>
       </c>
       <c r="R25" s="2" t="inlineStr">
@@ -5509,8 +5474,9 @@
       <c r="AV25" s="2" t="inlineStr"/>
       <c r="AW25" t="inlineStr">
         <is>
-          <t>narrateur|Amir s'accroupit, et il regarde.
-papa|Comment on fait, capitaine ?</t>
+          <t>narrateur|Le bateau attend dans les mains d'Amir.
+narrateur|Le caillou blanc reste hors d'atteinte.
+papa|Comment sauver ce voyage ?</t>
         </is>
       </c>
     </row>
@@ -5537,12 +5503,12 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Celle-ci s'en va. On prend l'autre. À côté, une flaque plus ronde tient encore. Amir y pose le bateau. Il avance. Ffff. On reprend plus loin, alors.</t>
+          <t>Je cherche une autre flaque. Amir regarde autour du bac. Sous le banc, une eau claire résiste. Il y pose vite son bateau. Le bateau contourne un galet gris. Une nouvelle île !</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Celle-ci s'en va. On prend l'autre. À côté, une flaque plus ronde tient encore. Amir y pose le bateau. Il avance. Ffff. On reprend plus loin, alors.</t>
+          <t>Je cherche une autre flaque. Amir regarde autour du bac. Sous le banc, une eau claire résiste. Il y pose vite son bateau. Le bateau contourne un galet gris. Une nouvelle île !</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -5677,13 +5643,12 @@
       <c r="AV26" s="2" t="inlineStr"/>
       <c r="AW26" t="inlineStr">
         <is>
-          <t>enfant-m|Celle-ci s'en va.
-enfant-m|On prend l'autre.
-narrateur|À côté, une flaque plus ronde tient encore.
-narrateur|Amir y pose le bateau.
-narrateur|Il avance.
-narrateur|Ffff.
-papa|On reprend plus loin, alors.</t>
+          <t>enfant-m|Je cherche une autre flaque.
+narrateur|Amir regarde autour du bac.
+narrateur|Sous le banc, une eau claire résiste.
+narrateur|Il y pose vite son bateau.
+narrateur|Le bateau contourne un galet gris.
+enfant-m|Une nouvelle île !</t>
         </is>
       </c>
     </row>
@@ -5710,12 +5675,12 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>La première flaque est partie. L'autre m'a emmené. Tu as trouvé une autre rivière. Amir hoche la tête. Le bateau sèche près du volet jaune. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
+          <t>Le galet gris devient le nouveau trésor. Amir le laisse près de la flaque. Il rapporte seulement son histoire. L'île a changé, mais le voyage continue. Demain, je chercherai encore. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>La première flaque est partie. L'autre m'a emmené. Tu as trouvé une autre rivière. Amir hoche la tête. Le bateau sèche près du volet jaune. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
+          <t>Le galet gris devient le nouveau trésor. Amir le laisse près de la flaque. Il rapporte seulement son histoire. L'île a changé, mais le voyage continue. Demain, je chercherai encore. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -5850,14 +5815,15 @@
       <c r="AV27" s="2" t="inlineStr"/>
       <c r="AW27" t="inlineStr">
         <is>
-          <t>enfant-m|La première flaque est partie.
-enfant-m|L'autre m'a emmené.
-papa|Tu as trouvé une autre rivière.
-narrateur|Amir hoche la tête.
+          <t>narrateur|Le galet gris devient le nouveau trésor.
+narrateur|Amir le laisse près de la flaque.
+narrateur|Il rapporte seulement son histoire.
+papa|L'île a changé, mais le voyage continue.
+enfant-m|Demain, je chercherai encore.
+narrateur|Amir suspend son manteau jaune.
+narrateur|Une goutte tombe de sa capuche.
 narrateur|Le bateau sèche près du volet jaune.
-narrateur|Il raccroche le manteau.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -5884,12 +5850,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Plus d'eau. Alors il marche. Amir pousse le bateau sur le sable humide. Une piste. Le papier glisse. Grain. Grain. Un bateau de terre, pour cette fois.</t>
+          <t>Je creuse un petit canal. Amir prend la pelle du bac. Papa verse doucement un fond d'arrosoir. L'eau suit le canal jusqu'au caillou. Le bateau avance dans cette rivière neuve. L'île revient !</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Plus d'eau. Alors il marche. Amir pousse le bateau sur le sable humide. Une piste. Le papier glisse. Grain. Grain. Un bateau de terre, pour cette fois.</t>
+          <t>Je creuse un petit canal. Amir prend la pelle du bac. Papa verse doucement un fond d'arrosoir. L'eau suit le canal jusqu'au caillou. Le bateau avance dans cette rivière neuve. L'île revient !</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -6024,14 +5990,12 @@
       <c r="AV28" s="2" t="inlineStr"/>
       <c r="AW28" t="inlineStr">
         <is>
-          <t>enfant-m|Plus d'eau.
-enfant-m|Alors il marche.
-narrateur|Amir pousse le bateau sur le sable humide.
-narrateur|Une piste.
-narrateur|Le papier glisse.
-narrateur|Grain.
-narrateur|Grain.
-papa|Un bateau de terre, pour cette fois.</t>
+          <t>enfant-m|Je creuse un petit canal.
+narrateur|Amir prend la pelle du bac.
+narrateur|Papa verse doucement un fond d'arrosoir.
+narrateur|L'eau suit le canal jusqu'au caillou.
+narrateur|Le bateau avance dans cette rivière neuve.
+enfant-m|L'île revient !</t>
         </is>
       </c>
     </row>
@@ -6058,12 +6022,12 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Mon bateau a marché sur le sable. Un capitaine de sable. Un grain reste sur la cheminée rouge. Amir le souffle. Ffff. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
+          <t>Le bateau atteint enfin le caillou blanc. Son reflet danse dans le petit canal. Puis l'eau disparaît doucement dans le sable. J'ai vu mon île revenir. Juste assez longtemps pour ton voyage. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Mon bateau a marché sur le sable. Un capitaine de sable. Un grain reste sur la cheminée rouge. Amir le souffle. Ffff. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
+          <t>Le bateau atteint enfin le caillou blanc. Son reflet danse dans le petit canal. Puis l'eau disparaît doucement dans le sable. J'ai vu mon île revenir. Juste assez longtemps pour ton voyage. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -6198,14 +6162,15 @@
       <c r="AV29" s="2" t="inlineStr"/>
       <c r="AW29" t="inlineStr">
         <is>
-          <t>enfant-m|Mon bateau a marché sur le sable.
-papa|Un capitaine de sable.
-narrateur|Un grain reste sur la cheminée rouge.
-narrateur|Amir le souffle.
-narrateur|Ffff.
-narrateur|Il raccroche le manteau.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|Le bateau atteint enfin le caillou blanc.
+narrateur|Son reflet danse dans le petit canal.
+narrateur|Puis l'eau disparaît doucement dans le sable.
+enfant-m|J'ai vu mon île revenir.
+papa|Juste assez longtemps pour ton voyage.
+narrateur|Amir suspend son manteau jaune.
+narrateur|Une goutte tombe de sa capuche.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -6232,12 +6197,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Celui-là est trop fragile. Amir pose le bateau en papier dans le sac. On en fabrique un autre, plus solide. Avec une feuille plus épaisse, ils plient une nouvelle coque. Celui-ci, pour le sable.</t>
+          <t>Je fabrique une piste de sable. Amir tasse une longue bande humide. Il pose la coque bien droite. Puis il souffle dans la voile. Le bateau glisse jusqu'au caillou blanc. Mon bateau roule aussi !</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Celui-là est trop fragile. Amir pose le bateau en papier dans le sac. On en fabrique un autre, plus solide. Avec une feuille plus épaisse, ils plient une nouvelle coque. Celui-ci, pour le sable.</t>
+          <t>Je fabrique une piste de sable. Amir tasse une longue bande humide. Il pose la coque bien droite. Puis il souffle dans la voile. Le bateau glisse jusqu'au caillou blanc. Mon bateau roule aussi !</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -6372,11 +6337,12 @@
       <c r="AV30" s="2" t="inlineStr"/>
       <c r="AW30" t="inlineStr">
         <is>
-          <t>enfant-m|Celui-là est trop fragile.
-narrateur|Amir pose le bateau en papier dans le sac.
-papa|On en fabrique un autre, plus solide.
-narrateur|Avec une feuille plus épaisse, ils plient une nouvelle coque.
-enfant-m|Celui-ci, pour le sable.</t>
+          <t>enfant-m|Je fabrique une piste de sable.
+narrateur|Amir tasse une longue bande humide.
+narrateur|Il pose la coque bien droite.
+narrateur|Puis il souffle dans la voile.
+narrateur|Le bateau glisse jusqu'au caillou blanc.
+enfant-m|Mon bateau roule aussi !</t>
         </is>
       </c>
     </row>
@@ -6403,12 +6369,12 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Deux bateaux maintenant. L'ancien dans le sac. Le nouveau sur la table. Celui-là, on le fera demain. On a bien fait. Le papier fragile se repose. L'autre attend le jardin. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
+          <t>Le devant touche doucement le caillou blanc. Un grain doré reste sur la coque. Amir le montre à papa en rentrant. Un vrai trésor de capitaine. Mon bateau connaît aussi les routes. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Deux bateaux maintenant. L'ancien dans le sac. Le nouveau sur la table. Celui-là, on le fera demain. On a bien fait. Le papier fragile se repose. L'autre attend le jardin. Il raccroche le manteau. Le sac se ferme. Zzz.</t>
+          <t>Le devant touche doucement le caillou blanc. Un grain doré reste sur la coque. Amir le montre à papa en rentrant. Un vrai trésor de capitaine. Mon bateau connaît aussi les routes. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -6543,16 +6509,15 @@
       <c r="AV31" s="2" t="inlineStr"/>
       <c r="AW31" t="inlineStr">
         <is>
-          <t>narrateur|Deux bateaux maintenant.
-narrateur|L'ancien dans le sac.
-narrateur|Le nouveau sur la table.
-enfant-m|Celui-là, on le fera demain.
-papa|On a bien fait.
-narrateur|Le papier fragile se repose.
-narrateur|L'autre attend le jardin.
-narrateur|Il raccroche le manteau.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|Le devant touche doucement le caillou blanc.
+narrateur|Un grain doré reste sur la coque.
+narrateur|Amir le montre à papa en rentrant.
+papa|Un vrai trésor de capitaine.
+enfant-m|Mon bateau connaît aussi les routes.
+narrateur|Amir suspend son manteau jaune.
+narrateur|Une goutte tombe de sa capuche.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -6579,12 +6544,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Amir glisse le bateau au fond du sac. Toc. La voile dépasse. Il la rentre. Les bottes sont près de la porte. Un peu mouillées dehors. Attends. Je les essuie. Maman passe le linge sur chaque botte. Voilà. Tes pieds resteront au sec.</t>
+          <t>Amir choisit d'abord ses bottes rouges. Une botte porte encore de la boue. Je te montre un petit coin de boue. Maman commence avec le linge. Puis Amir frotte jusqu'au bout. Elle est prête ! Le bateau rejoint le sac. Le manteau attend sur la chaise.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Amir glisse le bateau au fond du sac. Toc. La voile dépasse. Il la rentre. Les bottes sont près de la porte. Un peu mouillées dehors. Attends. Je les essuie. Maman passe le linge sur chaque botte. Voilà. Tes pieds resteront au sec.</t>
+          <t>Amir choisit d'abord ses bottes rouges. Une botte porte encore de la boue. Je te montre un petit coin de boue. Maman commence avec le linge. Puis Amir frotte jusqu'au bout. Elle est prête ! Le bateau rejoint le sac. Le manteau attend sur la chaise.</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -6719,17 +6684,14 @@
       <c r="AV32" s="2" t="inlineStr"/>
       <c r="AW32" t="inlineStr">
         <is>
-          <t>narrateur|Amir glisse le bateau au fond du sac.
-narrateur|Toc.
-narrateur|La voile dépasse.
-narrateur|Il la rentre.
-narrateur|Les bottes sont près de la porte.
-narrateur|Un peu mouillées dehors.
-maman|Attends.
-maman|Je les essuie.
-narrateur|Maman passe le linge sur chaque botte.
-maman|Voilà.
-maman|Tes pieds resteront au sec.</t>
+          <t>narrateur|Amir choisit d'abord ses bottes rouges.
+narrateur|Une botte porte encore de la boue.
+maman|Je te montre un petit coin de boue.
+narrateur|Maman commence avec le linge.
+narrateur|Puis Amir frotte jusqu'au bout.
+enfant-m|Elle est prête !
+narrateur|Le bateau rejoint le sac.
+narrateur|Le manteau attend sur la chaise.</t>
         </is>
       </c>
     </row>
@@ -6756,27 +6718,27 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
+          <t>Qui termine d'essuyer la botte ?</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Qui termine d'essuyer la botte ?</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
           <t>Qui essuie les bottes ?</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>Qui essuie les bottes ?</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>Qui essuie les bottes ?</t>
-        </is>
-      </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>maman</t>
+          <t>Amir</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>maman|ma maman|maman essuie</t>
+          <t>amir|c'est amir|amir termine|le garçon</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -6791,7 +6753,7 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>Maman essuie les bottes.</t>
+          <t>Amir termine d'essuyer la botte.</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr"/>
@@ -6916,7 +6878,7 @@
       </c>
       <c r="AW33" t="inlineStr">
         <is>
-          <t>narrateur|Qui essuie les bottes ?</t>
+          <t>narrateur|Qui termine d'essuyer la botte ?</t>
         </is>
       </c>
     </row>
@@ -6943,12 +6905,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Les bottes sont sèches. Elles attendent près de la porte. Le bateau est dans le sac. Capitaine, tes bottes sont prêtes. On va au jardin.</t>
+          <t>La semelle rouge est propre. Amir enfile les deux bottes. Et le manteau, capitaine ? Fermé jusqu'en haut !</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Les bottes sont sèches. Elles attendent près de la porte. Le bateau est dans le sac. Capitaine, tes bottes sont prêtes. On va au jardin.</t>
+          <t>La semelle rouge est propre. Amir enfile les deux bottes. Et le manteau, capitaine ? Fermé jusqu'en haut !</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -7087,11 +7049,10 @@
       </c>
       <c r="AW34" t="inlineStr">
         <is>
-          <t>narrateur|Les bottes sont sèches.
-narrateur|Elles attendent près de la porte.
-narrateur|Le bateau est dans le sac.
-papa|Capitaine, tes bottes sont prêtes.
-enfant-m|On va au jardin.</t>
+          <t>narrateur|La semelle rouge est propre.
+narrateur|Amir enfile les deux bottes.
+papa|Et le manteau, capitaine ?
+enfant-m|Fermé jusqu'en haut !</t>
         </is>
       </c>
     </row>
@@ -7118,12 +7079,12 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Dehors, l'eau a fait trois chemins. La rivière de la gouttière. Le port des choux. L'île du bac. Où commence le voyage, capitaine ?</t>
+          <t>Dehors, trois chemins brillent encore. La rivière de la gouttière. Le port caché entre les choux. Puis l'île devant le bac. Quelle route choisis-tu, capitaine ?</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Dehors, l'eau a fait trois chemins. La rivière de la gouttière. Le port des choux. L'île du bac. Où commence le voyage, capitaine ?</t>
+          <t>Dehors, trois chemins brillent encore. La rivière de la gouttière. Le port caché entre les choux. Puis l'île devant le bac. Quelle route choisis-tu, capitaine ?</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -7282,11 +7243,11 @@
       <c r="AV35" s="2" t="inlineStr"/>
       <c r="AW35" t="inlineStr">
         <is>
-          <t>narrateur|Dehors, l'eau a fait trois chemins.
+          <t>narrateur|Dehors, trois chemins brillent encore.
 narrateur|La rivière de la gouttière.
-narrateur|Le port des choux.
-narrateur|L'île du bac.
-papa|Où commence le voyage, capitaine ?</t>
+narrateur|Le port caché entre les choux.
+narrateur|Puis l'île devant le bac.
+papa|Quelle route choisis-tu, capitaine ?</t>
         </is>
       </c>
     </row>
@@ -7313,12 +7274,12 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Amir enfile les bottes. Elles sont un peu froides. Clap. Sous la gouttière, l'eau tremble. Plic. Ploc. Une grosse feuille barre le passage. La rivière est fermée. Le bateau ne peut pas passer. Amir s'accroupit. La feuille ne bouge presque pas. Les bottes font clap, déjà, dans l'entrée.</t>
+          <t>Ses bottes font floc sous la gouttière. Une rigole court sous la gouttière. Amir pose le bateau sur l'eau. Le voyage commence enfin. Soudain, une grande feuille tourne. Elle bouche toute la rivière. Le bateau s'arrête derrière elle. Vite, le soleil revient ! L'eau baisse déjà.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Amir enfile les bottes. Elles sont un peu froides. Clap. Sous la gouttière, l'eau tremble. Plic. Ploc. Une grosse feuille barre le passage. La rivière est fermée. Le bateau ne peut pas passer. Amir s'accroupit. La feuille ne bouge presque pas. Les bottes font clap, déjà, dans l'entrée.</t>
+          <t>Ses bottes font floc sous la gouttière. Une rigole court sous la gouttière. Amir pose le bateau sur l'eau. Le voyage commence enfin. Soudain, une grande feuille tourne. Elle bouche toute la rivière. Le bateau s'arrête derrière elle. Vite, le soleil revient ! L'eau baisse déjà.</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -7453,18 +7414,15 @@
       <c r="AV36" s="2" t="inlineStr"/>
       <c r="AW36" t="inlineStr">
         <is>
-          <t>narrateur|Amir enfile les bottes.
-narrateur|Elles sont un peu froides.
-narrateur|Clap.
-narrateur|Sous la gouttière, l'eau tremble.
-narrateur|Plic.
-narrateur|Ploc.
-narrateur|Une grosse feuille barre le passage.
-enfant-m|La rivière est fermée.
-papa|Le bateau ne peut pas passer.
-narrateur|Amir s'accroupit.
-narrateur|La feuille ne bouge presque pas.
-narrateur|Les bottes font clap, déjà, dans l'entrée.</t>
+          <t>narrateur|Ses bottes font floc sous la gouttière.
+narrateur|Une rigole court sous la gouttière.
+narrateur|Amir pose le bateau sur l'eau.
+narrateur|Le voyage commence enfin.
+narrateur|Soudain, une grande feuille tourne.
+narrateur|Elle bouche toute la rivière.
+narrateur|Le bateau s'arrête derrière elle.
+enfant-m|Vite, le soleil revient !
+papa|L'eau baisse déjà.</t>
         </is>
       </c>
     </row>
@@ -7491,12 +7449,12 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit, et il regarde. Comment on fait, capitaine ?</t>
+          <t>La feuille tient bon. L'eau devient moins profonde. Que tente le capitaine ?</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit, et il regarde. Comment on fait, capitaine ?</t>
+          <t>La feuille tient bon. L'eau devient moins profonde. Que tente le capitaine ?</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -7519,7 +7477,7 @@
       <c r="L37" s="2" t="inlineStr"/>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>attendre les gouttes</t>
+          <t>attendre trois gouttes</t>
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr">
@@ -7529,7 +7487,7 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>appeler papa</t>
+          <t>demander l'aide de papa</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
@@ -7539,7 +7497,7 @@
       </c>
       <c r="Q37" s="2" t="inlineStr">
         <is>
-          <t>changer de départ</t>
+          <t>chercher un autre départ</t>
         </is>
       </c>
       <c r="R37" s="2" t="inlineStr">
@@ -7655,8 +7613,9 @@
       <c r="AV37" s="2" t="inlineStr"/>
       <c r="AW37" t="inlineStr">
         <is>
-          <t>narrateur|Amir s'accroupit, et il regarde.
-papa|Comment on fait, capitaine ?</t>
+          <t>narrateur|La feuille tient bon.
+narrateur|L'eau devient moins profonde.
+papa|Que tente le capitaine ?</t>
         </is>
       </c>
     </row>
@@ -7683,12 +7642,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit près de la feuille. J'attends encore un peu. Une goutte. Plic. La feuille bouge à peine. Une deuxième. Ploc. La feuille tourne. Une troisième. Plouf. La feuille ouvre un passage. La rivière est libre !</t>
+          <t>J'attends trois gouttes. La première frappe la feuille. La deuxième soulève son bord. La troisième la fait pivoter. Un passage étroit apparaît. Maintenant, petit bateau ! Le bateau file sous une brindille.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit près de la feuille. J'attends encore un peu. Une goutte. Plic. La feuille bouge à peine. Une deuxième. Ploc. La feuille tourne. Une troisième. Plouf. La feuille ouvre un passage. La rivière est libre !</t>
+          <t>J'attends trois gouttes. La première frappe la feuille. La deuxième soulève son bord. La troisième la fait pivoter. Un passage étroit apparaît. Maintenant, petit bateau ! Le bateau file sous une brindille.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -7823,18 +7782,13 @@
       <c r="AV38" s="2" t="inlineStr"/>
       <c r="AW38" t="inlineStr">
         <is>
-          <t>narrateur|Amir s'accroupit près de la feuille.
-enfant-m|J'attends encore un peu.
-narrateur|Une goutte.
-narrateur|Plic.
-narrateur|La feuille bouge à peine.
-narrateur|Une deuxième.
-narrateur|Ploc.
-narrateur|La feuille tourne.
-narrateur|Une troisième.
-narrateur|Plouf.
-narrateur|La feuille ouvre un passage.
-enfant-m|La rivière est libre !</t>
+          <t>enfant-m|J'attends trois gouttes.
+narrateur|La première frappe la feuille.
+narrateur|La deuxième soulève son bord.
+narrateur|La troisième la fait pivoter.
+narrateur|Un passage étroit apparaît.
+enfant-m|Maintenant, petit bateau !
+narrateur|Le bateau file sous une brindille.</t>
         </is>
       </c>
     </row>
@@ -7861,12 +7815,12 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>De retour, Amir pose le bateau sur le petit linge. Alors, capitaine, jusqu'où es-tu allé ? Très loin. J'ai attendu trois gouttes. C'est vraiment loin. Une dernière goutte, dehors. Plic. Sur le linge, le bateau attend déjà le prochain voyage. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
+          <t>Le bateau atteint le pot violet. Une petite feuille colle devant. Amir la garde comme drapeau. Puis il rentre avant la dernière goutte. Quel trésor rapporte votre navire ? Un drapeau gagné après trois gouttes. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>De retour, Amir pose le bateau sur le petit linge. Alors, capitaine, jusqu'où es-tu allé ? Très loin. J'ai attendu trois gouttes. C'est vraiment loin. Une dernière goutte, dehors. Plic. Sur le linge, le bateau attend déjà le prochain voyage. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
+          <t>Le bateau atteint le pot violet. Une petite feuille colle devant. Amir la garde comme drapeau. Puis il rentre avant la dernière goutte. Quel trésor rapporte votre navire ? Un drapeau gagné après trois gouttes. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -8001,17 +7955,16 @@
       <c r="AV39" s="2" t="inlineStr"/>
       <c r="AW39" t="inlineStr">
         <is>
-          <t>narrateur|De retour, Amir pose le bateau sur le petit linge.
-papa|Alors, capitaine, jusqu'où es-tu allé ?
-enfant-m|Très loin.
-enfant-m|J'ai attendu trois gouttes.
-papa|C'est vraiment loin.
-narrateur|Une dernière goutte, dehors.
-narrateur|Plic.
-narrateur|Sur le linge, le bateau attend déjà le prochain voyage.
-narrateur|À la porte, il retire les bottes.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|Le bateau atteint le pot violet.
+narrateur|Une petite feuille colle devant.
+narrateur|Amir la garde comme drapeau.
+narrateur|Puis il rentre avant la dernière goutte.
+papa|Quel trésor rapporte votre navire ?
+enfant-m|Un drapeau gagné après trois gouttes.
+narrateur|À la porte, Amir retire ses bottes.
+narrateur|Deux traces rouges restent sur le tapis.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -8038,12 +7991,12 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu peux bouger la feuille ? On la pousse ensemble. Tout doux. Papa soulève le bord. Amir tient le bateau. La feuille glisse. L'eau circule. C'est à toi, capitaine.</t>
+          <t>Papa, j'ai besoin de toi. Tiens le bateau contre le courant. Papa soulève doucement la feuille. Amir maintient la coque bien droite. Maintenant, laisse-le partir. Le bateau bondit dans l'eau libre.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu peux bouger la feuille ? On la pousse ensemble. Tout doux. Papa soulève le bord. Amir tient le bateau. La feuille glisse. L'eau circule. C'est à toi, capitaine.</t>
+          <t>Papa, j'ai besoin de toi. Tiens le bateau contre le courant. Papa soulève doucement la feuille. Amir maintient la coque bien droite. Maintenant, laisse-le partir. Le bateau bondit dans l'eau libre.</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -8178,14 +8131,12 @@
       <c r="AV40" s="2" t="inlineStr"/>
       <c r="AW40" t="inlineStr">
         <is>
-          <t>enfant-m|Papa, tu peux bouger la feuille ?
-papa|On la pousse ensemble.
-papa|Tout doux.
-narrateur|Papa soulève le bord.
-narrateur|Amir tient le bateau.
-narrateur|La feuille glisse.
-narrateur|L'eau circule.
-papa|C'est à toi, capitaine.</t>
+          <t>enfant-m|Papa, j'ai besoin de toi.
+papa|Tiens le bateau contre le courant.
+narrateur|Papa soulève doucement la feuille.
+narrateur|Amir maintient la coque bien droite.
+papa|Maintenant, laisse-le partir.
+narrateur|Le bateau bondit dans l'eau libre.</t>
         </is>
       </c>
     </row>
@@ -8212,12 +8163,12 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Dans la maison. Amir pose le bateau près de la fenêtre. On a poussé la feuille ensemble. Oui. La rivière a dit oui. Papa reprend sa table. Amir regarde le jardin. La gouttière fait encore un tout petit plic. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
+          <t>Le bateau traverse la rivière délivrée. Une ligne brillante marque sa coque. Amir la montre en rentrant. Nous avons formé un bon équipage. Moi devant, et toi derrière ! À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Dans la maison. Amir pose le bateau près de la fenêtre. On a poussé la feuille ensemble. Oui. La rivière a dit oui. Papa reprend sa table. Amir regarde le jardin. La gouttière fait encore un tout petit plic. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
+          <t>Le bateau traverse la rivière délivrée. Une ligne brillante marque sa coque. Amir la montre en rentrant. Nous avons formé un bon équipage. Moi devant, et toi derrière ! À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -8352,17 +8303,15 @@
       <c r="AV41" s="2" t="inlineStr"/>
       <c r="AW41" t="inlineStr">
         <is>
-          <t>narrateur|Dans la maison.
-narrateur|Amir pose le bateau près de la fenêtre.
-papa|On a poussé la feuille ensemble.
-enfant-m|Oui.
-enfant-m|La rivière a dit oui.
-narrateur|Papa reprend sa table.
-narrateur|Amir regarde le jardin.
-narrateur|La gouttière fait encore un tout petit plic.
-narrateur|À la porte, il retire les bottes.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|Le bateau traverse la rivière délivrée.
+narrateur|Une ligne brillante marque sa coque.
+narrateur|Amir la montre en rentrant.
+papa|Nous avons formé un bon équipage.
+enfant-m|Moi devant, et toi derrière !
+narrateur|À la porte, Amir retire ses bottes.
+narrateur|Deux traces rouges restent sur le tapis.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -8389,12 +8338,12 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>On part d'ici, plus loin. Amir pose le bateau après la feuille. Là où l'eau court déjà. Un petit courant emmène le papier sous une brindille. Une autre rivière !</t>
+          <t>Je cherche un autre départ. Amir longe la rivière sans courir. Derrière un pot, l'eau recommence. Il pose le bateau après la feuille. Le courant l'emporte vers les violettes. J'ai trouvé le passage secret !</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>On part d'ici, plus loin. Amir pose le bateau après la feuille. Là où l'eau court déjà. Un petit courant emmène le papier sous une brindille. Une autre rivière !</t>
+          <t>Je cherche un autre départ. Amir longe la rivière sans courir. Derrière un pot, l'eau recommence. Il pose le bateau après la feuille. Le courant l'emporte vers les violettes. J'ai trouvé le passage secret !</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -8529,11 +8478,12 @@
       <c r="AV42" s="2" t="inlineStr"/>
       <c r="AW42" t="inlineStr">
         <is>
-          <t>enfant-m|On part d'ici, plus loin.
-narrateur|Amir pose le bateau après la feuille.
-narrateur|Là où l'eau court déjà.
-narrateur|Un petit courant emmène le papier sous une brindille.
-enfant-m|Une autre rivière !</t>
+          <t>enfant-m|Je cherche un autre départ.
+narrateur|Amir longe la rivière sans courir.
+narrateur|Derrière un pot, l'eau recommence.
+narrateur|Il pose le bateau après la feuille.
+narrateur|Le courant l'emporte vers les violettes.
+enfant-m|J'ai trouvé le passage secret !</t>
         </is>
       </c>
     </row>
@@ -8560,12 +8510,12 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Amir rentre. Le bateau a une brindille collée à la voile. On a trouvé un autre courant. Le bateau a choisi. Amir sourit. Le sac attend près de la porte. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
+          <t>Le courant dépose une brindille sur la voile. Amir rapporte le bateau ainsi décoré. Je reconnais le passage secret. Il commence derrière le grand pot. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Amir rentre. Le bateau a une brindille collée à la voile. On a trouvé un autre courant. Le bateau a choisi. Amir sourit. Le sac attend près de la porte. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
+          <t>Le courant dépose une brindille sur la voile. Amir rapporte le bateau ainsi décoré. Je reconnais le passage secret. Il commence derrière le grand pot. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -8700,15 +8650,14 @@
       <c r="AV43" s="2" t="inlineStr"/>
       <c r="AW43" t="inlineStr">
         <is>
-          <t>narrateur|Amir rentre.
-narrateur|Le bateau a une brindille collée à la voile.
-enfant-m|On a trouvé un autre courant.
-papa|Le bateau a choisi.
-narrateur|Amir sourit.
-narrateur|Le sac attend près de la porte.
-narrateur|À la porte, il retire les bottes.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|Le courant dépose une brindille sur la voile.
+narrateur|Amir rapporte le bateau ainsi décoré.
+papa|Je reconnais le passage secret.
+enfant-m|Il commence derrière le grand pot.
+narrateur|À la porte, Amir retire ses bottes.
+narrateur|Deux traces rouges restent sur le tapis.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -8735,12 +8684,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Amir enfile les bottes. Elles font clap-clap vers les choux. Entre deux choux, une flaque ronde. Comme un port. Trois petites feuilles flottent devant l'entrée. Les bateaux n'arrivent pas à accoster. Il y a trois feuilles. Amir compte. Une. Deux. Trois. Les bottes font clap, déjà, dans l'entrée.</t>
+          <t>Ses bottes traversent la terre molle. Entre les choux se cache un port. Trois feuilles flottent devant l'entrée. Le bateau avance vers elles. La première touche sa voile. La deuxième ferme le passage. La troisième frôle un jeune chou. Je ne veux rien abîmer. Amir retient aussitôt son bateau.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Amir enfile les bottes. Elles font clap-clap vers les choux. Entre deux choux, une flaque ronde. Comme un port. Trois petites feuilles flottent devant l'entrée. Les bateaux n'arrivent pas à accoster. Il y a trois feuilles. Amir compte. Une. Deux. Trois. Les bottes font clap, déjà, dans l'entrée.</t>
+          <t>Ses bottes traversent la terre molle. Entre les choux se cache un port. Trois feuilles flottent devant l'entrée. Le bateau avance vers elles. La première touche sa voile. La deuxième ferme le passage. La troisième frôle un jeune chou. Je ne veux rien abîmer. Amir retient aussitôt son bateau.</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -8875,18 +8824,15 @@
       <c r="AV44" s="2" t="inlineStr"/>
       <c r="AW44" t="inlineStr">
         <is>
-          <t>narrateur|Amir enfile les bottes.
-narrateur|Elles font clap-clap vers les choux.
-narrateur|Entre deux choux, une flaque ronde.
-narrateur|Comme un port.
-narrateur|Trois petites feuilles flottent devant l'entrée.
-enfant-m|Les bateaux n'arrivent pas à accoster.
-papa|Il y a trois feuilles.
-narrateur|Amir compte.
-narrateur|Une.
-narrateur|Deux.
-narrateur|Trois.
-narrateur|Les bottes font clap, déjà, dans l'entrée.</t>
+          <t>narrateur|Ses bottes traversent la terre molle.
+narrateur|Entre les choux se cache un port.
+narrateur|Trois feuilles flottent devant l'entrée.
+narrateur|Le bateau avance vers elles.
+narrateur|La première touche sa voile.
+narrateur|La deuxième ferme le passage.
+narrateur|La troisième frôle un jeune chou.
+enfant-m|Je ne veux rien abîmer.
+narrateur|Amir retient aussitôt son bateau.</t>
         </is>
       </c>
     </row>
@@ -8913,12 +8859,12 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit, et il regarde. Comment on fait, capitaine ?</t>
+          <t>Le port semble fermé. Derrière, la terre forme un petit quai. Comment entrera ton bateau ?</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit, et il regarde. Comment on fait, capitaine ?</t>
+          <t>Le port semble fermé. Derrière, la terre forme un petit quai. Comment entrera ton bateau ?</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -8941,7 +8887,7 @@
       <c r="L45" s="2" t="inlineStr"/>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>compter les feuilles</t>
+          <t>compter les passages</t>
         </is>
       </c>
       <c r="N45" s="2" t="inlineStr">
@@ -8961,7 +8907,7 @@
       </c>
       <c r="Q45" s="2" t="inlineStr">
         <is>
-          <t>demander à maman</t>
+          <t>demander conseil à maman</t>
         </is>
       </c>
       <c r="R45" s="2" t="inlineStr">
@@ -9077,8 +9023,9 @@
       <c r="AV45" s="2" t="inlineStr"/>
       <c r="AW45" t="inlineStr">
         <is>
-          <t>narrateur|Amir s'accroupit, et il regarde.
-papa|Comment on fait, capitaine ?</t>
+          <t>narrateur|Le port semble fermé.
+narrateur|Derrière, la terre forme un petit quai.
+maman|Comment entrera ton bateau ?</t>
         </is>
       </c>
     </row>
@@ -9105,12 +9052,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Amir compte encore. Une. Deux. Trois. Là. Un espace libre. Il glisse le bateau entre la deuxième. La troisième feuille. Le papier touche un quai de terre. Toc. Celui-ci, c'est le quai Deux.</t>
+          <t>Amir observe les trois feuilles. Une, deux, trois. Entre deux et trois, l'eau brille. Il guide doucement le bateau. Le bateau traverse sans toucher les choux. Quai numéro deux !</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Amir compte encore. Une. Deux. Trois. Là. Un espace libre. Il glisse le bateau entre la deuxième. La troisième feuille. Le papier touche un quai de terre. Toc. Celui-ci, c'est le quai Deux.</t>
+          <t>Amir observe les trois feuilles. Une, deux, trois. Entre deux et trois, l'eau brille. Il guide doucement le bateau. Le bateau traverse sans toucher les choux. Quai numéro deux !</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -9245,17 +9192,12 @@
       <c r="AV46" s="2" t="inlineStr"/>
       <c r="AW46" t="inlineStr">
         <is>
-          <t>narrateur|Amir compte encore.
-narrateur|Une.
-narrateur|Deux.
-narrateur|Trois.
-enfant-m|Là.
-enfant-m|Un espace libre.
-narrateur|Il glisse le bateau entre la deuxième.
-narrateur|La troisième feuille.
-narrateur|Le papier touche un quai de terre.
-narrateur|Toc.
-enfant-m|Celui-ci, c'est le quai Deux.</t>
+          <t>narrateur|Amir observe les trois feuilles.
+enfant-m|Une, deux, trois.
+narrateur|Entre deux et trois, l'eau brille.
+narrateur|Il guide doucement le bateau.
+narrateur|Le bateau traverse sans toucher les choux.
+enfant-m|Quai numéro deux !</t>
         </is>
       </c>
     </row>
@@ -9282,12 +9224,12 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>À table, Amir dit :. Quai Un. Quai Deux. Quai Trois. Ton bateau a visité le port. Sans déranger les choux. Le bateau sèche. Les choux, dehors, restent droits. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
+          <t>Au quai, une feuille devient drapeau. Amir la plante dans le sable humide. Les trois choux restent bien droits. À table, Amir dessine son port. Quel passage as-tu choisi ? Celui entre deux et trois. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>À table, Amir dit :. Quai Un. Quai Deux. Quai Trois. Ton bateau a visité le port. Sans déranger les choux. Le bateau sèche. Les choux, dehors, restent droits. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
+          <t>Au quai, une feuille devient drapeau. Amir la plante dans le sable humide. Les trois choux restent bien droits. À table, Amir dessine son port. Quel passage as-tu choisi ? Celui entre deux et trois. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -9422,17 +9364,16 @@
       <c r="AV47" s="2" t="inlineStr"/>
       <c r="AW47" t="inlineStr">
         <is>
-          <t>narrateur|À table, Amir dit :.
-enfant-m|Quai Un.
-enfant-m|Quai Deux.
-enfant-m|Quai Trois.
-maman|Ton bateau a visité le port.
-enfant-m|Sans déranger les choux.
-narrateur|Le bateau sèche.
-narrateur|Les choux, dehors, restent droits.
-narrateur|À la porte, il retire les bottes.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|Au quai, une feuille devient drapeau.
+narrateur|Amir la plante dans le sable humide.
+narrateur|Les trois choux restent bien droits.
+narrateur|À table, Amir dessine son port.
+maman|Quel passage as-tu choisi ?
+enfant-m|Celui entre deux et trois.
+narrateur|À la porte, Amir retire ses bottes.
+narrateur|Deux traces rouges restent sur le tapis.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -9459,12 +9400,12 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Amir attend. L'eau pousse tout doux. Une feuille s'écarte. Puis une autre. Le port s'ouvre. Le bateau avance tout seul jusqu'au chou.</t>
+          <t>J'attends le prochain courant. Amir garde le bateau contre sa botte. L'eau pousse lentement la première feuille. Puis la seconde s'écarte aussi. Le port s'ouvre juste assez. Le bateau glisse jusqu'au quai.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Amir attend. L'eau pousse tout doux. Une feuille s'écarte. Puis une autre. Le port s'ouvre. Le bateau avance tout seul jusqu'au chou.</t>
+          <t>J'attends le prochain courant. Amir garde le bateau contre sa botte. L'eau pousse lentement la première feuille. Puis la seconde s'écarte aussi. Le port s'ouvre juste assez. Le bateau glisse jusqu'au quai.</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -9599,12 +9540,12 @@
       <c r="AV48" s="2" t="inlineStr"/>
       <c r="AW48" t="inlineStr">
         <is>
-          <t>narrateur|Amir attend.
-narrateur|L'eau pousse tout doux.
-narrateur|Une feuille s'écarte.
-narrateur|Puis une autre.
-enfant-m|Le port s'ouvre.
-narrateur|Le bateau avance tout seul jusqu'au chou.</t>
+          <t>enfant-m|J'attends le prochain courant.
+narrateur|Amir garde le bateau contre sa botte.
+narrateur|L'eau pousse lentement la première feuille.
+narrateur|Puis la seconde s'écarte aussi.
+narrateur|Le port s'ouvre juste assez.
+narrateur|Le bateau glisse jusqu'au quai.</t>
         </is>
       </c>
     </row>
@@ -9631,12 +9572,12 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Amir raconte, tout doux. J'ai attendu. Les feuilles ont ouvert le port. Le courant a aidé. Le bateau sent encore un peu le chou. Amir rit. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
+          <t>Le bateau touche enfin le quai de terre. Une odeur de chou monte de sa coque. Amir éclate de rire en rentrant. Ton trésor sent vraiment le potager ! C'est le parfum de mon port. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Amir raconte, tout doux. J'ai attendu. Les feuilles ont ouvert le port. Le courant a aidé. Le bateau sent encore un peu le chou. Amir rit. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
+          <t>Le bateau touche enfin le quai de terre. Une odeur de chou monte de sa coque. Amir éclate de rire en rentrant. Ton trésor sent vraiment le potager ! C'est le parfum de mon port. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -9771,15 +9712,15 @@
       <c r="AV49" s="2" t="inlineStr"/>
       <c r="AW49" t="inlineStr">
         <is>
-          <t>narrateur|Amir raconte, tout doux.
-enfant-m|J'ai attendu.
-enfant-m|Les feuilles ont ouvert le port.
-papa|Le courant a aidé.
-narrateur|Le bateau sent encore un peu le chou.
-narrateur|Amir rit.
-narrateur|À la porte, il retire les bottes.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|Le bateau touche enfin le quai de terre.
+narrateur|Une odeur de chou monte de sa coque.
+narrateur|Amir éclate de rire en rentrant.
+papa|Ton trésor sent vraiment le potager !
+enfant-m|C'est le parfum de mon port.
+narrateur|À la porte, Amir retire ses bottes.
+narrateur|Deux traces rouges restent sur le tapis.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -9806,12 +9747,12 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Maman est venue jusqu'au potager. Maman, je veux jouer sans abîmer les choux. Passe entre les feuilles. Pas dessus. Amir pose le bateau dans l'espace libre. Les plants ne bougent pas. Ton port est gentil avec le jardin.</t>
+          <t>Maman, peux-tu regarder mon port ? Vois-tu cette rigole près du thym ? Amir suit la rigole avec son doigt. Elle contourne toutes les jeunes pousses. Voilà ma route ! Le bateau rejoint le quai sans rien plier.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Maman est venue jusqu'au potager. Maman, je veux jouer sans abîmer les choux. Passe entre les feuilles. Pas dessus. Amir pose le bateau dans l'espace libre. Les plants ne bougent pas. Ton port est gentil avec le jardin.</t>
+          <t>Maman, peux-tu regarder mon port ? Vois-tu cette rigole près du thym ? Amir suit la rigole avec son doigt. Elle contourne toutes les jeunes pousses. Voilà ma route ! Le bateau rejoint le quai sans rien plier.</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -9946,13 +9887,12 @@
       <c r="AV50" s="2" t="inlineStr"/>
       <c r="AW50" t="inlineStr">
         <is>
-          <t>narrateur|Maman est venue jusqu'au potager.
-enfant-m|Maman, je veux jouer sans abîmer les choux.
-maman|Passe entre les feuilles.
-maman|Pas dessus.
-narrateur|Amir pose le bateau dans l'espace libre.
-narrateur|Les plants ne bougent pas.
-maman|Ton port est gentil avec le jardin.</t>
+          <t>enfant-m|Maman, peux-tu regarder mon port ?
+maman|Vois-tu cette rigole près du thym ?
+narrateur|Amir suit la rigole avec son doigt.
+narrateur|Elle contourne toutes les jeunes pousses.
+enfant-m|Voilà ma route !
+narrateur|Le bateau rejoint le quai sans rien plier.</t>
         </is>
       </c>
     </row>
@@ -9979,12 +9919,12 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Merci d'avoir demandé. Le port est dans le jardin. On le garde. Amir pose le bateau. Maman pose la soupe. Deux voyages : l'eau, et la maison. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
+          <t>La rigole conduit le bateau au thym. Une minuscule fleur touche sa voile. Amir rentre avec son bateau parfumé. Tu as trouvé sans écraser mes choux. La route passait près du thym. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Merci d'avoir demandé. Le port est dans le jardin. On le garde. Amir pose le bateau. Maman pose la soupe. Deux voyages : l'eau, et la maison. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
+          <t>La rigole conduit le bateau au thym. Une minuscule fleur touche sa voile. Amir rentre avec son bateau parfumé. Tu as trouvé sans écraser mes choux. La route passait près du thym. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -10119,15 +10059,15 @@
       <c r="AV51" s="2" t="inlineStr"/>
       <c r="AW51" t="inlineStr">
         <is>
-          <t>maman|Merci d'avoir demandé.
-enfant-m|Le port est dans le jardin.
-enfant-m|On le garde.
-narrateur|Amir pose le bateau.
-narrateur|Maman pose la soupe.
-narrateur|Deux voyages : l'eau, et la maison.
-narrateur|À la porte, il retire les bottes.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|La rigole conduit le bateau au thym.
+narrateur|Une minuscule fleur touche sa voile.
+narrateur|Amir rentre avec son bateau parfumé.
+maman|Tu as trouvé sans écraser mes choux.
+enfant-m|La route passait près du thym.
+narrateur|À la porte, Amir retire ses bottes.
+narrateur|Deux traces rouges restent sur le tapis.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -10154,12 +10094,12 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Amir enfile les bottes. Elles s'arrêtent pile au bord du bac. Près du bac à sable. L'eau devient de plus en plus petite. Elle rentre dans le sol. Le bateau n'aurait plus assez d'eau. Mon chemin s'en va dans le sable. Le sable boit la flaque. Amir serre le bateau. Il avait imaginé cette île. Les bottes font clap, déjà, dans l'entrée.</t>
+          <t>Ses bottes s'arrêtent au bord du sable. Devant le bac brille une île ronde. Au milieu repose un caillou blanc. Voilà l'île au trésor ! Amir approche le bateau de l'eau. Mais la flaque devient soudain plus petite. Le sable boit ses derniers reflets. Mon île disparaît ! Il reste encore un peu de temps.</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Amir enfile les bottes. Elles s'arrêtent pile au bord du bac. Près du bac à sable. L'eau devient de plus en plus petite. Elle rentre dans le sol. Le bateau n'aurait plus assez d'eau. Mon chemin s'en va dans le sable. Le sable boit la flaque. Amir serre le bateau. Il avait imaginé cette île. Les bottes font clap, déjà, dans l'entrée.</t>
+          <t>Ses bottes s'arrêtent au bord du sable. Devant le bac brille une île ronde. Au milieu repose un caillou blanc. Voilà l'île au trésor ! Amir approche le bateau de l'eau. Mais la flaque devient soudain plus petite. Le sable boit ses derniers reflets. Mon île disparaît ! Il reste encore un peu de temps.</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -10294,17 +10234,15 @@
       <c r="AV52" s="2" t="inlineStr"/>
       <c r="AW52" t="inlineStr">
         <is>
-          <t>narrateur|Amir enfile les bottes.
-narrateur|Elles s'arrêtent pile au bord du bac.
-narrateur|Près du bac à sable.
-narrateur|L'eau devient de plus en plus petite.
-narrateur|Elle rentre dans le sol.
-narrateur|Le bateau n'aurait plus assez d'eau.
-enfant-m|Mon chemin s'en va dans le sable.
-papa|Le sable boit la flaque.
-narrateur|Amir serre le bateau.
-narrateur|Il avait imaginé cette île.
-narrateur|Les bottes font clap, déjà, dans l'entrée.</t>
+          <t>narrateur|Ses bottes s'arrêtent au bord du sable.
+narrateur|Devant le bac brille une île ronde.
+narrateur|Au milieu repose un caillou blanc.
+enfant-m|Voilà l'île au trésor !
+narrateur|Amir approche le bateau de l'eau.
+narrateur|Mais la flaque devient soudain plus petite.
+narrateur|Le sable boit ses derniers reflets.
+enfant-m|Mon île disparaît !
+papa|Il reste encore un peu de temps.</t>
         </is>
       </c>
     </row>
@@ -10331,12 +10269,12 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit, et il regarde. Comment on fait, capitaine ?</t>
+          <t>Le bateau attend dans les mains d'Amir. Le caillou blanc reste hors d'atteinte. Comment sauver ce voyage ?</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit, et il regarde. Comment on fait, capitaine ?</t>
+          <t>Le bateau attend dans les mains d'Amir. Le caillou blanc reste hors d'atteinte. Comment sauver ce voyage ?</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -10359,7 +10297,7 @@
       <c r="L53" s="2" t="inlineStr"/>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>une autre flaque</t>
+          <t>chercher une autre flaque</t>
         </is>
       </c>
       <c r="N53" s="2" t="inlineStr">
@@ -10369,7 +10307,7 @@
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>sur le sable</t>
+          <t>creuser un petit canal</t>
         </is>
       </c>
       <c r="P53" s="2" t="inlineStr">
@@ -10379,7 +10317,7 @@
       </c>
       <c r="Q53" s="2" t="inlineStr">
         <is>
-          <t>un autre bateau</t>
+          <t>faire une piste de sable</t>
         </is>
       </c>
       <c r="R53" s="2" t="inlineStr">
@@ -10495,8 +10433,9 @@
       <c r="AV53" s="2" t="inlineStr"/>
       <c r="AW53" t="inlineStr">
         <is>
-          <t>narrateur|Amir s'accroupit, et il regarde.
-papa|Comment on fait, capitaine ?</t>
+          <t>narrateur|Le bateau attend dans les mains d'Amir.
+narrateur|Le caillou blanc reste hors d'atteinte.
+papa|Comment sauver ce voyage ?</t>
         </is>
       </c>
     </row>
@@ -10523,12 +10462,12 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Celle-ci s'en va. On prend l'autre. À côté, une flaque plus ronde tient encore. Amir y pose le bateau. Il avance. Ffff. On reprend plus loin, alors.</t>
+          <t>Je cherche une autre flaque. Amir regarde autour du bac. Sous le banc, une eau claire résiste. Il y pose vite son bateau. Le bateau contourne un galet gris. Une nouvelle île !</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Celle-ci s'en va. On prend l'autre. À côté, une flaque plus ronde tient encore. Amir y pose le bateau. Il avance. Ffff. On reprend plus loin, alors.</t>
+          <t>Je cherche une autre flaque. Amir regarde autour du bac. Sous le banc, une eau claire résiste. Il y pose vite son bateau. Le bateau contourne un galet gris. Une nouvelle île !</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -10663,13 +10602,12 @@
       <c r="AV54" s="2" t="inlineStr"/>
       <c r="AW54" t="inlineStr">
         <is>
-          <t>enfant-m|Celle-ci s'en va.
-enfant-m|On prend l'autre.
-narrateur|À côté, une flaque plus ronde tient encore.
-narrateur|Amir y pose le bateau.
-narrateur|Il avance.
-narrateur|Ffff.
-papa|On reprend plus loin, alors.</t>
+          <t>enfant-m|Je cherche une autre flaque.
+narrateur|Amir regarde autour du bac.
+narrateur|Sous le banc, une eau claire résiste.
+narrateur|Il y pose vite son bateau.
+narrateur|Le bateau contourne un galet gris.
+enfant-m|Une nouvelle île !</t>
         </is>
       </c>
     </row>
@@ -10696,12 +10634,12 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>La première flaque est partie. L'autre m'a emmené. Tu as trouvé une autre rivière. Amir hoche la tête. Le bateau sèche près du volet jaune. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
+          <t>Le galet gris devient le nouveau trésor. Amir le laisse près de la flaque. Il rapporte seulement son histoire. L'île a changé, mais le voyage continue. Demain, je chercherai encore. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>La première flaque est partie. L'autre m'a emmené. Tu as trouvé une autre rivière. Amir hoche la tête. Le bateau sèche près du volet jaune. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
+          <t>Le galet gris devient le nouveau trésor. Amir le laisse près de la flaque. Il rapporte seulement son histoire. L'île a changé, mais le voyage continue. Demain, je chercherai encore. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -10836,14 +10774,15 @@
       <c r="AV55" s="2" t="inlineStr"/>
       <c r="AW55" t="inlineStr">
         <is>
-          <t>enfant-m|La première flaque est partie.
-enfant-m|L'autre m'a emmené.
-papa|Tu as trouvé une autre rivière.
-narrateur|Amir hoche la tête.
+          <t>narrateur|Le galet gris devient le nouveau trésor.
+narrateur|Amir le laisse près de la flaque.
+narrateur|Il rapporte seulement son histoire.
+papa|L'île a changé, mais le voyage continue.
+enfant-m|Demain, je chercherai encore.
+narrateur|À la porte, Amir retire ses bottes.
+narrateur|Deux traces rouges restent sur le tapis.
 narrateur|Le bateau sèche près du volet jaune.
-narrateur|À la porte, il retire les bottes.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -10870,12 +10809,12 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Plus d'eau. Alors il marche. Amir pousse le bateau sur le sable humide. Une piste. Le papier glisse. Grain. Grain. Un bateau de terre, pour cette fois.</t>
+          <t>Je creuse un petit canal. Amir prend la pelle du bac. Papa verse doucement un fond d'arrosoir. L'eau suit le canal jusqu'au caillou. Le bateau avance dans cette rivière neuve. L'île revient !</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Plus d'eau. Alors il marche. Amir pousse le bateau sur le sable humide. Une piste. Le papier glisse. Grain. Grain. Un bateau de terre, pour cette fois.</t>
+          <t>Je creuse un petit canal. Amir prend la pelle du bac. Papa verse doucement un fond d'arrosoir. L'eau suit le canal jusqu'au caillou. Le bateau avance dans cette rivière neuve. L'île revient !</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -11010,14 +10949,12 @@
       <c r="AV56" s="2" t="inlineStr"/>
       <c r="AW56" t="inlineStr">
         <is>
-          <t>enfant-m|Plus d'eau.
-enfant-m|Alors il marche.
-narrateur|Amir pousse le bateau sur le sable humide.
-narrateur|Une piste.
-narrateur|Le papier glisse.
-narrateur|Grain.
-narrateur|Grain.
-papa|Un bateau de terre, pour cette fois.</t>
+          <t>enfant-m|Je creuse un petit canal.
+narrateur|Amir prend la pelle du bac.
+narrateur|Papa verse doucement un fond d'arrosoir.
+narrateur|L'eau suit le canal jusqu'au caillou.
+narrateur|Le bateau avance dans cette rivière neuve.
+enfant-m|L'île revient !</t>
         </is>
       </c>
     </row>
@@ -11044,12 +10981,12 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Mon bateau a marché sur le sable. Un capitaine de sable. Un grain reste sur la cheminée rouge. Amir le souffle. Ffff. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
+          <t>Le bateau atteint enfin le caillou blanc. Son reflet danse dans le petit canal. Puis l'eau disparaît doucement dans le sable. J'ai vu mon île revenir. Juste assez longtemps pour ton voyage. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Mon bateau a marché sur le sable. Un capitaine de sable. Un grain reste sur la cheminée rouge. Amir le souffle. Ffff. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
+          <t>Le bateau atteint enfin le caillou blanc. Son reflet danse dans le petit canal. Puis l'eau disparaît doucement dans le sable. J'ai vu mon île revenir. Juste assez longtemps pour ton voyage. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -11184,14 +11121,15 @@
       <c r="AV57" s="2" t="inlineStr"/>
       <c r="AW57" t="inlineStr">
         <is>
-          <t>enfant-m|Mon bateau a marché sur le sable.
-papa|Un capitaine de sable.
-narrateur|Un grain reste sur la cheminée rouge.
-narrateur|Amir le souffle.
-narrateur|Ffff.
-narrateur|À la porte, il retire les bottes.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|Le bateau atteint enfin le caillou blanc.
+narrateur|Son reflet danse dans le petit canal.
+narrateur|Puis l'eau disparaît doucement dans le sable.
+enfant-m|J'ai vu mon île revenir.
+papa|Juste assez longtemps pour ton voyage.
+narrateur|À la porte, Amir retire ses bottes.
+narrateur|Deux traces rouges restent sur le tapis.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -11218,12 +11156,12 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Celui-là est trop fragile. Amir pose le bateau en papier dans le sac. On en fabrique un autre, plus solide. Avec une feuille plus épaisse, ils plient une nouvelle coque. Celui-ci, pour le sable.</t>
+          <t>Je fabrique une piste de sable. Amir tasse une longue bande humide. Il pose la coque bien droite. Puis il souffle dans la voile. Le bateau glisse jusqu'au caillou blanc. Mon bateau roule aussi !</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Celui-là est trop fragile. Amir pose le bateau en papier dans le sac. On en fabrique un autre, plus solide. Avec une feuille plus épaisse, ils plient une nouvelle coque. Celui-ci, pour le sable.</t>
+          <t>Je fabrique une piste de sable. Amir tasse une longue bande humide. Il pose la coque bien droite. Puis il souffle dans la voile. Le bateau glisse jusqu'au caillou blanc. Mon bateau roule aussi !</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -11358,11 +11296,12 @@
       <c r="AV58" s="2" t="inlineStr"/>
       <c r="AW58" t="inlineStr">
         <is>
-          <t>enfant-m|Celui-là est trop fragile.
-narrateur|Amir pose le bateau en papier dans le sac.
-papa|On en fabrique un autre, plus solide.
-narrateur|Avec une feuille plus épaisse, ils plient une nouvelle coque.
-enfant-m|Celui-ci, pour le sable.</t>
+          <t>enfant-m|Je fabrique une piste de sable.
+narrateur|Amir tasse une longue bande humide.
+narrateur|Il pose la coque bien droite.
+narrateur|Puis il souffle dans la voile.
+narrateur|Le bateau glisse jusqu'au caillou blanc.
+enfant-m|Mon bateau roule aussi !</t>
         </is>
       </c>
     </row>
@@ -11389,12 +11328,12 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Deux bateaux maintenant. L'ancien dans le sac. Le nouveau sur la table. Celui-là, on le fera demain. On a bien fait. Le papier fragile se repose. L'autre attend le jardin. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
+          <t>Le devant touche doucement le caillou blanc. Un grain doré reste sur la coque. Amir le montre à papa en rentrant. Un vrai trésor de capitaine. Mon bateau connaît aussi les routes. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Deux bateaux maintenant. L'ancien dans le sac. Le nouveau sur la table. Celui-là, on le fera demain. On a bien fait. Le papier fragile se repose. L'autre attend le jardin. À la porte, il retire les bottes. Le sac se ferme. Zzz.</t>
+          <t>Le devant touche doucement le caillou blanc. Un grain doré reste sur la coque. Amir le montre à papa en rentrant. Un vrai trésor de capitaine. Mon bateau connaît aussi les routes. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -11529,16 +11468,15 @@
       <c r="AV59" s="2" t="inlineStr"/>
       <c r="AW59" t="inlineStr">
         <is>
-          <t>narrateur|Deux bateaux maintenant.
-narrateur|L'ancien dans le sac.
-narrateur|Le nouveau sur la table.
-enfant-m|Celui-là, on le fera demain.
-papa|On a bien fait.
-narrateur|Le papier fragile se repose.
-narrateur|L'autre attend le jardin.
-narrateur|À la porte, il retire les bottes.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|Le devant touche doucement le caillou blanc.
+narrateur|Un grain doré reste sur la coque.
+narrateur|Amir le montre à papa en rentrant.
+papa|Un vrai trésor de capitaine.
+enfant-m|Mon bateau connaît aussi les routes.
+narrateur|À la porte, Amir retire ses bottes.
+narrateur|Deux traces rouges restent sur le tapis.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -11565,12 +11503,12 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Amir met le bateau dans le sac. Toc. La voile rentre sous son doigt. Le linge est sur le radiateur. Il sent le propre. Pour tes mains, après l'eau. Je le prends. Le linge rejoint le bateau dans le sac.</t>
+          <t>Amir choisit d'abord le petit linge bleu. Il est encore chaud du radiateur. À quoi servira-t-il ? À sauver mon bateau mouillé. Amir le roule comme un petit coussin. Le bateau se pose dessus. Le manteau et les bottes sont prêts.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Amir met le bateau dans le sac. Toc. La voile rentre sous son doigt. Le linge est sur le radiateur. Il sent le propre. Pour tes mains, après l'eau. Je le prends. Le linge rejoint le bateau dans le sac.</t>
+          <t>Amir choisit d'abord le petit linge bleu. Il est encore chaud du radiateur. À quoi servira-t-il ? À sauver mon bateau mouillé. Amir le roule comme un petit coussin. Le bateau se pose dessus. Le manteau et les bottes sont prêts.</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -11705,14 +11643,13 @@
       <c r="AV60" s="2" t="inlineStr"/>
       <c r="AW60" t="inlineStr">
         <is>
-          <t>narrateur|Amir met le bateau dans le sac.
-narrateur|Toc.
-narrateur|La voile rentre sous son doigt.
-narrateur|Le linge est sur le radiateur.
-narrateur|Il sent le propre.
-maman|Pour tes mains, après l'eau.
-enfant-m|Je le prends.
-narrateur|Le linge rejoint le bateau dans le sac.</t>
+          <t>narrateur|Amir choisit d'abord le petit linge bleu.
+narrateur|Il est encore chaud du radiateur.
+maman|À quoi servira-t-il ?
+enfant-m|À sauver mon bateau mouillé.
+narrateur|Amir le roule comme un petit coussin.
+narrateur|Le bateau se pose dessus.
+narrateur|Le manteau et les bottes sont prêts.</t>
         </is>
       </c>
     </row>
@@ -11739,19 +11676,19 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
+          <t>Où Amir met-il le petit linge ?</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Où Amir met-il le petit linge ?</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
           <t>On met le linge où ?</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr">
-        <is>
-          <t>On met le linge où ?</t>
-        </is>
-      </c>
-      <c r="G61" s="2" t="inlineStr">
-        <is>
-          <t>On met le linge où ?</t>
-        </is>
-      </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
           <t>dans le sac</t>
@@ -11774,7 +11711,7 @@
       </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>Le linge va dans le sac.</t>
+          <t>Le petit linge va dans le sac.</t>
         </is>
       </c>
       <c r="M61" s="2" t="inlineStr"/>
@@ -11899,7 +11836,7 @@
       </c>
       <c r="AW61" t="inlineStr">
         <is>
-          <t>narrateur|On met le linge où ?</t>
+          <t>narrateur|Où Amir met-il le petit linge ?</t>
         </is>
       </c>
     </row>
@@ -11926,12 +11863,12 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Le linge est dans le sac. Le bateau aussi. On ouvre la porte ? Oui. Le voyage commence.</t>
+          <t>Le linge protège le bateau. Amir ferme doucement le sac. Tout est prêt, capitaine ? Manteau, bottes et bateau !</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Le linge est dans le sac. Le bateau aussi. On ouvre la porte ? Oui. Le voyage commence.</t>
+          <t>Le linge protège le bateau. Amir ferme doucement le sac. Tout est prêt, capitaine ? Manteau, bottes et bateau !</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -12070,11 +12007,10 @@
       </c>
       <c r="AW62" t="inlineStr">
         <is>
-          <t>narrateur|Le linge est dans le sac.
-narrateur|Le bateau aussi.
-papa|On ouvre la porte ?
-enfant-m|Oui.
-enfant-m|Le voyage commence.</t>
+          <t>narrateur|Le linge protège le bateau.
+narrateur|Amir ferme doucement le sac.
+papa|Tout est prêt, capitaine ?
+enfant-m|Manteau, bottes et bateau !</t>
         </is>
       </c>
     </row>
@@ -12101,12 +12037,12 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Dehors, l'eau a fait trois chemins. La rivière de la gouttière. Le port des choux. L'île du bac. Où commence le voyage, capitaine ?</t>
+          <t>Dehors, trois chemins brillent encore. La rivière de la gouttière. Le port caché entre les choux. Puis l'île devant le bac. Quelle route choisis-tu, capitaine ?</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Dehors, l'eau a fait trois chemins. La rivière de la gouttière. Le port des choux. L'île du bac. Où commence le voyage, capitaine ?</t>
+          <t>Dehors, trois chemins brillent encore. La rivière de la gouttière. Le port caché entre les choux. Puis l'île devant le bac. Quelle route choisis-tu, capitaine ?</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -12265,11 +12201,11 @@
       <c r="AV63" s="2" t="inlineStr"/>
       <c r="AW63" t="inlineStr">
         <is>
-          <t>narrateur|Dehors, l'eau a fait trois chemins.
+          <t>narrateur|Dehors, trois chemins brillent encore.
 narrateur|La rivière de la gouttière.
-narrateur|Le port des choux.
-narrateur|L'île du bac.
-papa|Où commence le voyage, capitaine ?</t>
+narrateur|Le port caché entre les choux.
+narrateur|Puis l'île devant le bac.
+papa|Quelle route choisis-tu, capitaine ?</t>
         </is>
       </c>
     </row>
@@ -12296,12 +12232,12 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Amir porte le sac. Le linge est dedans, au chaud. Sous la gouttière, l'eau tremble. Plic. Ploc. Une grosse feuille barre le passage. La rivière est fermée. Le bateau ne peut pas passer. Amir s'accroupit. La feuille ne bouge presque pas. Le linge sent encore le radiateur.</t>
+          <t>Le linge bleu attend dans le sac. Une rigole court sous la gouttière. Amir pose le bateau sur l'eau. Le voyage commence enfin. Soudain, une grande feuille tourne. Elle bouche toute la rivière. Le bateau s'arrête derrière elle. Vite, le soleil revient ! L'eau baisse déjà.</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Amir porte le sac. Le linge est dedans, au chaud. Sous la gouttière, l'eau tremble. Plic. Ploc. Une grosse feuille barre le passage. La rivière est fermée. Le bateau ne peut pas passer. Amir s'accroupit. La feuille ne bouge presque pas. Le linge sent encore le radiateur.</t>
+          <t>Le linge bleu attend dans le sac. Une rigole court sous la gouttière. Amir pose le bateau sur l'eau. Le voyage commence enfin. Soudain, une grande feuille tourne. Elle bouche toute la rivière. Le bateau s'arrête derrière elle. Vite, le soleil revient ! L'eau baisse déjà.</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -12436,17 +12372,15 @@
       <c r="AV64" s="2" t="inlineStr"/>
       <c r="AW64" t="inlineStr">
         <is>
-          <t>narrateur|Amir porte le sac.
-narrateur|Le linge est dedans, au chaud.
-narrateur|Sous la gouttière, l'eau tremble.
-narrateur|Plic.
-narrateur|Ploc.
-narrateur|Une grosse feuille barre le passage.
-enfant-m|La rivière est fermée.
-papa|Le bateau ne peut pas passer.
-narrateur|Amir s'accroupit.
-narrateur|La feuille ne bouge presque pas.
-narrateur|Le linge sent encore le radiateur.</t>
+          <t>narrateur|Le linge bleu attend dans le sac.
+narrateur|Une rigole court sous la gouttière.
+narrateur|Amir pose le bateau sur l'eau.
+narrateur|Le voyage commence enfin.
+narrateur|Soudain, une grande feuille tourne.
+narrateur|Elle bouche toute la rivière.
+narrateur|Le bateau s'arrête derrière elle.
+enfant-m|Vite, le soleil revient !
+papa|L'eau baisse déjà.</t>
         </is>
       </c>
     </row>
@@ -12473,12 +12407,12 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit, et il regarde. Comment on fait, capitaine ?</t>
+          <t>La feuille tient bon. L'eau devient moins profonde. Que tente le capitaine ?</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit, et il regarde. Comment on fait, capitaine ?</t>
+          <t>La feuille tient bon. L'eau devient moins profonde. Que tente le capitaine ?</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -12501,7 +12435,7 @@
       <c r="L65" s="2" t="inlineStr"/>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>attendre les gouttes</t>
+          <t>attendre trois gouttes</t>
         </is>
       </c>
       <c r="N65" s="2" t="inlineStr">
@@ -12511,7 +12445,7 @@
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>appeler papa</t>
+          <t>demander l'aide de papa</t>
         </is>
       </c>
       <c r="P65" s="2" t="inlineStr">
@@ -12521,7 +12455,7 @@
       </c>
       <c r="Q65" s="2" t="inlineStr">
         <is>
-          <t>changer de départ</t>
+          <t>chercher un autre départ</t>
         </is>
       </c>
       <c r="R65" s="2" t="inlineStr">
@@ -12637,8 +12571,9 @@
       <c r="AV65" s="2" t="inlineStr"/>
       <c r="AW65" t="inlineStr">
         <is>
-          <t>narrateur|Amir s'accroupit, et il regarde.
-papa|Comment on fait, capitaine ?</t>
+          <t>narrateur|La feuille tient bon.
+narrateur|L'eau devient moins profonde.
+papa|Que tente le capitaine ?</t>
         </is>
       </c>
     </row>
@@ -12665,12 +12600,12 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit près de la feuille. J'attends encore un peu. Une goutte. Plic. La feuille bouge à peine. Une deuxième. Ploc. La feuille tourne. Une troisième. Plouf. La feuille ouvre un passage. La rivière est libre !</t>
+          <t>J'attends trois gouttes. La première frappe la feuille. La deuxième soulève son bord. La troisième la fait pivoter. Un passage étroit apparaît. Maintenant, petit bateau ! Le bateau file sous une brindille.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit près de la feuille. J'attends encore un peu. Une goutte. Plic. La feuille bouge à peine. Une deuxième. Ploc. La feuille tourne. Une troisième. Plouf. La feuille ouvre un passage. La rivière est libre !</t>
+          <t>J'attends trois gouttes. La première frappe la feuille. La deuxième soulève son bord. La troisième la fait pivoter. Un passage étroit apparaît. Maintenant, petit bateau ! Le bateau file sous une brindille.</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -12805,18 +12740,13 @@
       <c r="AV66" s="2" t="inlineStr"/>
       <c r="AW66" t="inlineStr">
         <is>
-          <t>narrateur|Amir s'accroupit près de la feuille.
-enfant-m|J'attends encore un peu.
-narrateur|Une goutte.
-narrateur|Plic.
-narrateur|La feuille bouge à peine.
-narrateur|Une deuxième.
-narrateur|Ploc.
-narrateur|La feuille tourne.
-narrateur|Une troisième.
-narrateur|Plouf.
-narrateur|La feuille ouvre un passage.
-enfant-m|La rivière est libre !</t>
+          <t>enfant-m|J'attends trois gouttes.
+narrateur|La première frappe la feuille.
+narrateur|La deuxième soulève son bord.
+narrateur|La troisième la fait pivoter.
+narrateur|Un passage étroit apparaît.
+enfant-m|Maintenant, petit bateau !
+narrateur|Le bateau file sous une brindille.</t>
         </is>
       </c>
     </row>
@@ -12843,12 +12773,12 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>De retour, Amir pose le bateau sur le petit linge. Alors, capitaine, jusqu'où es-tu allé ? Très loin. J'ai attendu trois gouttes. C'est vraiment loin. Une dernière goutte, dehors. Plic. Sur le linge, le bateau attend déjà le prochain voyage. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
+          <t>Le bateau atteint le pot violet. Une petite feuille colle devant. Amir la garde comme drapeau. Puis il rentre avant la dernière goutte. Quel trésor rapporte votre navire ? Un drapeau gagné après trois gouttes. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>De retour, Amir pose le bateau sur le petit linge. Alors, capitaine, jusqu'où es-tu allé ? Très loin. J'ai attendu trois gouttes. C'est vraiment loin. Une dernière goutte, dehors. Plic. Sur le linge, le bateau attend déjà le prochain voyage. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
+          <t>Le bateau atteint le pot violet. Une petite feuille colle devant. Amir la garde comme drapeau. Puis il rentre avant la dernière goutte. Quel trésor rapporte votre navire ? Un drapeau gagné après trois gouttes. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -12983,18 +12913,16 @@
       <c r="AV67" s="2" t="inlineStr"/>
       <c r="AW67" t="inlineStr">
         <is>
-          <t>narrateur|De retour, Amir pose le bateau sur le petit linge.
-papa|Alors, capitaine, jusqu'où es-tu allé ?
-enfant-m|Très loin.
-enfant-m|J'ai attendu trois gouttes.
-papa|C'est vraiment loin.
-narrateur|Une dernière goutte, dehors.
-narrateur|Plic.
-narrateur|Sur le linge, le bateau attend déjà le prochain voyage.
-narrateur|Il sèche ses doigts avec le linge.
-narrateur|Le linge rentre.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|Le bateau atteint le pot violet.
+narrateur|Une petite feuille colle devant.
+narrateur|Amir la garde comme drapeau.
+narrateur|Puis il rentre avant la dernière goutte.
+papa|Quel trésor rapporte votre navire ?
+enfant-m|Un drapeau gagné après trois gouttes.
+narrateur|Amir enveloppe le bateau dans le linge.
+narrateur|Une tache humide dessine une petite île.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -13021,12 +12949,12 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu peux bouger la feuille ? On la pousse ensemble. Tout doux. Papa soulève le bord. Amir tient le bateau. La feuille glisse. L'eau circule. C'est à toi, capitaine.</t>
+          <t>Papa, j'ai besoin de toi. Tiens le bateau contre le courant. Papa soulève doucement la feuille. Amir maintient la coque bien droite. Maintenant, laisse-le partir. Le bateau bondit dans l'eau libre.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu peux bouger la feuille ? On la pousse ensemble. Tout doux. Papa soulève le bord. Amir tient le bateau. La feuille glisse. L'eau circule. C'est à toi, capitaine.</t>
+          <t>Papa, j'ai besoin de toi. Tiens le bateau contre le courant. Papa soulève doucement la feuille. Amir maintient la coque bien droite. Maintenant, laisse-le partir. Le bateau bondit dans l'eau libre.</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -13161,14 +13089,12 @@
       <c r="AV68" s="2" t="inlineStr"/>
       <c r="AW68" t="inlineStr">
         <is>
-          <t>enfant-m|Papa, tu peux bouger la feuille ?
-papa|On la pousse ensemble.
-papa|Tout doux.
-narrateur|Papa soulève le bord.
-narrateur|Amir tient le bateau.
-narrateur|La feuille glisse.
-narrateur|L'eau circule.
-papa|C'est à toi, capitaine.</t>
+          <t>enfant-m|Papa, j'ai besoin de toi.
+papa|Tiens le bateau contre le courant.
+narrateur|Papa soulève doucement la feuille.
+narrateur|Amir maintient la coque bien droite.
+papa|Maintenant, laisse-le partir.
+narrateur|Le bateau bondit dans l'eau libre.</t>
         </is>
       </c>
     </row>
@@ -13195,12 +13121,12 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Dans la maison. Amir pose le bateau près de la fenêtre. On a poussé la feuille ensemble. Oui. La rivière a dit oui. Papa reprend sa table. Amir regarde le jardin. La gouttière fait encore un tout petit plic. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
+          <t>Le bateau traverse la rivière délivrée. Une ligne brillante marque sa coque. Amir la montre en rentrant. Nous avons formé un bon équipage. Moi devant, et toi derrière ! Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Dans la maison. Amir pose le bateau près de la fenêtre. On a poussé la feuille ensemble. Oui. La rivière a dit oui. Papa reprend sa table. Amir regarde le jardin. La gouttière fait encore un tout petit plic. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
+          <t>Le bateau traverse la rivière délivrée. Une ligne brillante marque sa coque. Amir la montre en rentrant. Nous avons formé un bon équipage. Moi devant, et toi derrière ! Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -13335,18 +13261,15 @@
       <c r="AV69" s="2" t="inlineStr"/>
       <c r="AW69" t="inlineStr">
         <is>
-          <t>narrateur|Dans la maison.
-narrateur|Amir pose le bateau près de la fenêtre.
-papa|On a poussé la feuille ensemble.
-enfant-m|Oui.
-enfant-m|La rivière a dit oui.
-narrateur|Papa reprend sa table.
-narrateur|Amir regarde le jardin.
-narrateur|La gouttière fait encore un tout petit plic.
-narrateur|Il sèche ses doigts avec le linge.
-narrateur|Le linge rentre.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|Le bateau traverse la rivière délivrée.
+narrateur|Une ligne brillante marque sa coque.
+narrateur|Amir la montre en rentrant.
+papa|Nous avons formé un bon équipage.
+enfant-m|Moi devant, et toi derrière !
+narrateur|Amir enveloppe le bateau dans le linge.
+narrateur|Une tache humide dessine une petite île.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -13373,12 +13296,12 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>On part d'ici, plus loin. Amir pose le bateau après la feuille. Là où l'eau court déjà. Un petit courant emmène le papier sous une brindille. Une autre rivière !</t>
+          <t>Je cherche un autre départ. Amir longe la rivière sans courir. Derrière un pot, l'eau recommence. Il pose le bateau après la feuille. Le courant l'emporte vers les violettes. J'ai trouvé le passage secret !</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>On part d'ici, plus loin. Amir pose le bateau après la feuille. Là où l'eau court déjà. Un petit courant emmène le papier sous une brindille. Une autre rivière !</t>
+          <t>Je cherche un autre départ. Amir longe la rivière sans courir. Derrière un pot, l'eau recommence. Il pose le bateau après la feuille. Le courant l'emporte vers les violettes. J'ai trouvé le passage secret !</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -13513,11 +13436,12 @@
       <c r="AV70" s="2" t="inlineStr"/>
       <c r="AW70" t="inlineStr">
         <is>
-          <t>enfant-m|On part d'ici, plus loin.
-narrateur|Amir pose le bateau après la feuille.
-narrateur|Là où l'eau court déjà.
-narrateur|Un petit courant emmène le papier sous une brindille.
-enfant-m|Une autre rivière !</t>
+          <t>enfant-m|Je cherche un autre départ.
+narrateur|Amir longe la rivière sans courir.
+narrateur|Derrière un pot, l'eau recommence.
+narrateur|Il pose le bateau après la feuille.
+narrateur|Le courant l'emporte vers les violettes.
+enfant-m|J'ai trouvé le passage secret !</t>
         </is>
       </c>
     </row>
@@ -13544,12 +13468,12 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Amir rentre. Le bateau a une brindille collée à la voile. On a trouvé un autre courant. Le bateau a choisi. Amir sourit. Le sac attend près de la porte. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
+          <t>Le courant dépose une brindille sur la voile. Amir rapporte le bateau ainsi décoré. Je reconnais le passage secret. Il commence derrière le grand pot. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Amir rentre. Le bateau a une brindille collée à la voile. On a trouvé un autre courant. Le bateau a choisi. Amir sourit. Le sac attend près de la porte. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
+          <t>Le courant dépose une brindille sur la voile. Amir rapporte le bateau ainsi décoré. Je reconnais le passage secret. Il commence derrière le grand pot. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -13684,16 +13608,14 @@
       <c r="AV71" s="2" t="inlineStr"/>
       <c r="AW71" t="inlineStr">
         <is>
-          <t>narrateur|Amir rentre.
-narrateur|Le bateau a une brindille collée à la voile.
-enfant-m|On a trouvé un autre courant.
-papa|Le bateau a choisi.
-narrateur|Amir sourit.
-narrateur|Le sac attend près de la porte.
-narrateur|Il sèche ses doigts avec le linge.
-narrateur|Le linge rentre.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|Le courant dépose une brindille sur la voile.
+narrateur|Amir rapporte le bateau ainsi décoré.
+papa|Je reconnais le passage secret.
+enfant-m|Il commence derrière le grand pot.
+narrateur|Amir enveloppe le bateau dans le linge.
+narrateur|Une tache humide dessine une petite île.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -13720,12 +13642,12 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Amir porte le sac. Le linge sent encore le radiateur. Entre deux choux, une flaque ronde. Comme un port. Trois petites feuilles flottent devant l'entrée. Les bateaux n'arrivent pas à accoster. Il y a trois feuilles. Amir compte. Une. Deux. Trois. Le linge sent encore le radiateur.</t>
+          <t>Le linge garde encore un peu de chaleur. Entre les choux se cache un port. Trois feuilles flottent devant l'entrée. Le bateau avance vers elles. La première touche sa voile. La deuxième ferme le passage. La troisième frôle un jeune chou. Je ne veux rien abîmer. Amir retient aussitôt son bateau.</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Amir porte le sac. Le linge sent encore le radiateur. Entre deux choux, une flaque ronde. Comme un port. Trois petites feuilles flottent devant l'entrée. Les bateaux n'arrivent pas à accoster. Il y a trois feuilles. Amir compte. Une. Deux. Trois. Le linge sent encore le radiateur.</t>
+          <t>Le linge garde encore un peu de chaleur. Entre les choux se cache un port. Trois feuilles flottent devant l'entrée. Le bateau avance vers elles. La première touche sa voile. La deuxième ferme le passage. La troisième frôle un jeune chou. Je ne veux rien abîmer. Amir retient aussitôt son bateau.</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -13860,18 +13782,15 @@
       <c r="AV72" s="2" t="inlineStr"/>
       <c r="AW72" t="inlineStr">
         <is>
-          <t>narrateur|Amir porte le sac.
-narrateur|Le linge sent encore le radiateur.
-narrateur|Entre deux choux, une flaque ronde.
-narrateur|Comme un port.
-narrateur|Trois petites feuilles flottent devant l'entrée.
-enfant-m|Les bateaux n'arrivent pas à accoster.
-papa|Il y a trois feuilles.
-narrateur|Amir compte.
-narrateur|Une.
-narrateur|Deux.
-narrateur|Trois.
-narrateur|Le linge sent encore le radiateur.</t>
+          <t>narrateur|Le linge garde encore un peu de chaleur.
+narrateur|Entre les choux se cache un port.
+narrateur|Trois feuilles flottent devant l'entrée.
+narrateur|Le bateau avance vers elles.
+narrateur|La première touche sa voile.
+narrateur|La deuxième ferme le passage.
+narrateur|La troisième frôle un jeune chou.
+enfant-m|Je ne veux rien abîmer.
+narrateur|Amir retient aussitôt son bateau.</t>
         </is>
       </c>
     </row>
@@ -13898,12 +13817,12 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit, et il regarde. Comment on fait, capitaine ?</t>
+          <t>Le port semble fermé. Derrière, la terre forme un petit quai. Comment entrera ton bateau ?</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit, et il regarde. Comment on fait, capitaine ?</t>
+          <t>Le port semble fermé. Derrière, la terre forme un petit quai. Comment entrera ton bateau ?</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -13926,7 +13845,7 @@
       <c r="L73" s="2" t="inlineStr"/>
       <c r="M73" s="2" t="inlineStr">
         <is>
-          <t>compter les feuilles</t>
+          <t>compter les passages</t>
         </is>
       </c>
       <c r="N73" s="2" t="inlineStr">
@@ -13946,7 +13865,7 @@
       </c>
       <c r="Q73" s="2" t="inlineStr">
         <is>
-          <t>demander à maman</t>
+          <t>demander conseil à maman</t>
         </is>
       </c>
       <c r="R73" s="2" t="inlineStr">
@@ -14062,8 +13981,9 @@
       <c r="AV73" s="2" t="inlineStr"/>
       <c r="AW73" t="inlineStr">
         <is>
-          <t>narrateur|Amir s'accroupit, et il regarde.
-papa|Comment on fait, capitaine ?</t>
+          <t>narrateur|Le port semble fermé.
+narrateur|Derrière, la terre forme un petit quai.
+maman|Comment entrera ton bateau ?</t>
         </is>
       </c>
     </row>
@@ -14090,12 +14010,12 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Amir compte encore. Une. Deux. Trois. Là. Un espace libre. Il glisse le bateau entre la deuxième. La troisième feuille. Le papier touche un quai de terre. Toc. Celui-ci, c'est le quai Deux.</t>
+          <t>Amir observe les trois feuilles. Une, deux, trois. Entre deux et trois, l'eau brille. Il guide doucement le bateau. Le bateau traverse sans toucher les choux. Quai numéro deux !</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Amir compte encore. Une. Deux. Trois. Là. Un espace libre. Il glisse le bateau entre la deuxième. La troisième feuille. Le papier touche un quai de terre. Toc. Celui-ci, c'est le quai Deux.</t>
+          <t>Amir observe les trois feuilles. Une, deux, trois. Entre deux et trois, l'eau brille. Il guide doucement le bateau. Le bateau traverse sans toucher les choux. Quai numéro deux !</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -14230,17 +14150,12 @@
       <c r="AV74" s="2" t="inlineStr"/>
       <c r="AW74" t="inlineStr">
         <is>
-          <t>narrateur|Amir compte encore.
-narrateur|Une.
-narrateur|Deux.
-narrateur|Trois.
-enfant-m|Là.
-enfant-m|Un espace libre.
-narrateur|Il glisse le bateau entre la deuxième.
-narrateur|La troisième feuille.
-narrateur|Le papier touche un quai de terre.
-narrateur|Toc.
-enfant-m|Celui-ci, c'est le quai Deux.</t>
+          <t>narrateur|Amir observe les trois feuilles.
+enfant-m|Une, deux, trois.
+narrateur|Entre deux et trois, l'eau brille.
+narrateur|Il guide doucement le bateau.
+narrateur|Le bateau traverse sans toucher les choux.
+enfant-m|Quai numéro deux !</t>
         </is>
       </c>
     </row>
@@ -14267,12 +14182,12 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>À table, Amir dit :. Quai Un. Quai Deux. Quai Trois. Ton bateau a visité le port. Sans déranger les choux. Le bateau sèche. Les choux, dehors, restent droits. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
+          <t>Au quai, une feuille devient drapeau. Amir la plante dans le sable humide. Les trois choux restent bien droits. À table, Amir dessine son port. Quel passage as-tu choisi ? Celui entre deux et trois. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>À table, Amir dit :. Quai Un. Quai Deux. Quai Trois. Ton bateau a visité le port. Sans déranger les choux. Le bateau sèche. Les choux, dehors, restent droits. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
+          <t>Au quai, une feuille devient drapeau. Amir la plante dans le sable humide. Les trois choux restent bien droits. À table, Amir dessine son port. Quel passage as-tu choisi ? Celui entre deux et trois. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -14407,18 +14322,16 @@
       <c r="AV75" s="2" t="inlineStr"/>
       <c r="AW75" t="inlineStr">
         <is>
-          <t>narrateur|À table, Amir dit :.
-enfant-m|Quai Un.
-enfant-m|Quai Deux.
-enfant-m|Quai Trois.
-maman|Ton bateau a visité le port.
-enfant-m|Sans déranger les choux.
-narrateur|Le bateau sèche.
-narrateur|Les choux, dehors, restent droits.
-narrateur|Il sèche ses doigts avec le linge.
-narrateur|Le linge rentre.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|Au quai, une feuille devient drapeau.
+narrateur|Amir la plante dans le sable humide.
+narrateur|Les trois choux restent bien droits.
+narrateur|À table, Amir dessine son port.
+maman|Quel passage as-tu choisi ?
+enfant-m|Celui entre deux et trois.
+narrateur|Amir enveloppe le bateau dans le linge.
+narrateur|Une tache humide dessine une petite île.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -14445,12 +14358,12 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Amir attend. L'eau pousse tout doux. Une feuille s'écarte. Puis une autre. Le port s'ouvre. Le bateau avance tout seul jusqu'au chou.</t>
+          <t>J'attends le prochain courant. Amir garde le bateau contre sa botte. L'eau pousse lentement la première feuille. Puis la seconde s'écarte aussi. Le port s'ouvre juste assez. Le bateau glisse jusqu'au quai.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Amir attend. L'eau pousse tout doux. Une feuille s'écarte. Puis une autre. Le port s'ouvre. Le bateau avance tout seul jusqu'au chou.</t>
+          <t>J'attends le prochain courant. Amir garde le bateau contre sa botte. L'eau pousse lentement la première feuille. Puis la seconde s'écarte aussi. Le port s'ouvre juste assez. Le bateau glisse jusqu'au quai.</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -14585,12 +14498,12 @@
       <c r="AV76" s="2" t="inlineStr"/>
       <c r="AW76" t="inlineStr">
         <is>
-          <t>narrateur|Amir attend.
-narrateur|L'eau pousse tout doux.
-narrateur|Une feuille s'écarte.
-narrateur|Puis une autre.
-enfant-m|Le port s'ouvre.
-narrateur|Le bateau avance tout seul jusqu'au chou.</t>
+          <t>enfant-m|J'attends le prochain courant.
+narrateur|Amir garde le bateau contre sa botte.
+narrateur|L'eau pousse lentement la première feuille.
+narrateur|Puis la seconde s'écarte aussi.
+narrateur|Le port s'ouvre juste assez.
+narrateur|Le bateau glisse jusqu'au quai.</t>
         </is>
       </c>
     </row>
@@ -14617,12 +14530,12 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Amir raconte, tout doux. J'ai attendu. Les feuilles ont ouvert le port. Le courant a aidé. Le bateau sent encore un peu le chou. Amir rit. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
+          <t>Le bateau touche enfin le quai de terre. Une odeur de chou monte de sa coque. Amir éclate de rire en rentrant. Ton trésor sent vraiment le potager ! C'est le parfum de mon port. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Amir raconte, tout doux. J'ai attendu. Les feuilles ont ouvert le port. Le courant a aidé. Le bateau sent encore un peu le chou. Amir rit. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
+          <t>Le bateau touche enfin le quai de terre. Une odeur de chou monte de sa coque. Amir éclate de rire en rentrant. Ton trésor sent vraiment le potager ! C'est le parfum de mon port. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -14757,16 +14670,15 @@
       <c r="AV77" s="2" t="inlineStr"/>
       <c r="AW77" t="inlineStr">
         <is>
-          <t>narrateur|Amir raconte, tout doux.
-enfant-m|J'ai attendu.
-enfant-m|Les feuilles ont ouvert le port.
-papa|Le courant a aidé.
-narrateur|Le bateau sent encore un peu le chou.
-narrateur|Amir rit.
-narrateur|Il sèche ses doigts avec le linge.
-narrateur|Le linge rentre.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|Le bateau touche enfin le quai de terre.
+narrateur|Une odeur de chou monte de sa coque.
+narrateur|Amir éclate de rire en rentrant.
+papa|Ton trésor sent vraiment le potager !
+enfant-m|C'est le parfum de mon port.
+narrateur|Amir enveloppe le bateau dans le linge.
+narrateur|Une tache humide dessine une petite île.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -14793,12 +14705,12 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Maman est venue jusqu'au potager. Maman, je veux jouer sans abîmer les choux. Passe entre les feuilles. Pas dessus. Amir pose le bateau dans l'espace libre. Les plants ne bougent pas. Ton port est gentil avec le jardin.</t>
+          <t>Maman, peux-tu regarder mon port ? Vois-tu cette rigole près du thym ? Amir suit la rigole avec son doigt. Elle contourne toutes les jeunes pousses. Voilà ma route ! Le bateau rejoint le quai sans rien plier.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Maman est venue jusqu'au potager. Maman, je veux jouer sans abîmer les choux. Passe entre les feuilles. Pas dessus. Amir pose le bateau dans l'espace libre. Les plants ne bougent pas. Ton port est gentil avec le jardin.</t>
+          <t>Maman, peux-tu regarder mon port ? Vois-tu cette rigole près du thym ? Amir suit la rigole avec son doigt. Elle contourne toutes les jeunes pousses. Voilà ma route ! Le bateau rejoint le quai sans rien plier.</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -14933,13 +14845,12 @@
       <c r="AV78" s="2" t="inlineStr"/>
       <c r="AW78" t="inlineStr">
         <is>
-          <t>narrateur|Maman est venue jusqu'au potager.
-enfant-m|Maman, je veux jouer sans abîmer les choux.
-maman|Passe entre les feuilles.
-maman|Pas dessus.
-narrateur|Amir pose le bateau dans l'espace libre.
-narrateur|Les plants ne bougent pas.
-maman|Ton port est gentil avec le jardin.</t>
+          <t>enfant-m|Maman, peux-tu regarder mon port ?
+maman|Vois-tu cette rigole près du thym ?
+narrateur|Amir suit la rigole avec son doigt.
+narrateur|Elle contourne toutes les jeunes pousses.
+enfant-m|Voilà ma route !
+narrateur|Le bateau rejoint le quai sans rien plier.</t>
         </is>
       </c>
     </row>
@@ -14966,12 +14877,12 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Merci d'avoir demandé. Le port est dans le jardin. On le garde. Amir pose le bateau. Maman pose la soupe. Deux voyages : l'eau, et la maison. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
+          <t>La rigole conduit le bateau au thym. Une minuscule fleur touche sa voile. Amir rentre avec son bateau parfumé. Tu as trouvé sans écraser mes choux. La route passait près du thym. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Merci d'avoir demandé. Le port est dans le jardin. On le garde. Amir pose le bateau. Maman pose la soupe. Deux voyages : l'eau, et la maison. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
+          <t>La rigole conduit le bateau au thym. Une minuscule fleur touche sa voile. Amir rentre avec son bateau parfumé. Tu as trouvé sans écraser mes choux. La route passait près du thym. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -15106,16 +15017,15 @@
       <c r="AV79" s="2" t="inlineStr"/>
       <c r="AW79" t="inlineStr">
         <is>
-          <t>maman|Merci d'avoir demandé.
-enfant-m|Le port est dans le jardin.
-enfant-m|On le garde.
-narrateur|Amir pose le bateau.
-narrateur|Maman pose la soupe.
-narrateur|Deux voyages : l'eau, et la maison.
-narrateur|Il sèche ses doigts avec le linge.
-narrateur|Le linge rentre.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|La rigole conduit le bateau au thym.
+narrateur|Une minuscule fleur touche sa voile.
+narrateur|Amir rentre avec son bateau parfumé.
+maman|Tu as trouvé sans écraser mes choux.
+enfant-m|La route passait près du thym.
+narrateur|Amir enveloppe le bateau dans le linge.
+narrateur|Une tache humide dessine une petite île.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -15142,12 +15052,12 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Amir porte le sac. Le linge attend les mains mouillées. Près du bac à sable. L'eau devient de plus en plus petite. Elle rentre dans le sol. Le bateau n'aurait plus assez d'eau. Mon chemin s'en va dans le sable. Le sable boit la flaque. Amir serre le bateau. Il avait imaginé cette île. Le linge sent encore le radiateur.</t>
+          <t>Le linge attend le bateau mouillé. Devant le bac brille une île ronde. Au milieu repose un caillou blanc. Voilà l'île au trésor ! Amir approche le bateau de l'eau. Mais la flaque devient soudain plus petite. Le sable boit ses derniers reflets. Mon île disparaît ! Il reste encore un peu de temps.</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Amir porte le sac. Le linge attend les mains mouillées. Près du bac à sable. L'eau devient de plus en plus petite. Elle rentre dans le sol. Le bateau n'aurait plus assez d'eau. Mon chemin s'en va dans le sable. Le sable boit la flaque. Amir serre le bateau. Il avait imaginé cette île. Le linge sent encore le radiateur.</t>
+          <t>Le linge attend le bateau mouillé. Devant le bac brille une île ronde. Au milieu repose un caillou blanc. Voilà l'île au trésor ! Amir approche le bateau de l'eau. Mais la flaque devient soudain plus petite. Le sable boit ses derniers reflets. Mon île disparaît ! Il reste encore un peu de temps.</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -15282,17 +15192,15 @@
       <c r="AV80" s="2" t="inlineStr"/>
       <c r="AW80" t="inlineStr">
         <is>
-          <t>narrateur|Amir porte le sac.
-narrateur|Le linge attend les mains mouillées.
-narrateur|Près du bac à sable.
-narrateur|L'eau devient de plus en plus petite.
-narrateur|Elle rentre dans le sol.
-narrateur|Le bateau n'aurait plus assez d'eau.
-enfant-m|Mon chemin s'en va dans le sable.
-papa|Le sable boit la flaque.
-narrateur|Amir serre le bateau.
-narrateur|Il avait imaginé cette île.
-narrateur|Le linge sent encore le radiateur.</t>
+          <t>narrateur|Le linge attend le bateau mouillé.
+narrateur|Devant le bac brille une île ronde.
+narrateur|Au milieu repose un caillou blanc.
+enfant-m|Voilà l'île au trésor !
+narrateur|Amir approche le bateau de l'eau.
+narrateur|Mais la flaque devient soudain plus petite.
+narrateur|Le sable boit ses derniers reflets.
+enfant-m|Mon île disparaît !
+papa|Il reste encore un peu de temps.</t>
         </is>
       </c>
     </row>
@@ -15319,12 +15227,12 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit, et il regarde. Comment on fait, capitaine ?</t>
+          <t>Le bateau attend dans les mains d'Amir. Le caillou blanc reste hors d'atteinte. Comment sauver ce voyage ?</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit, et il regarde. Comment on fait, capitaine ?</t>
+          <t>Le bateau attend dans les mains d'Amir. Le caillou blanc reste hors d'atteinte. Comment sauver ce voyage ?</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -15347,7 +15255,7 @@
       <c r="L81" s="2" t="inlineStr"/>
       <c r="M81" s="2" t="inlineStr">
         <is>
-          <t>une autre flaque</t>
+          <t>chercher une autre flaque</t>
         </is>
       </c>
       <c r="N81" s="2" t="inlineStr">
@@ -15357,7 +15265,7 @@
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>sur le sable</t>
+          <t>creuser un petit canal</t>
         </is>
       </c>
       <c r="P81" s="2" t="inlineStr">
@@ -15367,7 +15275,7 @@
       </c>
       <c r="Q81" s="2" t="inlineStr">
         <is>
-          <t>un autre bateau</t>
+          <t>faire une piste de sable</t>
         </is>
       </c>
       <c r="R81" s="2" t="inlineStr">
@@ -15483,8 +15391,9 @@
       <c r="AV81" s="2" t="inlineStr"/>
       <c r="AW81" t="inlineStr">
         <is>
-          <t>narrateur|Amir s'accroupit, et il regarde.
-papa|Comment on fait, capitaine ?</t>
+          <t>narrateur|Le bateau attend dans les mains d'Amir.
+narrateur|Le caillou blanc reste hors d'atteinte.
+papa|Comment sauver ce voyage ?</t>
         </is>
       </c>
     </row>
@@ -15511,12 +15420,12 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Celle-ci s'en va. On prend l'autre. À côté, une flaque plus ronde tient encore. Amir y pose le bateau. Il avance. Ffff. On reprend plus loin, alors.</t>
+          <t>Je cherche une autre flaque. Amir regarde autour du bac. Sous le banc, une eau claire résiste. Il y pose vite son bateau. Le bateau contourne un galet gris. Une nouvelle île !</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Celle-ci s'en va. On prend l'autre. À côté, une flaque plus ronde tient encore. Amir y pose le bateau. Il avance. Ffff. On reprend plus loin, alors.</t>
+          <t>Je cherche une autre flaque. Amir regarde autour du bac. Sous le banc, une eau claire résiste. Il y pose vite son bateau. Le bateau contourne un galet gris. Une nouvelle île !</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -15651,13 +15560,12 @@
       <c r="AV82" s="2" t="inlineStr"/>
       <c r="AW82" t="inlineStr">
         <is>
-          <t>enfant-m|Celle-ci s'en va.
-enfant-m|On prend l'autre.
-narrateur|À côté, une flaque plus ronde tient encore.
-narrateur|Amir y pose le bateau.
-narrateur|Il avance.
-narrateur|Ffff.
-papa|On reprend plus loin, alors.</t>
+          <t>enfant-m|Je cherche une autre flaque.
+narrateur|Amir regarde autour du bac.
+narrateur|Sous le banc, une eau claire résiste.
+narrateur|Il y pose vite son bateau.
+narrateur|Le bateau contourne un galet gris.
+enfant-m|Une nouvelle île !</t>
         </is>
       </c>
     </row>
@@ -15684,12 +15592,12 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>La première flaque est partie. L'autre m'a emmené. Tu as trouvé une autre rivière. Amir hoche la tête. Le bateau sèche près du volet jaune. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
+          <t>Le galet gris devient le nouveau trésor. Amir le laisse près de la flaque. Il rapporte seulement son histoire. L'île a changé, mais le voyage continue. Demain, je chercherai encore. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>La première flaque est partie. L'autre m'a emmené. Tu as trouvé une autre rivière. Amir hoche la tête. Le bateau sèche près du volet jaune. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
+          <t>Le galet gris devient le nouveau trésor. Amir le laisse près de la flaque. Il rapporte seulement son histoire. L'île a changé, mais le voyage continue. Demain, je chercherai encore. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -15824,15 +15732,15 @@
       <c r="AV83" s="2" t="inlineStr"/>
       <c r="AW83" t="inlineStr">
         <is>
-          <t>enfant-m|La première flaque est partie.
-enfant-m|L'autre m'a emmené.
-papa|Tu as trouvé une autre rivière.
-narrateur|Amir hoche la tête.
+          <t>narrateur|Le galet gris devient le nouveau trésor.
+narrateur|Amir le laisse près de la flaque.
+narrateur|Il rapporte seulement son histoire.
+papa|L'île a changé, mais le voyage continue.
+enfant-m|Demain, je chercherai encore.
+narrateur|Amir enveloppe le bateau dans le linge.
+narrateur|Une tache humide dessine une petite île.
 narrateur|Le bateau sèche près du volet jaune.
-narrateur|Il sèche ses doigts avec le linge.
-narrateur|Le linge rentre.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -15859,12 +15767,12 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Plus d'eau. Alors il marche. Amir pousse le bateau sur le sable humide. Une piste. Le papier glisse. Grain. Grain. Un bateau de terre, pour cette fois.</t>
+          <t>Je creuse un petit canal. Amir prend la pelle du bac. Papa verse doucement un fond d'arrosoir. L'eau suit le canal jusqu'au caillou. Le bateau avance dans cette rivière neuve. L'île revient !</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Plus d'eau. Alors il marche. Amir pousse le bateau sur le sable humide. Une piste. Le papier glisse. Grain. Grain. Un bateau de terre, pour cette fois.</t>
+          <t>Je creuse un petit canal. Amir prend la pelle du bac. Papa verse doucement un fond d'arrosoir. L'eau suit le canal jusqu'au caillou. Le bateau avance dans cette rivière neuve. L'île revient !</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -15999,14 +15907,12 @@
       <c r="AV84" s="2" t="inlineStr"/>
       <c r="AW84" t="inlineStr">
         <is>
-          <t>enfant-m|Plus d'eau.
-enfant-m|Alors il marche.
-narrateur|Amir pousse le bateau sur le sable humide.
-narrateur|Une piste.
-narrateur|Le papier glisse.
-narrateur|Grain.
-narrateur|Grain.
-papa|Un bateau de terre, pour cette fois.</t>
+          <t>enfant-m|Je creuse un petit canal.
+narrateur|Amir prend la pelle du bac.
+narrateur|Papa verse doucement un fond d'arrosoir.
+narrateur|L'eau suit le canal jusqu'au caillou.
+narrateur|Le bateau avance dans cette rivière neuve.
+enfant-m|L'île revient !</t>
         </is>
       </c>
     </row>
@@ -16033,12 +15939,12 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Mon bateau a marché sur le sable. Un capitaine de sable. Un grain reste sur la cheminée rouge. Amir le souffle. Ffff. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
+          <t>Le bateau atteint enfin le caillou blanc. Son reflet danse dans le petit canal. Puis l'eau disparaît doucement dans le sable. J'ai vu mon île revenir. Juste assez longtemps pour ton voyage. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Mon bateau a marché sur le sable. Un capitaine de sable. Un grain reste sur la cheminée rouge. Amir le souffle. Ffff. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
+          <t>Le bateau atteint enfin le caillou blanc. Son reflet danse dans le petit canal. Puis l'eau disparaît doucement dans le sable. J'ai vu mon île revenir. Juste assez longtemps pour ton voyage. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -16173,15 +16079,15 @@
       <c r="AV85" s="2" t="inlineStr"/>
       <c r="AW85" t="inlineStr">
         <is>
-          <t>enfant-m|Mon bateau a marché sur le sable.
-papa|Un capitaine de sable.
-narrateur|Un grain reste sur la cheminée rouge.
-narrateur|Amir le souffle.
-narrateur|Ffff.
-narrateur|Il sèche ses doigts avec le linge.
-narrateur|Le linge rentre.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|Le bateau atteint enfin le caillou blanc.
+narrateur|Son reflet danse dans le petit canal.
+narrateur|Puis l'eau disparaît doucement dans le sable.
+enfant-m|J'ai vu mon île revenir.
+papa|Juste assez longtemps pour ton voyage.
+narrateur|Amir enveloppe le bateau dans le linge.
+narrateur|Une tache humide dessine une petite île.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -16208,12 +16114,12 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Celui-là est trop fragile. Amir pose le bateau en papier dans le sac. On en fabrique un autre, plus solide. Avec une feuille plus épaisse, ils plient une nouvelle coque. Celui-ci, pour le sable.</t>
+          <t>Je fabrique une piste de sable. Amir tasse une longue bande humide. Il pose la coque bien droite. Puis il souffle dans la voile. Le bateau glisse jusqu'au caillou blanc. Mon bateau roule aussi !</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Celui-là est trop fragile. Amir pose le bateau en papier dans le sac. On en fabrique un autre, plus solide. Avec une feuille plus épaisse, ils plient une nouvelle coque. Celui-ci, pour le sable.</t>
+          <t>Je fabrique une piste de sable. Amir tasse une longue bande humide. Il pose la coque bien droite. Puis il souffle dans la voile. Le bateau glisse jusqu'au caillou blanc. Mon bateau roule aussi !</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -16348,11 +16254,12 @@
       <c r="AV86" s="2" t="inlineStr"/>
       <c r="AW86" t="inlineStr">
         <is>
-          <t>enfant-m|Celui-là est trop fragile.
-narrateur|Amir pose le bateau en papier dans le sac.
-papa|On en fabrique un autre, plus solide.
-narrateur|Avec une feuille plus épaisse, ils plient une nouvelle coque.
-enfant-m|Celui-ci, pour le sable.</t>
+          <t>enfant-m|Je fabrique une piste de sable.
+narrateur|Amir tasse une longue bande humide.
+narrateur|Il pose la coque bien droite.
+narrateur|Puis il souffle dans la voile.
+narrateur|Le bateau glisse jusqu'au caillou blanc.
+enfant-m|Mon bateau roule aussi !</t>
         </is>
       </c>
     </row>
@@ -16379,12 +16286,12 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Deux bateaux maintenant. L'ancien dans le sac. Le nouveau sur la table. Celui-là, on le fera demain. On a bien fait. Le papier fragile se repose. L'autre attend le jardin. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
+          <t>Le devant touche doucement le caillou blanc. Un grain doré reste sur la coque. Amir le montre à papa en rentrant. Un vrai trésor de capitaine. Mon bateau connaît aussi les routes. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Deux bateaux maintenant. L'ancien dans le sac. Le nouveau sur la table. Celui-là, on le fera demain. On a bien fait. Le papier fragile se repose. L'autre attend le jardin. Il sèche ses doigts avec le linge. Le linge rentre. Le sac se ferme. Zzz.</t>
+          <t>Le devant touche doucement le caillou blanc. Un grain doré reste sur la coque. Amir le montre à papa en rentrant. Un vrai trésor de capitaine. Mon bateau connaît aussi les routes. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -16519,17 +16426,15 @@
       <c r="AV87" s="2" t="inlineStr"/>
       <c r="AW87" t="inlineStr">
         <is>
-          <t>narrateur|Deux bateaux maintenant.
-narrateur|L'ancien dans le sac.
-narrateur|Le nouveau sur la table.
-enfant-m|Celui-là, on le fera demain.
-papa|On a bien fait.
-narrateur|Le papier fragile se repose.
-narrateur|L'autre attend le jardin.
-narrateur|Il sèche ses doigts avec le linge.
-narrateur|Le linge rentre.
-narrateur|Le sac se ferme.
-narrateur|Zzz.</t>
+          <t>narrateur|Le devant touche doucement le caillou blanc.
+narrateur|Un grain doré reste sur la coque.
+narrateur|Amir le montre à papa en rentrant.
+papa|Un vrai trésor de capitaine.
+enfant-m|Mon bateau connaît aussi les routes.
+narrateur|Amir enveloppe le bateau dans le linge.
+narrateur|Une tache humide dessine une petite île.
+narrateur|Le bateau sèche près du volet jaune.
+narrateur|Dans la cuisine, la soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -16550,7 +16455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16647,6 +16552,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-018): AUT-001 oral, plus de puces numérotées
Les gouttes et les feuilles s'enchaînent. Ouverture et fins liées.
T2 raconte les chemins au lieu de les lister.
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-AUT-001.xlsx
+++ b/stories/arbres/TREE-AUT-001.xlsx
@@ -1197,12 +1197,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Au bout d'une petite rue vit Amir. Sa maison a un jardin minuscule. Ce matin-là, la pluie vient de partir. Les pavés brillent derrière la fenêtre. Maman prépare une soupe dans la cuisine. Papa travaille près du volet jaune. Son ordinateur souffle comme un petit vent. En ce moment, Amir plie une feuille. Un pli devient coque. Un autre pli devient voile. Capitaine Amir est prêt ! Il pousse le bateau vers papa. Le bateau heurte sa pantoufle. Votre navire cherche-t-il la mer ? Oui, mais la mer est très loin. Une goutte tombe dehors. Puis une deuxième rejoint la gouttière. Amir colle son nez contre la vitre. L'eau dessine des chemins dans le jardin. Papa, mon bateau peut voyager ici ! Alors rapporte-nous une grande histoire. Et peut-être un trésor ! Merci, on t'attendra. Maman pose le petit sac près d'Amir. Prépare-toi, avant que le soleil sèche tout.</t>
+          <t>Au bout de la rue, une petite maison. Amir vit là, avec papa et maman. Le jardin derrière est minuscule, encore mouillé. Ce matin-là, la pluie vient de partir. Les pavés brillent derrière la fenêtre. Dans la cuisine, ça sent déjà la soupe. Papa travaille près du volet jaune. Son ordinateur souffle, tout doux. En ce moment, Amir plie une feuille. Les plis font une coque, puis une voile. Capitaine Amir est prêt ! Il pousse le bateau vers la pantoufle de papa. Votre navire cherche-t-il la mer ? Oui, mais la mer est très loin. Une goutte tombe dehors, puis une autre. Amir colle son nez contre la vitre. L'eau a dessiné des chemins dans le jardin. Papa, mon bateau peut voyager ici ! Alors rapporte-nous une grande histoire. Et peut-être un trésor ! Merci, on t'attendra. Maman pose le petit sac près d'Amir. Prépare-toi, avant que le soleil sèche tout.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Au bout d'une petite rue vit Amir. Sa maison a un jardin minuscule. Ce matin-là, la pluie vient de partir. Les pavés brillent derrière la fenêtre. Maman prépare une soupe dans la cuisine. Papa travaille près du volet jaune. Son ordinateur souffle comme un petit vent. En ce moment, Amir plie une feuille. Un pli devient coque. Un autre pli devient voile. Capitaine Amir est prêt ! Il pousse le bateau vers papa. Le bateau heurte sa pantoufle. Votre navire cherche-t-il la mer ? Oui, mais la mer est très loin. Une goutte tombe dehors. Puis une deuxième rejoint la gouttière. Amir colle son nez contre la vitre. L'eau dessine des chemins dans le jardin. Papa, mon bateau peut voyager ici ! Alors rapporte-nous une grande histoire. Et peut-être un trésor ! Merci, on t'attendra. Maman pose le petit sac près d'Amir. Prépare-toi, avant que le soleil sèche tout.</t>
+          <t>Au bout de la rue, une petite maison. Amir vit là, avec papa et maman. Le jardin derrière est minuscule, encore mouillé. Ce matin-là, la pluie vient de partir. Les pavés brillent derrière la fenêtre. Dans la cuisine, ça sent déjà la soupe. Papa travaille près du volet jaune. Son ordinateur souffle, tout doux. En ce moment, Amir plie une feuille. Les plis font une coque, puis une voile. Capitaine Amir est prêt ! Il pousse le bateau vers la pantoufle de papa. Votre navire cherche-t-il la mer ? Oui, mais la mer est très loin. Une goutte tombe dehors, puis une autre. Amir colle son nez contre la vitre. L'eau a dessiné des chemins dans le jardin. Papa, mon bateau peut voyager ici ! Alors rapporte-nous une grande histoire. Et peut-être un trésor ! Merci, on t'attendra. Maman pose le petit sac près d'Amir. Prépare-toi, avant que le soleil sèche tout.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1337,25 +1337,23 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Au bout d'une petite rue vit Amir.
-narrateur|Sa maison a un jardin minuscule.
+          <t>narrateur|Au bout de la rue, une petite maison.
+narrateur|Amir vit là, avec papa et maman.
+narrateur|Le jardin derrière est minuscule, encore mouillé.
 narrateur|Ce matin-là, la pluie vient de partir.
 narrateur|Les pavés brillent derrière la fenêtre.
-narrateur|Maman prépare une soupe dans la cuisine.
+narrateur|Dans la cuisine, ça sent déjà la soupe.
 narrateur|Papa travaille près du volet jaune.
-narrateur|Son ordinateur souffle comme un petit vent.
+narrateur|Son ordinateur souffle, tout doux.
 narrateur|En ce moment, Amir plie une feuille.
-narrateur|Un pli devient coque.
-narrateur|Un autre pli devient voile.
+narrateur|Les plis font une coque, puis une voile.
 enfant-m|Capitaine Amir est prêt !
-narrateur|Il pousse le bateau vers papa.
-narrateur|Le bateau heurte sa pantoufle.
+narrateur|Il pousse le bateau vers la pantoufle de papa.
 papa|Votre navire cherche-t-il la mer ?
 enfant-m|Oui, mais la mer est très loin.
-narrateur|Une goutte tombe dehors.
-narrateur|Puis une deuxième rejoint la gouttière.
+narrateur|Une goutte tombe dehors, puis une autre.
 narrateur|Amir colle son nez contre la vitre.
-narrateur|L'eau dessine des chemins dans le jardin.
+narrateur|L'eau a dessiné des chemins dans le jardin.
 enfant-m|Papa, mon bateau peut voyager ici !
 papa|Alors rapporte-nous une grande histoire.
 enfant-m|Et peut-être un trésor !
@@ -1388,12 +1386,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Amir doit préparer trois choses. Son manteau, ses bottes et un linge. Laquelle prépares-tu d'abord ?</t>
+          <t>Avant de sortir, Amir prépare ses affaires. Il y a le manteau, les bottes, et le linge. Laquelle prépares-tu d'abord ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Amir doit préparer trois choses. Son manteau, ses bottes et un linge. Laquelle prépares-tu d'abord ?</t>
+          <t>Avant de sortir, Amir prépare ses affaires. Il y a le manteau, les bottes, et le linge. Laquelle prépares-tu d'abord ?</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -1556,8 +1554,8 @@
       <c r="AV3" s="2" t="inlineStr"/>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Amir doit préparer trois choses.
-narrateur|Son manteau, ses bottes et un linge.
+          <t>narrateur|Avant de sortir, Amir prépare ses affaires.
+narrateur|Il y a le manteau, les bottes, et le linge.
 maman|Laquelle prépares-tu d'abord ?</t>
         </is>
       </c>
@@ -1585,12 +1583,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Amir choisit d'abord son manteau jaune. Il cherche la manche retournée. Je l'ai trouvée ! Il remet la manche dans le bon sens. Ton manteau est prêt. Amir glisse ensuite le bateau dans le sac. Maman ajoute le petit linge. Les bottes attendent près de la porte.</t>
+          <t>Amir cherche d'abord son manteau jaune. Une manche est encore retournée. Je l'ai trouvée ! Il la remet dans le bon sens. Ton manteau est prêt. Ensuite, le bateau glisse dans le sac. Maman glisse le petit linge à côté. Les bottes attendent déjà près de la porte.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Amir choisit d'abord son manteau jaune. Il cherche la manche retournée. Je l'ai trouvée ! Il remet la manche dans le bon sens. Ton manteau est prêt. Amir glisse ensuite le bateau dans le sac. Maman ajoute le petit linge. Les bottes attendent près de la porte.</t>
+          <t>Amir cherche d'abord son manteau jaune. Une manche est encore retournée. Je l'ai trouvée ! Il la remet dans le bon sens. Ton manteau est prêt. Ensuite, le bateau glisse dans le sac. Maman glisse le petit linge à côté. Les bottes attendent déjà près de la porte.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1725,14 +1723,14 @@
       <c r="AV4" s="2" t="inlineStr"/>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Amir choisit d'abord son manteau jaune.
-narrateur|Il cherche la manche retournée.
+          <t>narrateur|Amir cherche d'abord son manteau jaune.
+narrateur|Une manche est encore retournée.
 enfant-m|Je l'ai trouvée !
-narrateur|Il remet la manche dans le bon sens.
+narrateur|Il la remet dans le bon sens.
 maman|Ton manteau est prêt.
-narrateur|Amir glisse ensuite le bateau dans le sac.
-narrateur|Maman ajoute le petit linge.
-narrateur|Les bottes attendent près de la porte.</t>
+narrateur|Ensuite, le bateau glisse dans le sac.
+narrateur|Maman glisse le petit linge à côté.
+narrateur|Les bottes attendent déjà près de la porte.</t>
         </is>
       </c>
     </row>
@@ -1946,12 +1944,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le bateau repose au fond du sac. Le linge protège sa voile. Bottes aux pieds, capitaine ? Bottes aux pieds, manteau fermé !</t>
+          <t>Le bateau repose au fond du sac, sous le linge. Bottes aux pieds, capitaine ? Bottes aux pieds, manteau fermé !</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le bateau repose au fond du sac. Le linge protège sa voile. Bottes aux pieds, capitaine ? Bottes aux pieds, manteau fermé !</t>
+          <t>Le bateau repose au fond du sac, sous le linge. Bottes aux pieds, capitaine ? Bottes aux pieds, manteau fermé !</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2090,8 +2088,7 @@
       </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le bateau repose au fond du sac.
-narrateur|Le linge protège sa voile.
+          <t>narrateur|Le bateau repose au fond du sac, sous le linge.
 papa|Bottes aux pieds, capitaine ?
 enfant-m|Bottes aux pieds, manteau fermé !</t>
         </is>
@@ -2120,12 +2117,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Dehors, trois chemins brillent encore. La rivière de la gouttière. Le port caché entre les choux. Puis l'île devant le bac. Quelle route choisis-tu, capitaine ?</t>
+          <t>Dehors, l'eau brille encore un peu. Un chemin part de la gouttière. Un autre se cache entre les choux. Le bac a l'air d'une petite île. Quelle route choisis-tu, capitaine ?</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Dehors, trois chemins brillent encore. La rivière de la gouttière. Le port caché entre les choux. Puis l'île devant le bac. Quelle route choisis-tu, capitaine ?</t>
+          <t>Dehors, l'eau brille encore un peu. Un chemin part de la gouttière. Un autre se cache entre les choux. Le bac a l'air d'une petite île. Quelle route choisis-tu, capitaine ?</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -2284,10 +2281,10 @@
       <c r="AV7" s="2" t="inlineStr"/>
       <c r="AW7" t="inlineStr">
         <is>
-          <t>narrateur|Dehors, trois chemins brillent encore.
-narrateur|La rivière de la gouttière.
-narrateur|Le port caché entre les choux.
-narrateur|Puis l'île devant le bac.
+          <t>narrateur|Dehors, l'eau brille encore un peu.
+narrateur|Un chemin part de la gouttière.
+narrateur|Un autre se cache entre les choux.
+narrateur|Le bac a l'air d'une petite île.
 papa|Quelle route choisis-tu, capitaine ?</t>
         </is>
       </c>
@@ -2315,12 +2312,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Le manteau jaune brille sous la gouttière. Une rigole court sous la gouttière. Amir pose le bateau sur l'eau. Le voyage commence enfin. Soudain, une grande feuille tourne. Elle bouche toute la rivière. Le bateau s'arrête derrière elle. Vite, le soleil revient ! L'eau baisse déjà.</t>
+          <t>Le manteau jaune brille encore sous la gouttière. Une rigole court encore sous la gouttière. Amir pose le bateau sur l'eau, tout doux. Le voyage commence, enfin. Soudain, une grande feuille tourne et bouche tout. Le bateau s'arrête juste derrière. Vite, le soleil revient ! L'eau baisse déjà.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Le manteau jaune brille sous la gouttière. Une rigole court sous la gouttière. Amir pose le bateau sur l'eau. Le voyage commence enfin. Soudain, une grande feuille tourne. Elle bouche toute la rivière. Le bateau s'arrête derrière elle. Vite, le soleil revient ! L'eau baisse déjà.</t>
+          <t>Le manteau jaune brille encore sous la gouttière. Une rigole court encore sous la gouttière. Amir pose le bateau sur l'eau, tout doux. Le voyage commence, enfin. Soudain, une grande feuille tourne et bouche tout. Le bateau s'arrête juste derrière. Vite, le soleil revient ! L'eau baisse déjà.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -2455,13 +2452,12 @@
       <c r="AV8" s="2" t="inlineStr"/>
       <c r="AW8" t="inlineStr">
         <is>
-          <t>narrateur|Le manteau jaune brille sous la gouttière.
-narrateur|Une rigole court sous la gouttière.
-narrateur|Amir pose le bateau sur l'eau.
-narrateur|Le voyage commence enfin.
-narrateur|Soudain, une grande feuille tourne.
-narrateur|Elle bouche toute la rivière.
-narrateur|Le bateau s'arrête derrière elle.
+          <t>narrateur|Le manteau jaune brille encore sous la gouttière.
+narrateur|Une rigole court encore sous la gouttière.
+narrateur|Amir pose le bateau sur l'eau, tout doux.
+narrateur|Le voyage commence, enfin.
+narrateur|Soudain, une grande feuille tourne et bouche tout.
+narrateur|Le bateau s'arrête juste derrière.
 enfant-m|Vite, le soleil revient !
 papa|L'eau baisse déjà.</t>
         </is>
@@ -2490,12 +2486,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>La feuille tient bon. L'eau devient moins profonde. Que tente le capitaine ?</t>
+          <t>La feuille tient bon, et l'eau baisse. Que tente le capitaine ?</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>La feuille tient bon. L'eau devient moins profonde. Que tente le capitaine ?</t>
+          <t>La feuille tient bon, et l'eau baisse. Que tente le capitaine ?</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -2654,8 +2650,7 @@
       <c r="AV9" s="2" t="inlineStr"/>
       <c r="AW9" t="inlineStr">
         <is>
-          <t>narrateur|La feuille tient bon.
-narrateur|L'eau devient moins profonde.
+          <t>narrateur|La feuille tient bon, et l'eau baisse.
 papa|Que tente le capitaine ?</t>
         </is>
       </c>
@@ -2683,12 +2678,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>J'attends trois gouttes. La première frappe la feuille. La deuxième soulève son bord. La troisième la fait pivoter. Un passage étroit apparaît. Maintenant, petit bateau ! Le bateau file sous une brindille.</t>
+          <t>J'attends trois gouttes. Une goutte frappe la feuille. Puis une autre soulève le bord. La dernière la fait pivoter. Un passage étroit apparaît. Maintenant, petit bateau ! Le bateau file sous une brindille.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>J'attends trois gouttes. La première frappe la feuille. La deuxième soulève son bord. La troisième la fait pivoter. Un passage étroit apparaît. Maintenant, petit bateau ! Le bateau file sous une brindille.</t>
+          <t>J'attends trois gouttes. Une goutte frappe la feuille. Puis une autre soulève le bord. La dernière la fait pivoter. Un passage étroit apparaît. Maintenant, petit bateau ! Le bateau file sous une brindille.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -2824,9 +2819,9 @@
       <c r="AW10" t="inlineStr">
         <is>
           <t>enfant-m|J'attends trois gouttes.
-narrateur|La première frappe la feuille.
-narrateur|La deuxième soulève son bord.
-narrateur|La troisième la fait pivoter.
+narrateur|Une goutte frappe la feuille.
+narrateur|Puis une autre soulève le bord.
+narrateur|La dernière la fait pivoter.
 narrateur|Un passage étroit apparaît.
 enfant-m|Maintenant, petit bateau !
 narrateur|Le bateau file sous une brindille.</t>
@@ -2856,12 +2851,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Le bateau atteint le pot violet. Une petite feuille colle devant. Amir la garde comme drapeau. Puis il rentre avant la dernière goutte. Quel trésor rapporte votre navire ? Un drapeau gagné après trois gouttes. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau atteint le pot violet. Une petite feuille colle devant. Amir la garde comme drapeau. Puis il rentre avant la dernière goutte. Quel trésor rapporte votre navire ? Un drapeau gagné après trois gouttes. À la porte, Amir suspend son manteau. Une goutte glisse encore de la capuche. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Le bateau atteint le pot violet. Une petite feuille colle devant. Amir la garde comme drapeau. Puis il rentre avant la dernière goutte. Quel trésor rapporte votre navire ? Un drapeau gagné après trois gouttes. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau atteint le pot violet. Une petite feuille colle devant. Amir la garde comme drapeau. Puis il rentre avant la dernière goutte. Quel trésor rapporte votre navire ? Un drapeau gagné après trois gouttes. À la porte, Amir suspend son manteau. Une goutte glisse encore de la capuche. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -3002,10 +2997,10 @@
 narrateur|Puis il rentre avant la dernière goutte.
 papa|Quel trésor rapporte votre navire ?
 enfant-m|Un drapeau gagné après trois gouttes.
-narrateur|Amir suspend son manteau jaune.
-narrateur|Une goutte tombe de sa capuche.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|À la porte, Amir suspend son manteau.
+narrateur|Une goutte glisse encore de la capuche.
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -3204,12 +3199,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Le bateau traverse la rivière délivrée. Une ligne brillante marque sa coque. Amir la montre en rentrant. Nous avons formé un bon équipage. Moi devant, et toi derrière ! Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau traverse la rivière délivrée. Une ligne brillante marque sa coque. Amir la montre en rentrant. Nous avons formé un bon équipage. Moi devant, et toi derrière ! À la porte, Amir suspend son manteau. Une goutte glisse encore de la capuche. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Le bateau traverse la rivière délivrée. Une ligne brillante marque sa coque. Amir la montre en rentrant. Nous avons formé un bon équipage. Moi devant, et toi derrière ! Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau traverse la rivière délivrée. Une ligne brillante marque sa coque. Amir la montre en rentrant. Nous avons formé un bon équipage. Moi devant, et toi derrière ! À la porte, Amir suspend son manteau. Une goutte glisse encore de la capuche. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -3349,10 +3344,10 @@
 narrateur|Amir la montre en rentrant.
 papa|Nous avons formé un bon équipage.
 enfant-m|Moi devant, et toi derrière !
-narrateur|Amir suspend son manteau jaune.
-narrateur|Une goutte tombe de sa capuche.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|À la porte, Amir suspend son manteau.
+narrateur|Une goutte glisse encore de la capuche.
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -3551,12 +3546,12 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Le courant dépose une brindille sur la voile. Amir rapporte le bateau ainsi décoré. Je reconnais le passage secret. Il commence derrière le grand pot. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le courant dépose une brindille sur la voile. Amir rapporte le bateau ainsi décoré. Je reconnais le passage secret. Il commence derrière le grand pot. À la porte, Amir suspend son manteau. Une goutte glisse encore de la capuche. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Le courant dépose une brindille sur la voile. Amir rapporte le bateau ainsi décoré. Je reconnais le passage secret. Il commence derrière le grand pot. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le courant dépose une brindille sur la voile. Amir rapporte le bateau ainsi décoré. Je reconnais le passage secret. Il commence derrière le grand pot. À la porte, Amir suspend son manteau. Une goutte glisse encore de la capuche. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -3695,10 +3690,10 @@
 narrateur|Amir rapporte le bateau ainsi décoré.
 papa|Je reconnais le passage secret.
 enfant-m|Il commence derrière le grand pot.
-narrateur|Amir suspend son manteau jaune.
-narrateur|Une goutte tombe de sa capuche.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|À la porte, Amir suspend son manteau.
+narrateur|Une goutte glisse encore de la capuche.
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -3725,12 +3720,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Une odeur de soupe reste dans son col. Entre les choux se cache un port. Trois feuilles flottent devant l'entrée. Le bateau avance vers elles. La première touche sa voile. La deuxième ferme le passage. La troisième frôle un jeune chou. Je ne veux rien abîmer. Amir retient aussitôt son bateau.</t>
+          <t>Une odeur de soupe reste dans son col. Entre les choux se cache un petit port. Trois feuilles flottent devant l'entrée. Le bateau avance, tout doucement. L'une touche sa voile. Une autre ferme le passage. La dernière frôle un jeune chou. Je ne veux rien abîmer. Amir retient aussitôt son bateau.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Une odeur de soupe reste dans son col. Entre les choux se cache un port. Trois feuilles flottent devant l'entrée. Le bateau avance vers elles. La première touche sa voile. La deuxième ferme le passage. La troisième frôle un jeune chou. Je ne veux rien abîmer. Amir retient aussitôt son bateau.</t>
+          <t>Une odeur de soupe reste dans son col. Entre les choux se cache un petit port. Trois feuilles flottent devant l'entrée. Le bateau avance, tout doucement. L'une touche sa voile. Une autre ferme le passage. La dernière frôle un jeune chou. Je ne veux rien abîmer. Amir retient aussitôt son bateau.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -3866,12 +3861,12 @@
       <c r="AW16" t="inlineStr">
         <is>
           <t>narrateur|Une odeur de soupe reste dans son col.
-narrateur|Entre les choux se cache un port.
+narrateur|Entre les choux se cache un petit port.
 narrateur|Trois feuilles flottent devant l'entrée.
-narrateur|Le bateau avance vers elles.
-narrateur|La première touche sa voile.
-narrateur|La deuxième ferme le passage.
-narrateur|La troisième frôle un jeune chou.
+narrateur|Le bateau avance, tout doucement.
+narrateur|L'une touche sa voile.
+narrateur|Une autre ferme le passage.
+narrateur|La dernière frôle un jeune chou.
 enfant-m|Je ne veux rien abîmer.
 narrateur|Amir retient aussitôt son bateau.</t>
         </is>
@@ -4265,12 +4260,12 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Au quai, une feuille devient drapeau. Amir la plante dans le sable humide. Les trois choux restent bien droits. À table, Amir dessine son port. Quel passage as-tu choisi ? Celui entre deux et trois. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Au quai, une feuille devient drapeau. Amir la plante dans le sable humide. Les trois choux restent bien droits. À table, Amir dessine son port. Quel passage as-tu choisi ? Celui entre deux et trois. À la porte, Amir suspend son manteau. Une goutte glisse encore de la capuche. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Au quai, une feuille devient drapeau. Amir la plante dans le sable humide. Les trois choux restent bien droits. À table, Amir dessine son port. Quel passage as-tu choisi ? Celui entre deux et trois. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Au quai, une feuille devient drapeau. Amir la plante dans le sable humide. Les trois choux restent bien droits. À table, Amir dessine son port. Quel passage as-tu choisi ? Celui entre deux et trois. À la porte, Amir suspend son manteau. Une goutte glisse encore de la capuche. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -4411,10 +4406,10 @@
 narrateur|À table, Amir dessine son port.
 maman|Quel passage as-tu choisi ?
 enfant-m|Celui entre deux et trois.
-narrateur|Amir suspend son manteau jaune.
-narrateur|Une goutte tombe de sa capuche.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|À la porte, Amir suspend son manteau.
+narrateur|Une goutte glisse encore de la capuche.
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -4441,12 +4436,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>J'attends le prochain courant. Amir garde le bateau contre sa botte. L'eau pousse lentement la première feuille. Puis la seconde s'écarte aussi. Le port s'ouvre juste assez. Le bateau glisse jusqu'au quai.</t>
+          <t>J'attends le prochain courant. Amir garde le bateau contre sa botte. L'eau pousse lentement une feuille. Puis une autre s'écarte aussi. Le port s'ouvre juste assez. Le bateau glisse jusqu'au quai.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>J'attends le prochain courant. Amir garde le bateau contre sa botte. L'eau pousse lentement la première feuille. Puis la seconde s'écarte aussi. Le port s'ouvre juste assez. Le bateau glisse jusqu'au quai.</t>
+          <t>J'attends le prochain courant. Amir garde le bateau contre sa botte. L'eau pousse lentement une feuille. Puis une autre s'écarte aussi. Le port s'ouvre juste assez. Le bateau glisse jusqu'au quai.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -4583,8 +4578,8 @@
         <is>
           <t>enfant-m|J'attends le prochain courant.
 narrateur|Amir garde le bateau contre sa botte.
-narrateur|L'eau pousse lentement la première feuille.
-narrateur|Puis la seconde s'écarte aussi.
+narrateur|L'eau pousse lentement une feuille.
+narrateur|Puis une autre s'écarte aussi.
 narrateur|Le port s'ouvre juste assez.
 narrateur|Le bateau glisse jusqu'au quai.</t>
         </is>
@@ -4613,12 +4608,12 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Le bateau touche enfin le quai de terre. Une odeur de chou monte de sa coque. Amir éclate de rire en rentrant. Ton trésor sent vraiment le potager ! C'est le parfum de mon port. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau touche enfin le quai de terre. Une odeur de chou monte de sa coque. Amir éclate de rire en rentrant. Ton trésor sent vraiment le potager ! C'est le parfum de mon port. À la porte, Amir suspend son manteau. Une goutte glisse encore de la capuche. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Le bateau touche enfin le quai de terre. Une odeur de chou monte de sa coque. Amir éclate de rire en rentrant. Ton trésor sent vraiment le potager ! C'est le parfum de mon port. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau touche enfin le quai de terre. Une odeur de chou monte de sa coque. Amir éclate de rire en rentrant. Ton trésor sent vraiment le potager ! C'est le parfum de mon port. À la porte, Amir suspend son manteau. Une goutte glisse encore de la capuche. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -4758,10 +4753,10 @@
 narrateur|Amir éclate de rire en rentrant.
 papa|Ton trésor sent vraiment le potager !
 enfant-m|C'est le parfum de mon port.
-narrateur|Amir suspend son manteau jaune.
-narrateur|Une goutte tombe de sa capuche.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|À la porte, Amir suspend son manteau.
+narrateur|Une goutte glisse encore de la capuche.
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -4960,12 +4955,12 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>La rigole conduit le bateau au thym. Une minuscule fleur touche sa voile. Amir rentre avec son bateau parfumé. Tu as trouvé sans écraser mes choux. La route passait près du thym. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>La rigole conduit le bateau au thym. Une minuscule fleur touche sa voile. Amir rentre avec son bateau parfumé. Tu as trouvé sans écraser mes choux. La route passait près du thym. À la porte, Amir suspend son manteau. Une goutte glisse encore de la capuche. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>La rigole conduit le bateau au thym. Une minuscule fleur touche sa voile. Amir rentre avec son bateau parfumé. Tu as trouvé sans écraser mes choux. La route passait près du thym. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>La rigole conduit le bateau au thym. Une minuscule fleur touche sa voile. Amir rentre avec son bateau parfumé. Tu as trouvé sans écraser mes choux. La route passait près du thym. À la porte, Amir suspend son manteau. Une goutte glisse encore de la capuche. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -5105,10 +5100,10 @@
 narrateur|Amir rentre avec son bateau parfumé.
 maman|Tu as trouvé sans écraser mes choux.
 enfant-m|La route passait près du thym.
-narrateur|Amir suspend son manteau jaune.
-narrateur|Une goutte tombe de sa capuche.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|À la porte, Amir suspend son manteau.
+narrateur|Une goutte glisse encore de la capuche.
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -5675,12 +5670,12 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Le galet gris devient le nouveau trésor. Amir le laisse près de la flaque. Il rapporte seulement son histoire. L'île a changé, mais le voyage continue. Demain, je chercherai encore. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le galet gris devient le nouveau trésor. Amir le laisse près de la flaque. Il rapporte seulement son histoire. L'île a changé, mais le voyage continue. Demain, je chercherai encore. À la porte, Amir suspend son manteau. Une goutte glisse encore de la capuche. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Le galet gris devient le nouveau trésor. Amir le laisse près de la flaque. Il rapporte seulement son histoire. L'île a changé, mais le voyage continue. Demain, je chercherai encore. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le galet gris devient le nouveau trésor. Amir le laisse près de la flaque. Il rapporte seulement son histoire. L'île a changé, mais le voyage continue. Demain, je chercherai encore. À la porte, Amir suspend son manteau. Une goutte glisse encore de la capuche. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -5820,10 +5815,10 @@
 narrateur|Il rapporte seulement son histoire.
 papa|L'île a changé, mais le voyage continue.
 enfant-m|Demain, je chercherai encore.
-narrateur|Amir suspend son manteau jaune.
-narrateur|Une goutte tombe de sa capuche.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|À la porte, Amir suspend son manteau.
+narrateur|Une goutte glisse encore de la capuche.
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -6022,12 +6017,12 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Le bateau atteint enfin le caillou blanc. Son reflet danse dans le petit canal. Puis l'eau disparaît doucement dans le sable. J'ai vu mon île revenir. Juste assez longtemps pour ton voyage. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau atteint enfin le caillou blanc. Son reflet danse dans le petit canal. Puis l'eau disparaît doucement dans le sable. J'ai vu mon île revenir. Juste assez longtemps pour ton voyage. À la porte, Amir suspend son manteau. Une goutte glisse encore de la capuche. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Le bateau atteint enfin le caillou blanc. Son reflet danse dans le petit canal. Puis l'eau disparaît doucement dans le sable. J'ai vu mon île revenir. Juste assez longtemps pour ton voyage. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau atteint enfin le caillou blanc. Son reflet danse dans le petit canal. Puis l'eau disparaît doucement dans le sable. J'ai vu mon île revenir. Juste assez longtemps pour ton voyage. À la porte, Amir suspend son manteau. Une goutte glisse encore de la capuche. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -6167,10 +6162,10 @@
 narrateur|Puis l'eau disparaît doucement dans le sable.
 enfant-m|J'ai vu mon île revenir.
 papa|Juste assez longtemps pour ton voyage.
-narrateur|Amir suspend son manteau jaune.
-narrateur|Une goutte tombe de sa capuche.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|À la porte, Amir suspend son manteau.
+narrateur|Une goutte glisse encore de la capuche.
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -6369,12 +6364,12 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Le devant touche doucement le caillou blanc. Un grain doré reste sur la coque. Amir le montre à papa en rentrant. Un vrai trésor de capitaine. Mon bateau connaît aussi les routes. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le devant touche doucement le caillou blanc. Un grain doré reste sur la coque. Amir le montre à papa en rentrant. Un vrai trésor de capitaine. Mon bateau connaît aussi les routes. À la porte, Amir suspend son manteau. Une goutte glisse encore de la capuche. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Le devant touche doucement le caillou blanc. Un grain doré reste sur la coque. Amir le montre à papa en rentrant. Un vrai trésor de capitaine. Mon bateau connaît aussi les routes. Amir suspend son manteau jaune. Une goutte tombe de sa capuche. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le devant touche doucement le caillou blanc. Un grain doré reste sur la coque. Amir le montre à papa en rentrant. Un vrai trésor de capitaine. Mon bateau connaît aussi les routes. À la porte, Amir suspend son manteau. Une goutte glisse encore de la capuche. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -6514,10 +6509,10 @@
 narrateur|Amir le montre à papa en rentrant.
 papa|Un vrai trésor de capitaine.
 enfant-m|Mon bateau connaît aussi les routes.
-narrateur|Amir suspend son manteau jaune.
-narrateur|Une goutte tombe de sa capuche.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|À la porte, Amir suspend son manteau.
+narrateur|Une goutte glisse encore de la capuche.
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -6544,12 +6539,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Amir choisit d'abord ses bottes rouges. Une botte porte encore de la boue. Je te montre un petit coin de boue. Maman commence avec le linge. Puis Amir frotte jusqu'au bout. Elle est prête ! Le bateau rejoint le sac. Le manteau attend sur la chaise.</t>
+          <t>Amir choisit d'abord ses bottes rouges. Une botte porte encore un peu de boue. Je te montre un petit coin. Maman passe le linge, puis Amir frotte. Elle est prête ! Le bateau rejoint le sac. Le manteau attend encore sur la chaise.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Amir choisit d'abord ses bottes rouges. Une botte porte encore de la boue. Je te montre un petit coin de boue. Maman commence avec le linge. Puis Amir frotte jusqu'au bout. Elle est prête ! Le bateau rejoint le sac. Le manteau attend sur la chaise.</t>
+          <t>Amir choisit d'abord ses bottes rouges. Une botte porte encore un peu de boue. Je te montre un petit coin. Maman passe le linge, puis Amir frotte. Elle est prête ! Le bateau rejoint le sac. Le manteau attend encore sur la chaise.</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -6685,13 +6680,12 @@
       <c r="AW32" t="inlineStr">
         <is>
           <t>narrateur|Amir choisit d'abord ses bottes rouges.
-narrateur|Une botte porte encore de la boue.
-maman|Je te montre un petit coin de boue.
-narrateur|Maman commence avec le linge.
-narrateur|Puis Amir frotte jusqu'au bout.
+narrateur|Une botte porte encore un peu de boue.
+maman|Je te montre un petit coin.
+narrateur|Maman passe le linge, puis Amir frotte.
 enfant-m|Elle est prête !
 narrateur|Le bateau rejoint le sac.
-narrateur|Le manteau attend sur la chaise.</t>
+narrateur|Le manteau attend encore sur la chaise.</t>
         </is>
       </c>
     </row>
@@ -6905,12 +6899,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>La semelle rouge est propre. Amir enfile les deux bottes. Et le manteau, capitaine ? Fermé jusqu'en haut !</t>
+          <t>La semelle rouge est propre, enfin. Amir enfile les deux bottes. Et le manteau, capitaine ? Fermé jusqu'en haut !</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>La semelle rouge est propre. Amir enfile les deux bottes. Et le manteau, capitaine ? Fermé jusqu'en haut !</t>
+          <t>La semelle rouge est propre, enfin. Amir enfile les deux bottes. Et le manteau, capitaine ? Fermé jusqu'en haut !</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -7049,7 +7043,7 @@
       </c>
       <c r="AW34" t="inlineStr">
         <is>
-          <t>narrateur|La semelle rouge est propre.
+          <t>narrateur|La semelle rouge est propre, enfin.
 narrateur|Amir enfile les deux bottes.
 papa|Et le manteau, capitaine ?
 enfant-m|Fermé jusqu'en haut !</t>
@@ -7079,12 +7073,12 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Dehors, trois chemins brillent encore. La rivière de la gouttière. Le port caché entre les choux. Puis l'île devant le bac. Quelle route choisis-tu, capitaine ?</t>
+          <t>Dehors, l'eau brille encore un peu. Un chemin part de la gouttière. Un autre se cache entre les choux. Le bac a l'air d'une petite île. Quelle route choisis-tu, capitaine ?</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Dehors, trois chemins brillent encore. La rivière de la gouttière. Le port caché entre les choux. Puis l'île devant le bac. Quelle route choisis-tu, capitaine ?</t>
+          <t>Dehors, l'eau brille encore un peu. Un chemin part de la gouttière. Un autre se cache entre les choux. Le bac a l'air d'une petite île. Quelle route choisis-tu, capitaine ?</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -7243,10 +7237,10 @@
       <c r="AV35" s="2" t="inlineStr"/>
       <c r="AW35" t="inlineStr">
         <is>
-          <t>narrateur|Dehors, trois chemins brillent encore.
-narrateur|La rivière de la gouttière.
-narrateur|Le port caché entre les choux.
-narrateur|Puis l'île devant le bac.
+          <t>narrateur|Dehors, l'eau brille encore un peu.
+narrateur|Un chemin part de la gouttière.
+narrateur|Un autre se cache entre les choux.
+narrateur|Le bac a l'air d'une petite île.
 papa|Quelle route choisis-tu, capitaine ?</t>
         </is>
       </c>
@@ -7274,12 +7268,12 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Ses bottes font floc sous la gouttière. Une rigole court sous la gouttière. Amir pose le bateau sur l'eau. Le voyage commence enfin. Soudain, une grande feuille tourne. Elle bouche toute la rivière. Le bateau s'arrête derrière elle. Vite, le soleil revient ! L'eau baisse déjà.</t>
+          <t>Ses bottes font floc sous la gouttière. Une rigole court encore sous la gouttière. Amir pose le bateau sur l'eau, tout doux. Le voyage commence, enfin. Soudain, une grande feuille tourne et bouche tout. Le bateau s'arrête juste derrière. Vite, le soleil revient ! L'eau baisse déjà.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Ses bottes font floc sous la gouttière. Une rigole court sous la gouttière. Amir pose le bateau sur l'eau. Le voyage commence enfin. Soudain, une grande feuille tourne. Elle bouche toute la rivière. Le bateau s'arrête derrière elle. Vite, le soleil revient ! L'eau baisse déjà.</t>
+          <t>Ses bottes font floc sous la gouttière. Une rigole court encore sous la gouttière. Amir pose le bateau sur l'eau, tout doux. Le voyage commence, enfin. Soudain, une grande feuille tourne et bouche tout. Le bateau s'arrête juste derrière. Vite, le soleil revient ! L'eau baisse déjà.</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -7415,12 +7409,11 @@
       <c r="AW36" t="inlineStr">
         <is>
           <t>narrateur|Ses bottes font floc sous la gouttière.
-narrateur|Une rigole court sous la gouttière.
-narrateur|Amir pose le bateau sur l'eau.
-narrateur|Le voyage commence enfin.
-narrateur|Soudain, une grande feuille tourne.
-narrateur|Elle bouche toute la rivière.
-narrateur|Le bateau s'arrête derrière elle.
+narrateur|Une rigole court encore sous la gouttière.
+narrateur|Amir pose le bateau sur l'eau, tout doux.
+narrateur|Le voyage commence, enfin.
+narrateur|Soudain, une grande feuille tourne et bouche tout.
+narrateur|Le bateau s'arrête juste derrière.
 enfant-m|Vite, le soleil revient !
 papa|L'eau baisse déjà.</t>
         </is>
@@ -7449,12 +7442,12 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>La feuille tient bon. L'eau devient moins profonde. Que tente le capitaine ?</t>
+          <t>La feuille tient bon, et l'eau baisse. Que tente le capitaine ?</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>La feuille tient bon. L'eau devient moins profonde. Que tente le capitaine ?</t>
+          <t>La feuille tient bon, et l'eau baisse. Que tente le capitaine ?</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -7613,8 +7606,7 @@
       <c r="AV37" s="2" t="inlineStr"/>
       <c r="AW37" t="inlineStr">
         <is>
-          <t>narrateur|La feuille tient bon.
-narrateur|L'eau devient moins profonde.
+          <t>narrateur|La feuille tient bon, et l'eau baisse.
 papa|Que tente le capitaine ?</t>
         </is>
       </c>
@@ -7642,12 +7634,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>J'attends trois gouttes. La première frappe la feuille. La deuxième soulève son bord. La troisième la fait pivoter. Un passage étroit apparaît. Maintenant, petit bateau ! Le bateau file sous une brindille.</t>
+          <t>J'attends trois gouttes. Une goutte frappe la feuille. Puis une autre soulève le bord. La dernière la fait pivoter. Un passage étroit apparaît. Maintenant, petit bateau ! Le bateau file sous une brindille.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>J'attends trois gouttes. La première frappe la feuille. La deuxième soulève son bord. La troisième la fait pivoter. Un passage étroit apparaît. Maintenant, petit bateau ! Le bateau file sous une brindille.</t>
+          <t>J'attends trois gouttes. Une goutte frappe la feuille. Puis une autre soulève le bord. La dernière la fait pivoter. Un passage étroit apparaît. Maintenant, petit bateau ! Le bateau file sous une brindille.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -7783,9 +7775,9 @@
       <c r="AW38" t="inlineStr">
         <is>
           <t>enfant-m|J'attends trois gouttes.
-narrateur|La première frappe la feuille.
-narrateur|La deuxième soulève son bord.
-narrateur|La troisième la fait pivoter.
+narrateur|Une goutte frappe la feuille.
+narrateur|Puis une autre soulève le bord.
+narrateur|La dernière la fait pivoter.
 narrateur|Un passage étroit apparaît.
 enfant-m|Maintenant, petit bateau !
 narrateur|Le bateau file sous une brindille.</t>
@@ -7815,12 +7807,12 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Le bateau atteint le pot violet. Une petite feuille colle devant. Amir la garde comme drapeau. Puis il rentre avant la dernière goutte. Quel trésor rapporte votre navire ? Un drapeau gagné après trois gouttes. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau atteint le pot violet. Une petite feuille colle devant. Amir la garde comme drapeau. Puis il rentre avant la dernière goutte. Quel trésor rapporte votre navire ? Un drapeau gagné après trois gouttes. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Le bateau atteint le pot violet. Une petite feuille colle devant. Amir la garde comme drapeau. Puis il rentre avant la dernière goutte. Quel trésor rapporte votre navire ? Un drapeau gagné après trois gouttes. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau atteint le pot violet. Une petite feuille colle devant. Amir la garde comme drapeau. Puis il rentre avant la dernière goutte. Quel trésor rapporte votre navire ? Un drapeau gagné après trois gouttes. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -7963,8 +7955,8 @@
 enfant-m|Un drapeau gagné après trois gouttes.
 narrateur|À la porte, Amir retire ses bottes.
 narrateur|Deux traces rouges restent sur le tapis.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -8163,12 +8155,12 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Le bateau traverse la rivière délivrée. Une ligne brillante marque sa coque. Amir la montre en rentrant. Nous avons formé un bon équipage. Moi devant, et toi derrière ! À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau traverse la rivière délivrée. Une ligne brillante marque sa coque. Amir la montre en rentrant. Nous avons formé un bon équipage. Moi devant, et toi derrière ! À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Le bateau traverse la rivière délivrée. Une ligne brillante marque sa coque. Amir la montre en rentrant. Nous avons formé un bon équipage. Moi devant, et toi derrière ! À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau traverse la rivière délivrée. Une ligne brillante marque sa coque. Amir la montre en rentrant. Nous avons formé un bon équipage. Moi devant, et toi derrière ! À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -8310,8 +8302,8 @@
 enfant-m|Moi devant, et toi derrière !
 narrateur|À la porte, Amir retire ses bottes.
 narrateur|Deux traces rouges restent sur le tapis.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -8510,12 +8502,12 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Le courant dépose une brindille sur la voile. Amir rapporte le bateau ainsi décoré. Je reconnais le passage secret. Il commence derrière le grand pot. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le courant dépose une brindille sur la voile. Amir rapporte le bateau ainsi décoré. Je reconnais le passage secret. Il commence derrière le grand pot. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Le courant dépose une brindille sur la voile. Amir rapporte le bateau ainsi décoré. Je reconnais le passage secret. Il commence derrière le grand pot. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le courant dépose une brindille sur la voile. Amir rapporte le bateau ainsi décoré. Je reconnais le passage secret. Il commence derrière le grand pot. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -8656,8 +8648,8 @@
 enfant-m|Il commence derrière le grand pot.
 narrateur|À la porte, Amir retire ses bottes.
 narrateur|Deux traces rouges restent sur le tapis.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -8684,12 +8676,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Ses bottes traversent la terre molle. Entre les choux se cache un port. Trois feuilles flottent devant l'entrée. Le bateau avance vers elles. La première touche sa voile. La deuxième ferme le passage. La troisième frôle un jeune chou. Je ne veux rien abîmer. Amir retient aussitôt son bateau.</t>
+          <t>Ses bottes traversent la terre molle. Entre les choux se cache un petit port. Trois feuilles flottent devant l'entrée. Le bateau avance, tout doucement. L'une touche sa voile. Une autre ferme le passage. La dernière frôle un jeune chou. Je ne veux rien abîmer. Amir retient aussitôt son bateau.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Ses bottes traversent la terre molle. Entre les choux se cache un port. Trois feuilles flottent devant l'entrée. Le bateau avance vers elles. La première touche sa voile. La deuxième ferme le passage. La troisième frôle un jeune chou. Je ne veux rien abîmer. Amir retient aussitôt son bateau.</t>
+          <t>Ses bottes traversent la terre molle. Entre les choux se cache un petit port. Trois feuilles flottent devant l'entrée. Le bateau avance, tout doucement. L'une touche sa voile. Une autre ferme le passage. La dernière frôle un jeune chou. Je ne veux rien abîmer. Amir retient aussitôt son bateau.</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -8825,12 +8817,12 @@
       <c r="AW44" t="inlineStr">
         <is>
           <t>narrateur|Ses bottes traversent la terre molle.
-narrateur|Entre les choux se cache un port.
+narrateur|Entre les choux se cache un petit port.
 narrateur|Trois feuilles flottent devant l'entrée.
-narrateur|Le bateau avance vers elles.
-narrateur|La première touche sa voile.
-narrateur|La deuxième ferme le passage.
-narrateur|La troisième frôle un jeune chou.
+narrateur|Le bateau avance, tout doucement.
+narrateur|L'une touche sa voile.
+narrateur|Une autre ferme le passage.
+narrateur|La dernière frôle un jeune chou.
 enfant-m|Je ne veux rien abîmer.
 narrateur|Amir retient aussitôt son bateau.</t>
         </is>
@@ -9224,12 +9216,12 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Au quai, une feuille devient drapeau. Amir la plante dans le sable humide. Les trois choux restent bien droits. À table, Amir dessine son port. Quel passage as-tu choisi ? Celui entre deux et trois. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Au quai, une feuille devient drapeau. Amir la plante dans le sable humide. Les trois choux restent bien droits. À table, Amir dessine son port. Quel passage as-tu choisi ? Celui entre deux et trois. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Au quai, une feuille devient drapeau. Amir la plante dans le sable humide. Les trois choux restent bien droits. À table, Amir dessine son port. Quel passage as-tu choisi ? Celui entre deux et trois. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Au quai, une feuille devient drapeau. Amir la plante dans le sable humide. Les trois choux restent bien droits. À table, Amir dessine son port. Quel passage as-tu choisi ? Celui entre deux et trois. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -9372,8 +9364,8 @@
 enfant-m|Celui entre deux et trois.
 narrateur|À la porte, Amir retire ses bottes.
 narrateur|Deux traces rouges restent sur le tapis.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -9400,12 +9392,12 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>J'attends le prochain courant. Amir garde le bateau contre sa botte. L'eau pousse lentement la première feuille. Puis la seconde s'écarte aussi. Le port s'ouvre juste assez. Le bateau glisse jusqu'au quai.</t>
+          <t>J'attends le prochain courant. Amir garde le bateau contre sa botte. L'eau pousse lentement une feuille. Puis une autre s'écarte aussi. Le port s'ouvre juste assez. Le bateau glisse jusqu'au quai.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>J'attends le prochain courant. Amir garde le bateau contre sa botte. L'eau pousse lentement la première feuille. Puis la seconde s'écarte aussi. Le port s'ouvre juste assez. Le bateau glisse jusqu'au quai.</t>
+          <t>J'attends le prochain courant. Amir garde le bateau contre sa botte. L'eau pousse lentement une feuille. Puis une autre s'écarte aussi. Le port s'ouvre juste assez. Le bateau glisse jusqu'au quai.</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -9542,8 +9534,8 @@
         <is>
           <t>enfant-m|J'attends le prochain courant.
 narrateur|Amir garde le bateau contre sa botte.
-narrateur|L'eau pousse lentement la première feuille.
-narrateur|Puis la seconde s'écarte aussi.
+narrateur|L'eau pousse lentement une feuille.
+narrateur|Puis une autre s'écarte aussi.
 narrateur|Le port s'ouvre juste assez.
 narrateur|Le bateau glisse jusqu'au quai.</t>
         </is>
@@ -9572,12 +9564,12 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Le bateau touche enfin le quai de terre. Une odeur de chou monte de sa coque. Amir éclate de rire en rentrant. Ton trésor sent vraiment le potager ! C'est le parfum de mon port. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau touche enfin le quai de terre. Une odeur de chou monte de sa coque. Amir éclate de rire en rentrant. Ton trésor sent vraiment le potager ! C'est le parfum de mon port. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Le bateau touche enfin le quai de terre. Une odeur de chou monte de sa coque. Amir éclate de rire en rentrant. Ton trésor sent vraiment le potager ! C'est le parfum de mon port. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau touche enfin le quai de terre. Une odeur de chou monte de sa coque. Amir éclate de rire en rentrant. Ton trésor sent vraiment le potager ! C'est le parfum de mon port. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -9719,8 +9711,8 @@
 enfant-m|C'est le parfum de mon port.
 narrateur|À la porte, Amir retire ses bottes.
 narrateur|Deux traces rouges restent sur le tapis.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -9919,12 +9911,12 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>La rigole conduit le bateau au thym. Une minuscule fleur touche sa voile. Amir rentre avec son bateau parfumé. Tu as trouvé sans écraser mes choux. La route passait près du thym. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>La rigole conduit le bateau au thym. Une minuscule fleur touche sa voile. Amir rentre avec son bateau parfumé. Tu as trouvé sans écraser mes choux. La route passait près du thym. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>La rigole conduit le bateau au thym. Une minuscule fleur touche sa voile. Amir rentre avec son bateau parfumé. Tu as trouvé sans écraser mes choux. La route passait près du thym. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>La rigole conduit le bateau au thym. Une minuscule fleur touche sa voile. Amir rentre avec son bateau parfumé. Tu as trouvé sans écraser mes choux. La route passait près du thym. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -10066,8 +10058,8 @@
 enfant-m|La route passait près du thym.
 narrateur|À la porte, Amir retire ses bottes.
 narrateur|Deux traces rouges restent sur le tapis.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -10634,12 +10626,12 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Le galet gris devient le nouveau trésor. Amir le laisse près de la flaque. Il rapporte seulement son histoire. L'île a changé, mais le voyage continue. Demain, je chercherai encore. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le galet gris devient le nouveau trésor. Amir le laisse près de la flaque. Il rapporte seulement son histoire. L'île a changé, mais le voyage continue. Demain, je chercherai encore. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Le galet gris devient le nouveau trésor. Amir le laisse près de la flaque. Il rapporte seulement son histoire. L'île a changé, mais le voyage continue. Demain, je chercherai encore. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le galet gris devient le nouveau trésor. Amir le laisse près de la flaque. Il rapporte seulement son histoire. L'île a changé, mais le voyage continue. Demain, je chercherai encore. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -10781,8 +10773,8 @@
 enfant-m|Demain, je chercherai encore.
 narrateur|À la porte, Amir retire ses bottes.
 narrateur|Deux traces rouges restent sur le tapis.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -10981,12 +10973,12 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Le bateau atteint enfin le caillou blanc. Son reflet danse dans le petit canal. Puis l'eau disparaît doucement dans le sable. J'ai vu mon île revenir. Juste assez longtemps pour ton voyage. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau atteint enfin le caillou blanc. Son reflet danse dans le petit canal. Puis l'eau disparaît doucement dans le sable. J'ai vu mon île revenir. Juste assez longtemps pour ton voyage. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Le bateau atteint enfin le caillou blanc. Son reflet danse dans le petit canal. Puis l'eau disparaît doucement dans le sable. J'ai vu mon île revenir. Juste assez longtemps pour ton voyage. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau atteint enfin le caillou blanc. Son reflet danse dans le petit canal. Puis l'eau disparaît doucement dans le sable. J'ai vu mon île revenir. Juste assez longtemps pour ton voyage. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -11128,8 +11120,8 @@
 papa|Juste assez longtemps pour ton voyage.
 narrateur|À la porte, Amir retire ses bottes.
 narrateur|Deux traces rouges restent sur le tapis.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -11328,12 +11320,12 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Le devant touche doucement le caillou blanc. Un grain doré reste sur la coque. Amir le montre à papa en rentrant. Un vrai trésor de capitaine. Mon bateau connaît aussi les routes. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le devant touche doucement le caillou blanc. Un grain doré reste sur la coque. Amir le montre à papa en rentrant. Un vrai trésor de capitaine. Mon bateau connaît aussi les routes. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Le devant touche doucement le caillou blanc. Un grain doré reste sur la coque. Amir le montre à papa en rentrant. Un vrai trésor de capitaine. Mon bateau connaît aussi les routes. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le devant touche doucement le caillou blanc. Un grain doré reste sur la coque. Amir le montre à papa en rentrant. Un vrai trésor de capitaine. Mon bateau connaît aussi les routes. À la porte, Amir retire ses bottes. Deux traces rouges restent sur le tapis. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -11475,8 +11467,8 @@
 enfant-m|Mon bateau connaît aussi les routes.
 narrateur|À la porte, Amir retire ses bottes.
 narrateur|Deux traces rouges restent sur le tapis.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -11503,12 +11495,12 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Amir choisit d'abord le petit linge bleu. Il est encore chaud du radiateur. À quoi servira-t-il ? À sauver mon bateau mouillé. Amir le roule comme un petit coussin. Le bateau se pose dessus. Le manteau et les bottes sont prêts.</t>
+          <t>Amir prend d'abord le petit linge bleu. Il est encore chaud du radiateur. À quoi servira-t-il ? À sauver mon bateau mouillé. Il le roule comme un petit coussin. Le bateau se pose dessus, dans le sac. Le manteau et les bottes sont déjà prêts.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Amir choisit d'abord le petit linge bleu. Il est encore chaud du radiateur. À quoi servira-t-il ? À sauver mon bateau mouillé. Amir le roule comme un petit coussin. Le bateau se pose dessus. Le manteau et les bottes sont prêts.</t>
+          <t>Amir prend d'abord le petit linge bleu. Il est encore chaud du radiateur. À quoi servira-t-il ? À sauver mon bateau mouillé. Il le roule comme un petit coussin. Le bateau se pose dessus, dans le sac. Le manteau et les bottes sont déjà prêts.</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -11643,13 +11635,13 @@
       <c r="AV60" s="2" t="inlineStr"/>
       <c r="AW60" t="inlineStr">
         <is>
-          <t>narrateur|Amir choisit d'abord le petit linge bleu.
+          <t>narrateur|Amir prend d'abord le petit linge bleu.
 narrateur|Il est encore chaud du radiateur.
 maman|À quoi servira-t-il ?
 enfant-m|À sauver mon bateau mouillé.
-narrateur|Amir le roule comme un petit coussin.
-narrateur|Le bateau se pose dessus.
-narrateur|Le manteau et les bottes sont prêts.</t>
+narrateur|Il le roule comme un petit coussin.
+narrateur|Le bateau se pose dessus, dans le sac.
+narrateur|Le manteau et les bottes sont déjà prêts.</t>
         </is>
       </c>
     </row>
@@ -12037,12 +12029,12 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Dehors, trois chemins brillent encore. La rivière de la gouttière. Le port caché entre les choux. Puis l'île devant le bac. Quelle route choisis-tu, capitaine ?</t>
+          <t>Dehors, l'eau brille encore un peu. Un chemin part de la gouttière. Un autre se cache entre les choux. Le bac a l'air d'une petite île. Quelle route choisis-tu, capitaine ?</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Dehors, trois chemins brillent encore. La rivière de la gouttière. Le port caché entre les choux. Puis l'île devant le bac. Quelle route choisis-tu, capitaine ?</t>
+          <t>Dehors, l'eau brille encore un peu. Un chemin part de la gouttière. Un autre se cache entre les choux. Le bac a l'air d'une petite île. Quelle route choisis-tu, capitaine ?</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -12201,10 +12193,10 @@
       <c r="AV63" s="2" t="inlineStr"/>
       <c r="AW63" t="inlineStr">
         <is>
-          <t>narrateur|Dehors, trois chemins brillent encore.
-narrateur|La rivière de la gouttière.
-narrateur|Le port caché entre les choux.
-narrateur|Puis l'île devant le bac.
+          <t>narrateur|Dehors, l'eau brille encore un peu.
+narrateur|Un chemin part de la gouttière.
+narrateur|Un autre se cache entre les choux.
+narrateur|Le bac a l'air d'une petite île.
 papa|Quelle route choisis-tu, capitaine ?</t>
         </is>
       </c>
@@ -12232,12 +12224,12 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Le linge bleu attend dans le sac. Une rigole court sous la gouttière. Amir pose le bateau sur l'eau. Le voyage commence enfin. Soudain, une grande feuille tourne. Elle bouche toute la rivière. Le bateau s'arrête derrière elle. Vite, le soleil revient ! L'eau baisse déjà.</t>
+          <t>Le linge bleu attend dans le sac. Une rigole court encore sous la gouttière. Amir pose le bateau sur l'eau, tout doux. Le voyage commence, enfin. Soudain, une grande feuille tourne et bouche tout. Le bateau s'arrête juste derrière. Vite, le soleil revient ! L'eau baisse déjà.</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Le linge bleu attend dans le sac. Une rigole court sous la gouttière. Amir pose le bateau sur l'eau. Le voyage commence enfin. Soudain, une grande feuille tourne. Elle bouche toute la rivière. Le bateau s'arrête derrière elle. Vite, le soleil revient ! L'eau baisse déjà.</t>
+          <t>Le linge bleu attend dans le sac. Une rigole court encore sous la gouttière. Amir pose le bateau sur l'eau, tout doux. Le voyage commence, enfin. Soudain, une grande feuille tourne et bouche tout. Le bateau s'arrête juste derrière. Vite, le soleil revient ! L'eau baisse déjà.</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -12373,12 +12365,11 @@
       <c r="AW64" t="inlineStr">
         <is>
           <t>narrateur|Le linge bleu attend dans le sac.
-narrateur|Une rigole court sous la gouttière.
-narrateur|Amir pose le bateau sur l'eau.
-narrateur|Le voyage commence enfin.
-narrateur|Soudain, une grande feuille tourne.
-narrateur|Elle bouche toute la rivière.
-narrateur|Le bateau s'arrête derrière elle.
+narrateur|Une rigole court encore sous la gouttière.
+narrateur|Amir pose le bateau sur l'eau, tout doux.
+narrateur|Le voyage commence, enfin.
+narrateur|Soudain, une grande feuille tourne et bouche tout.
+narrateur|Le bateau s'arrête juste derrière.
 enfant-m|Vite, le soleil revient !
 papa|L'eau baisse déjà.</t>
         </is>
@@ -12407,12 +12398,12 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>La feuille tient bon. L'eau devient moins profonde. Que tente le capitaine ?</t>
+          <t>La feuille tient bon, et l'eau baisse. Que tente le capitaine ?</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>La feuille tient bon. L'eau devient moins profonde. Que tente le capitaine ?</t>
+          <t>La feuille tient bon, et l'eau baisse. Que tente le capitaine ?</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -12571,8 +12562,7 @@
       <c r="AV65" s="2" t="inlineStr"/>
       <c r="AW65" t="inlineStr">
         <is>
-          <t>narrateur|La feuille tient bon.
-narrateur|L'eau devient moins profonde.
+          <t>narrateur|La feuille tient bon, et l'eau baisse.
 papa|Que tente le capitaine ?</t>
         </is>
       </c>
@@ -12600,12 +12590,12 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>J'attends trois gouttes. La première frappe la feuille. La deuxième soulève son bord. La troisième la fait pivoter. Un passage étroit apparaît. Maintenant, petit bateau ! Le bateau file sous une brindille.</t>
+          <t>J'attends trois gouttes. Une goutte frappe la feuille. Puis une autre soulève le bord. La dernière la fait pivoter. Un passage étroit apparaît. Maintenant, petit bateau ! Le bateau file sous une brindille.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>J'attends trois gouttes. La première frappe la feuille. La deuxième soulève son bord. La troisième la fait pivoter. Un passage étroit apparaît. Maintenant, petit bateau ! Le bateau file sous une brindille.</t>
+          <t>J'attends trois gouttes. Une goutte frappe la feuille. Puis une autre soulève le bord. La dernière la fait pivoter. Un passage étroit apparaît. Maintenant, petit bateau ! Le bateau file sous une brindille.</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -12741,9 +12731,9 @@
       <c r="AW66" t="inlineStr">
         <is>
           <t>enfant-m|J'attends trois gouttes.
-narrateur|La première frappe la feuille.
-narrateur|La deuxième soulève son bord.
-narrateur|La troisième la fait pivoter.
+narrateur|Une goutte frappe la feuille.
+narrateur|Puis une autre soulève le bord.
+narrateur|La dernière la fait pivoter.
 narrateur|Un passage étroit apparaît.
 enfant-m|Maintenant, petit bateau !
 narrateur|Le bateau file sous une brindille.</t>
@@ -12773,12 +12763,12 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Le bateau atteint le pot violet. Une petite feuille colle devant. Amir la garde comme drapeau. Puis il rentre avant la dernière goutte. Quel trésor rapporte votre navire ? Un drapeau gagné après trois gouttes. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau atteint le pot violet. Une petite feuille colle devant. Amir la garde comme drapeau. Puis il rentre avant la dernière goutte. Quel trésor rapporte votre navire ? Un drapeau gagné après trois gouttes. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Le bateau atteint le pot violet. Une petite feuille colle devant. Amir la garde comme drapeau. Puis il rentre avant la dernière goutte. Quel trésor rapporte votre navire ? Un drapeau gagné après trois gouttes. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau atteint le pot violet. Une petite feuille colle devant. Amir la garde comme drapeau. Puis il rentre avant la dernière goutte. Quel trésor rapporte votre navire ? Un drapeau gagné après trois gouttes. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -12921,8 +12911,8 @@
 enfant-m|Un drapeau gagné après trois gouttes.
 narrateur|Amir enveloppe le bateau dans le linge.
 narrateur|Une tache humide dessine une petite île.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -13121,12 +13111,12 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Le bateau traverse la rivière délivrée. Une ligne brillante marque sa coque. Amir la montre en rentrant. Nous avons formé un bon équipage. Moi devant, et toi derrière ! Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau traverse la rivière délivrée. Une ligne brillante marque sa coque. Amir la montre en rentrant. Nous avons formé un bon équipage. Moi devant, et toi derrière ! Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Le bateau traverse la rivière délivrée. Une ligne brillante marque sa coque. Amir la montre en rentrant. Nous avons formé un bon équipage. Moi devant, et toi derrière ! Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau traverse la rivière délivrée. Une ligne brillante marque sa coque. Amir la montre en rentrant. Nous avons formé un bon équipage. Moi devant, et toi derrière ! Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -13268,8 +13258,8 @@
 enfant-m|Moi devant, et toi derrière !
 narrateur|Amir enveloppe le bateau dans le linge.
 narrateur|Une tache humide dessine une petite île.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -13468,12 +13458,12 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Le courant dépose une brindille sur la voile. Amir rapporte le bateau ainsi décoré. Je reconnais le passage secret. Il commence derrière le grand pot. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le courant dépose une brindille sur la voile. Amir rapporte le bateau ainsi décoré. Je reconnais le passage secret. Il commence derrière le grand pot. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Le courant dépose une brindille sur la voile. Amir rapporte le bateau ainsi décoré. Je reconnais le passage secret. Il commence derrière le grand pot. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le courant dépose une brindille sur la voile. Amir rapporte le bateau ainsi décoré. Je reconnais le passage secret. Il commence derrière le grand pot. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -13614,8 +13604,8 @@
 enfant-m|Il commence derrière le grand pot.
 narrateur|Amir enveloppe le bateau dans le linge.
 narrateur|Une tache humide dessine une petite île.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -13642,12 +13632,12 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Le linge garde encore un peu de chaleur. Entre les choux se cache un port. Trois feuilles flottent devant l'entrée. Le bateau avance vers elles. La première touche sa voile. La deuxième ferme le passage. La troisième frôle un jeune chou. Je ne veux rien abîmer. Amir retient aussitôt son bateau.</t>
+          <t>Le linge garde encore un peu de chaleur. Entre les choux se cache un petit port. Trois feuilles flottent devant l'entrée. Le bateau avance, tout doucement. L'une touche sa voile. Une autre ferme le passage. La dernière frôle un jeune chou. Je ne veux rien abîmer. Amir retient aussitôt son bateau.</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Le linge garde encore un peu de chaleur. Entre les choux se cache un port. Trois feuilles flottent devant l'entrée. Le bateau avance vers elles. La première touche sa voile. La deuxième ferme le passage. La troisième frôle un jeune chou. Je ne veux rien abîmer. Amir retient aussitôt son bateau.</t>
+          <t>Le linge garde encore un peu de chaleur. Entre les choux se cache un petit port. Trois feuilles flottent devant l'entrée. Le bateau avance, tout doucement. L'une touche sa voile. Une autre ferme le passage. La dernière frôle un jeune chou. Je ne veux rien abîmer. Amir retient aussitôt son bateau.</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -13783,12 +13773,12 @@
       <c r="AW72" t="inlineStr">
         <is>
           <t>narrateur|Le linge garde encore un peu de chaleur.
-narrateur|Entre les choux se cache un port.
+narrateur|Entre les choux se cache un petit port.
 narrateur|Trois feuilles flottent devant l'entrée.
-narrateur|Le bateau avance vers elles.
-narrateur|La première touche sa voile.
-narrateur|La deuxième ferme le passage.
-narrateur|La troisième frôle un jeune chou.
+narrateur|Le bateau avance, tout doucement.
+narrateur|L'une touche sa voile.
+narrateur|Une autre ferme le passage.
+narrateur|La dernière frôle un jeune chou.
 enfant-m|Je ne veux rien abîmer.
 narrateur|Amir retient aussitôt son bateau.</t>
         </is>
@@ -14182,12 +14172,12 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Au quai, une feuille devient drapeau. Amir la plante dans le sable humide. Les trois choux restent bien droits. À table, Amir dessine son port. Quel passage as-tu choisi ? Celui entre deux et trois. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Au quai, une feuille devient drapeau. Amir la plante dans le sable humide. Les trois choux restent bien droits. À table, Amir dessine son port. Quel passage as-tu choisi ? Celui entre deux et trois. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Au quai, une feuille devient drapeau. Amir la plante dans le sable humide. Les trois choux restent bien droits. À table, Amir dessine son port. Quel passage as-tu choisi ? Celui entre deux et trois. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Au quai, une feuille devient drapeau. Amir la plante dans le sable humide. Les trois choux restent bien droits. À table, Amir dessine son port. Quel passage as-tu choisi ? Celui entre deux et trois. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -14330,8 +14320,8 @@
 enfant-m|Celui entre deux et trois.
 narrateur|Amir enveloppe le bateau dans le linge.
 narrateur|Une tache humide dessine une petite île.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -14358,12 +14348,12 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>J'attends le prochain courant. Amir garde le bateau contre sa botte. L'eau pousse lentement la première feuille. Puis la seconde s'écarte aussi. Le port s'ouvre juste assez. Le bateau glisse jusqu'au quai.</t>
+          <t>J'attends le prochain courant. Amir garde le bateau contre sa botte. L'eau pousse lentement une feuille. Puis une autre s'écarte aussi. Le port s'ouvre juste assez. Le bateau glisse jusqu'au quai.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>J'attends le prochain courant. Amir garde le bateau contre sa botte. L'eau pousse lentement la première feuille. Puis la seconde s'écarte aussi. Le port s'ouvre juste assez. Le bateau glisse jusqu'au quai.</t>
+          <t>J'attends le prochain courant. Amir garde le bateau contre sa botte. L'eau pousse lentement une feuille. Puis une autre s'écarte aussi. Le port s'ouvre juste assez. Le bateau glisse jusqu'au quai.</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -14500,8 +14490,8 @@
         <is>
           <t>enfant-m|J'attends le prochain courant.
 narrateur|Amir garde le bateau contre sa botte.
-narrateur|L'eau pousse lentement la première feuille.
-narrateur|Puis la seconde s'écarte aussi.
+narrateur|L'eau pousse lentement une feuille.
+narrateur|Puis une autre s'écarte aussi.
 narrateur|Le port s'ouvre juste assez.
 narrateur|Le bateau glisse jusqu'au quai.</t>
         </is>
@@ -14530,12 +14520,12 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Le bateau touche enfin le quai de terre. Une odeur de chou monte de sa coque. Amir éclate de rire en rentrant. Ton trésor sent vraiment le potager ! C'est le parfum de mon port. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau touche enfin le quai de terre. Une odeur de chou monte de sa coque. Amir éclate de rire en rentrant. Ton trésor sent vraiment le potager ! C'est le parfum de mon port. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Le bateau touche enfin le quai de terre. Une odeur de chou monte de sa coque. Amir éclate de rire en rentrant. Ton trésor sent vraiment le potager ! C'est le parfum de mon port. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau touche enfin le quai de terre. Une odeur de chou monte de sa coque. Amir éclate de rire en rentrant. Ton trésor sent vraiment le potager ! C'est le parfum de mon port. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -14677,8 +14667,8 @@
 enfant-m|C'est le parfum de mon port.
 narrateur|Amir enveloppe le bateau dans le linge.
 narrateur|Une tache humide dessine une petite île.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -14877,12 +14867,12 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>La rigole conduit le bateau au thym. Une minuscule fleur touche sa voile. Amir rentre avec son bateau parfumé. Tu as trouvé sans écraser mes choux. La route passait près du thym. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>La rigole conduit le bateau au thym. Une minuscule fleur touche sa voile. Amir rentre avec son bateau parfumé. Tu as trouvé sans écraser mes choux. La route passait près du thym. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>La rigole conduit le bateau au thym. Une minuscule fleur touche sa voile. Amir rentre avec son bateau parfumé. Tu as trouvé sans écraser mes choux. La route passait près du thym. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>La rigole conduit le bateau au thym. Une minuscule fleur touche sa voile. Amir rentre avec son bateau parfumé. Tu as trouvé sans écraser mes choux. La route passait près du thym. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -15024,8 +15014,8 @@
 enfant-m|La route passait près du thym.
 narrateur|Amir enveloppe le bateau dans le linge.
 narrateur|Une tache humide dessine une petite île.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -15592,12 +15582,12 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Le galet gris devient le nouveau trésor. Amir le laisse près de la flaque. Il rapporte seulement son histoire. L'île a changé, mais le voyage continue. Demain, je chercherai encore. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le galet gris devient le nouveau trésor. Amir le laisse près de la flaque. Il rapporte seulement son histoire. L'île a changé, mais le voyage continue. Demain, je chercherai encore. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Le galet gris devient le nouveau trésor. Amir le laisse près de la flaque. Il rapporte seulement son histoire. L'île a changé, mais le voyage continue. Demain, je chercherai encore. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le galet gris devient le nouveau trésor. Amir le laisse près de la flaque. Il rapporte seulement son histoire. L'île a changé, mais le voyage continue. Demain, je chercherai encore. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -15739,8 +15729,8 @@
 enfant-m|Demain, je chercherai encore.
 narrateur|Amir enveloppe le bateau dans le linge.
 narrateur|Une tache humide dessine une petite île.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -15939,12 +15929,12 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Le bateau atteint enfin le caillou blanc. Son reflet danse dans le petit canal. Puis l'eau disparaît doucement dans le sable. J'ai vu mon île revenir. Juste assez longtemps pour ton voyage. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau atteint enfin le caillou blanc. Son reflet danse dans le petit canal. Puis l'eau disparaît doucement dans le sable. J'ai vu mon île revenir. Juste assez longtemps pour ton voyage. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Le bateau atteint enfin le caillou blanc. Son reflet danse dans le petit canal. Puis l'eau disparaît doucement dans le sable. J'ai vu mon île revenir. Juste assez longtemps pour ton voyage. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le bateau atteint enfin le caillou blanc. Son reflet danse dans le petit canal. Puis l'eau disparaît doucement dans le sable. J'ai vu mon île revenir. Juste assez longtemps pour ton voyage. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -16086,8 +16076,8 @@
 papa|Juste assez longtemps pour ton voyage.
 narrateur|Amir enveloppe le bateau dans le linge.
 narrateur|Une tache humide dessine une petite île.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -16286,12 +16276,12 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Le devant touche doucement le caillou blanc. Un grain doré reste sur la coque. Amir le montre à papa en rentrant. Un vrai trésor de capitaine. Mon bateau connaît aussi les routes. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le devant touche doucement le caillou blanc. Un grain doré reste sur la coque. Amir le montre à papa en rentrant. Un vrai trésor de capitaine. Mon bateau connaît aussi les routes. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Le devant touche doucement le caillou blanc. Un grain doré reste sur la coque. Amir le montre à papa en rentrant. Un vrai trésor de capitaine. Mon bateau connaît aussi les routes. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet jaune. Dans la cuisine, la soupe est prête.</t>
+          <t>Le devant touche doucement le caillou blanc. Un grain doré reste sur la coque. Amir le montre à papa en rentrant. Un vrai trésor de capitaine. Mon bateau connaît aussi les routes. Amir enveloppe le bateau dans le linge. Une tache humide dessine une petite île. Le bateau sèche près du volet. La soupe est prête.</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -16433,8 +16423,8 @@
 enfant-m|Mon bateau connaît aussi les routes.
 narrateur|Amir enveloppe le bateau dans le linge.
 narrateur|Une tache humide dessine une petite île.
-narrateur|Le bateau sèche près du volet jaune.
-narrateur|Dans la cuisine, la soupe est prête.</t>
+narrateur|Le bateau sèche près du volet.
+maman|La soupe est prête.</t>
         </is>
       </c>
     </row>
@@ -16455,7 +16445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16559,6 +16549,13 @@
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>